<commit_message>
IAM-071 Establish Excel-driven Codex agent foundation
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,14 +29,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'API Contracts'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DB Schema + RLS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Dependencies!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Release Checklist'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Risks &amp; Decisions'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Timeline + Gantt'!$A$1:$AX$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UI Screens'!$A$1:$H$12</definedName>
   </definedNames>
@@ -5528,7 +5528,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P71"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -8953,9 +8953,83 @@
       </c>
       <c r="P71" s="5"/>
     </row>
+    <row r="72" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>IAM-071</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>Developer Automation</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Establish Excel-driven Codex agent foundation</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E72" s="5">
+        <v>3</v>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>Establish repository instructions, tracker rules, and the package location for an Excel-driven Codex task agent.</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>AGENTS.md contains the agent rules; Excel temporary files are ignored; the workbook contains IAM-071 and CODE-041; completed tasks are not selected again; no commits occur without a task ID.</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="J72" s="6">
+        <v>46230</v>
+      </c>
+      <c r="K72" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="L72" s="5">
+        <v>1</v>
+      </c>
+      <c r="M72" s="6">
+        <v>46230</v>
+      </c>
+      <c r="N72" s="5" t="inlineStr">
+        <is>
+          <t>IAM-001,IAM-003</t>
+        </is>
+      </c>
+      <c r="O72" s="5" t="inlineStr">
+        <is>
+          <t>AGENTS.md; .gitignore; planning/IAMONIT_Full_Project_Control_Workbook.xlsx</t>
+        </is>
+      </c>
+      <c r="P72" s="5" t="inlineStr">
+        <is>
+          <t>Every Git commit must begin with the exact related task ID.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P71" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="F2:F71">
+  <autoFilter ref="A1:P72" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="F2:F72">
     <cfRule type="expression" dxfId="29" priority="1">
       <formula>$F2="Done"</formula>
     </cfRule>
@@ -8973,13 +9047,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="D2:D71" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D72" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F71" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F72" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:I71" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I72" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"Frontend,Backend,Database,DevOps,QA,Product,Security"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8993,7 +9067,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -9124,7 +9198,7 @@
         <v>5</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>49</v>
@@ -11277,9 +11351,59 @@
         <v>469</v>
       </c>
     </row>
+    <row r="72" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>IAM-071</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Developer Automation</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>Establish Excel-driven Codex agent foundation</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G72" s="5">
+        <v>3</v>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>IAM-001,IAM-003</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>Repository and workbook rules for the Excel-driven Codex agent are established.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J71" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="H2:H71">
+  <autoFilter ref="A1:J72" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="H2:H72">
     <cfRule type="expression" dxfId="24" priority="1">
       <formula>$H2="Done"</formula>
     </cfRule>
@@ -11297,7 +11421,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H71" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H72" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17956,7 +18080,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19158,9 +19282,56 @@
         <v>25</v>
       </c>
     </row>
+    <row r="42" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>CODE-041</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>task-agent</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>packages/task-agent/src/cli.ts</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Create read-only workbook reader and eligible-task selector</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Use ExcelJS to read the Backlog and IntelliJ Coding Tasks sheets. Skip Done, In Progress, Blocked, and Review tasks. Select a Todo task only when all dependencies are Done. Print one selected task and stop without changing the workbook or application code.</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>IAM-071</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>The CLI identifies exactly one eligible task, respects dependencies, skips completed work, and makes no workbook changes.</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I41" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I41">
+  <autoFilter ref="A1:I42" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <conditionalFormatting sqref="I2:I42">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -19178,7 +19349,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I41" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I42" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
CODE-041 Create read-only workbook task selector
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282641C4-3D80-D446-A338-EE232088BC70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5E26DD-3880-4541-8665-AE97E29BBC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3253" uniqueCount="986">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3283" uniqueCount="1003">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3015,6 +3015,57 @@
   </si>
   <si>
     <t>User guide created</t>
+  </si>
+  <si>
+    <t>IAM-071</t>
+  </si>
+  <si>
+    <t>Developer Automation</t>
+  </si>
+  <si>
+    <t>Establish Excel-driven Codex agent foundation</t>
+  </si>
+  <si>
+    <t>Establish repository instructions, tracker rules, and the package location for an Excel-driven Codex task agent.</t>
+  </si>
+  <si>
+    <t>AGENTS.md contains the agent rules; Excel temporary files are ignored; the workbook contains IAM-071 and CODE-041; completed tasks are not selected again; no commits occur without a task ID.</t>
+  </si>
+  <si>
+    <t>Sprint 10</t>
+  </si>
+  <si>
+    <t>IAM-001,IAM-003</t>
+  </si>
+  <si>
+    <t>AGENTS.md; .gitignore; planning/IAMONIT_Full_Project_Control_Workbook.xlsx</t>
+  </si>
+  <si>
+    <t>Every Git commit must begin with the exact related task ID.</t>
+  </si>
+  <si>
+    <t>Repository and workbook rules for the Excel-driven Codex agent are established.</t>
+  </si>
+  <si>
+    <t>CODE-041</t>
+  </si>
+  <si>
+    <t>Tooling</t>
+  </si>
+  <si>
+    <t>task-agent</t>
+  </si>
+  <si>
+    <t>packages/task-agent/src/cli.ts</t>
+  </si>
+  <si>
+    <t>Create read-only workbook reader and eligible-task selector</t>
+  </si>
+  <si>
+    <t>Use ExcelJS to read the Backlog and IntelliJ Coding Tasks sheets. Skip Done, In Progress, Blocked, and Review tasks. Select a Todo task only when all dependencies are Done. Print one selected task and stop without changing the workbook or application code.</t>
+  </si>
+  <si>
+    <t>The CLI identifies exactly one eligible task, respects dependencies, skips completed work, and makes no workbook changes.</t>
   </si>
 </sst>
 </file>
@@ -3171,21 +3222,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3193,6 +3229,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3887,161 +3938,161 @@
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="4" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="8" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="12" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
     </row>
     <row r="16" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -5131,87 +5182,87 @@
       <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="D4" s="15" t="s">
+      <c r="B4" s="13"/>
+      <c r="D4" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="G4" s="15" t="s">
+      <c r="E4" s="13"/>
+      <c r="G4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="10"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:9" ht="24" x14ac:dyDescent="0.3">
-      <c r="A5" s="14">
+      <c r="A5" s="17">
         <f>COUNTA(Backlog!A2:A500)</f>
         <v>70</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="D5" s="14">
+      <c r="B5" s="13"/>
+      <c r="D5" s="17">
         <f>COUNTIF(Backlog!F2:F500,"Done")</f>
         <v>3</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="G5" s="14">
+      <c r="E5" s="13"/>
+      <c r="G5" s="17">
         <f>COUNTIF(Backlog!F2:F500,"In Progress")</f>
         <v>0</v>
       </c>
-      <c r="H5" s="10"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="D7" s="15" t="s">
+      <c r="B7" s="13"/>
+      <c r="D7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="10"/>
-      <c r="G7" s="15" t="s">
+      <c r="E7" s="13"/>
+      <c r="G7" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="10"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:9" ht="24" x14ac:dyDescent="0.3">
-      <c r="A8" s="14">
+      <c r="A8" s="17">
         <f>COUNTIF(Backlog!F2:F500,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="D8" s="14">
+      <c r="B8" s="13"/>
+      <c r="D8" s="17">
         <f>SUM(Backlog!E2:E500)</f>
         <v>358</v>
       </c>
-      <c r="E8" s="10"/>
-      <c r="G8" s="14">
+      <c r="E8" s="13"/>
+      <c r="G8" s="17">
         <f>SUMIF(Backlog!F2:F500,"Done",Backlog!E2:E500)</f>
         <v>13</v>
       </c>
-      <c r="H8" s="10"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -5595,147 +5646,147 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="18" customFormat="1" ht="32" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:16" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="16">
+      <c r="E2" s="9">
         <v>3</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="17">
+      <c r="J2" s="10">
         <v>46153</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="16">
+      <c r="L2" s="9">
         <v>1</v>
       </c>
-      <c r="M2" s="17">
+      <c r="M2" s="10">
         <v>46153</v>
       </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16" t="s">
+      <c r="N2" s="9"/>
+      <c r="O2" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="P2" s="16"/>
-    </row>
-    <row r="3" spans="1:16" s="18" customFormat="1" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="16" t="s">
+      <c r="P2" s="9"/>
+    </row>
+    <row r="3" spans="1:16" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A3" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="9">
         <v>5</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="J3" s="17">
+      <c r="J3" s="10">
         <v>46153</v>
       </c>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="16">
+      <c r="L3" s="9">
         <v>2</v>
       </c>
-      <c r="M3" s="17">
+      <c r="M3" s="10">
         <v>46154</v>
       </c>
-      <c r="N3" s="16" t="s">
+      <c r="N3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="O3" s="16" t="s">
+      <c r="O3" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="P3" s="16"/>
-    </row>
-    <row r="4" spans="1:16" s="18" customFormat="1" ht="32" x14ac:dyDescent="0.2">
-      <c r="A4" s="16" t="s">
+      <c r="P3" s="9"/>
+    </row>
+    <row r="4" spans="1:16" s="11" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+      <c r="A4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="9">
         <v>5</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="J4" s="17">
+      <c r="J4" s="10">
         <v>46153</v>
       </c>
-      <c r="K4" s="16" t="s">
+      <c r="K4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="16">
+      <c r="L4" s="9">
         <v>2</v>
       </c>
-      <c r="M4" s="17">
+      <c r="M4" s="10">
         <v>46154</v>
       </c>
-      <c r="N4" s="16" t="s">
+      <c r="N4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="O4" s="16" t="s">
+      <c r="O4" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="P4" s="16"/>
+      <c r="P4" s="9"/>
     </row>
     <row r="5" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
@@ -8954,56 +9005,38 @@
       <c r="P71" s="5"/>
     </row>
     <row r="72" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>IAM-071</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>Developer Automation</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Establish Excel-driven Codex agent foundation</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+      <c r="A72" s="5" t="s">
+        <v>986</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>987</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>988</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>71</v>
       </c>
       <c r="E72" s="5">
         <v>3</v>
       </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="inlineStr">
-        <is>
-          <t>Establish repository instructions, tracker rules, and the package location for an Excel-driven Codex task agent.</t>
-        </is>
-      </c>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>AGENTS.md contains the agent rules; Excel temporary files are ignored; the workbook contains IAM-071 and CODE-041; completed tasks are not selected again; no commits occur without a task ID.</t>
-        </is>
-      </c>
-      <c r="I72" s="5" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
+      <c r="F72" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>989</v>
+      </c>
+      <c r="H72" s="5" t="s">
+        <v>990</v>
+      </c>
+      <c r="I72" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="J72" s="6">
         <v>46230</v>
       </c>
-      <c r="K72" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 10</t>
-        </is>
+      <c r="K72" s="5" t="s">
+        <v>991</v>
       </c>
       <c r="L72" s="5">
         <v>1</v>
@@ -9011,20 +9044,14 @@
       <c r="M72" s="6">
         <v>46230</v>
       </c>
-      <c r="N72" s="5" t="inlineStr">
-        <is>
-          <t>IAM-001,IAM-003</t>
-        </is>
-      </c>
-      <c r="O72" s="5" t="inlineStr">
-        <is>
-          <t>AGENTS.md; .gitignore; planning/IAMONIT_Full_Project_Control_Workbook.xlsx</t>
-        </is>
-      </c>
-      <c r="P72" s="5" t="inlineStr">
-        <is>
-          <t>Every Git commit must begin with the exact related task ID.</t>
-        </is>
+      <c r="N72" s="5" t="s">
+        <v>992</v>
+      </c>
+      <c r="O72" s="5" t="s">
+        <v>993</v>
+      </c>
+      <c r="P72" s="5" t="s">
+        <v>994</v>
       </c>
     </row>
   </sheetData>
@@ -11352,53 +11379,35 @@
       </c>
     </row>
     <row r="72" spans="1:10" ht="32" x14ac:dyDescent="0.2">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 10</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>IAM-071</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Developer Automation</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>Establish Excel-driven Codex agent foundation</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+      <c r="A72" s="5" t="s">
+        <v>991</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>986</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>987</v>
+      </c>
+      <c r="D72" s="5" t="s">
+        <v>988</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F72" s="5" t="s">
+        <v>71</v>
       </c>
       <c r="G72" s="5">
         <v>3</v>
       </c>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="I72" s="5" t="inlineStr">
-        <is>
-          <t>IAM-001,IAM-003</t>
-        </is>
-      </c>
-      <c r="J72" s="5" t="inlineStr">
-        <is>
-          <t>Repository and workbook rules for the Excel-driven Codex agent are established.</t>
-        </is>
+      <c r="H72" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I72" s="5" t="s">
+        <v>992</v>
+      </c>
+      <c r="J72" s="5" t="s">
+        <v>995</v>
       </c>
     </row>
   </sheetData>
@@ -19283,50 +19292,32 @@
       </c>
     </row>
     <row r="42" spans="1:9" ht="64" x14ac:dyDescent="0.2">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>CODE-041</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>task-agent</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>packages/task-agent/src/cli.ts</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Create read-only workbook reader and eligible-task selector</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Use ExcelJS to read the Backlog and IntelliJ Coding Tasks sheets. Skip Done, In Progress, Blocked, and Review tasks. Select a Todo task only when all dependencies are Done. Print one selected task and stop without changing the workbook or application code.</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>IAM-071</t>
-        </is>
-      </c>
-      <c r="H42" s="5" t="inlineStr">
-        <is>
-          <t>The CLI identifies exactly one eligible task, respects dependencies, skips completed work, and makes no workbook changes.</t>
-        </is>
-      </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
+      <c r="A42" s="5" t="s">
+        <v>996</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>997</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>998</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>999</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>1000</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>986</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>1002</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
IAM-072 Align tracker paths with workspace structure
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,14 +29,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'API Contracts'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DB Schema + RLS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Dependencies!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Release Checklist'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Risks &amp; Decisions'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$73</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Timeline + Gantt'!$A$1:$AX$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UI Screens'!$A$1:$H$12</definedName>
   </definedNames>
@@ -5579,7 +5579,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -5735,8 +5735,10 @@
       <c r="N3" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="O3" s="9" t="s">
-        <v>62</v>
+      <c r="O3" s="9" t="inlineStr">
+        <is>
+          <t>apps/web/package.json; apps/web/app/layout.tsx; apps/web/tailwind.config.ts</t>
+        </is>
       </c>
       <c r="P3" s="9"/>
     </row>
@@ -5783,8 +5785,10 @@
       <c r="N4" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="O4" s="9" t="s">
-        <v>68</v>
+      <c r="O4" s="9" t="inlineStr">
+        <is>
+          <t>apps/api/src/main.ts; apps/api/src/app.module.ts</t>
+        </is>
       </c>
       <c r="P4" s="9"/>
     </row>
@@ -5831,8 +5835,10 @@
       <c r="N5" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="O5" s="5" t="s">
-        <v>75</v>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/config/env.ts; apps/web/.env.example</t>
+        </is>
       </c>
       <c r="P5" s="5"/>
     </row>
@@ -5879,8 +5885,10 @@
       <c r="N6" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="O6" s="5" t="s">
-        <v>80</v>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/.eslintrc; apps/api/.eslintrc</t>
+        </is>
       </c>
       <c r="P6" s="5"/>
     </row>
@@ -6023,8 +6031,10 @@
       <c r="N9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="O9" s="5" t="s">
-        <v>98</v>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/dto/register.dto.ts; login.dto.ts</t>
+        </is>
       </c>
       <c r="P9" s="5"/>
     </row>
@@ -6071,8 +6081,10 @@
       <c r="N10" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="O10" s="5" t="s">
-        <v>103</v>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(auth)/login/page.tsx; apps/web/app/(auth)/register/page.tsx</t>
+        </is>
       </c>
       <c r="P10" s="5"/>
     </row>
@@ -6359,8 +6371,10 @@
       <c r="N16" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="O16" s="5" t="s">
-        <v>138</v>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.service.ts; tenants.service.ts</t>
+        </is>
       </c>
       <c r="P16" s="5"/>
     </row>
@@ -6407,8 +6421,10 @@
       <c r="N17" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="O17" s="5" t="s">
-        <v>144</v>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.controller.ts; jwt.strategy.ts</t>
+        </is>
       </c>
       <c r="P17" s="5"/>
     </row>
@@ -6455,8 +6471,10 @@
       <c r="N18" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="O18" s="5" t="s">
-        <v>151</v>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/lib/auth.ts; apps/web/app/(auth)/*</t>
+        </is>
       </c>
       <c r="P18" s="5"/>
     </row>
@@ -6503,8 +6521,10 @@
       <c r="N19" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="O19" s="5" t="s">
-        <v>157</v>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/common/guards/auth.guard.ts; roles.guard.ts</t>
+        </is>
       </c>
       <c r="P19" s="5"/>
     </row>
@@ -6599,8 +6619,10 @@
       <c r="N21" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="O21" s="5" t="s">
-        <v>169</v>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/invitations/invitations.controller.ts; invitations.service.ts</t>
+        </is>
       </c>
       <c r="P21" s="5"/>
     </row>
@@ -6647,8 +6669,10 @@
       <c r="N22" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="O22" s="5" t="s">
-        <v>174</v>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/invitations/invitations.service.ts</t>
+        </is>
       </c>
       <c r="P22" s="5"/>
     </row>
@@ -6695,8 +6719,10 @@
       <c r="N23" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="O23" s="5" t="s">
-        <v>180</v>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/users/users.controller.ts; users.service.ts</t>
+        </is>
       </c>
       <c r="P23" s="5"/>
     </row>
@@ -6743,8 +6769,10 @@
       <c r="N24" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="O24" s="5" t="s">
-        <v>187</v>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/users/page.tsx; components/users/InviteUserModal.tsx</t>
+        </is>
       </c>
       <c r="P24" s="5"/>
     </row>
@@ -6791,8 +6819,10 @@
       <c r="N25" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="O25" s="5" t="s">
-        <v>193</v>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/layout.tsx; components/layout/Sidebar.tsx; Topbar.tsx</t>
+        </is>
       </c>
       <c r="P25" s="5"/>
     </row>
@@ -6839,8 +6869,10 @@
       <c r="N26" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="O26" s="5" t="s">
-        <v>201</v>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tenants/*; apps/web/app/(dashboard)/settings/company/page.tsx</t>
+        </is>
       </c>
       <c r="P26" s="5"/>
     </row>
@@ -6983,8 +7015,10 @@
       <c r="N29" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="O29" s="5" t="s">
-        <v>218</v>
+      <c r="O29" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/dto/create-task.dto.ts; update-task-status.dto.ts</t>
+        </is>
       </c>
       <c r="P29" s="5"/>
     </row>
@@ -7031,8 +7065,10 @@
       <c r="N30" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="O30" s="5" t="s">
-        <v>224</v>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/tasks.controller.ts; tasks.service.ts</t>
+        </is>
       </c>
       <c r="P30" s="5"/>
     </row>
@@ -7079,8 +7115,10 @@
       <c r="N31" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="O31" s="5" t="s">
-        <v>229</v>
+      <c r="O31" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/tasks.repository.ts</t>
+        </is>
       </c>
       <c r="P31" s="5"/>
     </row>
@@ -7127,8 +7165,10 @@
       <c r="N32" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="O32" s="5" t="s">
-        <v>234</v>
+      <c r="O32" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/tasks.service.ts</t>
+        </is>
       </c>
       <c r="P32" s="5"/>
     </row>
@@ -7175,8 +7215,10 @@
       <c r="N33" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="O33" s="5" t="s">
-        <v>240</v>
+      <c r="O33" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/task-status.service.ts</t>
+        </is>
       </c>
       <c r="P33" s="5"/>
     </row>
@@ -7223,8 +7265,10 @@
       <c r="N34" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="O34" s="5" t="s">
-        <v>247</v>
+      <c r="O34" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/page.tsx; components/tasks/TaskCard.tsx</t>
+        </is>
       </c>
       <c r="P34" s="5"/>
     </row>
@@ -7271,8 +7315,10 @@
       <c r="N35" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="O35" s="5" t="s">
-        <v>253</v>
+      <c r="O35" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/new/page.tsx; components/tasks/CreateTaskForm.tsx</t>
+        </is>
       </c>
       <c r="P35" s="5"/>
     </row>
@@ -7319,8 +7365,10 @@
       <c r="N36" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="O36" s="5" t="s">
-        <v>259</v>
+      <c r="O36" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/[id]/page.tsx; components/tasks/TaskDetail.tsx</t>
+        </is>
       </c>
       <c r="P36" s="5"/>
     </row>
@@ -7415,8 +7463,10 @@
       <c r="N38" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="O38" s="5" t="s">
-        <v>272</v>
+      <c r="O38" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/uploads/uploads.controller.ts; uploads.service.ts</t>
+        </is>
       </c>
       <c r="P38" s="5"/>
     </row>
@@ -7463,8 +7513,10 @@
       <c r="N39" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="O39" s="5" t="s">
-        <v>277</v>
+      <c r="O39" s="5" t="inlineStr">
+        <is>
+          <t>supabase/migrations/038_files.sql; apps/api/src/modules/uploads/file-metadata.service.ts</t>
+        </is>
       </c>
       <c r="P39" s="5"/>
     </row>
@@ -7511,8 +7563,10 @@
       <c r="N40" s="5" t="s">
         <v>266</v>
       </c>
-      <c r="O40" s="5" t="s">
-        <v>283</v>
+      <c r="O40" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/uploads/FileUploader.tsx</t>
+        </is>
       </c>
       <c r="P40" s="5"/>
     </row>
@@ -7607,8 +7661,10 @@
       <c r="N42" s="5" t="s">
         <v>284</v>
       </c>
-      <c r="O42" s="5" t="s">
-        <v>295</v>
+      <c r="O42" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/task-updates/task-updates.controller.ts; service.ts</t>
+        </is>
       </c>
       <c r="P42" s="5"/>
     </row>
@@ -7655,8 +7711,10 @@
       <c r="N43" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="O43" s="5" t="s">
-        <v>301</v>
+      <c r="O43" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/tasks/TaskTimeline.tsx; TaskUpdateComposer.tsx</t>
+        </is>
       </c>
       <c r="P43" s="5"/>
     </row>
@@ -7703,8 +7761,10 @@
       <c r="N44" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="O44" s="5" t="s">
-        <v>307</v>
+      <c r="O44" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/my-tasks/[id]/page.tsx</t>
+        </is>
       </c>
       <c r="P44" s="5"/>
     </row>
@@ -7799,8 +7859,10 @@
       <c r="N46" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="O46" s="5" t="s">
-        <v>319</v>
+      <c r="O46" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/notifications/notifications.service.ts</t>
+        </is>
       </c>
       <c r="P46" s="5"/>
     </row>
@@ -7847,8 +7909,10 @@
       <c r="N47" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="O47" s="5" t="s">
-        <v>324</v>
+      <c r="O47" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/notifications/notifications.controller.ts</t>
+        </is>
       </c>
       <c r="P47" s="5"/>
     </row>
@@ -7895,8 +7959,10 @@
       <c r="N48" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="O48" s="5" t="s">
-        <v>330</v>
+      <c r="O48" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/notifications/NotificationBell.tsx</t>
+        </is>
       </c>
       <c r="P48" s="5"/>
     </row>
@@ -7943,8 +8009,10 @@
       <c r="N49" s="5" t="s">
         <v>336</v>
       </c>
-      <c r="O49" s="5" t="s">
-        <v>337</v>
+      <c r="O49" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/page.tsx; components/dashboard/KpiCard.tsx</t>
+        </is>
       </c>
       <c r="P49" s="5"/>
     </row>
@@ -7991,8 +8059,10 @@
       <c r="N50" s="5" t="s">
         <v>302</v>
       </c>
-      <c r="O50" s="5" t="s">
-        <v>342</v>
+      <c r="O50" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/my-tasks/page.tsx</t>
+        </is>
       </c>
       <c r="P50" s="5"/>
     </row>
@@ -8039,8 +8109,10 @@
       <c r="N51" s="5" t="s">
         <v>225</v>
       </c>
-      <c r="O51" s="5" t="s">
-        <v>348</v>
+      <c r="O51" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/task-query.dto.ts</t>
+        </is>
       </c>
       <c r="P51" s="5"/>
     </row>
@@ -8087,8 +8159,10 @@
       <c r="N52" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="O52" s="5" t="s">
-        <v>354</v>
+      <c r="O52" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/tasks/TaskFilters.tsx</t>
+        </is>
       </c>
       <c r="P52" s="5"/>
     </row>
@@ -8279,8 +8353,10 @@
       <c r="N56" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="O56" s="5" t="s">
-        <v>380</v>
+      <c r="O56" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/test/auth.spec.ts; tenants.spec.ts</t>
+        </is>
       </c>
       <c r="P56" s="5"/>
     </row>
@@ -8327,8 +8403,10 @@
       <c r="N57" s="5" t="s">
         <v>385</v>
       </c>
-      <c r="O57" s="5" t="s">
-        <v>386</v>
+      <c r="O57" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/test/tasks.spec.ts; uploads.spec.ts</t>
+        </is>
       </c>
       <c r="P57" s="5"/>
     </row>
@@ -8375,8 +8453,10 @@
       <c r="N58" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="O58" s="5" t="s">
-        <v>392</v>
+      <c r="O58" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/__tests__/*</t>
+        </is>
       </c>
       <c r="P58" s="5"/>
     </row>
@@ -8567,8 +8647,10 @@
       <c r="N62" s="5" t="s">
         <v>399</v>
       </c>
-      <c r="O62" s="5" t="s">
-        <v>415</v>
+      <c r="O62" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/Dockerfile; railway.json/render.yaml</t>
+        </is>
       </c>
       <c r="P62" s="5"/>
     </row>
@@ -8903,8 +8985,10 @@
       <c r="N69" s="5" t="s">
         <v>456</v>
       </c>
-      <c r="O69" s="5" t="s">
-        <v>457</v>
+      <c r="O69" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/payments/PaymentPanel.tsx</t>
+        </is>
       </c>
       <c r="P69" s="5"/>
     </row>
@@ -8951,8 +9035,10 @@
       <c r="N70" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="O70" s="5" t="s">
-        <v>465</v>
+      <c r="O70" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/lib/realtime.ts; backend events</t>
+        </is>
       </c>
       <c r="P70" s="5"/>
     </row>
@@ -8999,8 +9085,10 @@
       <c r="N71" s="5" t="s">
         <v>470</v>
       </c>
-      <c r="O71" s="5" t="s">
-        <v>330</v>
+      <c r="O71" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/notifications/NotificationBell.tsx</t>
+        </is>
       </c>
       <c r="P71" s="5"/>
     </row>
@@ -9054,9 +9142,83 @@
         <v>994</v>
       </c>
     </row>
+    <row r="73" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>IAM-072</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Developer Automation</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Align tracker paths with workspace structure</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E73" s="5">
+        <v>3</v>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>Align legacy backend and frontend file paths in the IAMONIT project tracker with the repository’s pnpm workspace structure.</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Legacy backend paths use apps/api; legacy frontend paths use apps/web; canonical paths remain unchanged; no formulas, dropdowns, styles, or unrelated tracker content are damaged; remaining invalid path prefixes are reported.</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="J73" s="6">
+        <v>46230</v>
+      </c>
+      <c r="K73" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="L73" s="5">
+        <v>1</v>
+      </c>
+      <c r="M73" s="6">
+        <v>46230</v>
+      </c>
+      <c r="N73" s="5" t="inlineStr">
+        <is>
+          <t>IAM-071</t>
+        </is>
+      </c>
+      <c r="O73" s="5" t="inlineStr">
+        <is>
+          <t>planning/IAMONIT_Full_Project_Control_Workbook.xlsx</t>
+        </is>
+      </c>
+      <c r="P73" s="5" t="inlineStr">
+        <is>
+          <t>Normalize path-bearing tracker cells only. Do not change descriptive prose, URLs, package names, commands, class names, or task IDs.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P72" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="F2:F72">
+  <autoFilter ref="A1:P73" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="F2:F73">
     <cfRule type="expression" dxfId="29" priority="1">
       <formula>$F2="Done"</formula>
     </cfRule>
@@ -9074,13 +9236,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="D2:D72" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D73" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F72" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F73" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:I72" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I73" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"Frontend,Backend,Database,DevOps,QA,Product,Security"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9094,7 +9256,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -11410,9 +11572,59 @@
         <v>995</v>
       </c>
     </row>
+    <row r="73" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>IAM-072</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Developer Automation</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Align tracker paths with workspace structure</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G73" s="5">
+        <v>3</v>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>IAM-071</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>Tracker file paths match the actual apps/api and apps/web workspace structure.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J72" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="H2:H72">
+  <autoFilter ref="A1:J73" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="H2:H73">
     <cfRule type="expression" dxfId="24" priority="1">
       <formula>$H2="Done"</formula>
     </cfRule>
@@ -11430,7 +11642,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H72" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H73" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -18089,7 +18301,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -18141,8 +18353,10 @@
       <c r="C2" s="5" t="s">
         <v>534</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>535</v>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/config/env.ts</t>
+        </is>
       </c>
       <c r="E2" s="5" t="s">
         <v>536</v>
@@ -18170,8 +18384,10 @@
       <c r="C3" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>541</v>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/dto/register.dto.ts</t>
+        </is>
       </c>
       <c r="E3" s="5" t="s">
         <v>542</v>
@@ -18199,8 +18415,10 @@
       <c r="C4" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>546</v>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/dto/login.dto.ts</t>
+        </is>
       </c>
       <c r="E4" s="5" t="s">
         <v>547</v>
@@ -18228,8 +18446,10 @@
       <c r="C5" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>551</v>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.controller.ts</t>
+        </is>
       </c>
       <c r="E5" s="5" t="s">
         <v>552</v>
@@ -18257,8 +18477,10 @@
       <c r="C6" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>557</v>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.service.ts</t>
+        </is>
       </c>
       <c r="E6" s="5" t="s">
         <v>558</v>
@@ -18286,8 +18508,10 @@
       <c r="C7" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>562</v>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/jwt.strategy.ts</t>
+        </is>
       </c>
       <c r="E7" s="5" t="s">
         <v>563</v>
@@ -18315,8 +18539,10 @@
       <c r="C8" s="5" t="s">
         <v>567</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>568</v>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/common/guards/auth.guard.ts</t>
+        </is>
       </c>
       <c r="E8" s="5" t="s">
         <v>569</v>
@@ -18344,8 +18570,10 @@
       <c r="C9" s="5" t="s">
         <v>567</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>573</v>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/common/guards/roles.guard.ts</t>
+        </is>
       </c>
       <c r="E9" s="5" t="s">
         <v>574</v>
@@ -18373,8 +18601,10 @@
       <c r="C10" s="5" t="s">
         <v>578</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>579</v>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tenants/tenants.service.ts</t>
+        </is>
       </c>
       <c r="E10" s="5" t="s">
         <v>580</v>
@@ -18402,8 +18632,10 @@
       <c r="C11" s="5" t="s">
         <v>584</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>585</v>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/users/users.controller.ts</t>
+        </is>
       </c>
       <c r="E11" s="5" t="s">
         <v>586</v>
@@ -18431,8 +18663,10 @@
       <c r="C12" s="5" t="s">
         <v>584</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>590</v>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/users/users.service.ts</t>
+        </is>
       </c>
       <c r="E12" s="5" t="s">
         <v>591</v>
@@ -18460,8 +18694,10 @@
       <c r="C13" s="5" t="s">
         <v>595</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>596</v>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/invitations/invitations.controller.ts</t>
+        </is>
       </c>
       <c r="E13" s="5" t="s">
         <v>597</v>
@@ -18489,8 +18725,10 @@
       <c r="C14" s="5" t="s">
         <v>595</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>174</v>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/invitations/invitations.service.ts</t>
+        </is>
       </c>
       <c r="E14" s="5" t="s">
         <v>602</v>
@@ -18518,8 +18756,10 @@
       <c r="C15" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>607</v>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/dto/create-task.dto.ts</t>
+        </is>
       </c>
       <c r="E15" s="5" t="s">
         <v>608</v>
@@ -18547,8 +18787,10 @@
       <c r="C16" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>612</v>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/tasks.controller.ts</t>
+        </is>
       </c>
       <c r="E16" s="5" t="s">
         <v>613</v>
@@ -18576,8 +18818,10 @@
       <c r="C17" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>234</v>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/tasks.service.ts</t>
+        </is>
       </c>
       <c r="E17" s="5" t="s">
         <v>618</v>
@@ -18605,8 +18849,10 @@
       <c r="C18" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>240</v>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/task-status.service.ts</t>
+        </is>
       </c>
       <c r="E18" s="5" t="s">
         <v>622</v>
@@ -18634,8 +18880,10 @@
       <c r="C19" s="5" t="s">
         <v>626</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>627</v>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/uploads/uploads.controller.ts</t>
+        </is>
       </c>
       <c r="E19" s="5" t="s">
         <v>628</v>
@@ -18663,8 +18911,10 @@
       <c r="C20" s="5" t="s">
         <v>626</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>632</v>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/uploads/uploads.service.ts</t>
+        </is>
       </c>
       <c r="E20" s="5" t="s">
         <v>633</v>
@@ -18692,8 +18942,10 @@
       <c r="C21" s="5" t="s">
         <v>637</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>638</v>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/task-updates/task-updates.controller.ts</t>
+        </is>
       </c>
       <c r="E21" s="5" t="s">
         <v>639</v>
@@ -18721,8 +18973,10 @@
       <c r="C22" s="5" t="s">
         <v>643</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>319</v>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/notifications/notifications.service.ts</t>
+        </is>
       </c>
       <c r="E22" s="5" t="s">
         <v>644</v>
@@ -18750,8 +19004,10 @@
       <c r="C23" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>648</v>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(auth)/login/page.tsx</t>
+        </is>
       </c>
       <c r="E23" s="5" t="s">
         <v>649</v>
@@ -18779,8 +19035,10 @@
       <c r="C24" s="5" t="s">
         <v>540</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>654</v>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(auth)/register/page.tsx</t>
+        </is>
       </c>
       <c r="E24" s="5" t="s">
         <v>655</v>
@@ -18808,8 +19066,10 @@
       <c r="C25" s="5" t="s">
         <v>659</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>660</v>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/lib/api.ts</t>
+        </is>
       </c>
       <c r="E25" s="5" t="s">
         <v>661</v>
@@ -18837,8 +19097,10 @@
       <c r="C26" s="5" t="s">
         <v>659</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>665</v>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/lib/auth.ts</t>
+        </is>
       </c>
       <c r="E26" s="5" t="s">
         <v>666</v>
@@ -18866,8 +19128,10 @@
       <c r="C27" s="5" t="s">
         <v>670</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>671</v>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/layout/Sidebar.tsx</t>
+        </is>
       </c>
       <c r="E27" s="5" t="s">
         <v>672</v>
@@ -18895,8 +19159,10 @@
       <c r="C28" s="5" t="s">
         <v>670</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>676</v>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/layout/Topbar.tsx</t>
+        </is>
       </c>
       <c r="E28" s="5" t="s">
         <v>677</v>
@@ -18924,8 +19190,10 @@
       <c r="C29" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>682</v>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/page.tsx</t>
+        </is>
       </c>
       <c r="E29" s="5" t="s">
         <v>243</v>
@@ -18953,8 +19221,10 @@
       <c r="C30" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>687</v>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/new/page.tsx</t>
+        </is>
       </c>
       <c r="E30" s="5" t="s">
         <v>249</v>
@@ -18982,8 +19252,10 @@
       <c r="C31" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D31" s="5" t="s">
-        <v>691</v>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/[id]/page.tsx</t>
+        </is>
       </c>
       <c r="E31" s="5" t="s">
         <v>255</v>
@@ -19011,8 +19283,10 @@
       <c r="C32" s="5" t="s">
         <v>606</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>695</v>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/tasks/TaskTimeline.tsx</t>
+        </is>
       </c>
       <c r="E32" s="5" t="s">
         <v>696</v>
@@ -19040,8 +19314,10 @@
       <c r="C33" s="5" t="s">
         <v>626</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>283</v>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/uploads/FileUploader.tsx</t>
+        </is>
       </c>
       <c r="E33" s="5" t="s">
         <v>700</v>
@@ -19069,8 +19345,10 @@
       <c r="C34" s="5" t="s">
         <v>704</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>307</v>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/my-tasks/[id]/page.tsx</t>
+        </is>
       </c>
       <c r="E34" s="5" t="s">
         <v>705</v>
@@ -19098,8 +19376,10 @@
       <c r="C35" s="5" t="s">
         <v>643</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>330</v>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/notifications/NotificationBell.tsx</t>
+        </is>
       </c>
       <c r="E35" s="5" t="s">
         <v>709</v>
@@ -19243,8 +19523,10 @@
       <c r="C40" s="5" t="s">
         <v>731</v>
       </c>
-      <c r="D40" s="5" t="s">
-        <v>732</v>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/test/tasks.spec.ts</t>
+        </is>
       </c>
       <c r="E40" s="5" t="s">
         <v>733</v>
@@ -19320,9 +19602,56 @@
         <v>13</v>
       </c>
     </row>
+    <row r="43" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>CODE-042</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>task-agent</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>packages/task-agent/src/path-normalizer.ts</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Validate and normalize coding-task file paths</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Add runtime path normalization and validation to the read-only task agent. Convert known legacy prefixes to canonical workspace paths, reject unsafe paths, preserve already canonical paths, and print both original and normalized task paths.</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>IAM-072</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>backend paths normalize to apps/api; frontend paths normalize to apps/web; canonical paths remain unchanged; absolute paths and directory traversal are rejected; future files are allowed to be absent; tests cover valid, legacy, unsafe, and multiple-path inputs.</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I42" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I42">
+  <autoFilter ref="A1:I43" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <conditionalFormatting sqref="I2:I43">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -19340,7 +19669,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I42" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I43" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19385,8 +19714,10 @@
       <c r="A2" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>535</v>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/config/env.ts</t>
+        </is>
       </c>
       <c r="C2" s="5" t="s">
         <v>536</v>
@@ -19402,8 +19733,10 @@
       <c r="A3" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>541</v>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/dto/register.dto.ts</t>
+        </is>
       </c>
       <c r="C3" s="5" t="s">
         <v>542</v>
@@ -19419,8 +19752,10 @@
       <c r="A4" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>546</v>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/dto/login.dto.ts</t>
+        </is>
       </c>
       <c r="C4" s="5" t="s">
         <v>547</v>
@@ -19436,8 +19771,10 @@
       <c r="A5" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>551</v>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.controller.ts</t>
+        </is>
       </c>
       <c r="C5" s="5" t="s">
         <v>552</v>
@@ -19453,8 +19790,10 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>557</v>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.service.ts</t>
+        </is>
       </c>
       <c r="C6" s="5" t="s">
         <v>558</v>
@@ -19470,8 +19809,10 @@
       <c r="A7" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>562</v>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/jwt.strategy.ts</t>
+        </is>
       </c>
       <c r="C7" s="5" t="s">
         <v>563</v>
@@ -19487,8 +19828,10 @@
       <c r="A8" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>568</v>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/common/guards/auth.guard.ts</t>
+        </is>
       </c>
       <c r="C8" s="5" t="s">
         <v>569</v>
@@ -19504,8 +19847,10 @@
       <c r="A9" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>573</v>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/common/guards/roles.guard.ts</t>
+        </is>
       </c>
       <c r="C9" s="5" t="s">
         <v>574</v>
@@ -19521,8 +19866,10 @@
       <c r="A10" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>579</v>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tenants/tenants.service.ts</t>
+        </is>
       </c>
       <c r="C10" s="5" t="s">
         <v>580</v>
@@ -19538,8 +19885,10 @@
       <c r="A11" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>585</v>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/users/users.controller.ts</t>
+        </is>
       </c>
       <c r="C11" s="5" t="s">
         <v>586</v>
@@ -19555,8 +19904,10 @@
       <c r="A12" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>590</v>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/users/users.service.ts</t>
+        </is>
       </c>
       <c r="C12" s="5" t="s">
         <v>591</v>
@@ -19572,8 +19923,10 @@
       <c r="A13" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>596</v>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/invitations/invitations.controller.ts</t>
+        </is>
       </c>
       <c r="C13" s="5" t="s">
         <v>597</v>
@@ -19589,8 +19942,10 @@
       <c r="A14" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>174</v>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/invitations/invitations.service.ts</t>
+        </is>
       </c>
       <c r="C14" s="5" t="s">
         <v>602</v>
@@ -19606,8 +19961,10 @@
       <c r="A15" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>607</v>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/dto/create-task.dto.ts</t>
+        </is>
       </c>
       <c r="C15" s="5" t="s">
         <v>608</v>
@@ -19623,8 +19980,10 @@
       <c r="A16" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>612</v>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/tasks.controller.ts</t>
+        </is>
       </c>
       <c r="C16" s="5" t="s">
         <v>613</v>
@@ -19640,8 +19999,10 @@
       <c r="A17" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B17" s="5" t="s">
-        <v>234</v>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/tasks.service.ts</t>
+        </is>
       </c>
       <c r="C17" s="5" t="s">
         <v>618</v>
@@ -19657,8 +20018,10 @@
       <c r="A18" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B18" s="5" t="s">
-        <v>240</v>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/tasks/task-status.service.ts</t>
+        </is>
       </c>
       <c r="C18" s="5" t="s">
         <v>622</v>
@@ -19674,8 +20037,10 @@
       <c r="A19" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="5" t="s">
-        <v>627</v>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/uploads/uploads.controller.ts</t>
+        </is>
       </c>
       <c r="C19" s="5" t="s">
         <v>628</v>
@@ -19691,8 +20056,10 @@
       <c r="A20" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>632</v>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/uploads/uploads.service.ts</t>
+        </is>
       </c>
       <c r="C20" s="5" t="s">
         <v>633</v>
@@ -19708,8 +20075,10 @@
       <c r="A21" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>638</v>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/task-updates/task-updates.controller.ts</t>
+        </is>
       </c>
       <c r="C21" s="5" t="s">
         <v>639</v>
@@ -19725,8 +20094,10 @@
       <c r="A22" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>319</v>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/notifications/notifications.service.ts</t>
+        </is>
       </c>
       <c r="C22" s="5" t="s">
         <v>644</v>
@@ -19742,8 +20113,10 @@
       <c r="A23" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="5" t="s">
-        <v>648</v>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(auth)/login/page.tsx</t>
+        </is>
       </c>
       <c r="C23" s="5" t="s">
         <v>649</v>
@@ -19759,8 +20132,10 @@
       <c r="A24" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>654</v>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(auth)/register/page.tsx</t>
+        </is>
       </c>
       <c r="C24" s="5" t="s">
         <v>655</v>
@@ -19776,8 +20151,10 @@
       <c r="A25" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>660</v>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/lib/api.ts</t>
+        </is>
       </c>
       <c r="C25" s="5" t="s">
         <v>661</v>
@@ -19793,8 +20170,10 @@
       <c r="A26" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>665</v>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/lib/auth.ts</t>
+        </is>
       </c>
       <c r="C26" s="5" t="s">
         <v>666</v>
@@ -19810,8 +20189,10 @@
       <c r="A27" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>671</v>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/layout/Sidebar.tsx</t>
+        </is>
       </c>
       <c r="C27" s="5" t="s">
         <v>672</v>
@@ -19827,8 +20208,10 @@
       <c r="A28" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>676</v>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/layout/Topbar.tsx</t>
+        </is>
       </c>
       <c r="C28" s="5" t="s">
         <v>677</v>
@@ -19844,8 +20227,10 @@
       <c r="A29" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B29" s="5" t="s">
-        <v>682</v>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/page.tsx</t>
+        </is>
       </c>
       <c r="C29" s="5" t="s">
         <v>243</v>
@@ -19861,8 +20246,10 @@
       <c r="A30" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="5" t="s">
-        <v>687</v>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/new/page.tsx</t>
+        </is>
       </c>
       <c r="C30" s="5" t="s">
         <v>249</v>
@@ -19878,8 +20265,10 @@
       <c r="A31" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B31" s="5" t="s">
-        <v>691</v>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/tasks/[id]/page.tsx</t>
+        </is>
       </c>
       <c r="C31" s="5" t="s">
         <v>255</v>
@@ -19895,8 +20284,10 @@
       <c r="A32" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>695</v>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/tasks/TaskTimeline.tsx</t>
+        </is>
       </c>
       <c r="C32" s="5" t="s">
         <v>696</v>
@@ -19912,8 +20303,10 @@
       <c r="A33" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B33" s="5" t="s">
-        <v>283</v>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/uploads/FileUploader.tsx</t>
+        </is>
       </c>
       <c r="C33" s="5" t="s">
         <v>700</v>
@@ -19929,8 +20322,10 @@
       <c r="A34" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>307</v>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/app/(dashboard)/my-tasks/[id]/page.tsx</t>
+        </is>
       </c>
       <c r="C34" s="5" t="s">
         <v>705</v>
@@ -19946,8 +20341,10 @@
       <c r="A35" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B35" s="5" t="s">
-        <v>330</v>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>apps/web/components/notifications/NotificationBell.tsx</t>
+        </is>
       </c>
       <c r="C35" s="5" t="s">
         <v>709</v>
@@ -20031,8 +20428,10 @@
       <c r="A40" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="B40" s="5" t="s">
-        <v>732</v>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/test/tasks.spec.ts</t>
+        </is>
       </c>
       <c r="C40" s="5" t="s">
         <v>733</v>

</xml_diff>

<commit_message>
IAM-073 Add controlled Codex execution pipeline
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,14 +29,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'API Contracts'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DB Schema + RLS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Dependencies!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Release Checklist'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Risks &amp; Decisions'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Timeline + Gantt'!$A$1:$AX$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'UI Screens'!$A$1:$H$12</definedName>
   </definedNames>
@@ -5615,7 +5615,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P73"/>
+  <dimension ref="A1:P74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -9140,9 +9140,83 @@
         <v>980</v>
       </c>
     </row>
+    <row r="74" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>IAM-073</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>Developer Automation</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Add controlled Codex execution pipeline</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E74" s="5">
+        <v>5</v>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>Extend the IAMONIT task-agent so it can generate a task-specific Codex prompt and invoke Codex non-interactively under explicit safety controls.</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>The agent supports a non-mutating plan mode; execution requires an explicit flag; execution is blocked on a dirty working tree or protected branch; Codex runs only inside the repository workspace; results and exit status are captured; the workbook is never modified; no commit or push occurs automatically.</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="J74" s="6">
+        <v>46230</v>
+      </c>
+      <c r="K74" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="L74" s="5">
+        <v>2</v>
+      </c>
+      <c r="M74" s="6">
+        <v>46231</v>
+      </c>
+      <c r="N74" s="5" t="inlineStr">
+        <is>
+          <t>IAM-071,IAM-072</t>
+        </is>
+      </c>
+      <c r="O74" s="5" t="inlineStr">
+        <is>
+          <t>packages/task-agent/src/prompt-builder.ts; packages/task-agent/src/codex-executor.ts; packages/task-agent/src/git-preflight.ts; packages/task-agent/src/cli.ts</t>
+        </is>
+      </c>
+      <c r="P74" s="5" t="inlineStr">
+        <is>
+          <t>Plan mode is the default. Real execution requires explicit user action and must stop at human review.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P73" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="F2:F73">
+  <autoFilter ref="A1:P74" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="F2:F74">
     <cfRule type="expression" dxfId="29" priority="1">
       <formula>$F2="Done"</formula>
     </cfRule>
@@ -9160,13 +9234,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" sqref="D2:D73" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D2:D74" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F73" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F74" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I2:I73" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I74" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"Frontend,Backend,Database,DevOps,QA,Product,Security"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9180,7 +9254,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -11528,9 +11602,59 @@
         <v>981</v>
       </c>
     </row>
+    <row r="74" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Sprint 10</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>IAM-073</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Developer Automation</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Add controlled Codex execution pipeline</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G74" s="5">
+        <v>5</v>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>IAM-071,IAM-072</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>The task-agent can safely prepare and explicitly launch one Codex coding task without committing, pushing, or updating the workbook.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J73" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="H2:H73">
+  <autoFilter ref="A1:J74" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="H2:H74">
     <cfRule type="expression" dxfId="24" priority="1">
       <formula>$H2="Done"</formula>
     </cfRule>
@@ -11548,7 +11672,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="H2:H73" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H74" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -18207,7 +18331,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19467,9 +19591,56 @@
         <v>13</v>
       </c>
     </row>
+    <row r="44" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>CODE-043</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Tooling</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>task-agent</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>packages/task-agent/src/prompt-builder.ts; packages/task-agent/src/codex-executor.ts; packages/task-agent/src/git-preflight.ts; packages/task-agent/src/cli.ts</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Build task prompt generation and controlled Codex execution</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Generate a detailed prompt from the single selected workbook task. Keep plan mode as the default. Add an explicit execution mode that invokes codex exec using Node child_process.spawn without a shell. Pass the prompt through stdin. Use workspace-write sandboxing, disable network access, capture JSONL events and the final assistant message, verify a clean Git working tree, reject protected branches, preserve the workbook checksum, and never commit or push.</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>IAM-073</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Plan mode prints the exact generated prompt without invoking Codex; execution requires an explicit flag; dirty repositories and main/master branches are rejected; unsafe or unresolved task paths remain rejected; Codex output and exit code are captured; workbook checksum remains unchanged; no automatic commit, push, or tracker update occurs; unit tests cover prompt creation, argument construction, Git preflight, execution failure, and dry-run behavior.</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I43" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I43">
+  <autoFilter ref="A1:I44" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <conditionalFormatting sqref="I2:I44">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -19487,7 +19658,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I43" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I44" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
CODE-043 Build controlled Codex execution pipeline
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B21EA4D5-C3C2-1C47-A93D-229E87C46C63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B33F21D-B10C-CE48-81E0-0537066FF46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3313" uniqueCount="1015">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3343" uniqueCount="1027">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3102,6 +3102,42 @@
   </si>
   <si>
     <t>backend paths normalize to apps/api; frontend paths normalize to apps/web; canonical paths remain unchanged; absolute paths and directory traversal are rejected; future files are allowed to be absent; tests cover valid, legacy, unsafe, and multiple-path inputs.</t>
+  </si>
+  <si>
+    <t>IAM-073</t>
+  </si>
+  <si>
+    <t>Add controlled Codex execution pipeline</t>
+  </si>
+  <si>
+    <t>Extend the IAMONIT task-agent so it can generate a task-specific Codex prompt and invoke Codex non-interactively under explicit safety controls.</t>
+  </si>
+  <si>
+    <t>The agent supports a non-mutating plan mode; execution requires an explicit flag; execution is blocked on a dirty working tree or protected branch; Codex runs only inside the repository workspace; results and exit status are captured; the workbook is never modified; no commit or push occurs automatically.</t>
+  </si>
+  <si>
+    <t>IAM-071,IAM-072</t>
+  </si>
+  <si>
+    <t>packages/task-agent/src/prompt-builder.ts; packages/task-agent/src/codex-executor.ts; packages/task-agent/src/git-preflight.ts; packages/task-agent/src/cli.ts</t>
+  </si>
+  <si>
+    <t>Plan mode is the default. Real execution requires explicit user action and must stop at human review.</t>
+  </si>
+  <si>
+    <t>The task-agent can safely prepare and explicitly launch one Codex coding task without committing, pushing, or updating the workbook.</t>
+  </si>
+  <si>
+    <t>CODE-043</t>
+  </si>
+  <si>
+    <t>Build task prompt generation and controlled Codex execution</t>
+  </si>
+  <si>
+    <t>Generate a detailed prompt from the single selected workbook task. Keep plan mode as the default. Add an explicit execution mode that invokes codex exec using Node child_process.spawn without a shell. Pass the prompt through stdin. Use workspace-write sandboxing, disable network access, capture JSONL events and the final assistant message, verify a clean Git working tree, reject protected branches, preserve the workbook checksum, and never commit or push.</t>
+  </si>
+  <si>
+    <t>Plan mode prints the exact generated prompt without invoking Codex; execution requires an explicit flag; dirty repositories and main/master branches are rejected; unsafe or unresolved task paths remain rejected; Codex output and exit code are captured; workbook checksum remains unchanged; no automatic commit, push, or tracker update occurs; unit tests cover prompt creation, argument construction, Git preflight, execution failure, and dry-run behavior.</t>
   </si>
 </sst>
 </file>
@@ -3265,15 +3301,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3971,7 +4007,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -3983,7 +4019,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4007,7 +4043,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4041,7 +4077,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="14" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4075,7 +4111,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="14" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4109,7 +4145,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="14" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4132,16 +4168,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A17:H18"/>
+    <mergeCell ref="A9:H10"/>
+    <mergeCell ref="A13:H14"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A5:H6"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A17:H18"/>
-    <mergeCell ref="A9:H10"/>
-    <mergeCell ref="A13:H14"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -5215,7 +5251,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5227,7 +5263,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -9140,57 +9176,39 @@
         <v>980</v>
       </c>
     </row>
-    <row r="74" spans="1:16" ht="64" x14ac:dyDescent="0.2">
-      <c r="A74" s="5" t="inlineStr">
-        <is>
-          <t>IAM-073</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>Developer Automation</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>Add controlled Codex execution pipeline</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+    <row r="74" spans="1:16" ht="96" x14ac:dyDescent="0.2">
+      <c r="A74" s="5" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>916</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="E74" s="5">
         <v>5</v>
       </c>
-      <c r="F74" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="G74" s="5" t="inlineStr">
-        <is>
-          <t>Extend the IAMONIT task-agent so it can generate a task-specific Codex prompt and invoke Codex non-interactively under explicit safety controls.</t>
-        </is>
-      </c>
-      <c r="H74" s="5" t="inlineStr">
-        <is>
-          <t>The agent supports a non-mutating plan mode; execution requires an explicit flag; execution is blocked on a dirty working tree or protected branch; Codex runs only inside the repository workspace; results and exit status are captured; the workbook is never modified; no commit or push occurs automatically.</t>
-        </is>
-      </c>
-      <c r="I74" s="5" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
+      <c r="F74" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>1017</v>
+      </c>
+      <c r="H74" s="5" t="s">
+        <v>1018</v>
+      </c>
+      <c r="I74" s="5" t="s">
+        <v>55</v>
       </c>
       <c r="J74" s="6">
         <v>46230</v>
       </c>
-      <c r="K74" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 10</t>
-        </is>
+      <c r="K74" s="5" t="s">
+        <v>920</v>
       </c>
       <c r="L74" s="5">
         <v>2</v>
@@ -9198,20 +9216,14 @@
       <c r="M74" s="6">
         <v>46231</v>
       </c>
-      <c r="N74" s="5" t="inlineStr">
-        <is>
-          <t>IAM-071,IAM-072</t>
-        </is>
-      </c>
-      <c r="O74" s="5" t="inlineStr">
-        <is>
-          <t>packages/task-agent/src/prompt-builder.ts; packages/task-agent/src/codex-executor.ts; packages/task-agent/src/git-preflight.ts; packages/task-agent/src/cli.ts</t>
-        </is>
-      </c>
-      <c r="P74" s="5" t="inlineStr">
-        <is>
-          <t>Plan mode is the default. Real execution requires explicit user action and must stop at human review.</t>
-        </is>
+      <c r="N74" s="5" t="s">
+        <v>1019</v>
+      </c>
+      <c r="O74" s="5" t="s">
+        <v>1020</v>
+      </c>
+      <c r="P74" s="5" t="s">
+        <v>1021</v>
       </c>
     </row>
   </sheetData>
@@ -11602,54 +11614,36 @@
         <v>981</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="32" x14ac:dyDescent="0.2">
-      <c r="A74" s="5" t="inlineStr">
-        <is>
-          <t>Sprint 10</t>
-        </is>
-      </c>
-      <c r="B74" s="5" t="inlineStr">
-        <is>
-          <t>IAM-073</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>Developer Automation</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>Add controlled Codex execution pipeline</t>
-        </is>
-      </c>
-      <c r="E74" s="5" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="F74" s="5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+    <row r="74" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+      <c r="A74" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>916</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="G74" s="5">
         <v>5</v>
       </c>
-      <c r="H74" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="I74" s="5" t="inlineStr">
-        <is>
-          <t>IAM-071,IAM-072</t>
-        </is>
-      </c>
-      <c r="J74" s="5" t="inlineStr">
-        <is>
-          <t>The task-agent can safely prepare and explicitly launch one Codex coding task without committing, pushing, or updating the workbook.</t>
-        </is>
+      <c r="H74" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I74" s="5" t="s">
+        <v>1019</v>
+      </c>
+      <c r="J74" s="5" t="s">
+        <v>1022</v>
       </c>
     </row>
   </sheetData>
@@ -19591,51 +19585,33 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="64" x14ac:dyDescent="0.2">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>CODE-043</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>Tooling</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>task-agent</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>packages/task-agent/src/prompt-builder.ts; packages/task-agent/src/codex-executor.ts; packages/task-agent/src/git-preflight.ts; packages/task-agent/src/cli.ts</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Build task prompt generation and controlled Codex execution</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>Generate a detailed prompt from the single selected workbook task. Keep plan mode as the default. Add an explicit execution mode that invokes codex exec using Node child_process.spawn without a shell. Pass the prompt through stdin. Use workspace-write sandboxing, disable network access, capture JSONL events and the final assistant message, verify a clean Git working tree, reject protected branches, preserve the workbook checksum, and never commit or push.</t>
-        </is>
-      </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>IAM-073</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>Plan mode prints the exact generated prompt without invoking Codex; execution requires an explicit flag; dirty repositories and main/master branches are rejected; unsafe or unresolved task paths remain rejected; Codex output and exit code are captured; workbook checksum remains unchanged; no automatic commit, push, or tracker update occurs; unit tests cover prompt creation, argument construction, Git preflight, execution failure, and dry-run behavior.</t>
-        </is>
-      </c>
-      <c r="I44" s="5" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
+    <row r="44" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>926</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>927</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>1024</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>1025</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>1015</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>1026</v>
+      </c>
+      <c r="I44" s="5" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
IAM-073 Complete controlled Codex execution pipeline
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2049A0ED-A1AF-494E-8777-39E52A6A1D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068F4DCC-5E9E-2B49-B828-4A3986E2149E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -3301,15 +3301,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3635,7 +3635,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4007,7 +4007,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -4019,7 +4019,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4043,7 +4043,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4077,7 +4077,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="14" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4111,7 +4111,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="14" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4145,7 +4145,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="14" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4168,16 +4168,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A17:H18"/>
+    <mergeCell ref="A9:H10"/>
+    <mergeCell ref="A13:H14"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A5:H6"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A17:H18"/>
-    <mergeCell ref="A9:H10"/>
-    <mergeCell ref="A13:H14"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -5251,7 +5251,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5263,7 +5263,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -5296,7 +5296,7 @@
       <c r="B5" s="13"/>
       <c r="D5" s="17">
         <f>COUNTIF(Backlog!F2:F500,"Done")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="13"/>
       <c r="G5" s="17">
@@ -5332,7 +5332,7 @@
       <c r="E8" s="13"/>
       <c r="G8" s="17">
         <f>SUMIF(Backlog!F2:F500,"Done",Backlog!E2:E500)</f>
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="H8" s="13"/>
     </row>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="I16">
         <f>COUNTIF(Backlog!F:F,H16)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -9193,7 +9193,7 @@
         <v>5</v>
       </c>
       <c r="F74" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G74" s="5" t="s">
         <v>1017</v>
@@ -11637,7 +11637,7 @@
         <v>5</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>1019</v>
@@ -19611,7 +19611,7 @@
         <v>1026</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-022 Correct login page task dependency
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC39DFD-21FE-0B45-A260-C16567637F5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523A407C-10A5-F949-BD1A-E29F5E96E142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -3298,15 +3298,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4004,7 +4004,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -4016,7 +4016,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4040,7 +4040,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="12" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4074,7 +4074,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4108,7 +4108,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4142,7 +4142,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4165,16 +4165,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A5:H6"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="A17:H18"/>
     <mergeCell ref="A9:H10"/>
     <mergeCell ref="A13:H14"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H6"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A4:H4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -5248,7 +5248,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5260,7 +5260,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -18991,7 +18991,7 @@
         <v>588</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>589</v>
+        <v>94</v>
       </c>
       <c r="H23" s="5" t="s">
         <v>590</v>

</xml_diff>

<commit_message>
IAM-002 Reopen Next.js app initialization
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -33,7 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DB Schema + RLS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Dependencies!$A$1:$F$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Release Checklist'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Risks &amp; Decisions'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$74</definedName>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3345" uniqueCount="1026">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1034">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3135,6 +3135,30 @@
   </si>
   <si>
     <t>Plan mode prints the exact generated prompt without invoking Codex; execution requires an explicit flag; dirty repositories and main/master branches are rejected; unsafe or unresolved task paths remain rejected; Codex output and exit code are captured; workbook checksum remains unchanged; no automatic commit, push, or tracker update occurs; unit tests cover prompt creation, argument construction, Git preflight, execution failure, and dry-run behavior.</t>
+  </si>
+  <si>
+    <t>Initialize the Next.js frontend under apps/web using TypeScript, App Router, Tailwind CSS, and ESLint as part of the existing pnpm workspace.</t>
+  </si>
+  <si>
+    <t>apps/web/package.json exists; TypeScript is configured; App Router is configured; Tailwind CSS is configured; ESLint is configured; apps/web/app/layout.tsx exists; apps/web/app/page.tsx exists; the package participates in the existing pnpm workspace; the existing root dev:web command works with the web package; pnpm --filter &lt;web-package&gt; build passes</t>
+  </si>
+  <si>
+    <t>CODE-044</t>
+  </si>
+  <si>
+    <t>web</t>
+  </si>
+  <si>
+    <t>apps/web/package.json; apps/web/app/layout.tsx; apps/web/app/page.tsx</t>
+  </si>
+  <si>
+    <t>Initialize Next.js frontend application</t>
+  </si>
+  <si>
+    <t>Initialize apps/web as a pnpm-managed Next.js application using TypeScript, App Router, Tailwind CSS, and ESLint. Keep the app directory at apps/web/app rather than apps/web/src/app so existing tracker paths remain valid. Inspect the root workspace scripts and choose a package name compatible with dev:web. Preserve the existing monorepo structure.</t>
+  </si>
+  <si>
+    <t>Next.js application exists under apps/web; package participates in the pnpm workspace; layout and home page render; Tailwind and ESLint are configured; root dev:web resolves the package; web build passes.</t>
   </si>
 </sst>
 </file>
@@ -5778,13 +5802,13 @@
         <v>5</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>59</v>
+        <v>1026</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>60</v>
+        <v>1027</v>
       </c>
       <c r="I3" s="9" t="s">
         <v>61</v>
@@ -9362,13 +9386,13 @@
         <v>5</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>49</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>60</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -18320,7 +18344,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19609,9 +19633,38 @@
         <v>13</v>
       </c>
     </row>
+    <row r="45" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+      <c r="A45" s="5" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>1029</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>1030</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>1031</v>
+      </c>
+      <c r="F45" s="5" t="s">
+        <v>1032</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>1033</v>
+      </c>
+      <c r="I45" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I44" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I44">
+  <autoFilter ref="A1:I45" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <conditionalFormatting sqref="I2:I45">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -19629,7 +19682,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I44" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I45" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
CODE-022 Align login page scope with UI shell
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1032">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1034">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3153,6 +3153,12 @@
   </si>
   <si>
     <t>Next.js application exists under apps/web; package participates in the pnpm workspace; layout and home page render; Tailwind and ESLint are configured; root dev:web resolves the package; web build passes.</t>
+  </si>
+  <si>
+    <t>Create the client-side login page UI shell with email and password fields, client-side validation, accessible labels, validation and error messages, loading/disabled-state presentation, and navigation to the registration page. Do not call the backend, store authentication state, create sessions, or redirect to the dashboard. Those behaviors belong to later integration tasks.</t>
+  </si>
+  <si>
+    <t>Login page renders email and password fields; invalid input displays clear validation messages; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and a registration navigation link is available. No backend request, authentication persistence, or dashboard redirect is implemented.</t>
   </si>
 </sst>
 </file>
@@ -19006,13 +19012,13 @@
         <v>585</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>586</v>
+        <v>1032</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>92</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>588</v>
+        <v>1033</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>25</v>
@@ -20085,7 +20091,7 @@
         <v>585</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>587</v>
+        <v>92</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>584</v>

</xml_diff>

<commit_message>
CODE-022 Build login page UI shell
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3C07D20-814B-6B41-80C8-5345DBE557B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD903231-F54D-8246-99F3-BA5E76AE8D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1034">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1032">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -1817,13 +1817,7 @@
     <t>Build login page</t>
   </si>
   <si>
-    <t>Email/password form with loading/error states.</t>
-  </si>
-  <si>
     <t>IAM-009,IAM-017</t>
-  </si>
-  <si>
-    <t>Login redirects to dashboard</t>
   </si>
   <si>
     <t>CODE-023</t>
@@ -3322,15 +3316,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4028,7 +4022,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -4040,7 +4034,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4064,7 +4058,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="12" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4098,7 +4092,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4132,7 +4126,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4166,7 +4160,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4189,16 +4183,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A5:H6"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="A17:H18"/>
     <mergeCell ref="A9:H10"/>
     <mergeCell ref="A13:H14"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H6"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A4:H4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -4222,22 +4216,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>747</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>748</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>749</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>669</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>750</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>751</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>752</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -4245,76 +4239,76 @@
         <v>524</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>751</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>752</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>753</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>754</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>755</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>756</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>757</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
+        <v>756</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>757</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>758</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>759</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="E3" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>760</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>761</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>756</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>762</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>762</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>763</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>764</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="E4" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>765</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>766</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>756</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>766</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>767</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>768</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>769</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>770</v>
-      </c>
       <c r="D5" s="5" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>112</v>
@@ -4325,19 +4319,19 @@
         <v>538</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>769</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>770</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>771</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="E6" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>772</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>773</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>756</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>774</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -4345,56 +4339,56 @@
         <v>548</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>774</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>775</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="E7" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>776</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>777</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>756</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>778</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
+        <v>777</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>778</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>779</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>780</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>781</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>782</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>783</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>784</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
+        <v>783</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>784</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>785</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>786</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>787</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>788</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>246</v>
@@ -4402,22 +4396,22 @@
     </row>
     <row r="10" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>787</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>788</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>789</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>790</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>791</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>792</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>756</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>793</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -4425,36 +4419,36 @@
         <v>580</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>792</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>793</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>794</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>795</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>796</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>797</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>798</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
+        <v>797</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>798</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>799</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>800</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>801</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>802</v>
-      </c>
       <c r="E12" s="5" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>323</v>
@@ -4486,25 +4480,25 @@
   <sheetData>
     <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>801</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>802</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>803</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>804</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>805</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>806</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>669</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>807</v>
-      </c>
       <c r="G1" s="4" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>22</v>
@@ -4512,25 +4506,25 @@
     </row>
     <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>806</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>807</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>808</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>809</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>810</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>811</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>812</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>813</v>
-      </c>
       <c r="G2" s="5" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>25</v>
@@ -4538,25 +4532,25 @@
     </row>
     <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>813</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>814</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>815</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>816</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>811</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>817</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>818</v>
-      </c>
       <c r="G3" s="5" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>25</v>
@@ -4564,22 +4558,22 @@
     </row>
     <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>297</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>818</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>819</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>820</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>821</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>822</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>823</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>296</v>
@@ -4590,22 +4584,22 @@
     </row>
     <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>823</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>824</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>825</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>826</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>827</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>828</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>829</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>302</v>
@@ -4616,25 +4610,25 @@
     </row>
     <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
+        <v>828</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>703</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>819</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>830</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>831</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>821</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>832</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>833</v>
-      </c>
       <c r="G6" s="5" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>25</v>
@@ -4642,25 +4636,25 @@
     </row>
     <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>833</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>834</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="D7" s="5" t="s">
+        <v>819</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>835</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>836</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>821</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>837</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>839</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>25</v>
@@ -4668,25 +4662,25 @@
     </row>
     <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
+        <v>838</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>839</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>840</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>841</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>842</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>843</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>844</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>845</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>846</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>25</v>
@@ -4694,22 +4688,22 @@
     </row>
     <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
+        <v>845</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>847</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="D9" s="5" t="s">
+        <v>825</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>848</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>849</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>827</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>850</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>851</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>271</v>
@@ -4720,22 +4714,22 @@
     </row>
     <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>850</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>851</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>852</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>853</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>690</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>692</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>854</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>855</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>166</v>
@@ -4746,22 +4740,22 @@
     </row>
     <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>856</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="D11" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>857</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>858</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>692</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>859</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>860</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>177</v>
@@ -4772,22 +4766,22 @@
     </row>
     <row r="12" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
+        <v>859</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>860</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>861</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="D12" s="5" t="s">
+        <v>809</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>862</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>863</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>811</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>864</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>865</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>291</v>
@@ -4844,19 +4838,19 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>866</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>867</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>868</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>869</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>870</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>426</v>
@@ -4867,140 +4861,140 @@
     </row>
     <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>869</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>870</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>871</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>872</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>873</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>122</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>168</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>390</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>390</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
+        <v>883</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>884</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>885</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>886</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>887</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E6" s="5" t="s">
+        <v>886</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>887</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>888</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>889</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>890</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>80</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
     </row>
   </sheetData>
@@ -5028,13 +5022,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>426</v>
@@ -5043,7 +5037,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -5051,10 +5045,10 @@
         <v>122</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>122</v>
@@ -5069,10 +5063,10 @@
         <v>88</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>64</v>
@@ -5087,10 +5081,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>182</v>
@@ -5102,13 +5096,13 @@
     </row>
     <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>59</v>
@@ -5120,13 +5114,13 @@
     </row>
     <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>182</v>
@@ -5141,10 +5135,10 @@
         <v>277</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>182</v>
@@ -5159,10 +5153,10 @@
         <v>335</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>339</v>
@@ -5177,10 +5171,10 @@
         <v>358</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>55</v>
@@ -5195,10 +5189,10 @@
         <v>358</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>55</v>
@@ -5210,13 +5204,13 @@
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>390</v>
@@ -5272,7 +5266,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5284,7 +5278,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -5805,10 +5799,10 @@
         <v>13</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="I3" s="9" t="s">
         <v>59</v>
@@ -5829,7 +5823,7 @@
         <v>49</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="P3" s="9"/>
     </row>
@@ -5877,7 +5871,7 @@
         <v>49</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="P4" s="9"/>
     </row>
@@ -5925,7 +5919,7 @@
         <v>70</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="P5" s="5"/>
     </row>
@@ -5973,7 +5967,7 @@
         <v>70</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="P6" s="5"/>
     </row>
@@ -6117,7 +6111,7 @@
         <v>60</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="P9" s="5"/>
     </row>
@@ -6165,7 +6159,7 @@
         <v>57</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="P10" s="5"/>
     </row>
@@ -6453,7 +6447,7 @@
         <v>129</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="P16" s="5"/>
     </row>
@@ -6501,7 +6495,7 @@
         <v>134</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="P17" s="5"/>
     </row>
@@ -6549,7 +6543,7 @@
         <v>140</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="P18" s="5"/>
     </row>
@@ -6597,7 +6591,7 @@
         <v>130</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="P19" s="5"/>
     </row>
@@ -6693,7 +6687,7 @@
         <v>156</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="P21" s="5"/>
     </row>
@@ -6741,7 +6735,7 @@
         <v>152</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="P22" s="5"/>
     </row>
@@ -6789,7 +6783,7 @@
         <v>141</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="P23" s="5"/>
     </row>
@@ -6837,7 +6831,7 @@
         <v>171</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="P24" s="5"/>
     </row>
@@ -6885,7 +6879,7 @@
         <v>135</v>
       </c>
       <c r="O25" s="5" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="P25" s="5"/>
     </row>
@@ -6933,7 +6927,7 @@
         <v>183</v>
       </c>
       <c r="O26" s="5" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="P26" s="5"/>
     </row>
@@ -7077,7 +7071,7 @@
         <v>184</v>
       </c>
       <c r="O29" s="5" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="P29" s="5"/>
     </row>
@@ -7125,7 +7119,7 @@
         <v>204</v>
       </c>
       <c r="O30" s="5" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="P30" s="5"/>
     </row>
@@ -7173,7 +7167,7 @@
         <v>200</v>
       </c>
       <c r="O31" s="5" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="P31" s="5"/>
     </row>
@@ -7221,7 +7215,7 @@
         <v>205</v>
       </c>
       <c r="O32" s="5" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="P32" s="5"/>
     </row>
@@ -7269,7 +7263,7 @@
         <v>217</v>
       </c>
       <c r="O33" s="5" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="P33" s="5"/>
     </row>
@@ -7317,7 +7311,7 @@
         <v>223</v>
       </c>
       <c r="O34" s="5" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="P34" s="5"/>
     </row>
@@ -7365,7 +7359,7 @@
         <v>228</v>
       </c>
       <c r="O35" s="5" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="P35" s="5"/>
     </row>
@@ -7413,7 +7407,7 @@
         <v>233</v>
       </c>
       <c r="O36" s="5" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="P36" s="5"/>
     </row>
@@ -7509,7 +7503,7 @@
         <v>245</v>
       </c>
       <c r="O38" s="5" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="P38" s="5"/>
     </row>
@@ -7557,7 +7551,7 @@
         <v>240</v>
       </c>
       <c r="O39" s="5" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="P39" s="5"/>
     </row>
@@ -7605,7 +7599,7 @@
         <v>240</v>
       </c>
       <c r="O40" s="5" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="P40" s="5"/>
     </row>
@@ -7701,7 +7695,7 @@
         <v>255</v>
       </c>
       <c r="O42" s="5" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="P42" s="5"/>
     </row>
@@ -7749,7 +7743,7 @@
         <v>270</v>
       </c>
       <c r="O43" s="5" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="P43" s="5"/>
     </row>
@@ -7797,7 +7791,7 @@
         <v>275</v>
       </c>
       <c r="O44" s="5" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="P44" s="5"/>
     </row>
@@ -7893,7 +7887,7 @@
         <v>286</v>
       </c>
       <c r="O46" s="5" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="P46" s="5"/>
     </row>
@@ -7941,7 +7935,7 @@
         <v>282</v>
       </c>
       <c r="O47" s="5" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="P47" s="5"/>
     </row>
@@ -7989,7 +7983,7 @@
         <v>295</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="P48" s="5"/>
     </row>
@@ -8037,7 +8031,7 @@
         <v>301</v>
       </c>
       <c r="O49" s="5" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="P49" s="5"/>
     </row>
@@ -8085,7 +8079,7 @@
         <v>271</v>
       </c>
       <c r="O50" s="5" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="P50" s="5"/>
     </row>
@@ -8133,7 +8127,7 @@
         <v>205</v>
       </c>
       <c r="O51" s="5" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="P51" s="5"/>
     </row>
@@ -8181,7 +8175,7 @@
         <v>315</v>
       </c>
       <c r="O52" s="5" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="P52" s="5"/>
     </row>
@@ -8373,7 +8367,7 @@
         <v>340</v>
       </c>
       <c r="O56" s="5" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="P56" s="5"/>
     </row>
@@ -8421,7 +8415,7 @@
         <v>345</v>
       </c>
       <c r="O57" s="5" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="P57" s="5"/>
     </row>
@@ -8469,7 +8463,7 @@
         <v>350</v>
       </c>
       <c r="O58" s="5" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="P58" s="5"/>
     </row>
@@ -8661,7 +8655,7 @@
         <v>357</v>
       </c>
       <c r="O62" s="5" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="P62" s="5"/>
     </row>
@@ -8997,7 +8991,7 @@
         <v>413</v>
       </c>
       <c r="O69" s="5" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="P69" s="5"/>
     </row>
@@ -9045,7 +9039,7 @@
         <v>420</v>
       </c>
       <c r="O70" s="5" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
       <c r="P70" s="5"/>
     </row>
@@ -9093,19 +9087,19 @@
         <v>425</v>
       </c>
       <c r="O71" s="5" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="P71" s="5"/>
     </row>
     <row r="72" spans="1:16" ht="64" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
+        <v>910</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>911</v>
+      </c>
+      <c r="C72" s="5" t="s">
         <v>912</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>913</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>914</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>67</v>
@@ -9117,10 +9111,10 @@
         <v>14</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="I72" s="5" t="s">
         <v>55</v>
@@ -9129,7 +9123,7 @@
         <v>46230</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="L72" s="5">
         <v>1</v>
@@ -9138,24 +9132,24 @@
         <v>46230</v>
       </c>
       <c r="N72" s="5" t="s">
+        <v>916</v>
+      </c>
+      <c r="O72" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="P72" s="5" t="s">
         <v>918</v>
-      </c>
-      <c r="O72" s="5" t="s">
-        <v>919</v>
-      </c>
-      <c r="P72" s="5" t="s">
-        <v>920</v>
       </c>
     </row>
     <row r="73" spans="1:16" ht="80" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>67</v>
@@ -9167,10 +9161,10 @@
         <v>13</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="I73" s="5" t="s">
         <v>55</v>
@@ -9179,7 +9173,7 @@
         <v>46230</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="L73" s="5">
         <v>1</v>
@@ -9188,24 +9182,24 @@
         <v>46230</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="O73" s="5" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="P73" s="5" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
     </row>
     <row r="74" spans="1:16" ht="96" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>67</v>
@@ -9217,10 +9211,10 @@
         <v>13</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>55</v>
@@ -9229,7 +9223,7 @@
         <v>46230</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="L74" s="5">
         <v>2</v>
@@ -9238,13 +9232,13 @@
         <v>46231</v>
       </c>
       <c r="N74" s="5" t="s">
+        <v>1014</v>
+      </c>
+      <c r="O74" s="5" t="s">
+        <v>1015</v>
+      </c>
+      <c r="P74" s="5" t="s">
         <v>1016</v>
-      </c>
-      <c r="O74" s="5" t="s">
-        <v>1017</v>
-      </c>
-      <c r="P74" s="5" t="s">
-        <v>1018</v>
       </c>
     </row>
   </sheetData>
@@ -9392,7 +9386,7 @@
         <v>49</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -11573,16 +11567,16 @@
     </row>
     <row r="72" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="B72" s="5" t="s">
+        <v>910</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>911</v>
+      </c>
+      <c r="D72" s="5" t="s">
         <v>912</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>913</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>914</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>55</v>
@@ -11597,24 +11591,24 @@
         <v>14</v>
       </c>
       <c r="I72" s="5" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>921</v>
+        <v>919</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>55</v>
@@ -11629,24 +11623,24 @@
         <v>13</v>
       </c>
       <c r="I73" s="5" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="J73" s="5" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>917</v>
+        <v>915</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>1012</v>
+        <v>1010</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>55</v>
@@ -11661,10 +11655,10 @@
         <v>13</v>
       </c>
       <c r="I74" s="5" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
     </row>
   </sheetData>
@@ -18397,7 +18391,7 @@
         <v>488</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>489</v>
@@ -18426,7 +18420,7 @@
         <v>493</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>494</v>
@@ -18455,7 +18449,7 @@
         <v>493</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>498</v>
@@ -18484,7 +18478,7 @@
         <v>493</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>502</v>
@@ -18513,7 +18507,7 @@
         <v>493</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>507</v>
@@ -18542,7 +18536,7 @@
         <v>493</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>511</v>
@@ -18571,7 +18565,7 @@
         <v>515</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>516</v>
@@ -18600,7 +18594,7 @@
         <v>515</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>520</v>
@@ -18629,7 +18623,7 @@
         <v>524</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>525</v>
@@ -18658,7 +18652,7 @@
         <v>529</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>530</v>
@@ -18687,7 +18681,7 @@
         <v>529</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>534</v>
@@ -18716,7 +18710,7 @@
         <v>538</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>539</v>
@@ -18745,7 +18739,7 @@
         <v>538</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>544</v>
@@ -18774,7 +18768,7 @@
         <v>548</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>549</v>
@@ -18803,7 +18797,7 @@
         <v>548</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>553</v>
@@ -18832,7 +18826,7 @@
         <v>548</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>558</v>
@@ -18861,7 +18855,7 @@
         <v>548</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>562</v>
@@ -18890,7 +18884,7 @@
         <v>566</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>567</v>
@@ -18919,7 +18913,7 @@
         <v>566</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>571</v>
@@ -18948,7 +18942,7 @@
         <v>575</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>576</v>
@@ -18977,7 +18971,7 @@
         <v>580</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>581</v>
@@ -18995,7 +18989,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="112" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>584</v>
       </c>
@@ -19006,27 +19000,27 @@
         <v>493</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>585</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>92</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>59</v>
@@ -19035,19 +19029,19 @@
         <v>493</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="E24" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>589</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="H24" s="5" t="s">
         <v>590</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>591</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>587</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>592</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>25</v>
@@ -19055,28 +19049,28 @@
     </row>
     <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>996</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>593</v>
+      </c>
+      <c r="F25" s="5" t="s">
         <v>594</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>998</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>595</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>596</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>135</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>25</v>
@@ -19084,28 +19078,28 @@
     </row>
     <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>135</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>25</v>
@@ -19113,28 +19107,28 @@
     </row>
     <row r="27" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>998</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="F27" s="5" t="s">
         <v>603</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>604</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>605</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>172</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>25</v>
@@ -19142,28 +19136,28 @@
     </row>
     <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="E28" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>607</v>
+      </c>
+      <c r="G28" s="5" t="s">
         <v>608</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="H28" s="5" t="s">
         <v>609</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>610</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>611</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>25</v>
@@ -19171,7 +19165,7 @@
     </row>
     <row r="29" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>59</v>
@@ -19180,19 +19174,19 @@
         <v>548</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>220</v>
       </c>
       <c r="F29" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>612</v>
+      </c>
+      <c r="H29" s="5" t="s">
         <v>613</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>614</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>615</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>25</v>
@@ -19200,7 +19194,7 @@
     </row>
     <row r="30" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>59</v>
@@ -19209,19 +19203,19 @@
         <v>548</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>225</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>224</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>25</v>
@@ -19229,7 +19223,7 @@
     </row>
     <row r="31" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>59</v>
@@ -19238,19 +19232,19 @@
         <v>548</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>230</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>229</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>25</v>
@@ -19258,7 +19252,7 @@
     </row>
     <row r="32" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>59</v>
@@ -19267,19 +19261,19 @@
         <v>548</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>266</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>25</v>
@@ -19287,7 +19281,7 @@
     </row>
     <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>59</v>
@@ -19296,19 +19290,19 @@
         <v>566</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>250</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>25</v>
@@ -19316,28 +19310,28 @@
     </row>
     <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C34" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>956</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="F34" s="5" t="s">
         <v>631</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>958</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>632</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>633</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>271</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>25</v>
@@ -19345,7 +19339,7 @@
     </row>
     <row r="35" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>59</v>
@@ -19354,19 +19348,19 @@
         <v>580</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>291</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>25</v>
@@ -19374,28 +19368,28 @@
     </row>
     <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>101</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>96</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>25</v>
@@ -19403,28 +19397,28 @@
     </row>
     <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>189</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>184</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>25</v>
@@ -19432,28 +19426,28 @@
     </row>
     <row r="38" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>124</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>117</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>25</v>
@@ -19461,28 +19455,28 @@
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="D39" s="5" t="s">
+        <v>651</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>652</v>
+      </c>
+      <c r="F39" s="5" t="s">
         <v>653</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>654</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>655</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>234</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>25</v>
@@ -19490,28 +19484,28 @@
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>339</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>656</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>657</v>
+      </c>
+      <c r="F40" s="5" t="s">
         <v>658</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>1006</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>659</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>660</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>341</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>25</v>
@@ -19519,28 +19513,28 @@
     </row>
     <row r="41" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>339</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>356</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>351</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>25</v>
@@ -19548,28 +19542,28 @@
     </row>
     <row r="42" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>921</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>922</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>923</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>924</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="F42" s="5" t="s">
         <v>925</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="G42" s="5" t="s">
+        <v>910</v>
+      </c>
+      <c r="H42" s="5" t="s">
         <v>926</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>927</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>912</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>928</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>13</v>
@@ -19577,28 +19571,28 @@
     </row>
     <row r="43" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>921</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>922</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>1006</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>1007</v>
       </c>
-      <c r="B43" s="5" t="s">
-        <v>923</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>924</v>
-      </c>
-      <c r="D43" s="5" t="s">
+      <c r="F43" s="5" t="s">
         <v>1008</v>
       </c>
-      <c r="E43" s="5" t="s">
+      <c r="G43" s="5" t="s">
+        <v>970</v>
+      </c>
+      <c r="H43" s="5" t="s">
         <v>1009</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>1010</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>972</v>
-      </c>
-      <c r="H43" s="5" t="s">
-        <v>1011</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>13</v>
@@ -19606,28 +19600,28 @@
     </row>
     <row r="44" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
+        <v>1018</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>921</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>922</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>1015</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>1019</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>1020</v>
       </c>
-      <c r="B44" s="5" t="s">
-        <v>923</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>924</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>1017</v>
-      </c>
-      <c r="E44" s="5" t="s">
+      <c r="G44" s="5" t="s">
+        <v>1010</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>1021</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>1022</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>1012</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>1023</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>13</v>
@@ -19635,28 +19629,28 @@
     </row>
     <row r="45" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C45" s="5" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E45" s="5" t="s">
         <v>1027</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="F45" s="5" t="s">
         <v>1028</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>1029</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>1030</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>57</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>13</v>
@@ -19708,19 +19702,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>666</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>667</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>668</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>669</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>670</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>671</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19728,7 +19722,7 @@
         <v>64</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>489</v>
@@ -19745,7 +19739,7 @@
         <v>64</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>494</v>
@@ -19762,7 +19756,7 @@
         <v>64</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>498</v>
@@ -19779,7 +19773,7 @@
         <v>64</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>502</v>
@@ -19796,7 +19790,7 @@
         <v>64</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>507</v>
@@ -19813,7 +19807,7 @@
         <v>64</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>511</v>
@@ -19830,7 +19824,7 @@
         <v>64</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>516</v>
@@ -19847,7 +19841,7 @@
         <v>64</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>520</v>
@@ -19864,7 +19858,7 @@
         <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>525</v>
@@ -19881,7 +19875,7 @@
         <v>64</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>530</v>
@@ -19898,7 +19892,7 @@
         <v>64</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>534</v>
@@ -19915,7 +19909,7 @@
         <v>64</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>539</v>
@@ -19932,7 +19926,7 @@
         <v>64</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>544</v>
@@ -19949,7 +19943,7 @@
         <v>64</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>549</v>
@@ -19966,7 +19960,7 @@
         <v>64</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>553</v>
@@ -19983,7 +19977,7 @@
         <v>64</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>558</v>
@@ -20000,7 +19994,7 @@
         <v>64</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>562</v>
@@ -20017,7 +20011,7 @@
         <v>64</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>567</v>
@@ -20034,7 +20028,7 @@
         <v>64</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>571</v>
@@ -20051,7 +20045,7 @@
         <v>64</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>576</v>
@@ -20068,7 +20062,7 @@
         <v>64</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>581</v>
@@ -20085,7 +20079,7 @@
         <v>59</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>585</v>
@@ -20102,16 +20096,16 @@
         <v>59</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D24" s="5" t="s">
+        <v>586</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>587</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>589</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20119,16 +20113,16 @@
         <v>59</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>135</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20136,16 +20130,16 @@
         <v>59</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>135</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20153,16 +20147,16 @@
         <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>1000</v>
+        <v>998</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>172</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20170,16 +20164,16 @@
         <v>59</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>1001</v>
+        <v>999</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="D28" s="5" t="s">
         <v>608</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>610</v>
-      </c>
       <c r="E28" s="5" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20187,16 +20181,16 @@
         <v>59</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>220</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20204,7 +20198,7 @@
         <v>59</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>1003</v>
+        <v>1001</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>225</v>
@@ -20213,7 +20207,7 @@
         <v>224</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20221,7 +20215,7 @@
         <v>59</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>230</v>
@@ -20230,7 +20224,7 @@
         <v>229</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20238,16 +20232,16 @@
         <v>59</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>266</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20255,16 +20249,16 @@
         <v>59</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>250</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20272,16 +20266,16 @@
         <v>59</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>271</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20289,16 +20283,16 @@
         <v>59</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>291</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20309,13 +20303,13 @@
         <v>101</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>96</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20326,13 +20320,13 @@
         <v>189</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>184</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20343,13 +20337,13 @@
         <v>124</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>117</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20357,16 +20351,16 @@
         <v>80</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>234</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20374,16 +20368,16 @@
         <v>339</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>341</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20394,13 +20388,13 @@
         <v>356</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>351</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
     </row>
   </sheetData>
@@ -20429,114 +20423,114 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>672</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>673</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>669</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>674</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>675</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>676</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>677</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>679</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>680</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>681</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>682</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>684</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>684</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>685</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>686</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>681</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>687</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>688</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>687</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>689</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>690</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>691</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>692</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>693</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>694</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>695</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>695</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>696</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>697</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>692</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>698</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>699</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>152</v>
@@ -20544,22 +20538,22 @@
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>698</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>699</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>700</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>701</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>702</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>703</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>704</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>157</v>
@@ -20567,186 +20561,186 @@
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>703</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>706</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>707</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>708</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>709</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>710</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>711</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>712</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>713</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>714</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>715</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>714</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>715</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>716</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>717</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>718</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="G9" s="5" t="s">
         <v>719</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>720</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>722</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>723</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>724</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>725</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>726</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>727</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>728</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>727</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>729</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>730</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>731</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>732</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>733</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>734</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>733</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>734</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>735</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>736</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>718</v>
-      </c>
-      <c r="E12" s="5" t="s">
+      <c r="G12" s="5" t="s">
         <v>737</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>738</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>738</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>739</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>729</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>740</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="F13" s="5" t="s">
         <v>741</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>731</v>
-      </c>
-      <c r="E13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>742</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>743</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>744</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>743</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>744</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>729</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>745</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>746</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>731</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>747</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>748</v>
-      </c>
       <c r="G14" s="5" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-023 Align registration page scope with UI shell
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1032">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1034">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3153,6 +3153,12 @@
   </si>
   <si>
     <t>Login page renders email and password fields; invalid input displays clear validation messages; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and a registration navigation link is available. No backend request, authentication persistence, or dashboard redirect is implemented.</t>
+  </si>
+  <si>
+    <t>Create the client-side registration page UI shell with full name, company name, email, phone, password, and role-selection fields. Include client-side validation, accessible labels, field-level validation messages, loading and disabled-state presentation, and navigation to the login page. Do not call the backend, create an account, store authentication state, create a session, persist tokens, or redirect after submission. Those behaviors belong to later integration tasks.</t>
+  </si>
+  <si>
+    <t>Registration page renders all required fields and role selection; invalid input displays clear field-level validation messages; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and a navigation link to the login page is available. No backend request, account creation, authentication persistence, session creation, or post-registration redirect is implemented.</t>
   </si>
 </sst>
 </file>
@@ -19035,13 +19041,13 @@
         <v>588</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>589</v>
+        <v>1032</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>586</v>
+        <v>92</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>590</v>
+        <v>1033</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>25</v>
@@ -20102,7 +20108,7 @@
         <v>588</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>586</v>
+        <v>92</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>587</v>

</xml_diff>

<commit_message>
CODE-023 Complete registration page UI shell
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1034">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1036">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3159,6 +3159,12 @@
   </si>
   <si>
     <t>Registration page renders all required fields and role selection; invalid input displays clear field-level validation messages; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and a navigation link to the login page is available. No backend request, account creation, authentication persistence, session creation, or post-registration redirect is implemented.</t>
+  </si>
+  <si>
+    <t>Create the client-side registration page UI shell with full name, company name, email, phone, password, required confirm-password, and role-selection fields. Require a minimum of 8 password characters and require password and confirm password to match. Include client-side validation, accessible labels and field-level errors, loading and disabled states, and navigation to /login. Do not call the backend, create an account, store authentication state, create a session or token, persist data, or redirect after submission. Those behaviors belong to later integration tasks.</t>
+  </si>
+  <si>
+    <t>Registration page renders all required fields and role selection; password requires at least 8 characters; confirm password is required and must match password; invalid input displays accessible field-level validation errors; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and navigation to /login is available. No backend call, account creation, session, token, authentication persistence, other persistence, or post-registration redirect is implemented.</t>
   </si>
 </sst>
 </file>
@@ -6138,7 +6144,7 @@
         <v>5</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>94</v>
@@ -9610,7 +9616,7 @@
         <v>5</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>57</v>
@@ -19041,16 +19047,16 @@
         <v>588</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>92</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>1033</v>
+        <v>1035</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
IAM-008 Complete authentication DTO validation
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -6096,7 +6096,7 @@
         <v>3</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>90</v>
@@ -9584,7 +9584,7 @@
         <v>3</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
CODE-001 Reopen environment configuration validation
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1036">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1040">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3165,6 +3165,18 @@
   </si>
   <si>
     <t>Registration page renders all required fields and role selection; password requires at least 8 characters; confirm password is required and must match password; invalid input displays accessible field-level validation errors; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and navigation to /login is available. No backend call, account creation, session, token, authentication persistence, other persistence, or post-registration redirect is implemented.</t>
+  </si>
+  <si>
+    <t>apps/api/src/config/env.config.ts; apps/api/src/app.module.ts; apps/api/.env.example; apps/web/.env.example</t>
+  </si>
+  <si>
+    <t>Complete environment configuration and validation</t>
+  </si>
+  <si>
+    <t>Validate required API environment variables and fail clearly during startup when required values are missing or invalid. Keep configuration typed and centralized. Add repository-safe .env.example documentation for required API variables and add frontend public-environment examples or conventions where needed, using the appropriate NEXT_PUBLIC_ prefix for browser-exposed values. Do not add real credentials, tokens, passwords, URLs containing secrets, or production values. Do not provision Supabase or perform database migrations in this task.</t>
+  </si>
+  <si>
+    <t>Required API environment values are validated; invalid or missing required values produce a clear startup failure; API and frontend example-environment files document required variables; no secrets are committed; existing development configuration continues to work; TypeScript, lint, and relevant tests pass.</t>
   </si>
 </sst>
 </file>
@@ -18403,22 +18415,22 @@
         <v>488</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>977</v>
+        <v>1036</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>489</v>
+        <v>1037</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>490</v>
+        <v>1038</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>65</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>491</v>
+        <v>1039</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="32" x14ac:dyDescent="0.2">
@@ -19734,10 +19746,10 @@
         <v>64</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>977</v>
+        <v>1036</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>489</v>
+        <v>1037</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>65</v>

</xml_diff>

<commit_message>
CODE-001 Complete environment configuration validation
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD903231-F54D-8246-99F3-BA5E76AE8D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A97464-F48F-9047-BE86-279E36B024CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1040">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1032">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -1526,15 +1526,6 @@
     <t>config</t>
   </si>
   <si>
-    <t>Create typed env validation</t>
-  </si>
-  <si>
-    <t>Validate DATABASE_URL, JWT_SECRET, SUPABASE_URL, SUPABASE_SERVICE_KEY.</t>
-  </si>
-  <si>
-    <t>App fails fast when required env missing</t>
-  </si>
-  <si>
     <t>CODE-002</t>
   </si>
   <si>
@@ -1826,12 +1817,6 @@
     <t>Build registration page</t>
   </si>
   <si>
-    <t>Role selector and transporter/car puller fields.</t>
-  </si>
-  <si>
-    <t>Registration completes successfully</t>
-  </si>
-  <si>
     <t>CODE-024</t>
   </si>
   <si>
@@ -2990,9 +2975,6 @@
     <t>Tracker file paths match the actual apps/api and apps/web workspace structure.</t>
   </si>
   <si>
-    <t>apps/api/src/config/env.ts</t>
-  </si>
-  <si>
     <t>apps/api/src/modules/auth/dto/register.dto.ts</t>
   </si>
   <si>
@@ -3153,12 +3135,6 @@
   </si>
   <si>
     <t>Login page renders email and password fields; invalid input displays clear validation messages; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and a registration navigation link is available. No backend request, authentication persistence, or dashboard redirect is implemented.</t>
-  </si>
-  <si>
-    <t>Create the client-side registration page UI shell with full name, company name, email, phone, password, and role-selection fields. Include client-side validation, accessible labels, field-level validation messages, loading and disabled-state presentation, and navigation to the login page. Do not call the backend, create an account, store authentication state, create a session, persist tokens, or redirect after submission. Those behaviors belong to later integration tasks.</t>
-  </si>
-  <si>
-    <t>Registration page renders all required fields and role selection; invalid input displays clear field-level validation messages; loading and error presentation states are supported; the submit button has appropriate disabled behavior; and a navigation link to the login page is available. No backend request, account creation, authentication persistence, session creation, or post-registration redirect is implemented.</t>
   </si>
   <si>
     <t>Create the client-side registration page UI shell with full name, company name, email, phone, password, required confirm-password, and role-selection fields. Require a minimum of 8 password characters and require password and confirm password to match. Include client-side validation, accessible labels and field-level errors, loading and disabled states, and navigation to /login. Do not call the backend, create an account, store authentication state, create a session or token, persist data, or redirect after submission. Those behaviors belong to later integration tasks.</t>
@@ -3340,15 +3316,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3662,7 +3638,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>67</c:v>
+                  <c:v>64</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
@@ -3674,7 +3650,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4046,7 +4022,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -4058,7 +4034,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4082,7 +4058,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4116,7 +4092,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="14" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4150,7 +4126,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="14" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4184,7 +4160,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="14" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4207,16 +4183,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A17:H18"/>
+    <mergeCell ref="A9:H10"/>
+    <mergeCell ref="A13:H14"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A5:H6"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A17:H18"/>
-    <mergeCell ref="A9:H10"/>
-    <mergeCell ref="A13:H14"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -4240,99 +4216,99 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>747</v>
+        <v>742</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>749</v>
+        <v>744</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>750</v>
+        <v>745</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>751</v>
+        <v>746</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>755</v>
+        <v>750</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>758</v>
+        <v>753</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>760</v>
+        <v>755</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>762</v>
+        <v>757</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>763</v>
+        <v>758</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>764</v>
+        <v>759</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>765</v>
+        <v>760</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>766</v>
+        <v>761</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>767</v>
+        <v>762</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>768</v>
+        <v>763</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>764</v>
+        <v>759</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>112</v>
@@ -4340,79 +4316,79 @@
     </row>
     <row r="6" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>769</v>
+        <v>764</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>772</v>
+        <v>767</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>774</v>
+        <v>769</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>776</v>
+        <v>771</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
+        <v>772</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>774</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>776</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>777</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>778</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>779</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>780</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>781</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>783</v>
+        <v>778</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>784</v>
+        <v>779</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>785</v>
+        <v>780</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>786</v>
+        <v>781</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>246</v>
@@ -4420,59 +4396,59 @@
     </row>
     <row r="10" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>787</v>
+        <v>782</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>788</v>
+        <v>783</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>789</v>
+        <v>784</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>790</v>
+        <v>785</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>791</v>
+        <v>786</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>792</v>
+        <v>787</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>793</v>
+        <v>788</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>794</v>
+        <v>789</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>795</v>
+        <v>790</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>797</v>
+        <v>792</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>798</v>
+        <v>793</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>799</v>
+        <v>794</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>800</v>
+        <v>795</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>781</v>
+        <v>776</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>323</v>
@@ -4504,25 +4480,25 @@
   <sheetData>
     <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>801</v>
+        <v>796</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>802</v>
+        <v>797</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>803</v>
+        <v>798</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>804</v>
+        <v>799</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>805</v>
+        <v>800</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>22</v>
@@ -4530,25 +4506,25 @@
     </row>
     <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>802</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>803</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>804</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>805</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>806</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>807</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>808</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>809</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>810</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>811</v>
-      </c>
       <c r="G2" s="5" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>25</v>
@@ -4556,25 +4532,25 @@
     </row>
     <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>812</v>
+        <v>807</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>813</v>
+        <v>808</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>814</v>
+        <v>809</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>815</v>
+        <v>810</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>816</v>
+        <v>811</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>25</v>
@@ -4582,22 +4558,22 @@
     </row>
     <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>817</v>
+        <v>812</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>297</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>818</v>
+        <v>813</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>820</v>
+        <v>815</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>821</v>
+        <v>816</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>296</v>
@@ -4608,22 +4584,22 @@
     </row>
     <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>817</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>818</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>819</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>821</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>822</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>823</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>824</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>825</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>826</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>827</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>302</v>
@@ -4634,25 +4610,25 @@
     </row>
     <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>829</v>
+        <v>824</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>703</v>
+        <v>698</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>830</v>
+        <v>825</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>831</v>
+        <v>826</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>25</v>
@@ -4660,25 +4636,25 @@
     </row>
     <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
+        <v>827</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>828</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>814</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>832</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>833</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>834</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>819</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>835</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>836</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>837</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>25</v>
@@ -4686,25 +4662,25 @@
     </row>
     <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
+        <v>833</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>834</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>835</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>836</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>837</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>838</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>839</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>840</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>841</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>842</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>843</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>844</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>25</v>
@@ -4712,22 +4688,22 @@
     </row>
     <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>845</v>
+        <v>840</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>846</v>
+        <v>841</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>847</v>
+        <v>842</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>825</v>
+        <v>820</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>848</v>
+        <v>843</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>849</v>
+        <v>844</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>271</v>
@@ -4738,22 +4714,22 @@
     </row>
     <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>850</v>
+        <v>845</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>852</v>
+        <v>847</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>853</v>
+        <v>848</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>166</v>
@@ -4764,22 +4740,22 @@
     </row>
     <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>854</v>
+        <v>849</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>855</v>
+        <v>850</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>856</v>
+        <v>851</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>857</v>
+        <v>852</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>858</v>
+        <v>853</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>177</v>
@@ -4790,22 +4766,22 @@
     </row>
     <row r="12" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>859</v>
+        <v>854</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>861</v>
+        <v>856</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>862</v>
+        <v>857</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>863</v>
+        <v>858</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>291</v>
@@ -4862,19 +4838,19 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>864</v>
+        <v>859</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>865</v>
+        <v>860</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>866</v>
+        <v>861</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>867</v>
+        <v>862</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>868</v>
+        <v>863</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>426</v>
@@ -4885,140 +4861,140 @@
     </row>
     <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>869</v>
+        <v>864</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>871</v>
+        <v>866</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>872</v>
+        <v>867</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>122</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>874</v>
+        <v>869</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>865</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>870</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>875</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>876</v>
+        <v>871</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>877</v>
+        <v>872</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>878</v>
+        <v>873</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>168</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>879</v>
+        <v>874</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>390</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>880</v>
+        <v>875</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>870</v>
+        <v>865</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>881</v>
+        <v>876</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>882</v>
+        <v>877</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>390</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>873</v>
+        <v>868</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>883</v>
+        <v>878</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>885</v>
+        <v>880</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>886</v>
+        <v>881</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>887</v>
+        <v>882</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>889</v>
+        <v>884</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>884</v>
+        <v>879</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>890</v>
+        <v>885</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>891</v>
+        <v>886</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>80</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>888</v>
+        <v>883</v>
       </c>
     </row>
   </sheetData>
@@ -5046,13 +5022,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>892</v>
+        <v>887</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>426</v>
@@ -5061,7 +5037,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -5069,10 +5045,10 @@
         <v>122</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>895</v>
+        <v>890</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>122</v>
@@ -5087,10 +5063,10 @@
         <v>88</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>897</v>
+        <v>892</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>64</v>
@@ -5105,10 +5081,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>898</v>
+        <v>893</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>182</v>
@@ -5120,13 +5096,13 @@
     </row>
     <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>899</v>
+        <v>894</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>900</v>
+        <v>895</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>59</v>
@@ -5138,13 +5114,13 @@
     </row>
     <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>902</v>
+        <v>897</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>182</v>
@@ -5159,10 +5135,10 @@
         <v>277</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>903</v>
+        <v>898</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>182</v>
@@ -5177,10 +5153,10 @@
         <v>335</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>905</v>
+        <v>900</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>339</v>
@@ -5195,10 +5171,10 @@
         <v>358</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>906</v>
+        <v>901</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>55</v>
@@ -5213,10 +5189,10 @@
         <v>358</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>907</v>
+        <v>902</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>896</v>
+        <v>891</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>55</v>
@@ -5228,13 +5204,13 @@
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>908</v>
+        <v>903</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>909</v>
+        <v>904</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>904</v>
+        <v>899</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>390</v>
@@ -5290,7 +5266,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5302,7 +5278,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -5335,7 +5311,7 @@
       <c r="B5" s="13"/>
       <c r="D5" s="17">
         <f>COUNTIF(Backlog!F2:F500,"Done")</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E5" s="13"/>
       <c r="G5" s="17">
@@ -5366,12 +5342,12 @@
       <c r="B8" s="13"/>
       <c r="D8" s="17">
         <f>SUM(Backlog!E2:E500)</f>
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="E8" s="13"/>
       <c r="G8" s="17">
         <f>SUMIF(Backlog!F2:F500,"Done",Backlog!E2:E500)</f>
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="H8" s="13"/>
     </row>
@@ -5412,7 +5388,7 @@
       </c>
       <c r="C12">
         <f>COUNTIFS(Backlog!K:K,A12,Backlog!F:F,"Done")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D12">
         <f>COUNTIFS(Backlog!K:K,A12,Backlog!F:F,"Blocked")</f>
@@ -5424,14 +5400,14 @@
       </c>
       <c r="F12" s="3">
         <f t="shared" ref="F12:F20" si="0">IF(B12=0,0,C12/B12)</f>
-        <v>0.33333333333333331</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H12" t="s">
         <v>25</v>
       </c>
       <c r="I12">
         <f>COUNTIF(Backlog!F:F,H12)</f>
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -5559,7 +5535,7 @@
       </c>
       <c r="I16">
         <f>COUNTIF(Backlog!F:F,H16)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -5823,10 +5799,10 @@
         <v>13</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>1022</v>
+        <v>1016</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>1023</v>
+        <v>1017</v>
       </c>
       <c r="I3" s="9" t="s">
         <v>59</v>
@@ -5847,7 +5823,7 @@
         <v>49</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>927</v>
+        <v>922</v>
       </c>
       <c r="P3" s="9"/>
     </row>
@@ -5895,7 +5871,7 @@
         <v>49</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>928</v>
+        <v>923</v>
       </c>
       <c r="P4" s="9"/>
     </row>
@@ -5916,7 +5892,7 @@
         <v>3</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>68</v>
@@ -5943,7 +5919,7 @@
         <v>70</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>929</v>
+        <v>924</v>
       </c>
       <c r="P5" s="5"/>
     </row>
@@ -5991,7 +5967,7 @@
         <v>70</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>930</v>
+        <v>925</v>
       </c>
       <c r="P6" s="5"/>
     </row>
@@ -6135,7 +6111,7 @@
         <v>60</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>931</v>
+        <v>926</v>
       </c>
       <c r="P9" s="5"/>
     </row>
@@ -6183,7 +6159,7 @@
         <v>57</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>932</v>
+        <v>927</v>
       </c>
       <c r="P10" s="5"/>
     </row>
@@ -6471,7 +6447,7 @@
         <v>129</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>933</v>
+        <v>928</v>
       </c>
       <c r="P16" s="5"/>
     </row>
@@ -6519,7 +6495,7 @@
         <v>134</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>934</v>
+        <v>929</v>
       </c>
       <c r="P17" s="5"/>
     </row>
@@ -6567,7 +6543,7 @@
         <v>140</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>935</v>
+        <v>930</v>
       </c>
       <c r="P18" s="5"/>
     </row>
@@ -6615,7 +6591,7 @@
         <v>130</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>936</v>
+        <v>931</v>
       </c>
       <c r="P19" s="5"/>
     </row>
@@ -6711,7 +6687,7 @@
         <v>156</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>937</v>
+        <v>932</v>
       </c>
       <c r="P21" s="5"/>
     </row>
@@ -6759,7 +6735,7 @@
         <v>152</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="P22" s="5"/>
     </row>
@@ -6807,7 +6783,7 @@
         <v>141</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>939</v>
+        <v>934</v>
       </c>
       <c r="P23" s="5"/>
     </row>
@@ -6855,7 +6831,7 @@
         <v>171</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>940</v>
+        <v>935</v>
       </c>
       <c r="P24" s="5"/>
     </row>
@@ -6903,7 +6879,7 @@
         <v>135</v>
       </c>
       <c r="O25" s="5" t="s">
-        <v>941</v>
+        <v>936</v>
       </c>
       <c r="P25" s="5"/>
     </row>
@@ -6951,7 +6927,7 @@
         <v>183</v>
       </c>
       <c r="O26" s="5" t="s">
-        <v>942</v>
+        <v>937</v>
       </c>
       <c r="P26" s="5"/>
     </row>
@@ -7095,7 +7071,7 @@
         <v>184</v>
       </c>
       <c r="O29" s="5" t="s">
-        <v>943</v>
+        <v>938</v>
       </c>
       <c r="P29" s="5"/>
     </row>
@@ -7143,7 +7119,7 @@
         <v>204</v>
       </c>
       <c r="O30" s="5" t="s">
-        <v>944</v>
+        <v>939</v>
       </c>
       <c r="P30" s="5"/>
     </row>
@@ -7191,7 +7167,7 @@
         <v>200</v>
       </c>
       <c r="O31" s="5" t="s">
-        <v>945</v>
+        <v>940</v>
       </c>
       <c r="P31" s="5"/>
     </row>
@@ -7239,7 +7215,7 @@
         <v>205</v>
       </c>
       <c r="O32" s="5" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="P32" s="5"/>
     </row>
@@ -7287,7 +7263,7 @@
         <v>217</v>
       </c>
       <c r="O33" s="5" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="P33" s="5"/>
     </row>
@@ -7335,7 +7311,7 @@
         <v>223</v>
       </c>
       <c r="O34" s="5" t="s">
-        <v>948</v>
+        <v>943</v>
       </c>
       <c r="P34" s="5"/>
     </row>
@@ -7383,7 +7359,7 @@
         <v>228</v>
       </c>
       <c r="O35" s="5" t="s">
-        <v>949</v>
+        <v>944</v>
       </c>
       <c r="P35" s="5"/>
     </row>
@@ -7431,7 +7407,7 @@
         <v>233</v>
       </c>
       <c r="O36" s="5" t="s">
-        <v>950</v>
+        <v>945</v>
       </c>
       <c r="P36" s="5"/>
     </row>
@@ -7527,7 +7503,7 @@
         <v>245</v>
       </c>
       <c r="O38" s="5" t="s">
-        <v>951</v>
+        <v>946</v>
       </c>
       <c r="P38" s="5"/>
     </row>
@@ -7575,7 +7551,7 @@
         <v>240</v>
       </c>
       <c r="O39" s="5" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
       <c r="P39" s="5"/>
     </row>
@@ -7623,7 +7599,7 @@
         <v>240</v>
       </c>
       <c r="O40" s="5" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="P40" s="5"/>
     </row>
@@ -7719,7 +7695,7 @@
         <v>255</v>
       </c>
       <c r="O42" s="5" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
       <c r="P42" s="5"/>
     </row>
@@ -7767,7 +7743,7 @@
         <v>270</v>
       </c>
       <c r="O43" s="5" t="s">
-        <v>955</v>
+        <v>950</v>
       </c>
       <c r="P43" s="5"/>
     </row>
@@ -7815,7 +7791,7 @@
         <v>275</v>
       </c>
       <c r="O44" s="5" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="P44" s="5"/>
     </row>
@@ -7911,7 +7887,7 @@
         <v>286</v>
       </c>
       <c r="O46" s="5" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
       <c r="P46" s="5"/>
     </row>
@@ -7959,7 +7935,7 @@
         <v>282</v>
       </c>
       <c r="O47" s="5" t="s">
-        <v>958</v>
+        <v>953</v>
       </c>
       <c r="P47" s="5"/>
     </row>
@@ -8007,7 +7983,7 @@
         <v>295</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="P48" s="5"/>
     </row>
@@ -8055,7 +8031,7 @@
         <v>301</v>
       </c>
       <c r="O49" s="5" t="s">
-        <v>960</v>
+        <v>955</v>
       </c>
       <c r="P49" s="5"/>
     </row>
@@ -8103,7 +8079,7 @@
         <v>271</v>
       </c>
       <c r="O50" s="5" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
       <c r="P50" s="5"/>
     </row>
@@ -8151,7 +8127,7 @@
         <v>205</v>
       </c>
       <c r="O51" s="5" t="s">
-        <v>962</v>
+        <v>957</v>
       </c>
       <c r="P51" s="5"/>
     </row>
@@ -8199,7 +8175,7 @@
         <v>315</v>
       </c>
       <c r="O52" s="5" t="s">
-        <v>963</v>
+        <v>958</v>
       </c>
       <c r="P52" s="5"/>
     </row>
@@ -8391,7 +8367,7 @@
         <v>340</v>
       </c>
       <c r="O56" s="5" t="s">
-        <v>964</v>
+        <v>959</v>
       </c>
       <c r="P56" s="5"/>
     </row>
@@ -8439,7 +8415,7 @@
         <v>345</v>
       </c>
       <c r="O57" s="5" t="s">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="P57" s="5"/>
     </row>
@@ -8487,7 +8463,7 @@
         <v>350</v>
       </c>
       <c r="O58" s="5" t="s">
-        <v>966</v>
+        <v>961</v>
       </c>
       <c r="P58" s="5"/>
     </row>
@@ -8679,7 +8655,7 @@
         <v>357</v>
       </c>
       <c r="O62" s="5" t="s">
-        <v>967</v>
+        <v>962</v>
       </c>
       <c r="P62" s="5"/>
     </row>
@@ -9015,7 +8991,7 @@
         <v>413</v>
       </c>
       <c r="O69" s="5" t="s">
-        <v>968</v>
+        <v>963</v>
       </c>
       <c r="P69" s="5"/>
     </row>
@@ -9063,7 +9039,7 @@
         <v>420</v>
       </c>
       <c r="O70" s="5" t="s">
-        <v>969</v>
+        <v>964</v>
       </c>
       <c r="P70" s="5"/>
     </row>
@@ -9111,19 +9087,19 @@
         <v>425</v>
       </c>
       <c r="O71" s="5" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="P71" s="5"/>
     </row>
     <row r="72" spans="1:16" ht="64" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>67</v>
@@ -9135,10 +9111,10 @@
         <v>14</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>913</v>
+        <v>908</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>914</v>
+        <v>909</v>
       </c>
       <c r="I72" s="5" t="s">
         <v>55</v>
@@ -9147,7 +9123,7 @@
         <v>46230</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="L72" s="5">
         <v>1</v>
@@ -9156,24 +9132,24 @@
         <v>46230</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="O72" s="5" t="s">
-        <v>917</v>
+        <v>912</v>
       </c>
       <c r="P72" s="5" t="s">
-        <v>918</v>
+        <v>913</v>
       </c>
     </row>
     <row r="73" spans="1:16" ht="80" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>971</v>
+        <v>966</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>67</v>
@@ -9185,10 +9161,10 @@
         <v>13</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>972</v>
+        <v>967</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>973</v>
+        <v>968</v>
       </c>
       <c r="I73" s="5" t="s">
         <v>55</v>
@@ -9197,7 +9173,7 @@
         <v>46230</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="L73" s="5">
         <v>1</v>
@@ -9206,24 +9182,24 @@
         <v>46230</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="O73" s="5" t="s">
-        <v>974</v>
+        <v>969</v>
       </c>
       <c r="P73" s="5" t="s">
-        <v>975</v>
+        <v>970</v>
       </c>
     </row>
     <row r="74" spans="1:16" ht="96" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>1010</v>
+        <v>1004</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>1011</v>
+        <v>1005</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>67</v>
@@ -9235,10 +9211,10 @@
         <v>13</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>1012</v>
+        <v>1006</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>1013</v>
+        <v>1007</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>55</v>
@@ -9247,7 +9223,7 @@
         <v>46230</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="L74" s="5">
         <v>2</v>
@@ -9256,13 +9232,13 @@
         <v>46231</v>
       </c>
       <c r="N74" s="5" t="s">
-        <v>1014</v>
+        <v>1008</v>
       </c>
       <c r="O74" s="5" t="s">
-        <v>1015</v>
+        <v>1009</v>
       </c>
       <c r="P74" s="5" t="s">
-        <v>1016</v>
+        <v>1010</v>
       </c>
     </row>
   </sheetData>
@@ -9410,7 +9386,7 @@
         <v>49</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>1023</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9468,7 +9444,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>70</v>
@@ -11591,16 +11567,16 @@
     </row>
     <row r="72" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>912</v>
+        <v>907</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>55</v>
@@ -11615,24 +11591,24 @@
         <v>14</v>
       </c>
       <c r="I72" s="5" t="s">
-        <v>916</v>
+        <v>911</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>919</v>
+        <v>914</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>971</v>
+        <v>966</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>55</v>
@@ -11647,24 +11623,24 @@
         <v>13</v>
       </c>
       <c r="I73" s="5" t="s">
-        <v>910</v>
+        <v>905</v>
       </c>
       <c r="J73" s="5" t="s">
-        <v>976</v>
+        <v>971</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>915</v>
+        <v>910</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>1010</v>
+        <v>1004</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>911</v>
+        <v>906</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>1011</v>
+        <v>1005</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>55</v>
@@ -11679,10 +11655,10 @@
         <v>13</v>
       </c>
       <c r="I74" s="5" t="s">
-        <v>1014</v>
+        <v>1008</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>1017</v>
+        <v>1011</v>
       </c>
     </row>
   </sheetData>
@@ -18404,7 +18380,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>487</v>
       </c>
@@ -18415,48 +18391,48 @@
         <v>488</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>1036</v>
+        <v>1028</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>1037</v>
+        <v>1029</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>1038</v>
+        <v>1030</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>65</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>1039</v>
+        <v>1031</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>978</v>
+        <v>972</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>87</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>13</v>
@@ -18464,28 +18440,28 @@
     </row>
     <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>979</v>
+        <v>973</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>87</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>13</v>
@@ -18493,28 +18469,28 @@
     </row>
     <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>980</v>
+        <v>974</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>502</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>503</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>504</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>505</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>25</v>
@@ -18522,28 +18498,28 @@
     </row>
     <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>981</v>
+        <v>975</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>125</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>25</v>
@@ -18551,28 +18527,28 @@
     </row>
     <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>982</v>
+        <v>976</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>130</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>25</v>
@@ -18580,28 +18556,28 @@
     </row>
     <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>983</v>
+        <v>977</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>141</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>25</v>
@@ -18609,28 +18585,28 @@
     </row>
     <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>141</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>25</v>
@@ -18638,28 +18614,28 @@
     </row>
     <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>985</v>
+        <v>979</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>177</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>25</v>
@@ -18667,28 +18643,28 @@
     </row>
     <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>986</v>
+        <v>980</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>161</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>25</v>
@@ -18696,28 +18672,28 @@
     </row>
     <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>987</v>
+        <v>981</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>161</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>25</v>
@@ -18725,28 +18701,28 @@
     </row>
     <row r="13" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>982</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="G13" s="5" t="s">
         <v>538</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>988</v>
-      </c>
-      <c r="E13" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>539</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>540</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>541</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>542</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>25</v>
@@ -18754,28 +18730,28 @@
     </row>
     <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>542</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>538</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>938</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>544</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>545</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>541</v>
-      </c>
       <c r="H14" s="5" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>25</v>
@@ -18783,28 +18759,28 @@
     </row>
     <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>989</v>
+        <v>983</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>195</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>25</v>
@@ -18812,28 +18788,28 @@
     </row>
     <row r="16" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>990</v>
+        <v>984</v>
       </c>
       <c r="E16" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>552</v>
+      </c>
+      <c r="H16" s="5" t="s">
         <v>553</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>554</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>555</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>556</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>25</v>
@@ -18841,28 +18817,28 @@
     </row>
     <row r="17" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>25</v>
@@ -18870,28 +18846,28 @@
     </row>
     <row r="18" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>213</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>25</v>
@@ -18899,28 +18875,28 @@
     </row>
     <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>991</v>
+        <v>985</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>240</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>25</v>
@@ -18928,28 +18904,28 @@
     </row>
     <row r="20" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>992</v>
+        <v>986</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>240</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>25</v>
@@ -18957,28 +18933,28 @@
     </row>
     <row r="21" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>993</v>
+        <v>987</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>262</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>25</v>
@@ -18986,28 +18962,28 @@
     </row>
     <row r="22" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>282</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>25</v>
@@ -19015,57 +18991,57 @@
     </row>
     <row r="23" spans="1:9" ht="112" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>1030</v>
+        <v>1024</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>92</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>1031</v>
+        <v>1025</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="160" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>995</v>
+        <v>989</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>1034</v>
+        <v>1026</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>92</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>1035</v>
+        <v>1027</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>13</v>
@@ -19073,28 +19049,28 @@
     </row>
     <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
-        <v>591</v>
+        <v>586</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>592</v>
+        <v>587</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>135</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>595</v>
+        <v>590</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>25</v>
@@ -19102,28 +19078,28 @@
     </row>
     <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>587</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>991</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>592</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>997</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>597</v>
-      </c>
       <c r="F26" s="5" t="s">
-        <v>598</v>
+        <v>593</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>135</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>25</v>
@@ -19131,28 +19107,28 @@
     </row>
     <row r="27" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>600</v>
+        <v>595</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>601</v>
+        <v>596</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>172</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>604</v>
+        <v>599</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>25</v>
@@ -19160,28 +19136,28 @@
     </row>
     <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>993</v>
+      </c>
+      <c r="E28" s="5" t="s">
         <v>601</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>999</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>606</v>
-      </c>
       <c r="F28" s="5" t="s">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>25</v>
@@ -19189,28 +19165,28 @@
     </row>
     <row r="29" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>1000</v>
+        <v>994</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>220</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>613</v>
+        <v>608</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>25</v>
@@ -19218,28 +19194,28 @@
     </row>
     <row r="30" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>614</v>
+        <v>609</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>1001</v>
+        <v>995</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>225</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>615</v>
+        <v>610</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>224</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>616</v>
+        <v>611</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>25</v>
@@ -19247,28 +19223,28 @@
     </row>
     <row r="31" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>1002</v>
+        <v>996</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>230</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>229</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>619</v>
+        <v>614</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>25</v>
@@ -19276,28 +19252,28 @@
     </row>
     <row r="32" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>620</v>
+        <v>615</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>1003</v>
+        <v>997</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>621</v>
+        <v>616</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>266</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>623</v>
+        <v>618</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>25</v>
@@ -19305,28 +19281,28 @@
     </row>
     <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>250</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>25</v>
@@ -19334,28 +19310,28 @@
     </row>
     <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>629</v>
+        <v>624</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>271</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>25</v>
@@ -19363,28 +19339,28 @@
     </row>
     <row r="35" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>291</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="I35" s="5" t="s">
         <v>25</v>
@@ -19392,28 +19368,28 @@
     </row>
     <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>101</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>639</v>
+        <v>634</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>640</v>
+        <v>635</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>96</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>641</v>
+        <v>636</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>25</v>
@@ -19421,28 +19397,28 @@
     </row>
     <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>189</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>184</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>25</v>
@@ -19450,28 +19426,28 @@
     </row>
     <row r="38" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>124</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>117</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>649</v>
+        <v>644</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>25</v>
@@ -19479,28 +19455,28 @@
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>650</v>
+        <v>645</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>638</v>
+        <v>633</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>234</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>25</v>
@@ -19508,28 +19484,28 @@
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>339</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>1004</v>
+        <v>998</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>341</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>25</v>
@@ -19537,28 +19513,28 @@
     </row>
     <row r="41" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>339</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>661</v>
+        <v>656</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>356</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>662</v>
+        <v>657</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>663</v>
+        <v>658</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>351</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>664</v>
+        <v>659</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>25</v>
@@ -19566,28 +19542,28 @@
     </row>
     <row r="42" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>916</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>918</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="F42" s="5" t="s">
         <v>920</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="G42" s="5" t="s">
+        <v>905</v>
+      </c>
+      <c r="H42" s="5" t="s">
         <v>921</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>922</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>923</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>924</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>925</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>910</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>926</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>13</v>
@@ -19595,28 +19571,28 @@
     </row>
     <row r="43" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
-        <v>1005</v>
+        <v>999</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>1006</v>
+        <v>1000</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>1007</v>
+        <v>1001</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>1008</v>
+        <v>1002</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>1009</v>
+        <v>1003</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>13</v>
@@ -19624,28 +19600,28 @@
     </row>
     <row r="44" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>921</v>
+        <v>916</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>922</v>
+        <v>917</v>
       </c>
       <c r="D44" s="5" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>1013</v>
+      </c>
+      <c r="F44" s="5" t="s">
+        <v>1014</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>1004</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>1015</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>1019</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>1020</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>1010</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>1021</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>13</v>
@@ -19653,28 +19629,28 @@
     </row>
     <row r="45" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>1024</v>
+        <v>1018</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>1025</v>
+        <v>1019</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>1026</v>
+        <v>1020</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>1027</v>
+        <v>1021</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>1028</v>
+        <v>1022</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>57</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>1029</v>
+        <v>1023</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>13</v>
@@ -19726,30 +19702,30 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>669</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>64</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>1036</v>
+        <v>1028</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>1037</v>
+        <v>1029</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>65</v>
@@ -19763,16 +19739,16 @@
         <v>64</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>978</v>
+        <v>972</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19780,16 +19756,16 @@
         <v>64</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>979</v>
+        <v>973</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>87</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19797,16 +19773,16 @@
         <v>64</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>980</v>
+        <v>974</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19814,16 +19790,16 @@
         <v>64</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>981</v>
+        <v>975</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>125</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19831,16 +19807,16 @@
         <v>64</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>982</v>
+        <v>976</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>130</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19848,16 +19824,16 @@
         <v>64</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>983</v>
+        <v>977</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>141</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19865,16 +19841,16 @@
         <v>64</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>984</v>
+        <v>978</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>141</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19882,16 +19858,16 @@
         <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>985</v>
+        <v>979</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>177</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19899,16 +19875,16 @@
         <v>64</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>986</v>
+        <v>980</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>161</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19916,16 +19892,16 @@
         <v>64</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>987</v>
+        <v>981</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>161</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19933,16 +19909,16 @@
         <v>64</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>988</v>
+        <v>982</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19950,16 +19926,16 @@
         <v>64</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>938</v>
+        <v>933</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19967,16 +19943,16 @@
         <v>64</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>989</v>
+        <v>983</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>195</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -19984,16 +19960,16 @@
         <v>64</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>990</v>
+        <v>984</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20001,16 +19977,16 @@
         <v>64</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>946</v>
+        <v>941</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20018,16 +19994,16 @@
         <v>64</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>947</v>
+        <v>942</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>213</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20035,16 +20011,16 @@
         <v>64</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>991</v>
+        <v>985</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>240</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20052,16 +20028,16 @@
         <v>64</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>992</v>
+        <v>986</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>240</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20069,16 +20045,16 @@
         <v>64</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>993</v>
+        <v>987</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>262</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20086,16 +20062,16 @@
         <v>64</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>957</v>
+        <v>952</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>282</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20103,16 +20079,16 @@
         <v>59</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>994</v>
+        <v>988</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>92</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20120,16 +20096,16 @@
         <v>59</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>995</v>
+        <v>989</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>92</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20137,16 +20113,16 @@
         <v>59</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>996</v>
+        <v>990</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>135</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>591</v>
+        <v>586</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20154,16 +20130,16 @@
         <v>59</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>997</v>
+        <v>991</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>135</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>596</v>
+        <v>591</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20171,16 +20147,16 @@
         <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>998</v>
+        <v>992</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>172</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>600</v>
+        <v>595</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20188,16 +20164,16 @@
         <v>59</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>999</v>
+        <v>993</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20205,16 +20181,16 @@
         <v>59</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>1000</v>
+        <v>994</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>220</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20222,7 +20198,7 @@
         <v>59</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>1001</v>
+        <v>995</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>225</v>
@@ -20231,7 +20207,7 @@
         <v>224</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>614</v>
+        <v>609</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20239,7 +20215,7 @@
         <v>59</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>1002</v>
+        <v>996</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>230</v>
@@ -20248,7 +20224,7 @@
         <v>229</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20256,16 +20232,16 @@
         <v>59</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>1003</v>
+        <v>997</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>621</v>
+        <v>616</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>266</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>620</v>
+        <v>615</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20273,16 +20249,16 @@
         <v>59</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>953</v>
+        <v>948</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>250</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>624</v>
+        <v>619</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20290,16 +20266,16 @@
         <v>59</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>956</v>
+        <v>951</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>271</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>628</v>
+        <v>623</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20307,16 +20283,16 @@
         <v>59</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>291</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20327,13 +20303,13 @@
         <v>101</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>639</v>
+        <v>634</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>96</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>637</v>
+        <v>632</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20344,13 +20320,13 @@
         <v>189</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>184</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20361,13 +20337,13 @@
         <v>124</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>117</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20375,16 +20351,16 @@
         <v>80</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>234</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>650</v>
+        <v>645</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20392,16 +20368,16 @@
         <v>339</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>1004</v>
+        <v>998</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>341</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20412,13 +20388,13 @@
         <v>356</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>662</v>
+        <v>657</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>351</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
     </row>
   </sheetData>
@@ -20447,114 +20423,114 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>666</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>668</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>670</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>671</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>667</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>672</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>673</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>674</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>671</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>675</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>676</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>677</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>678</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>679</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>680</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>681</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>682</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
+        <v>671</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>678</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>679</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>680</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>676</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>684</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>679</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>685</v>
-      </c>
-      <c r="F3" s="5" t="s">
+      <c r="G3" s="5" t="s">
         <v>681</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>686</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>682</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>684</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>685</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>686</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>687</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>688</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>689</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>690</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>691</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>692</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>693</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>694</v>
+        <v>689</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>695</v>
+        <v>690</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>696</v>
+        <v>691</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>697</v>
+        <v>692</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>152</v>
@@ -20562,22 +20538,22 @@
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>698</v>
+        <v>693</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>699</v>
+        <v>694</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>700</v>
+        <v>695</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>702</v>
+        <v>697</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>157</v>
@@ -20585,186 +20561,186 @@
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>698</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>699</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>703</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>704</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>705</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>706</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>707</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>708</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>703</v>
+        <v>698</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>711</v>
+        <v>706</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>712</v>
+        <v>707</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>713</v>
+        <v>708</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>711</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>712</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>714</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>715</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>716</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>717</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>718</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>719</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>715</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>716</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>717</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>718</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>719</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>720</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>721</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>722</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>723</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>724</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>725</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>726</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>723</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>724</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>725</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>726</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>727</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>728</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>729</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>730</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>731</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>732</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>734</v>
+        <v>729</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>716</v>
+        <v>711</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>735</v>
+        <v>730</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>737</v>
+        <v>732</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>738</v>
+        <v>733</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>739</v>
+        <v>734</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>743</v>
+        <v>738</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>729</v>
+        <v>724</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>745</v>
+        <v>740</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>746</v>
+        <v>741</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>742</v>
+        <v>737</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-045 Add local Supabase configuration task
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -32,8 +32,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DB Schema + RLS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Dependencies!$A$1:$F$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Release Checklist'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Risks &amp; Decisions'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$74</definedName>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="1032">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3368" uniqueCount="1037">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3153,6 +3153,21 @@
   </si>
   <si>
     <t>Required API environment values are validated; invalid or missing required values produce a clear startup failure; API and frontend example-environment files document required variables; no secrets are committed; existing development configuration continues to work; TypeScript, lint, and relevant tests pass.</t>
+  </si>
+  <si>
+    <t>CODE-045</t>
+  </si>
+  <si>
+    <t>supabase</t>
+  </si>
+  <si>
+    <t>Initialize local Supabase configuration</t>
+  </si>
+  <si>
+    <t>Initialize repository-local Supabase configuration without secrets. Create supabase/config.toml using safe local-development settings and the standard migration directory expected by the project. Do not provision a hosted Supabase project, access credentials, configure production values, or create database migrations. Hosted-project creation, connection-string configuration, database reachability, and external connection verification remain manual IAM-006 completion requirements.</t>
+  </si>
+  <si>
+    <t>supabase/config.toml exists; it contains no credentials, tokens, passwords, or production secrets; local Supabase project and migration discovery settings are configured; the repository structure supports the documented local migration workflow; configuration syntax is valid; and no hosted Supabase project or database migration is created.</t>
   </si>
 </sst>
 </file>
@@ -18338,7 +18353,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19656,9 +19671,38 @@
         <v>13</v>
       </c>
     </row>
+    <row r="46" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+      <c r="A46" s="5" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>1034</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>1035</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>1036</v>
+      </c>
+      <c r="I46" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I45" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I45">
+  <autoFilter ref="A1:I46" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <conditionalFormatting sqref="I2:I46">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -19676,7 +19720,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I45" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I46" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19690,7 +19734,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -20397,8 +20441,25 @@
         <v>655</v>
       </c>
     </row>
+    <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>1032</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E41" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
+  <autoFilter ref="A1:E42" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
IAM-006 Complete Supabase project setup
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -6003,7 +6003,7 @@
         <v>3</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G7" s="5" t="s">
         <v>78</v>
@@ -9523,7 +9523,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>65</v>

</xml_diff>

<commit_message>
CODE-046 Add audit trigger migration task
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A97464-F48F-9047-BE86-279E36B024CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E473DA-4262-DF49-BE8C-854A03E5771E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3368" uniqueCount="1037">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3372" uniqueCount="1039">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3168,6 +3168,12 @@
   </si>
   <si>
     <t>supabase/config.toml exists; it contains no credentials, tokens, passwords, or production secrets; local Supabase project and migration discovery settings are configured; the repository structure supports the documented local migration workflow; configuration syntax is valid; and no hosted Supabase project or database migration is created.</t>
+  </si>
+  <si>
+    <t>CODE-046</t>
+  </si>
+  <si>
+    <t>Create reusable audit trigger migration</t>
   </si>
 </sst>
 </file>
@@ -3304,7 +3310,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3331,21 +3337,24 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4037,7 +4046,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -4049,7 +4058,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4073,7 +4082,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="12" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4107,7 +4116,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4141,7 +4150,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4175,7 +4184,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4198,16 +4207,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A5:H6"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="A17:H18"/>
     <mergeCell ref="A9:H10"/>
     <mergeCell ref="A13:H14"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H6"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A4:H4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -5281,7 +5290,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5293,7 +5302,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -18353,7 +18362,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19671,7 +19680,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="128" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
         <v>1032</v>
       </c>
@@ -19700,9 +19709,23 @@
         <v>13</v>
       </c>
     </row>
+    <row r="47" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A47" s="19" t="s">
+        <v>1037</v>
+      </c>
+      <c r="E47" t="s">
+        <v>1038</v>
+      </c>
+      <c r="G47" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="I47" s="19" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I46" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I46">
+  <conditionalFormatting sqref="I2:I47">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>

</xml_diff>

<commit_message>
CODE-046 Create reusable audit trigger migration
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9E9E24-878D-1748-BF91-19E4A6E4A569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D1E3EF-536F-5443-AA45-A3F15C98CE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3373" uniqueCount="1039">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3382" uniqueCount="1042">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3174,6 +3174,15 @@
   </si>
   <si>
     <t>Create reusable audit trigger migration</t>
+  </si>
+  <si>
+    <t>Create an ordered PostgreSQL migration that defines reusable audit timestamp behavior for IAMONIT tables. Define a reusable trigger function that sets updated_at to the current timestamp whenever a row is updated. Use timestamptz for created_at and updated_at conventions. Keep the migration compatible with Supabase PostgreSQL and safe to apply through the existing local migration workflow. Do not create tenants, app_users, authentication endpoints, or unrelated tables in this task. Do not apply the migration to the hosted Supabase project automatically.</t>
+  </si>
+  <si>
+    <t>supabase/migrations/20260804164436_audit_trigger.sql exists; it defines a reusable PostgreSQL updated_at trigger function; audit timestamp conventions use timestamptz; the SQL is valid and safely ordered; the migration applies successfully to the local Supabase database; local verification confirms that a table using the trigger receives a changed updated_at value after an update; no unrelated tables are created; and no hosted-project migration is applied.</t>
+  </si>
+  <si>
+    <t>supabase/migrations/20260804164436_audit_trigger.sql</t>
   </si>
 </sst>
 </file>
@@ -3310,7 +3319,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3337,9 +3346,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -3662,7 +3668,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>64</c:v>
+                  <c:v>62</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
@@ -3674,7 +3680,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4046,164 +4052,164 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="4" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
     </row>
     <row r="8" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
+      <c r="A10" s="13"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="12" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
     </row>
     <row r="16" spans="1:8" ht="19" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -5290,90 +5296,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
     </row>
     <row r="4" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="D4" s="19" t="s">
+      <c r="B4" s="13"/>
+      <c r="D4" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="14"/>
-      <c r="G4" s="19" t="s">
+      <c r="E4" s="13"/>
+      <c r="G4" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="14"/>
+      <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:9" ht="24" x14ac:dyDescent="0.3">
-      <c r="A5" s="18">
+      <c r="A5" s="17">
         <f>COUNTA(Backlog!A2:A500)</f>
         <v>70</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="D5" s="18">
+      <c r="B5" s="13"/>
+      <c r="D5" s="17">
         <f>COUNTIF(Backlog!F2:F500,"Done")</f>
-        <v>8</v>
-      </c>
-      <c r="E5" s="14"/>
-      <c r="G5" s="18">
+        <v>10</v>
+      </c>
+      <c r="E5" s="13"/>
+      <c r="G5" s="17">
         <f>COUNTIF(Backlog!F2:F500,"In Progress")</f>
         <v>1</v>
       </c>
-      <c r="H5" s="14"/>
+      <c r="H5" s="13"/>
     </row>
     <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="D7" s="19" t="s">
+      <c r="B7" s="13"/>
+      <c r="D7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="G7" s="19" t="s">
+      <c r="E7" s="13"/>
+      <c r="G7" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="14"/>
+      <c r="H7" s="13"/>
     </row>
     <row r="8" spans="1:9" ht="24" x14ac:dyDescent="0.3">
-      <c r="A8" s="18">
+      <c r="A8" s="17">
         <f>COUNTIF(Backlog!F2:F500,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="D8" s="18">
+      <c r="B8" s="13"/>
+      <c r="D8" s="17">
         <f>SUM(Backlog!E2:E500)</f>
         <v>369</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="G8" s="18">
+      <c r="E8" s="13"/>
+      <c r="G8" s="17">
         <f>SUMIF(Backlog!F2:F500,"Done",Backlog!E2:E500)</f>
-        <v>32</v>
-      </c>
-      <c r="H8" s="14"/>
+        <v>40</v>
+      </c>
+      <c r="H8" s="13"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -5412,7 +5418,7 @@
       </c>
       <c r="C12">
         <f>COUNTIFS(Backlog!K:K,A12,Backlog!F:F,"Done")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D12">
         <f>COUNTIFS(Backlog!K:K,A12,Backlog!F:F,"Blocked")</f>
@@ -5424,14 +5430,14 @@
       </c>
       <c r="F12" s="3">
         <f t="shared" ref="F12:F20" si="0">IF(B12=0,0,C12/B12)</f>
-        <v>0.66666666666666663</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="H12" t="s">
         <v>25</v>
       </c>
       <c r="I12">
         <f>COUNTIF(Backlog!F:F,H12)</f>
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -5559,7 +5565,7 @@
       </c>
       <c r="I16">
         <f>COUNTIF(Backlog!F:F,H16)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -6060,7 +6066,7 @@
         <v>5</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G8" s="5" t="s">
         <v>84</v>
@@ -9564,7 +9570,7 @@
         <v>5</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>75</v>
@@ -19709,7 +19715,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="128" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
         <v>1037</v>
       </c>
@@ -19720,26 +19726,22 @@
         <v>633</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>86</v>
+        <v>1041</v>
       </c>
       <c r="E47" s="5" t="s">
         <v>1038</v>
       </c>
-      <c r="F47" s="5" t="inlineStr">
-        <is>
-          <t>Create an ordered PostgreSQL migration that defines reusable audit timestamp behavior for IAMONIT tables. Define a reusable trigger function that sets updated_at to the current timestamp whenever a row is updated. Use timestamptz for created_at and updated_at conventions. Keep the migration compatible with Supabase PostgreSQL and safe to apply through the existing local migration workflow. Do not create tenants, app_users, authentication endpoints, or unrelated tables in this task. Do not apply the migration to the hosted Supabase project automatically.</t>
-        </is>
+      <c r="F47" s="5" t="s">
+        <v>1039</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="H47" s="5" t="inlineStr">
-        <is>
-          <t>supabase/migrations/001_audit.sql exists; it defines a reusable PostgreSQL updated_at trigger function; audit timestamp conventions use timestamptz; the SQL is valid and safely ordered; the migration applies successfully to the local Supabase database; local verification confirms that a table using the trigger receives a changed updated_at value after an update; no unrelated tables are created; and no hosted-project migration is applied.</t>
-        </is>
+      <c r="H47" s="5" t="s">
+        <v>1040</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -20505,7 +20507,7 @@
         <v>80</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>86</v>
+        <v>1041</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>1038</v>

</xml_diff>

<commit_message>
CODE-035 Align tenants migration scope
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -19406,20 +19406,51 @@
       <c r="C36" s="5" t="s">
         <v>633</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>101</v>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>supabase/migrations/20260804165923_create_tenants.sql</t>
+        </is>
       </c>
       <c r="E36" s="5" t="s">
         <v>634</v>
       </c>
-      <c r="F36" s="5" t="s">
-        <v>635</v>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Create one ordered Supabase PostgreSQL migration for public.tenants. Define id
+as uuid primary key with default gen_random_uuid(); define name as text, required,
+and unique; define status as text, required, with default 'active'; and define
+created_by and updated_by as nullable uuid columns without foreign keys at this
+stage.
+Follow the IAM-007 audit convention by defining created_at and updated_at as
+timestamptz NOT NULL DEFAULT now() and attach a BEFORE UPDATE trigger that
+executes public.set_updated_at().
+Enable row-level security on public.tenants, but do not create tenant-access
+policies because policy implementation belongs to IAM-014. Do not create or
+depend on app_users, memberships, profiles, authentication endpoints, API code,
+or other application files.
+Apply and verify the migration only against the local Supabase database. Do not
+apply it to the hosted Supabase project.</t>
+        </is>
       </c>
       <c r="G36" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="5" t="s">
-        <v>636</v>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>The timestamped migration
+supabase/migrations/20260804165923_create_tenants.sql creates public.tenants
+with id, name, status, created_at, updated_at, created_by, and updated_by.
+id is a uuid primary key with default gen_random_uuid(); name is required and
+unique; status is required and defaults to 'active'; created_by and updated_by
+are nullable uuid columns without foreign keys; created_at and updated_at use
+timestamptz NOT NULL DEFAULT now().
+A BEFORE UPDATE trigger invokes public.set_updated_at(); row-level security is
+enabled without adding IAM-014 tenant-access policies; the migration applies
+successfully to the local Supabase database; a privileged local insert succeeds;
+a duplicate tenant name is rejected; updating a tenant changes updated_at; no
+app_users, memberships, profiles, API files, or unrelated tables are created;
+and no hosted-project migration is applied.</t>
+        </is>
       </c>
       <c r="I36" s="5" t="s">
         <v>25</v>
@@ -20387,8 +20418,10 @@
       <c r="A36" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="5" t="s">
-        <v>101</v>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>supabase/migrations/20260804165923_create_tenants.sql</t>
+        </is>
       </c>
       <c r="C36" s="5" t="s">
         <v>634</v>

</xml_diff>

<commit_message>
CODE-035 Create tenants migration
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D1E3EF-536F-5443-AA45-A3F15C98CE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5976D16-CB74-D341-B99F-6DD1BFD3DEFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3382" uniqueCount="1042">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3382" uniqueCount="1043">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -1964,12 +1964,6 @@
     <t>Create tenants migration</t>
   </si>
   <si>
-    <t>tenants table with audit fields and RLS.</t>
-  </si>
-  <si>
-    <t>Migration applies</t>
-  </si>
-  <si>
     <t>CODE-036</t>
   </si>
   <si>
@@ -3183,6 +3177,40 @@
   </si>
   <si>
     <t>supabase/migrations/20260804164436_audit_trigger.sql</t>
+  </si>
+  <si>
+    <t>supabase/migrations/20260804165923_create_tenants.sql</t>
+  </si>
+  <si>
+    <t>Create one ordered Supabase PostgreSQL migration for public.tenants. Define id
+as uuid primary key with default gen_random_uuid(); define name as text, required,
+and unique; define status as text, required, with default 'active'; and define
+created_by and updated_by as nullable uuid columns without foreign keys at this
+stage.
+Follow the IAM-007 audit convention by defining created_at and updated_at as
+timestamptz NOT NULL DEFAULT now() and attach a BEFORE UPDATE trigger that
+executes public.set_updated_at().
+Enable row-level security on public.tenants, but do not create tenant-access
+policies because policy implementation belongs to IAM-014. Do not create or
+depend on app_users, memberships, profiles, authentication endpoints, API code,
+or other application files.
+Apply and verify the migration only against the local Supabase database. Do not
+apply it to the hosted Supabase project.</t>
+  </si>
+  <si>
+    <t>The timestamped migration
+supabase/migrations/20260804165923_create_tenants.sql creates public.tenants
+with id, name, status, created_at, updated_at, created_by, and updated_by.
+id is a uuid primary key with default gen_random_uuid(); name is required and
+unique; status is required and defaults to 'active'; created_by and updated_by
+are nullable uuid columns without foreign keys; created_at and updated_at use
+timestamptz NOT NULL DEFAULT now().
+A BEFORE UPDATE trigger invokes public.set_updated_at(); row-level security is
+enabled without adding IAM-014 tenant-access policies; the migration applies
+successfully to the local Supabase database; a privileged local insert succeeds;
+a duplicate tenant name is rejected; updating a tenant changes updated_at; no
+app_users, memberships, profiles, API files, or unrelated tables are created;
+and no hosted-project migration is applied.</t>
   </si>
 </sst>
 </file>
@@ -3346,15 +3374,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3668,7 +3696,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>62</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1</c:v>
@@ -3680,7 +3708,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4052,7 +4080,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -4064,7 +4092,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4088,7 +4116,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4122,7 +4150,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="14" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4156,7 +4184,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="14" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4190,7 +4218,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="14" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4213,16 +4241,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A17:H18"/>
+    <mergeCell ref="A9:H10"/>
+    <mergeCell ref="A13:H14"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A5:H6"/>
     <mergeCell ref="A8:H8"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A17:H18"/>
-    <mergeCell ref="A9:H10"/>
-    <mergeCell ref="A13:H14"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -4246,22 +4274,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>740</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>741</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>742</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>662</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>743</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>744</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>745</v>
-      </c>
       <c r="F1" s="4" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -4269,76 +4297,76 @@
         <v>521</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>744</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>745</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>746</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>747</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>748</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>749</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>750</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
+        <v>749</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>750</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>751</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>752</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="E3" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>753</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>754</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>749</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>755</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>754</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>755</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>756</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>757</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="E4" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>758</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>759</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>749</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>759</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>760</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>761</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>762</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>763</v>
-      </c>
       <c r="D5" s="5" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>112</v>
@@ -4349,19 +4377,19 @@
         <v>535</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>762</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>763</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>764</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="E6" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>765</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>766</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>749</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="32" x14ac:dyDescent="0.2">
@@ -4369,56 +4397,56 @@
         <v>545</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>766</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>767</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>768</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="E7" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>769</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>770</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>749</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>771</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
+        <v>770</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>772</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>773</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>774</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>775</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>776</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>777</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
+        <v>776</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>777</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>778</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>779</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>780</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>781</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>246</v>
@@ -4426,22 +4454,22 @@
     </row>
     <row r="10" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>781</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>782</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>783</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="5" t="s">
+        <v>747</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>784</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>785</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>749</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>786</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -4449,36 +4477,36 @@
         <v>577</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>785</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>786</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>787</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>788</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>789</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>790</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
+        <v>790</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>791</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>792</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>793</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>794</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>795</v>
-      </c>
       <c r="E12" s="5" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>323</v>
@@ -4510,25 +4538,25 @@
   <sheetData>
     <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>794</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>795</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>796</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>797</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>798</v>
       </c>
-      <c r="D1" s="4" t="s">
-        <v>799</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>662</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>800</v>
-      </c>
       <c r="G1" s="4" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>22</v>
@@ -4536,22 +4564,22 @@
     </row>
     <row r="2" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>799</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>800</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>801</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>802</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>803</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>804</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>805</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>806</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>583</v>
@@ -4562,22 +4590,22 @@
     </row>
     <row r="3" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
+        <v>805</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>806</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>807</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="5" t="s">
+        <v>802</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>808</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
         <v>809</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>804</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>810</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>811</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>583</v>
@@ -4588,22 +4616,22 @@
     </row>
     <row r="4" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>297</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>811</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>813</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>814</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>815</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>816</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>296</v>
@@ -4614,22 +4642,22 @@
     </row>
     <row r="5" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>817</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>818</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>819</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>820</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>821</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>822</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>302</v>
@@ -4640,22 +4668,22 @@
     </row>
     <row r="6" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
+        <v>821</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>696</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>823</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>824</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>698</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>814</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>825</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>826</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>607</v>
@@ -4666,25 +4694,25 @@
     </row>
     <row r="7" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
+        <v>825</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>826</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>827</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="D7" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>828</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>829</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>814</v>
-      </c>
-      <c r="E7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>830</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>831</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>832</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>25</v>
@@ -4692,25 +4720,25 @@
     </row>
     <row r="8" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>833</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>834</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>835</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>836</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>837</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>839</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>25</v>
@@ -4718,22 +4746,22 @@
     </row>
     <row r="9" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
+        <v>838</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>839</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>840</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="D9" s="5" t="s">
+        <v>818</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>841</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>842</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>820</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>843</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>844</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>271</v>
@@ -4744,22 +4772,22 @@
     </row>
     <row r="10" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>843</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>844</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>845</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>846</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>683</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>685</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>847</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>848</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>166</v>
@@ -4770,22 +4798,22 @@
     </row>
     <row r="11" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
+        <v>847</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>848</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>849</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="D11" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>850</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>851</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>685</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>852</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>853</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>177</v>
@@ -4796,22 +4824,22 @@
     </row>
     <row r="12" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
+        <v>852</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>854</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="D12" s="5" t="s">
+        <v>802</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>855</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>856</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>804</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>857</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>858</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>291</v>
@@ -4868,19 +4896,19 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>857</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>858</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>859</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>860</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>861</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>862</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>863</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>426</v>
@@ -4891,140 +4919,140 @@
     </row>
     <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>862</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>863</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>864</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>865</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>866</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>122</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>64</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>168</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>390</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>390</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
+        <v>876</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>877</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>878</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>879</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>880</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E6" s="5" t="s">
+        <v>879</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>880</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>881</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>882</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>883</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>67</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>80</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
     </row>
   </sheetData>
@@ -5052,13 +5080,13 @@
   <sheetData>
     <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>426</v>
@@ -5067,7 +5095,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
@@ -5075,10 +5103,10 @@
         <v>122</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>122</v>
@@ -5093,10 +5121,10 @@
         <v>88</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>64</v>
@@ -5111,10 +5139,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>182</v>
@@ -5126,13 +5154,13 @@
     </row>
     <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>59</v>
@@ -5144,13 +5172,13 @@
     </row>
     <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>182</v>
@@ -5165,10 +5193,10 @@
         <v>277</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>182</v>
@@ -5183,10 +5211,10 @@
         <v>335</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>339</v>
@@ -5201,10 +5229,10 @@
         <v>358</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>55</v>
@@ -5219,10 +5247,10 @@
         <v>358</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>55</v>
@@ -5234,13 +5262,13 @@
     </row>
     <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>390</v>
@@ -5296,7 +5324,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="12" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5308,7 +5336,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="16" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -5341,7 +5369,7 @@
       <c r="B5" s="13"/>
       <c r="D5" s="17">
         <f>COUNTIF(Backlog!F2:F500,"Done")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="13"/>
       <c r="G5" s="17">
@@ -5377,7 +5405,7 @@
       <c r="E8" s="13"/>
       <c r="G8" s="17">
         <f>SUMIF(Backlog!F2:F500,"Done",Backlog!E2:E500)</f>
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="H8" s="13"/>
     </row>
@@ -5437,7 +5465,7 @@
       </c>
       <c r="I12">
         <f>COUNTIF(Backlog!F:F,H12)</f>
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -5450,7 +5478,7 @@
       </c>
       <c r="C13">
         <f>COUNTIFS(Backlog!K:K,A13,Backlog!F:F,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13">
         <f>COUNTIFS(Backlog!K:K,A13,Backlog!F:F,"Blocked")</f>
@@ -5462,7 +5490,7 @@
       </c>
       <c r="F13" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="H13" t="s">
         <v>14</v>
@@ -5565,7 +5593,7 @@
       </c>
       <c r="I16">
         <f>COUNTIF(Backlog!F:F,H16)</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -5829,10 +5857,10 @@
         <v>13</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="I3" s="9" t="s">
         <v>59</v>
@@ -5853,7 +5881,7 @@
         <v>49</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>922</v>
+        <v>920</v>
       </c>
       <c r="P3" s="9"/>
     </row>
@@ -5901,7 +5929,7 @@
         <v>49</v>
       </c>
       <c r="O4" s="9" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="P4" s="9"/>
     </row>
@@ -5949,7 +5977,7 @@
         <v>70</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>924</v>
+        <v>922</v>
       </c>
       <c r="P5" s="5"/>
     </row>
@@ -5997,7 +6025,7 @@
         <v>70</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>925</v>
+        <v>923</v>
       </c>
       <c r="P6" s="5"/>
     </row>
@@ -6141,7 +6169,7 @@
         <v>60</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>926</v>
+        <v>924</v>
       </c>
       <c r="P9" s="5"/>
     </row>
@@ -6189,7 +6217,7 @@
         <v>57</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>927</v>
+        <v>925</v>
       </c>
       <c r="P10" s="5"/>
     </row>
@@ -6210,7 +6238,7 @@
         <v>5</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>99</v>
@@ -6477,7 +6505,7 @@
         <v>129</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="P16" s="5"/>
     </row>
@@ -6525,7 +6553,7 @@
         <v>134</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="P17" s="5"/>
     </row>
@@ -6573,7 +6601,7 @@
         <v>140</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>930</v>
+        <v>928</v>
       </c>
       <c r="P18" s="5"/>
     </row>
@@ -6621,7 +6649,7 @@
         <v>130</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>931</v>
+        <v>929</v>
       </c>
       <c r="P19" s="5"/>
     </row>
@@ -6717,7 +6745,7 @@
         <v>156</v>
       </c>
       <c r="O21" s="5" t="s">
-        <v>932</v>
+        <v>930</v>
       </c>
       <c r="P21" s="5"/>
     </row>
@@ -6765,7 +6793,7 @@
         <v>152</v>
       </c>
       <c r="O22" s="5" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="P22" s="5"/>
     </row>
@@ -6813,7 +6841,7 @@
         <v>141</v>
       </c>
       <c r="O23" s="5" t="s">
-        <v>934</v>
+        <v>932</v>
       </c>
       <c r="P23" s="5"/>
     </row>
@@ -6861,7 +6889,7 @@
         <v>171</v>
       </c>
       <c r="O24" s="5" t="s">
-        <v>935</v>
+        <v>933</v>
       </c>
       <c r="P24" s="5"/>
     </row>
@@ -6909,7 +6937,7 @@
         <v>135</v>
       </c>
       <c r="O25" s="5" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="P25" s="5"/>
     </row>
@@ -6957,7 +6985,7 @@
         <v>183</v>
       </c>
       <c r="O26" s="5" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="P26" s="5"/>
     </row>
@@ -7101,7 +7129,7 @@
         <v>184</v>
       </c>
       <c r="O29" s="5" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="P29" s="5"/>
     </row>
@@ -7149,7 +7177,7 @@
         <v>204</v>
       </c>
       <c r="O30" s="5" t="s">
-        <v>939</v>
+        <v>937</v>
       </c>
       <c r="P30" s="5"/>
     </row>
@@ -7197,7 +7225,7 @@
         <v>200</v>
       </c>
       <c r="O31" s="5" t="s">
-        <v>940</v>
+        <v>938</v>
       </c>
       <c r="P31" s="5"/>
     </row>
@@ -7245,7 +7273,7 @@
         <v>205</v>
       </c>
       <c r="O32" s="5" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="P32" s="5"/>
     </row>
@@ -7293,7 +7321,7 @@
         <v>217</v>
       </c>
       <c r="O33" s="5" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="P33" s="5"/>
     </row>
@@ -7341,7 +7369,7 @@
         <v>223</v>
       </c>
       <c r="O34" s="5" t="s">
-        <v>943</v>
+        <v>941</v>
       </c>
       <c r="P34" s="5"/>
     </row>
@@ -7389,7 +7417,7 @@
         <v>228</v>
       </c>
       <c r="O35" s="5" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="P35" s="5"/>
     </row>
@@ -7437,7 +7465,7 @@
         <v>233</v>
       </c>
       <c r="O36" s="5" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="P36" s="5"/>
     </row>
@@ -7533,7 +7561,7 @@
         <v>245</v>
       </c>
       <c r="O38" s="5" t="s">
-        <v>946</v>
+        <v>944</v>
       </c>
       <c r="P38" s="5"/>
     </row>
@@ -7581,7 +7609,7 @@
         <v>240</v>
       </c>
       <c r="O39" s="5" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="P39" s="5"/>
     </row>
@@ -7629,7 +7657,7 @@
         <v>240</v>
       </c>
       <c r="O40" s="5" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="P40" s="5"/>
     </row>
@@ -7725,7 +7753,7 @@
         <v>255</v>
       </c>
       <c r="O42" s="5" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="P42" s="5"/>
     </row>
@@ -7773,7 +7801,7 @@
         <v>270</v>
       </c>
       <c r="O43" s="5" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="P43" s="5"/>
     </row>
@@ -7821,7 +7849,7 @@
         <v>275</v>
       </c>
       <c r="O44" s="5" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="P44" s="5"/>
     </row>
@@ -7917,7 +7945,7 @@
         <v>286</v>
       </c>
       <c r="O46" s="5" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="P46" s="5"/>
     </row>
@@ -7965,7 +7993,7 @@
         <v>282</v>
       </c>
       <c r="O47" s="5" t="s">
-        <v>953</v>
+        <v>951</v>
       </c>
       <c r="P47" s="5"/>
     </row>
@@ -8013,7 +8041,7 @@
         <v>295</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="P48" s="5"/>
     </row>
@@ -8061,7 +8089,7 @@
         <v>301</v>
       </c>
       <c r="O49" s="5" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="P49" s="5"/>
     </row>
@@ -8109,7 +8137,7 @@
         <v>271</v>
       </c>
       <c r="O50" s="5" t="s">
-        <v>956</v>
+        <v>954</v>
       </c>
       <c r="P50" s="5"/>
     </row>
@@ -8157,7 +8185,7 @@
         <v>205</v>
       </c>
       <c r="O51" s="5" t="s">
-        <v>957</v>
+        <v>955</v>
       </c>
       <c r="P51" s="5"/>
     </row>
@@ -8205,7 +8233,7 @@
         <v>315</v>
       </c>
       <c r="O52" s="5" t="s">
-        <v>958</v>
+        <v>956</v>
       </c>
       <c r="P52" s="5"/>
     </row>
@@ -8397,7 +8425,7 @@
         <v>340</v>
       </c>
       <c r="O56" s="5" t="s">
-        <v>959</v>
+        <v>957</v>
       </c>
       <c r="P56" s="5"/>
     </row>
@@ -8445,7 +8473,7 @@
         <v>345</v>
       </c>
       <c r="O57" s="5" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="P57" s="5"/>
     </row>
@@ -8493,7 +8521,7 @@
         <v>350</v>
       </c>
       <c r="O58" s="5" t="s">
-        <v>961</v>
+        <v>959</v>
       </c>
       <c r="P58" s="5"/>
     </row>
@@ -8685,7 +8713,7 @@
         <v>357</v>
       </c>
       <c r="O62" s="5" t="s">
-        <v>962</v>
+        <v>960</v>
       </c>
       <c r="P62" s="5"/>
     </row>
@@ -9021,7 +9049,7 @@
         <v>413</v>
       </c>
       <c r="O69" s="5" t="s">
-        <v>963</v>
+        <v>961</v>
       </c>
       <c r="P69" s="5"/>
     </row>
@@ -9069,7 +9097,7 @@
         <v>420</v>
       </c>
       <c r="O70" s="5" t="s">
-        <v>964</v>
+        <v>962</v>
       </c>
       <c r="P70" s="5"/>
     </row>
@@ -9117,19 +9145,19 @@
         <v>425</v>
       </c>
       <c r="O71" s="5" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="P71" s="5"/>
     </row>
     <row r="72" spans="1:16" ht="64" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
+        <v>903</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>904</v>
+      </c>
+      <c r="C72" s="5" t="s">
         <v>905</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>906</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>907</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>67</v>
@@ -9141,10 +9169,10 @@
         <v>14</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="H72" s="5" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="I72" s="5" t="s">
         <v>55</v>
@@ -9153,7 +9181,7 @@
         <v>46230</v>
       </c>
       <c r="K72" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="L72" s="5">
         <v>1</v>
@@ -9162,24 +9190,24 @@
         <v>46230</v>
       </c>
       <c r="N72" s="5" t="s">
+        <v>909</v>
+      </c>
+      <c r="O72" s="5" t="s">
+        <v>910</v>
+      </c>
+      <c r="P72" s="5" t="s">
         <v>911</v>
-      </c>
-      <c r="O72" s="5" t="s">
-        <v>912</v>
-      </c>
-      <c r="P72" s="5" t="s">
-        <v>913</v>
       </c>
     </row>
     <row r="73" spans="1:16" ht="80" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>67</v>
@@ -9191,10 +9219,10 @@
         <v>13</v>
       </c>
       <c r="G73" s="5" t="s">
-        <v>967</v>
+        <v>965</v>
       </c>
       <c r="H73" s="5" t="s">
-        <v>968</v>
+        <v>966</v>
       </c>
       <c r="I73" s="5" t="s">
         <v>55</v>
@@ -9203,7 +9231,7 @@
         <v>46230</v>
       </c>
       <c r="K73" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="L73" s="5">
         <v>1</v>
@@ -9212,24 +9240,24 @@
         <v>46230</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="O73" s="5" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="P73" s="5" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
     </row>
     <row r="74" spans="1:16" ht="96" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>67</v>
@@ -9241,10 +9269,10 @@
         <v>13</v>
       </c>
       <c r="G74" s="5" t="s">
-        <v>1006</v>
+        <v>1004</v>
       </c>
       <c r="H74" s="5" t="s">
-        <v>1007</v>
+        <v>1005</v>
       </c>
       <c r="I74" s="5" t="s">
         <v>55</v>
@@ -9253,7 +9281,7 @@
         <v>46230</v>
       </c>
       <c r="K74" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="L74" s="5">
         <v>2</v>
@@ -9262,13 +9290,13 @@
         <v>46231</v>
       </c>
       <c r="N74" s="5" t="s">
+        <v>1006</v>
+      </c>
+      <c r="O74" s="5" t="s">
+        <v>1007</v>
+      </c>
+      <c r="P74" s="5" t="s">
         <v>1008</v>
-      </c>
-      <c r="O74" s="5" t="s">
-        <v>1009</v>
-      </c>
-      <c r="P74" s="5" t="s">
-        <v>1010</v>
       </c>
     </row>
   </sheetData>
@@ -9416,7 +9444,7 @@
         <v>49</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -9666,7 +9694,7 @@
         <v>5</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>82</v>
@@ -11597,16 +11625,16 @@
     </row>
     <row r="72" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A72" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="B72" s="5" t="s">
+        <v>903</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>904</v>
+      </c>
+      <c r="D72" s="5" t="s">
         <v>905</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>906</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>907</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>55</v>
@@ -11621,24 +11649,24 @@
         <v>14</v>
       </c>
       <c r="I72" s="5" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="J72" s="5" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
     </row>
     <row r="73" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A73" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>965</v>
+        <v>963</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>966</v>
+        <v>964</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>55</v>
@@ -11653,24 +11681,24 @@
         <v>13</v>
       </c>
       <c r="I73" s="5" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="J73" s="5" t="s">
-        <v>971</v>
+        <v>969</v>
       </c>
     </row>
     <row r="74" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A74" s="5" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>55</v>
@@ -11685,10 +11713,10 @@
         <v>13</v>
       </c>
       <c r="I74" s="5" t="s">
-        <v>1008</v>
+        <v>1006</v>
       </c>
       <c r="J74" s="5" t="s">
-        <v>1011</v>
+        <v>1009</v>
       </c>
     </row>
   </sheetData>
@@ -18421,19 +18449,19 @@
         <v>488</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>1027</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>1028</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>1029</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>1030</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>65</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>13</v>
@@ -18450,7 +18478,7 @@
         <v>490</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>491</v>
@@ -18479,7 +18507,7 @@
         <v>490</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>495</v>
@@ -18508,7 +18536,7 @@
         <v>490</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>499</v>
@@ -18537,7 +18565,7 @@
         <v>490</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>504</v>
@@ -18566,7 +18594,7 @@
         <v>490</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>508</v>
@@ -18595,7 +18623,7 @@
         <v>512</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>513</v>
@@ -18624,7 +18652,7 @@
         <v>512</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>517</v>
@@ -18653,7 +18681,7 @@
         <v>521</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>522</v>
@@ -18682,7 +18710,7 @@
         <v>526</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>527</v>
@@ -18711,7 +18739,7 @@
         <v>526</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>531</v>
@@ -18740,7 +18768,7 @@
         <v>535</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>536</v>
@@ -18769,7 +18797,7 @@
         <v>535</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>541</v>
@@ -18798,7 +18826,7 @@
         <v>545</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>546</v>
@@ -18827,7 +18855,7 @@
         <v>545</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>550</v>
@@ -18856,7 +18884,7 @@
         <v>545</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="E17" s="5" t="s">
         <v>555</v>
@@ -18885,7 +18913,7 @@
         <v>545</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>559</v>
@@ -18914,7 +18942,7 @@
         <v>563</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>564</v>
@@ -18943,7 +18971,7 @@
         <v>563</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>568</v>
@@ -18972,7 +19000,7 @@
         <v>572</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>573</v>
@@ -19001,7 +19029,7 @@
         <v>577</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>578</v>
@@ -19030,19 +19058,19 @@
         <v>490</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>582</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>92</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>13</v>
@@ -19059,19 +19087,19 @@
         <v>490</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>585</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>92</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>13</v>
@@ -19088,7 +19116,7 @@
         <v>587</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>588</v>
@@ -19117,7 +19145,7 @@
         <v>587</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>592</v>
@@ -19146,7 +19174,7 @@
         <v>596</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="E27" s="5" t="s">
         <v>597</v>
@@ -19175,7 +19203,7 @@
         <v>596</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="E28" s="5" t="s">
         <v>601</v>
@@ -19204,7 +19232,7 @@
         <v>545</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="E29" s="5" t="s">
         <v>220</v>
@@ -19233,7 +19261,7 @@
         <v>545</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>225</v>
@@ -19262,7 +19290,7 @@
         <v>545</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>230</v>
@@ -19291,7 +19319,7 @@
         <v>545</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="E32" s="5" t="s">
         <v>616</v>
@@ -19320,7 +19348,7 @@
         <v>563</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="E33" s="5" t="s">
         <v>620</v>
@@ -19349,7 +19377,7 @@
         <v>624</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="E34" s="5" t="s">
         <v>625</v>
@@ -19378,7 +19406,7 @@
         <v>577</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>629</v>
@@ -19396,7 +19424,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>632</v>
       </c>
@@ -19406,59 +19434,28 @@
       <c r="C36" s="5" t="s">
         <v>633</v>
       </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>supabase/migrations/20260804165923_create_tenants.sql</t>
-        </is>
+      <c r="D36" s="5" t="s">
+        <v>1040</v>
       </c>
       <c r="E36" s="5" t="s">
         <v>634</v>
       </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Create one ordered Supabase PostgreSQL migration for public.tenants. Define id
-as uuid primary key with default gen_random_uuid(); define name as text, required,
-and unique; define status as text, required, with default 'active'; and define
-created_by and updated_by as nullable uuid columns without foreign keys at this
-stage.
-Follow the IAM-007 audit convention by defining created_at and updated_at as
-timestamptz NOT NULL DEFAULT now() and attach a BEFORE UPDATE trigger that
-executes public.set_updated_at().
-Enable row-level security on public.tenants, but do not create tenant-access
-policies because policy implementation belongs to IAM-014. Do not create or
-depend on app_users, memberships, profiles, authentication endpoints, API code,
-or other application files.
-Apply and verify the migration only against the local Supabase database. Do not
-apply it to the hosted Supabase project.</t>
-        </is>
+      <c r="F36" s="5" t="s">
+        <v>1041</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>The timestamped migration
-supabase/migrations/20260804165923_create_tenants.sql creates public.tenants
-with id, name, status, created_at, updated_at, created_by, and updated_by.
-id is a uuid primary key with default gen_random_uuid(); name is required and
-unique; status is required and defaults to 'active'; created_by and updated_by
-are nullable uuid columns without foreign keys; created_at and updated_at use
-timestamptz NOT NULL DEFAULT now().
-A BEFORE UPDATE trigger invokes public.set_updated_at(); row-level security is
-enabled without adding IAM-014 tenant-access policies; the migration applies
-successfully to the local Supabase database; a privileged local insert succeeds;
-a duplicate tenant name is rejected; updating a tenant changes updated_at; no
-app_users, memberships, profiles, API files, or unrelated tables are created;
-and no hosted-project migration is applied.</t>
-        </is>
+      <c r="H36" s="5" t="s">
+        <v>1042</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>80</v>
@@ -19470,16 +19467,16 @@
         <v>189</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>184</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="I37" s="5" t="s">
         <v>25</v>
@@ -19487,7 +19484,7 @@
     </row>
     <row r="38" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>80</v>
@@ -19499,16 +19496,16 @@
         <v>124</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>117</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="I38" s="5" t="s">
         <v>25</v>
@@ -19516,7 +19513,7 @@
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>80</v>
@@ -19525,19 +19522,19 @@
         <v>633</v>
       </c>
       <c r="D39" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>645</v>
+      </c>
+      <c r="F39" s="5" t="s">
         <v>646</v>
-      </c>
-      <c r="E39" s="5" t="s">
-        <v>647</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>648</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>234</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>25</v>
@@ -19545,28 +19542,28 @@
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>339</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>649</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>996</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>650</v>
+      </c>
+      <c r="F40" s="5" t="s">
         <v>651</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>998</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>652</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>653</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>341</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>25</v>
@@ -19574,28 +19571,28 @@
     </row>
     <row r="41" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>339</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>356</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>351</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="I41" s="5" t="s">
         <v>25</v>
@@ -19603,28 +19600,28 @@
     </row>
     <row r="42" spans="1:9" ht="64" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
+        <v>913</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>914</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>915</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>916</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>917</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="F42" s="5" t="s">
         <v>918</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="G42" s="5" t="s">
+        <v>903</v>
+      </c>
+      <c r="H42" s="5" t="s">
         <v>919</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>920</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>905</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>921</v>
       </c>
       <c r="I42" s="5" t="s">
         <v>13</v>
@@ -19632,28 +19629,28 @@
     </row>
     <row r="43" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
+        <v>997</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>914</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>998</v>
+      </c>
+      <c r="E43" s="5" t="s">
         <v>999</v>
       </c>
-      <c r="B43" s="5" t="s">
-        <v>916</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>917</v>
-      </c>
-      <c r="D43" s="5" t="s">
+      <c r="F43" s="5" t="s">
         <v>1000</v>
       </c>
-      <c r="E43" s="5" t="s">
+      <c r="G43" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="H43" s="5" t="s">
         <v>1001</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>1002</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>965</v>
-      </c>
-      <c r="H43" s="5" t="s">
-        <v>1003</v>
       </c>
       <c r="I43" s="5" t="s">
         <v>13</v>
@@ -19661,28 +19658,28 @@
     </row>
     <row r="44" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>914</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>1011</v>
+      </c>
+      <c r="F44" s="5" t="s">
         <v>1012</v>
       </c>
-      <c r="B44" s="5" t="s">
-        <v>916</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>917</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>1009</v>
-      </c>
-      <c r="E44" s="5" t="s">
+      <c r="G44" s="5" t="s">
+        <v>1002</v>
+      </c>
+      <c r="H44" s="5" t="s">
         <v>1013</v>
-      </c>
-      <c r="F44" s="5" t="s">
-        <v>1014</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>1004</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>1015</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>13</v>
@@ -19690,28 +19687,28 @@
     </row>
     <row r="45" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C45" s="5" t="s">
+        <v>1017</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>1018</v>
+      </c>
+      <c r="E45" s="5" t="s">
         <v>1019</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="F45" s="5" t="s">
         <v>1020</v>
-      </c>
-      <c r="E45" s="5" t="s">
-        <v>1021</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>1022</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>57</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>13</v>
@@ -19719,28 +19716,28 @@
     </row>
     <row r="46" spans="1:9" ht="128" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>81</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>75</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="I46" s="5" t="s">
         <v>13</v>
@@ -19748,7 +19745,7 @@
     </row>
     <row r="47" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>80</v>
@@ -19757,19 +19754,19 @@
         <v>633</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>82</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>13</v>
@@ -19821,19 +19818,19 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>658</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>659</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>660</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="D1" s="4" t="s">
         <v>661</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>662</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>663</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="32" x14ac:dyDescent="0.2">
@@ -19841,10 +19838,10 @@
         <v>64</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>65</v>
@@ -19858,7 +19855,7 @@
         <v>64</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>972</v>
+        <v>970</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>491</v>
@@ -19875,7 +19872,7 @@
         <v>64</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>973</v>
+        <v>971</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>495</v>
@@ -19892,7 +19889,7 @@
         <v>64</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>974</v>
+        <v>972</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>499</v>
@@ -19909,7 +19906,7 @@
         <v>64</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>975</v>
+        <v>973</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>504</v>
@@ -19926,7 +19923,7 @@
         <v>64</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>508</v>
@@ -19943,7 +19940,7 @@
         <v>64</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>513</v>
@@ -19960,7 +19957,7 @@
         <v>64</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>517</v>
@@ -19977,7 +19974,7 @@
         <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>522</v>
@@ -19994,7 +19991,7 @@
         <v>64</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>527</v>
@@ -20011,7 +20008,7 @@
         <v>64</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>981</v>
+        <v>979</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>531</v>
@@ -20028,7 +20025,7 @@
         <v>64</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>536</v>
@@ -20045,7 +20042,7 @@
         <v>64</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>541</v>
@@ -20062,7 +20059,7 @@
         <v>64</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>983</v>
+        <v>981</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>546</v>
@@ -20079,7 +20076,7 @@
         <v>64</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>984</v>
+        <v>982</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>550</v>
@@ -20096,7 +20093,7 @@
         <v>64</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>555</v>
@@ -20113,7 +20110,7 @@
         <v>64</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>559</v>
@@ -20130,7 +20127,7 @@
         <v>64</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>564</v>
@@ -20147,7 +20144,7 @@
         <v>64</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>986</v>
+        <v>984</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>568</v>
@@ -20164,7 +20161,7 @@
         <v>64</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>573</v>
@@ -20181,7 +20178,7 @@
         <v>64</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>952</v>
+        <v>950</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>578</v>
@@ -20198,7 +20195,7 @@
         <v>59</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>582</v>
@@ -20215,7 +20212,7 @@
         <v>59</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>585</v>
@@ -20232,7 +20229,7 @@
         <v>59</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>588</v>
@@ -20249,7 +20246,7 @@
         <v>59</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>592</v>
@@ -20266,7 +20263,7 @@
         <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>597</v>
@@ -20283,7 +20280,7 @@
         <v>59</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>601</v>
@@ -20300,7 +20297,7 @@
         <v>59</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>220</v>
@@ -20317,7 +20314,7 @@
         <v>59</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>225</v>
@@ -20334,7 +20331,7 @@
         <v>59</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>996</v>
+        <v>994</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>230</v>
@@ -20351,7 +20348,7 @@
         <v>59</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>616</v>
@@ -20368,7 +20365,7 @@
         <v>59</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>620</v>
@@ -20385,7 +20382,7 @@
         <v>59</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>951</v>
+        <v>949</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>625</v>
@@ -20402,7 +20399,7 @@
         <v>59</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>629</v>
@@ -20418,10 +20415,8 @@
       <c r="A36" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>supabase/migrations/20260804165923_create_tenants.sql</t>
-        </is>
+      <c r="B36" s="5" t="s">
+        <v>1040</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>634</v>
@@ -20441,13 +20436,13 @@
         <v>189</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>184</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20458,13 +20453,13 @@
         <v>124</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>117</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20472,16 +20467,16 @@
         <v>80</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>234</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20489,16 +20484,16 @@
         <v>339</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>998</v>
+        <v>996</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>341</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20509,13 +20504,13 @@
         <v>356</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>351</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20526,13 +20521,13 @@
         <v>81</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>75</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20540,16 +20535,16 @@
         <v>80</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>82</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
     </row>
   </sheetData>
@@ -20578,114 +20573,114 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>664</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>660</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>665</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>666</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>662</v>
-      </c>
-      <c r="D1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>667</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>668</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>669</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>669</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>670</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>671</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>672</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>673</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>674</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>675</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>676</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>677</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>678</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="F3" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>679</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>674</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>680</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>676</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
+        <v>680</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>682</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>683</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>684</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>685</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>686</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>687</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>688</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>687</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>689</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="F5" s="5" t="s">
         <v>690</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>685</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>691</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>692</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>152</v>
@@ -20693,22 +20688,22 @@
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>691</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>692</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>693</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>694</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="F6" s="5" t="s">
         <v>695</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>696</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>697</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>157</v>
@@ -20716,186 +20711,186 @@
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>696</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>697</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>698</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>699</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="F7" s="5" t="s">
         <v>700</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="G7" s="5" t="s">
         <v>701</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>702</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>703</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>704</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="F8" s="5" t="s">
         <v>705</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>706</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>707</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>708</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>707</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>708</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>709</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>710</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>711</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="G9" s="5" t="s">
         <v>712</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>713</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>714</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>714</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>715</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>716</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>717</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>718</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>719</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>720</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>722</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>723</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>724</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="G11" s="5" t="s">
         <v>725</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>726</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>726</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>727</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>728</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>729</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>711</v>
-      </c>
-      <c r="E12" s="5" t="s">
+      <c r="G12" s="5" t="s">
         <v>730</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>731</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>732</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>731</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>732</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>733</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="F13" s="5" t="s">
         <v>734</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>724</v>
-      </c>
-      <c r="E13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>735</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>736</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>736</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>737</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>738</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>739</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>724</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>740</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>741</v>
-      </c>
       <c r="G14" s="5" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-047 Add app users migration task
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -32,8 +32,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DB Schema + RLS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Dependencies!$A$1:$F$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Release Checklist'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Risks &amp; Decisions'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$74</definedName>
@@ -18396,7 +18396,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19772,9 +19772,101 @@
         <v>13</v>
       </c>
     </row>
+    <row r="48" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>CODE-047</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>migrations</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>supabase/migrations/20260804184922_create_app_users.sql</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Create app_users migration</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Create one ordered, timestamped Supabase PostgreSQL migration for
+public.app_users.
+Define id as uuid primary key referencing auth.users(id), with no generated
+default and ON DELETE CASCADE, so each Supabase authentication identity has at
+most one application profile.
+Define tenant_id as uuid NOT NULL referencing public.tenants(id) with
+ON DELETE RESTRICT, modeling one tenant per app user.
+Define role as text NOT NULL with an exact check constraint allowing only:
+- admin
+- dispatcher
+- car_puller
+Define full_name and phone as text NOT NULL. Do not duplicate authentication
+email and do not add status, membership, invitation, or separate profile fields.
+Add created_at and updated_at as timestamptz NOT NULL DEFAULT now(). Add
+created_by and updated_by as nullable uuid columns without foreign keys at this
+stage.
+Attach a BEFORE UPDATE trigger that executes public.set_updated_at(). Add an
+index on tenant_id.
+Enable row-level security, but do not create access policies because app-user
+and tenant policies belong to IAM-014.
+Do not modify authentication, API, frontend, invitation, profile, membership,
+or other application files. Apply and verify only against the local Supabase
+database. Do not apply the migration to the hosted project.</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>IAM-011</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>The timestamped migration creates public.app_users with id, tenant_id, role,
+full_name, phone, created_at, updated_at, created_by, and updated_by.
+id is a uuid primary key referencing auth.users(id), has no generated default,
+and uses ON DELETE CASCADE. Inserting an app-user requires an existing auth user,
+and duplicate profiles for one authentication identity are rejected.
+tenant_id is required, references public.tenants(id), and uses ON DELETE
+RESTRICT.
+role is required and accepts only admin, dispatcher, or car_puller. Invalid role
+values are rejected. full_name and phone are required.
+created_at and updated_at use timestamptz NOT NULL DEFAULT now(). created_by and
+updated_by are nullable uuid columns without foreign keys.
+A BEFORE UPDATE trigger invokes public.set_updated_at(), and updating a profile
+changes updated_at. An index exists on tenant_id.
+RLS is enabled without adding IAM-014 access policies. The migration applies
+successfully to the local Supabase database. Privileged local verification
+confirms:
+- A valid linked app-user can be inserted.
+- An invalid auth-user ID is rejected.
+- An invalid tenant ID is rejected.
+- A duplicate auth-user ID is rejected.
+- An invalid role is rejected.
+- updated_at advances after an update.
+No membership, invitation, API, frontend, or unrelated tables or files are
+created, and no hosted-project migration is applied.</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I47" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I47">
+  <autoFilter ref="A1:I48" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <conditionalFormatting sqref="I2:I48">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -19792,7 +19884,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I47" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I48" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19806,7 +19898,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -20547,8 +20639,35 @@
         <v>1035</v>
       </c>
     </row>
+    <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>supabase/migrations/20260804184922_create_app_users.sql</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Create app_users migration</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>IAM-011</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>CODE-047</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E43" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
+  <autoFilter ref="A1:E44" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
CODE-047 Correct app users migration path
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andu_zed/Desktop/IAMONIT/iamonit-platform/planning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5976D16-CB74-D341-B99F-6DD1BFD3DEFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A36D3FCF-31B5-2542-9119-558448E42844}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3382" uniqueCount="1043">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3396" uniqueCount="1048">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3211,6 +3211,66 @@
 a duplicate tenant name is rejected; updating a tenant changes updated_at; no
 app_users, memberships, profiles, API files, or unrelated tables are created;
 and no hosted-project migration is applied.</t>
+  </si>
+  <si>
+    <t>CODE-047</t>
+  </si>
+  <si>
+    <t>supabase/migrations/20260804234822_create_app_users.sql</t>
+  </si>
+  <si>
+    <t>Create app_users migration</t>
+  </si>
+  <si>
+    <t>Create one ordered, timestamped Supabase PostgreSQL migration for
+public.app_users.
+Define id as uuid primary key referencing auth.users(id), with no generated
+default and ON DELETE CASCADE, so each Supabase authentication identity has at
+most one application profile.
+Define tenant_id as uuid NOT NULL referencing public.tenants(id) with
+ON DELETE RESTRICT, modeling one tenant per app user.
+Define role as text NOT NULL with an exact check constraint allowing only:
+- admin
+- dispatcher
+- car_puller
+Define full_name and phone as text NOT NULL. Do not duplicate authentication
+email and do not add status, membership, invitation, or separate profile fields.
+Add created_at and updated_at as timestamptz NOT NULL DEFAULT now(). Add
+created_by and updated_by as nullable uuid columns without foreign keys at this
+stage.
+Attach a BEFORE UPDATE trigger that executes public.set_updated_at(). Add an
+index on tenant_id.
+Enable row-level security, but do not create access policies because app-user
+and tenant policies belong to IAM-014.
+Do not modify authentication, API, frontend, invitation, profile, membership,
+or other application files. Apply and verify only against the local Supabase
+database. Do not apply the migration to the hosted project.</t>
+  </si>
+  <si>
+    <t>The timestamped migration creates public.app_users with id, tenant_id, role,
+full_name, phone, created_at, updated_at, created_by, and updated_by.
+id is a uuid primary key referencing auth.users(id), has no generated default,
+and uses ON DELETE CASCADE. Inserting an app-user requires an existing auth user,
+and duplicate profiles for one authentication identity are rejected.
+tenant_id is required, references public.tenants(id), and uses ON DELETE
+RESTRICT.
+role is required and accepts only admin, dispatcher, or car_puller. Invalid role
+values are rejected. full_name and phone are required.
+created_at and updated_at use timestamptz NOT NULL DEFAULT now(). created_by and
+updated_by are nullable uuid columns without foreign keys.
+A BEFORE UPDATE trigger invokes public.set_updated_at(), and updating a profile
+changes updated_at. An index exists on tenant_id.
+RLS is enabled without adding IAM-014 access policies. The migration applies
+successfully to the local Supabase database. Privileged local verification
+confirms:
+- A valid linked app-user can be inserted.
+- An invalid auth-user ID is rejected.
+- An invalid tenant ID is rejected.
+- A duplicate auth-user ID is rejected.
+- An invalid role is rejected.
+- updated_at advances after an update.
+No membership, invitation, API, frontend, or unrelated tables or files are
+created, and no hosted-project migration is applied.</t>
   </si>
 </sst>
 </file>
@@ -3374,15 +3434,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4080,7 +4140,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="13"/>
@@ -4092,7 +4152,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="13"/>
@@ -4116,7 +4176,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="12" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="13"/>
@@ -4150,7 +4210,7 @@
       <c r="H8" s="13"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B9" s="13"/>
@@ -4184,7 +4244,7 @@
       <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="13"/>
@@ -4218,7 +4278,7 @@
       <c r="H16" s="13"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B17" s="13"/>
@@ -4241,16 +4301,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A5:H6"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A4:H4"/>
     <mergeCell ref="A17:H18"/>
     <mergeCell ref="A9:H10"/>
     <mergeCell ref="A13:H14"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H6"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A4:H4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
@@ -5324,7 +5384,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="16" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="13"/>
@@ -5336,7 +5396,7 @@
       <c r="H1" s="13"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="13"/>
@@ -19773,95 +19833,32 @@
       </c>
     </row>
     <row r="48" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>CODE-047</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>migrations</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>supabase/migrations/20260804184922_create_app_users.sql</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Create app_users migration</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>Create one ordered, timestamped Supabase PostgreSQL migration for
-public.app_users.
-Define id as uuid primary key referencing auth.users(id), with no generated
-default and ON DELETE CASCADE, so each Supabase authentication identity has at
-most one application profile.
-Define tenant_id as uuid NOT NULL referencing public.tenants(id) with
-ON DELETE RESTRICT, modeling one tenant per app user.
-Define role as text NOT NULL with an exact check constraint allowing only:
-- admin
-- dispatcher
-- car_puller
-Define full_name and phone as text NOT NULL. Do not duplicate authentication
-email and do not add status, membership, invitation, or separate profile fields.
-Add created_at and updated_at as timestamptz NOT NULL DEFAULT now(). Add
-created_by and updated_by as nullable uuid columns without foreign keys at this
-stage.
-Attach a BEFORE UPDATE trigger that executes public.set_updated_at(). Add an
-index on tenant_id.
-Enable row-level security, but do not create access policies because app-user
-and tenant policies belong to IAM-014.
-Do not modify authentication, API, frontend, invitation, profile, membership,
-or other application files. Apply and verify only against the local Supabase
-database. Do not apply the migration to the hosted project.</t>
-        </is>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>IAM-011</t>
-        </is>
-      </c>
-      <c r="H48" s="5" t="inlineStr">
-        <is>
-          <t>The timestamped migration creates public.app_users with id, tenant_id, role,
-full_name, phone, created_at, updated_at, created_by, and updated_by.
-id is a uuid primary key referencing auth.users(id), has no generated default,
-and uses ON DELETE CASCADE. Inserting an app-user requires an existing auth user,
-and duplicate profiles for one authentication identity are rejected.
-tenant_id is required, references public.tenants(id), and uses ON DELETE
-RESTRICT.
-role is required and accepts only admin, dispatcher, or car_puller. Invalid role
-values are rejected. full_name and phone are required.
-created_at and updated_at use timestamptz NOT NULL DEFAULT now(). created_by and
-updated_by are nullable uuid columns without foreign keys.
-A BEFORE UPDATE trigger invokes public.set_updated_at(), and updating a profile
-changes updated_at. An index exists on tenant_id.
-RLS is enabled without adding IAM-014 access policies. The migration applies
-successfully to the local Supabase database. Privileged local verification
-confirms:
-- A valid linked app-user can be inserted.
-- An invalid auth-user ID is rejected.
-- An invalid tenant ID is rejected.
-- A duplicate auth-user ID is rejected.
-- An invalid role is rejected.
-- updated_at advances after an update.
-No membership, invitation, API, frontend, or unrelated tables or files are
-created, and no hosted-project migration is applied.</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Todo</t>
-        </is>
+      <c r="A48" s="5" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>1045</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>1046</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -20640,30 +20637,20 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Database</t>
-        </is>
-      </c>
-      <c r="B44" s="5" t="inlineStr">
-        <is>
-          <t>supabase/migrations/20260804184922_create_app_users.sql</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>Create app_users migration</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>IAM-011</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>CODE-047</t>
-        </is>
+      <c r="A44" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>1044</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>1043</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-047 Create app users migration
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -6346,7 +6346,7 @@
         <v>5</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>104</v>
@@ -9786,7 +9786,7 @@
         <v>5</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>96</v>
@@ -19858,7 +19858,7 @@
         <v>1047</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-004 Split authentication implementation scope
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -32,8 +32,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Backlog!$A$1:$P$74</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'DB Schema + RLS'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Dependencies!$A$1:$F$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'File-Class Map'!$A$1:$E$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IntelliJ Coding Tasks'!$A$1:$I$50</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Release Checklist'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Risks &amp; Decisions'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint Board'!$A$1:$J$74</definedName>
@@ -18456,7 +18456,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -18585,146 +18585,311 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>498</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>972</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>499</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>500</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>501</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>502</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>503</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>973</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>504</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>505</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>506</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>507</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>974</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>508</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>509</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>510</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>511</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>512</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>975</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>513</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>514</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>515</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>25</v>
+    <row r="5" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>CODE-048</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>auth / supabase</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/common/supabase/supabase.constants.ts; apps/api/src/common/supabase/supabase.provider.ts; apps/api/src/common/supabase/supabase.module.ts; apps/api/src/common/supabase/supabase.provider.spec.ts; apps/api/src/modules/auth/auth.types.ts; apps/api/src/modules/auth/dto/auth-response.dto.ts; apps/api/src/modules/auth/dto/register.dto.ts; apps/api/src/modules/auth/auth.module.ts; apps/api/package.json; ././pnpm-lock.yaml</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Create authentication integration foundation</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Install and configure @supabase/supabase-js and pg for the NestJS API. Create
+separate injectable Supabase public and admin clients. The public client uses
+SUPABASE_URL and SUPABASE_ANON_KEY. The admin client uses SUPABASE_URL and
+SUPABASE_SERVICE_ROLE_KEY and must remain server-only.
+Read configuration only through ConfigService. Never return, log, serialize, or
+otherwise expose the service-role key.
+Define the approved authentication response contract:
+- session is either null or an object containing accessToken, refreshToken,
+  expiresIn, expiresAt, and tokenType.
+- requiresEmailConfirmation is boolean.
+- user contains id, email, tenantId, role, fullName, and phone.
+Update RegisterDto so registration accepts only email, password, companyName,
+fullName, and phone. Remove the client-supplied role field. LoginDto remains
+email and password.
+Register the providers and authentication types through AuthModule. Add focused
+unit tests for provider construction, configuration validation, response
+mapping types, and secret boundaries.
+Do not implement registration orchestration, login behavior, controllers,
+database writes, JWT validation, guards, frontend changes, or hosted calls.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>IAM-015,IAM-016</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>The API package contains @supabase/supabase-js, pg, and required type
+dependencies. Injectable public and admin Supabase clients are available through
+Nest dependency injection. The public client uses only the anonymous key and the
+admin client uses the server-only service-role key.
+RegisterDto accepts email, password, companyName, fullName, and phone and no
+longer accepts role. Auth response DTOs represent the approved nullable-session,
+requiresEmailConfirmation, and user-context contract.
+Configuration is loaded through ConfigService. No secret value is printed,
+returned, committed, or exposed to frontend code. Unit tests pass. No Auth user,
+tenant, app-user, session, controller, RLS policy, frontend, or hosted-project
+operation is created.</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>CODE-005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.service.ts; apps/api/src/modules/auth/auth.repository.ts; apps/api/src/modules/auth/auth.service.spec.ts; apps/api/src/modules/auth/auth.repository.spec.ts</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Implement company registration orchestration</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Implement the registration service using the injectable Supabase clients and a
+PostgreSQL repository backed by pg and DATABASE_URL.
+Accept RegisterDto containing email, password, companyName, fullName, and phone.
+Do not accept or trust a client-supplied role. Assign admin to the first user.
+Create the Supabase Auth identity through the public sign-up capability and
+respect the Supabase email-confirmation setting. Then create exactly one tenant
+and one app_users record in one PostgreSQL transaction. The app_users id equals
+the Supabase Auth user id and references the new tenant.
+If the database transaction fails after Auth creation, roll back all database
+writes and attempt compensating deletion of the Auth identity through the admin
+client. If compensation fails, log only the orphaned Auth user identifier and a
+safe internal error; never log keys, passwords, access tokens, refresh tokens,
+or provider response bodies.
+Return the approved auth response. When Supabase returns no session because
+email confirmation is required, return session null and
+requiresEmailConfirmation true.
+Map duplicate email or tenant name to 409, provider unavailability to 503, and
+unexpected or failed-compensation errors to 500.
+Do not create transporter_profiles, controllers, login behavior, guards, JWT
+strategy code, RLS policies, frontend code, or hosted operations.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>IAM-015</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Successful registration creates exactly one Supabase Auth identity, one tenant,
+and one linked app_users row with role admin. Tenant and app-user writes occur
+in one PostgreSQL transaction.
+The returned response follows the approved session and user-context contract.
+When email confirmation is required, session is null and
+requiresEmailConfirmation is true.
+A database failure leaves no tenant or app_users records and triggers
+compensating Auth-user deletion. Tests cover successful registration, role
+derivation, duplicate email, duplicate company name, Auth failure, transaction
+rollback, successful compensation, failed compensation, confirmation-required
+responses, session responses, and secret-safe errors.
+No transporter profile, controller, login implementation, RLS policy, frontend
+file, hosted database, or hosted Auth operation is modified.</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>CODE-049</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.service.ts; apps/api/src/modules/auth/auth.repository.ts; apps/api/src/modules/auth/auth.service.spec.ts; apps/api/src/modules/auth/auth.repository.spec.ts</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Implement login service and user context</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Add login behavior to AuthService using the public Supabase client.
+Authenticate email and password through Supabase Auth. For a successful session,
+load the linked public.app_users record and return user context containing id,
+email, tenantId, role, fullName, and phone.
+Return the approved non-null session object containing accessToken,
+refreshToken, expiresIn, expiresAt, and tokenType, with
+requiresEmailConfirmation false.
+Map invalid credentials to 401. Map a valid Auth identity without a linked
+app_users profile to 403. Map Supabase availability errors to 503 and unexpected
+consistency failures to a safe 500.
+Never use or expose the service-role key for password authentication. Do not
+implement controllers, JWT strategy, guards, refresh endpoints, logout,
+frontend integration, RLS policies, or hosted operations.</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>IAM-016</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Valid credentials return a Supabase session and linked app-user context
+containing user id, email, tenant id, role, full name, and phone. Invalid
+credentials return 401 without revealing whether the email exists.
+A valid Auth identity without an app_users row returns 403. Provider
+unavailability returns 503. Unexpected failures return a safe 500.
+Tests cover valid login, invalid credentials, missing profile, session mapping,
+tenant and role context, provider failure, and absence of secrets in responses
+and logs.
+No controller, JWT strategy, guard, registration side effect, frontend file,
+RLS policy, hosted database, or hosted Auth project is modified.</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="288" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>CODE-004</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>auth</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.controller.ts; apps/api/src/modules/auth/auth.controller.spec.ts</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Implement register and login controllers</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Implement thin NestJS controller endpoints backed only by AuthService.
+POST /auth/register accepts RegisterDto, delegates to AuthService.register, and
+returns the approved AuthResponseDto with HTTP 201.
+POST /auth/login accepts LoginDto, delegates to AuthService.login, and returns
+the approved AuthResponseDto with HTTP 200.
+The controller must not instantiate Supabase clients, access ConfigService,
+perform database queries, manage transactions, create JWTs, or expose provider
+errors. Preserve Nest DTO validation and service-level safe exception mappings.
+Do not modify services, repositories, Supabase providers, JWT strategy, guards,
+frontend files, RLS policies, or hosted resources.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>IAM-015,IAM-016</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>POST /auth/register returns HTTP 201 and the AuthService registration response.
+POST /auth/login returns HTTP 200 and the AuthService login response.
+Controller tests verify DTO delegation, status codes, response forwarding, and
+safe propagation of documented HTTP exceptions. The controller contains no
+Supabase, database, transaction, JWT-signing, or secret-handling logic.</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Todo</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>512</v>
+        <v>490</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>518</v>
+        <v>509</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>25</v>
@@ -18732,28 +18897,28 @@
     </row>
     <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>522</v>
+        <v>513</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>523</v>
+        <v>514</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>524</v>
+        <v>515</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>25</v>
@@ -18761,28 +18926,28 @@
     </row>
     <row r="11" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>525</v>
+        <v>516</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>526</v>
+        <v>512</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>528</v>
+        <v>518</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>529</v>
+        <v>519</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>25</v>
@@ -18790,57 +18955,57 @@
     </row>
     <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>530</v>
+        <v>520</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>532</v>
+        <v>523</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>533</v>
+        <v>524</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>534</v>
+        <v>525</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>535</v>
+        <v>526</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>536</v>
+        <v>527</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>537</v>
+        <v>528</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>538</v>
+        <v>161</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>539</v>
+        <v>529</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>25</v>
@@ -18848,94 +19013,94 @@
     </row>
     <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>535</v>
+        <v>526</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>931</v>
+        <v>979</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>541</v>
+        <v>531</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>538</v>
+        <v>161</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>543</v>
+        <v>533</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>546</v>
+        <v>536</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>547</v>
+        <v>537</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>195</v>
+        <v>538</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>548</v>
+        <v>539</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>549</v>
+        <v>540</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>982</v>
+        <v>931</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>551</v>
+        <v>542</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>553</v>
+        <v>543</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>554</v>
+        <v>544</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>64</v>
@@ -18944,19 +19109,19 @@
         <v>545</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>939</v>
+        <v>981</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>555</v>
+        <v>546</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>556</v>
+        <v>547</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>552</v>
+        <v>195</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>557</v>
+        <v>548</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>25</v>
@@ -18964,7 +19129,7 @@
     </row>
     <row r="18" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>558</v>
+        <v>549</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>64</v>
@@ -18973,280 +19138,280 @@
         <v>545</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>940</v>
+        <v>982</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>559</v>
+        <v>550</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>560</v>
+        <v>551</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>213</v>
+        <v>552</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>563</v>
+        <v>545</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>983</v>
+        <v>939</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>564</v>
+        <v>555</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>565</v>
+        <v>556</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>240</v>
+        <v>552</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>566</v>
+        <v>557</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>567</v>
+        <v>558</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>563</v>
+        <v>545</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>984</v>
+        <v>940</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>568</v>
+        <v>559</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>569</v>
+        <v>560</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>240</v>
+        <v>213</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>570</v>
+        <v>561</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>571</v>
+        <v>562</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>572</v>
+        <v>563</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>573</v>
+        <v>564</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>574</v>
+        <v>565</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>575</v>
+        <v>566</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C22" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>984</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>568</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A23" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>985</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>574</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>575</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>577</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>950</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>578</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F24" s="5" t="s">
         <v>579</v>
       </c>
-      <c r="G22" s="5" t="s">
+      <c r="G24" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="H22" s="5" t="s">
+      <c r="H24" s="5" t="s">
         <v>580</v>
       </c>
-      <c r="I22" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" ht="112" x14ac:dyDescent="0.2">
-      <c r="A23" s="5" t="s">
+      <c r="I24" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
         <v>581</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>986</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>582</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>1022</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>1023</v>
-      </c>
-      <c r="I23" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" ht="160" x14ac:dyDescent="0.2">
-      <c r="A24" s="5" t="s">
-        <v>584</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>987</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>585</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>1024</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>1025</v>
-      </c>
-      <c r="I24" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="5" t="s">
-        <v>586</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>587</v>
+        <v>490</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>589</v>
+        <v>1022</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>590</v>
+        <v>1023</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="160" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
-        <v>591</v>
+        <v>584</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>587</v>
+        <v>490</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>593</v>
+        <v>1024</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>594</v>
+        <v>1025</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
-        <v>595</v>
+        <v>586</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>596</v>
+        <v>587</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>597</v>
+        <v>588</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>598</v>
+        <v>589</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>599</v>
+        <v>590</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>25</v>
@@ -19254,28 +19419,28 @@
     </row>
     <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>600</v>
+        <v>591</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>596</v>
+        <v>587</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>601</v>
+        <v>592</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>602</v>
+        <v>593</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>603</v>
+        <v>135</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>604</v>
+        <v>594</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>25</v>
@@ -19283,28 +19448,28 @@
     </row>
     <row r="29" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>605</v>
+        <v>595</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>545</v>
+        <v>596</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>220</v>
+        <v>597</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>606</v>
+        <v>598</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>607</v>
+        <v>172</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>608</v>
+        <v>599</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>25</v>
@@ -19312,28 +19477,28 @@
     </row>
     <row r="30" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
-        <v>609</v>
+        <v>600</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>545</v>
+        <v>596</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>225</v>
+        <v>601</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>610</v>
+        <v>602</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>224</v>
+        <v>603</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>611</v>
+        <v>604</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>25</v>
@@ -19341,7 +19506,7 @@
     </row>
     <row r="31" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
-        <v>612</v>
+        <v>605</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>59</v>
@@ -19350,19 +19515,19 @@
         <v>545</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>613</v>
+        <v>606</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>229</v>
+        <v>607</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>614</v>
+        <v>608</v>
       </c>
       <c r="I31" s="5" t="s">
         <v>25</v>
@@ -19370,7 +19535,7 @@
     </row>
     <row r="32" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>59</v>
@@ -19379,19 +19544,19 @@
         <v>545</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>616</v>
+        <v>225</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>617</v>
+        <v>610</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>266</v>
+        <v>224</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>618</v>
+        <v>611</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>25</v>
@@ -19399,28 +19564,28 @@
     </row>
     <row r="33" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
-        <v>619</v>
+        <v>612</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>563</v>
+        <v>545</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>946</v>
+        <v>994</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>620</v>
+        <v>230</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>250</v>
+        <v>229</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>622</v>
+        <v>614</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>25</v>
@@ -19428,123 +19593,123 @@
     </row>
     <row r="34" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
-        <v>623</v>
+        <v>615</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>624</v>
+        <v>545</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>949</v>
+        <v>995</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>626</v>
+        <v>617</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>627</v>
+        <v>618</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C35" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>946</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>621</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A36" s="5" t="s">
+        <v>623</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>949</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>626</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="I36" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A37" s="5" t="s">
+        <v>628</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>577</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>952</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E37" s="5" t="s">
         <v>629</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="F37" s="5" t="s">
         <v>630</v>
       </c>
-      <c r="G35" s="5" t="s">
+      <c r="G37" s="5" t="s">
         <v>291</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="H37" s="5" t="s">
         <v>631</v>
       </c>
-      <c r="I35" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A36" s="5" t="s">
+      <c r="I37" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A38" s="5" t="s">
         <v>632</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>633</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>1040</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>634</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>1041</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>1042</v>
-      </c>
-      <c r="I36" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="5" t="s">
-        <v>635</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>633</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="E37" s="5" t="s">
-        <v>636</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>637</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>638</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38" s="5" t="s">
-        <v>639</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>80</v>
@@ -19553,27 +19718,27 @@
         <v>633</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>124</v>
+        <v>1040</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>640</v>
+        <v>634</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>641</v>
+        <v>1041</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>642</v>
+        <v>1042</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
-        <v>643</v>
+        <v>635</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>80</v>
@@ -19582,19 +19747,19 @@
         <v>633</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>644</v>
+        <v>189</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>645</v>
+        <v>636</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>646</v>
+        <v>637</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>234</v>
+        <v>184</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>647</v>
+        <v>638</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>25</v>
@@ -19602,28 +19767,28 @@
     </row>
     <row r="40" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>648</v>
+        <v>639</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>339</v>
+        <v>80</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>649</v>
+        <v>633</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>996</v>
+        <v>124</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>650</v>
+        <v>640</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>651</v>
+        <v>641</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>341</v>
+        <v>117</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>652</v>
+        <v>642</v>
       </c>
       <c r="I40" s="5" t="s">
         <v>25</v>
@@ -19631,94 +19796,94 @@
     </row>
     <row r="41" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
+        <v>643</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>645</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>646</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>647</v>
+      </c>
+      <c r="I41" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>649</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>996</v>
+      </c>
+      <c r="E42" s="5" t="s">
+        <v>650</v>
+      </c>
+      <c r="F42" s="5" t="s">
+        <v>651</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>652</v>
+      </c>
+      <c r="I42" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+      <c r="A43" s="5" t="s">
         <v>653</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B43" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C43" s="5" t="s">
         <v>654</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D43" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E43" s="5" t="s">
         <v>655</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F43" s="5" t="s">
         <v>656</v>
       </c>
-      <c r="G41" s="5" t="s">
+      <c r="G43" s="5" t="s">
         <v>351</v>
       </c>
-      <c r="H41" s="5" t="s">
+      <c r="H43" s="5" t="s">
         <v>657</v>
       </c>
-      <c r="I41" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="64" x14ac:dyDescent="0.2">
-      <c r="A42" s="5" t="s">
+      <c r="I43" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="64" x14ac:dyDescent="0.2">
+      <c r="A44" s="5" t="s">
         <v>913</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>914</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>915</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>916</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>917</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>918</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>903</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>919</v>
-      </c>
-      <c r="I42" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" ht="80" x14ac:dyDescent="0.2">
-      <c r="A43" s="5" t="s">
-        <v>997</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>914</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>915</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>998</v>
-      </c>
-      <c r="E43" s="5" t="s">
-        <v>999</v>
-      </c>
-      <c r="F43" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>963</v>
-      </c>
-      <c r="H43" s="5" t="s">
-        <v>1001</v>
-      </c>
-      <c r="I43" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" ht="144" x14ac:dyDescent="0.2">
-      <c r="A44" s="5" t="s">
-        <v>1010</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>914</v>
@@ -19727,143 +19892,201 @@
         <v>915</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>1007</v>
+        <v>916</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>1011</v>
+        <v>917</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>1012</v>
+        <v>918</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>1002</v>
+        <v>903</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>1013</v>
+        <v>919</v>
       </c>
       <c r="I44" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
-        <v>1016</v>
+        <v>997</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>59</v>
+        <v>914</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>1017</v>
+        <v>915</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>1018</v>
+        <v>998</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>1019</v>
+        <v>999</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>1020</v>
+        <v>1000</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>57</v>
+        <v>963</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>1021</v>
+        <v>1001</v>
       </c>
       <c r="I45" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="128" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="144" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
-        <v>1030</v>
+        <v>1010</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>80</v>
+        <v>914</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>1031</v>
+        <v>915</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>81</v>
+        <v>1007</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>1032</v>
+        <v>1011</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>1033</v>
+        <v>1012</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>75</v>
+        <v>1002</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>1034</v>
+        <v>1013</v>
       </c>
       <c r="I46" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" ht="96" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
-        <v>1035</v>
+        <v>1016</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>633</v>
+        <v>1017</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>1039</v>
+        <v>1018</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>1036</v>
+        <v>1019</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>1037</v>
+        <v>1020</v>
       </c>
       <c r="G47" s="5" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>1038</v>
+        <v>1021</v>
       </c>
       <c r="I47" s="5" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" ht="128" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
-        <v>1043</v>
+        <v>1030</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>80</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>633</v>
+        <v>1031</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>1044</v>
+        <v>81</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>1045</v>
+        <v>1032</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>1046</v>
+        <v>1033</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>1047</v>
+        <v>1034</v>
       </c>
       <c r="I48" s="5" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="49" spans="1:9" ht="144" x14ac:dyDescent="0.2">
+      <c r="A49" s="5" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>1039</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>1036</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>1037</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H49" s="5" t="s">
+        <v>1038</v>
+      </c>
+      <c r="I49" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A50" s="5" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>1045</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>1046</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>1047</v>
+      </c>
+      <c r="I50" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I48" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
-  <conditionalFormatting sqref="I2:I48">
+  <autoFilter ref="A1:I50" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <conditionalFormatting sqref="I2:I50">
     <cfRule type="expression" dxfId="14" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -19881,7 +20104,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="I2:I48" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="I2:I50" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Todo,In Progress,Blocked,Review,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -19895,7 +20118,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -19973,72 +20196,112 @@
         <v>494</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>972</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>499</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>501</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>973</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>504</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>974</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>508</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>975</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>513</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>511</v>
+    <row r="5" spans="1:5" ht="64" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/common/supabase/supabase.constants.ts; apps/api/src/common/supabase/supabase.provider.ts; apps/api/src/common/supabase/supabase.module.ts; apps/api/src/common/supabase/supabase.provider.spec.ts; apps/api/src/modules/auth/auth.types.ts; apps/api/src/modules/auth/dto/auth-response.dto.ts; apps/api/src/modules/auth/dto/register.dto.ts; apps/api/src/modules/auth/auth.module.ts; apps/api/package.json; ././pnpm-lock.yaml</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Create authentication integration foundation</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>IAM-015,IAM-016</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>CODE-048</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.service.ts; apps/api/src/modules/auth/auth.repository.ts; apps/api/src/modules/auth/auth.service.spec.ts; apps/api/src/modules/auth/auth.repository.spec.ts</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Implement company registration orchestration</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>IAM-015</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>CODE-005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="48" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.service.ts; apps/api/src/modules/auth/auth.repository.ts; apps/api/src/modules/auth/auth.service.spec.ts; apps/api/src/modules/auth/auth.repository.spec.ts</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Implement login service and user context</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>IAM-016</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>CODE-049</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="32" x14ac:dyDescent="0.2">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>apps/api/src/modules/auth/auth.controller.ts; apps/api/src/modules/auth/auth.controller.spec.ts</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Implement register and login controllers</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>IAM-015,IAM-016</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>CODE-004</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20046,16 +20309,16 @@
         <v>64</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>976</v>
+        <v>974</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20063,16 +20326,16 @@
         <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>977</v>
+        <v>975</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>522</v>
+        <v>513</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20080,16 +20343,16 @@
         <v>64</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>978</v>
+        <v>976</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>527</v>
+        <v>517</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>161</v>
+        <v>141</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>525</v>
+        <v>516</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20097,16 +20360,16 @@
         <v>64</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>979</v>
+        <v>977</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>530</v>
+        <v>520</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20114,16 +20377,16 @@
         <v>64</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>536</v>
+        <v>527</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>538</v>
+        <v>161</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>534</v>
+        <v>525</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20131,16 +20394,16 @@
         <v>64</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>931</v>
+        <v>979</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>541</v>
+        <v>531</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>538</v>
+        <v>161</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20148,16 +20411,16 @@
         <v>64</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>546</v>
+        <v>536</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>195</v>
+        <v>538</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20165,16 +20428,16 @@
         <v>64</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>982</v>
+        <v>931</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>549</v>
+        <v>540</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20182,16 +20445,16 @@
         <v>64</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>939</v>
+        <v>981</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>555</v>
+        <v>546</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>552</v>
+        <v>195</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>554</v>
+        <v>544</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20199,16 +20462,16 @@
         <v>64</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>940</v>
+        <v>982</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>559</v>
+        <v>550</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>213</v>
+        <v>552</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>558</v>
+        <v>549</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20216,16 +20479,16 @@
         <v>64</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>983</v>
+        <v>939</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>564</v>
+        <v>555</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>240</v>
+        <v>552</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20233,16 +20496,16 @@
         <v>64</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>984</v>
+        <v>940</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>568</v>
+        <v>559</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>240</v>
+        <v>213</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>567</v>
+        <v>558</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20250,16 +20513,16 @@
         <v>64</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>573</v>
+        <v>564</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>571</v>
+        <v>562</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20267,50 +20530,50 @@
         <v>64</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>950</v>
+        <v>984</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>578</v>
+        <v>568</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>282</v>
+        <v>240</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>582</v>
+        <v>573</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>92</v>
+        <v>262</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>581</v>
+        <v>571</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>987</v>
+        <v>950</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>92</v>
+        <v>282</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>584</v>
+        <v>576</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20318,16 +20581,16 @@
         <v>59</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20335,16 +20598,16 @@
         <v>59</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>591</v>
+        <v>584</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20352,16 +20615,16 @@
         <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>990</v>
+        <v>988</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>597</v>
+        <v>588</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>172</v>
+        <v>135</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>595</v>
+        <v>586</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20369,16 +20632,16 @@
         <v>59</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>991</v>
+        <v>989</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>601</v>
+        <v>592</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>603</v>
+        <v>135</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>600</v>
+        <v>591</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20386,16 +20649,16 @@
         <v>59</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>220</v>
+        <v>597</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>607</v>
+        <v>172</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>605</v>
+        <v>595</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20403,16 +20666,16 @@
         <v>59</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>225</v>
+        <v>601</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>224</v>
+        <v>603</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>609</v>
+        <v>600</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20420,16 +20683,16 @@
         <v>59</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>994</v>
+        <v>992</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>229</v>
+        <v>607</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>612</v>
+        <v>605</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20437,16 +20700,16 @@
         <v>59</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>995</v>
+        <v>993</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>616</v>
+        <v>225</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>266</v>
+        <v>224</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20454,16 +20717,16 @@
         <v>59</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>946</v>
+        <v>994</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>620</v>
+        <v>230</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>250</v>
+        <v>229</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>619</v>
+        <v>612</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20471,16 +20734,16 @@
         <v>59</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>949</v>
+        <v>995</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>625</v>
+        <v>616</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>623</v>
+        <v>615</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20488,50 +20751,50 @@
         <v>59</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>952</v>
+        <v>946</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>629</v>
+        <v>620</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>291</v>
+        <v>250</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>628</v>
+        <v>619</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>1040</v>
+        <v>949</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>634</v>
+        <v>625</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>96</v>
+        <v>271</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>632</v>
+        <v>623</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>189</v>
+        <v>952</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>636</v>
+        <v>629</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>184</v>
+        <v>291</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>635</v>
+        <v>628</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20539,16 +20802,16 @@
         <v>80</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>124</v>
+        <v>1040</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>640</v>
+        <v>634</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>117</v>
+        <v>96</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20556,84 +20819,84 @@
         <v>80</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>644</v>
+        <v>189</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>645</v>
+        <v>636</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>234</v>
+        <v>184</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>643</v>
+        <v>635</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
-        <v>339</v>
+        <v>80</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>996</v>
+        <v>124</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>650</v>
+        <v>640</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>341</v>
+        <v>117</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>648</v>
+        <v>639</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
-        <v>339</v>
+        <v>80</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>356</v>
+        <v>644</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>655</v>
+        <v>645</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>351</v>
+        <v>234</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>653</v>
+        <v>643</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
-        <v>80</v>
+        <v>339</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>81</v>
+        <v>996</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1032</v>
+        <v>650</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>75</v>
+        <v>341</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>1030</v>
+        <v>648</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
-        <v>80</v>
+        <v>339</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>1039</v>
+        <v>356</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>1036</v>
+        <v>655</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>82</v>
+        <v>351</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>1035</v>
+        <v>653</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -20641,20 +20904,54 @@
         <v>80</v>
       </c>
       <c r="B44" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>1032</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A45" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E45" s="5" t="s">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A46" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B46" s="5" t="s">
         <v>1044</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>1045</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="D46" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="E46" s="5" t="s">
         <v>1043</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E44" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
+  <autoFilter ref="A1:E46" xr:uid="{00000000-0009-0000-0000-000007000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
CODE-004 Implement register and login controllers
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -6538,7 +6538,7 @@
         <v>8</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>127</v>
@@ -9914,7 +9914,7 @@
         <v>8</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>129</v>
@@ -18862,7 +18862,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CODE-006 Correct Supabase token verification scope
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3396" uniqueCount="1048">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3400" uniqueCount="1052">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3271,6 +3271,93 @@
 - updated_at advances after an update.
 No membership, invitation, API, frontend, or unrelated tables or files are
 created, and no hosted-project migration is applied.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps/api/src/modules/auth/jwt.strategy.ts;
+apps/api/src/modules/auth/jwt.strategy.spec.ts;
+apps/api/src/modules/auth/auth.repository.ts;
+apps/api/src/modules/auth/auth.repository.spec.ts;
+apps/api/src/modules/auth/auth.types.ts;
+apps/api/src/modules/auth/auth.module.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement Supabase token verification and authenticated context</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement an injectable Supabase access-token verifier through the existing
+public Supabase client. Do not mint or verify a separate application JWT and do
+not use JWT_SECRET.
+Accept an access-token string from the later CODE-007 authentication guard.
+Verify it using supabase.auth.getClaims(token). Require successful provider
+verification, an unexpired token, the configured Supabase issuer, an audience
+containing authenticated, an authenticated Supabase Auth role, and a valid UUID
+subject. Reject malformed, expired, wrongly issued, wrongly scoped, or
+unverifiable tokens with a safe UnauthorizedException.
+Treat the verified subject as the Supabase Auth user ID. Extend AuthRepository
+with an authoritative query joining public.app_users and public.tenants. Load
+tenant ID, application role, tenant existence, and tenant status from
+PostgreSQL. Do not trust JWT metadata for the IAMONIT tenant or application
+role.
+Require an existing app-user profile, an existing tenant, tenant status exactly
+active, and an application role exactly equal to admin, dispatcher, or
+car_puller.
+Return a typed authenticated context exactly containing:
+{
+  userId: string;
+  tenantId: string;
+  role: 'admin' | 'dispatcher' | 'car_puller';
+}
+Map invalid token or claim validation to 401. Map a missing app-user profile,
+missing tenant, or non-active tenant to 403. Map Supabase Auth or PostgreSQL
+availability failures to 503. Map invalid stored role/context and unexpected
+consistency failures to a safe 500.
+Register and export the verifier through AuthModule.
+Never expose or log an access token, refresh token, password, anonymous key,
+service-role key, JWT secret, provider response body, database URL, or database
+connection value.
+Token validation is signature-and-claims based. Immediate server-side session
+revocation checking is outside this task.
+Do not implement bearer-header extraction, an HTTP authentication guard,
+request.user attachment, role decorators, role authorization, custom JWT
+creation, refresh/logout behavior, controller changes, frontend changes, RLS
+changes, hosted Auth calls, or hosted database operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A valid Supabase access token is verified through the existing public Supabase
+client and explicitly checked for expiration, configured issuer, authenticated
+audience, authenticated Auth role, and valid UUID subject. JWT_SECRET is not
+used, and no custom application JWT is created.
+The verified subject is used to load current application access by joining
+public.app_users and public.tenants. The returned context is exactly
+{ userId, tenantId, role }. Tenant ID and application role come from PostgreSQL,
+not JWT metadata.
+Invalid, malformed, expired, wrongly issued, wrongly scoped, or unverifiable
+tokens return a safe 401.
+A missing app-user profile, missing tenant, or non-active tenant returns 403.
+Supabase Auth or PostgreSQL unavailability returns 503. An invalid stored
+application role or unexpected consistency failure returns a safe 500.
+Tests cover:
+- Valid token verification and context return
+- Correct subject-to-userId mapping
+- Database-derived tenant and role
+- admin, dispatcher, and car_puller roles
+- Missing or malformed token input
+- Invalid or expired token
+- Wrong issuer
+- Wrong audience
+- Missing or malformed subject
+- Missing app-user profile
+- Missing tenant
+- Non-active tenant
+- Invalid stored role
+- Supabase availability failure
+- PostgreSQL availability failure
+- Safe unexpected failures
+- Absence of tokens, secrets, provider bodies, and database URLs from errors
+  and logs
+Only the six authorized CODE-006 source/test/module/type paths are modified.
+No guard, request.user attachment, role authorization, controller, frontend,
+RLS policy, hosted Auth operation, or hosted database operation is created.</t>
   </si>
 </sst>
 </file>
@@ -18877,19 +18964,19 @@
         <v>490</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>974</v>
+        <v>1048</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>508</v>
+        <v>1049</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>509</v>
+        <v>1050</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>130</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>510</v>
+        <v>1051</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>25</v>
@@ -20309,10 +20396,10 @@
         <v>64</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>974</v>
+        <v>1048</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>508</v>
+        <v>1049</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>130</v>

</xml_diff>

<commit_message>
CODE-006 Implement Supabase token verification and authenticated context
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -6673,7 +6673,7 @@
         <v>5</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>132</v>
@@ -10033,7 +10033,7 @@
         <v>5</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>134</v>
@@ -18979,7 +18979,7 @@
         <v>1051</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
CODE-007 Correct authentication guard scope
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3400" uniqueCount="1052">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3404" uniqueCount="1056">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3358,6 +3358,67 @@
 Only the six authorized CODE-006 source/test/module/type paths are modified.
 No guard, request.user attachment, role authorization, controller, frontend,
 RLS policy, hosted Auth operation, or hosted database operation is created.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps/api/src/common/guards/auth.guard.ts;
+apps/api/src/common/guards/auth.guard.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create bearer authentication guard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implement an injectable NestJS CanActivate guard.
+Read the HTTP Authorization header from the request. Require exactly one
+Bearer access token using the case-insensitive Bearer authentication scheme.
+Reject these cases with a safe UnauthorizedException:
+- Missing Authorization header
+- Non-string Authorization header
+- Empty bearer token
+- Unsupported authentication scheme
+- Malformed header
+- Multiple credential values
+Pass only the extracted access-token string to the Supabase token verifier
+implemented by CODE-006. Do not decode, verify, or inspect JWT claims directly
+inside the guard.
+After successful verification, attach the returned authenticated context to:
+request.user
+The attached value must be exactly:
+{
+  userId: string;
+  tenantId: string;
+  role: 'admin' | 'dispatcher' | 'car_puller';
+}
+Return true only after request.user has been populated.
+Preserve the verifier's safe 401, 403, 500, and 503 exceptions without exposing
+provider details.
+Do not log or expose the Authorization header, token, password, access token,
+refresh token, anonymous key, service-role key, JWT secret, provider response,
+or database value.
+Do not perform:
+- Supabase calls directly
+- PostgreSQL queries
+- JWT decoding or cryptography
+- Application-role authorization
+- Controller changes
+- Global guard registration
+- Frontend changes
+- RLS changes
+- Hosted operations
+CODE-008 remains responsible for @Roles metadata and role authorization.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- A valid Bearer token is passed exactly once to the CODE-006 verifier.
+- Successful verification attaches exactly { userId, tenantId, role } to
+  request.user and returns true.
+- A missing token returns 401.
+- A malformed Authorization header returns 401.
+- Unsupported authentication schemes return 401.
+- Empty or multiple credentials return 401.
+- Verifier exceptions propagate safely.
+- Tests confirm tokens and secrets never appear in errors or logs.
+- Only auth.guard.ts and auth.guard.spec.ts are modified.
+- No role comparison, database access, Supabase access, JWT verification,
+  controller change, frontend change, or hosted operation is implemented.</t>
   </si>
 </sst>
 </file>
@@ -18993,19 +19054,19 @@
         <v>512</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>975</v>
+        <v>1052</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>513</v>
+        <v>1053</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>514</v>
+        <v>1054</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>141</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>515</v>
+        <v>1055</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>25</v>
@@ -20413,10 +20474,10 @@
         <v>64</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>975</v>
+        <v>1052</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>513</v>
+        <v>1053</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>141</v>

</xml_diff>

<commit_message>
CODE-008 Correct role authorization scope
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3404" uniqueCount="1056">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3408" uniqueCount="1060">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3419,6 +3419,59 @@
 - Only auth.guard.ts and auth.guard.spec.ts are modified.
 - No role comparison, database access, Supabase access, JWT verification,
   controller change, frontend change, or hosted operation is implemented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps/api/src/common/decorators/roles.decorator.ts;
+apps/api/src/common/guards/roles.guard.ts;
+apps/api/src/common/guards/roles.guard.spec.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create roles decorator and role authorization guard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a typed @Roles(...roles) decorator using NestJS SetMetadata.
+Supported application roles are exactly:
+- admin
+- dispatcher
+- car_puller
+Implement an injectable NestJS CanActivate RolesGuard using Reflector.
+Read required role metadata from the current handler and controller class.
+Handler-level metadata may override class-level metadata.
+When no role metadata exists, allow the request.
+When roles are required:
+- Read request.user populated by the CODE-007 authentication guard.
+- Require request.user to contain userId, tenantId, and a supported role.
+- Return true when the authenticated user's role matches one of the required
+  roles.
+- Return 403 ForbiddenException when the authenticated user has the wrong role.
+- Return 401 UnauthorizedException when authenticated user context is absent.
+Do not read or validate bearer tokens.
+Do not call Supabase.
+Do not query PostgreSQL.
+Do not decode or verify JWTs.
+Do not alter request.user.
+Do not implement controller endpoints.
+Do not register the guard globally.
+Do not change AuthModule.
+Do not modify frontend files, RLS policies, or hosted resources.
+Do not log or expose tokens, credentials, secrets, provider responses, database
+values, or authenticated personal information.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- @Roles('admin') stores typed role metadata.
+- Multiple allowed roles are supported.
+- No role metadata allows the request.
+- Matching method-level role allows the request.
+- Matching class-level role allows the request.
+- Handler-level metadata correctly overrides class-level metadata.
+- Wrong role returns 403.
+- Missing authenticated request.user returns 401 when roles are required.
+- The guard uses only request.user supplied by CODE-007.
+- Tests cover admin, dispatcher, car_puller, multiple roles, no metadata,
+  class metadata, handler metadata, wrong role, and missing user context.
+- Only the three authorized files are modified.
+- No authentication, token verification, database access, controller change,
+  frontend change, global registration, or hosted operation is implemented.</t>
   </si>
 </sst>
 </file>
@@ -19083,19 +19136,19 @@
         <v>512</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>976</v>
+        <v>1056</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>517</v>
+        <v>1057</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>518</v>
+        <v>1058</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>141</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>519</v>
+        <v>1059</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>25</v>
@@ -20491,10 +20544,10 @@
         <v>64</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>976</v>
+        <v>1056</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>517</v>
+        <v>1057</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>141</v>

</xml_diff>

<commit_message>
CODE-008 Create role authorization guard
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -6883,7 +6883,7 @@
         <v>5</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>144</v>
@@ -10211,7 +10211,7 @@
         <v>5</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>130</v>
@@ -19151,7 +19151,7 @@
         <v>1059</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
CODE-024 Correct frontend authentication integration scope
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3408" uniqueCount="1060">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3416" uniqueCount="1068">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3472,6 +3472,187 @@
 - Only the three authorized files are modified.
 - No authentication, token verification, database access, controller change,
   frontend change, global registration, or hosted operation is implemented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps/web/lib/api.ts;
+apps/web/lib/api.test.ts;
+apps/web/lib/auth.types.ts;
+apps/web/vitest.config.ts;
+apps/web/vitest.setup.ts;
+apps/web/package.json;
+././pnpm-lock.yaml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create typed frontend authentication API client and test foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configure a focused Vitest frontend test foundation using jsdom and React
+Testing Library dependencies needed by CODE-024 and the later CODE-025 page
+tests. Do not replace or modify Next.js runtime behavior.
+Create approved frontend authentication request and response types:
+RegisterRequest:
+{
+  email: string;
+  password: string;
+  companyName: string;
+  fullName: string;
+  phone: string;
+}
+LoginRequest:
+{
+  email: string;
+  password: string;
+}
+AuthSession:
+{
+  accessToken: string;
+  refreshToken: string;
+  expiresIn: number;
+  expiresAt: number;
+  tokenType: string;
+}
+AuthUserContext:
+{
+  id: string;
+  email: string;
+  tenantId: string;
+  role: 'admin' | 'dispatcher' | 'car_puller';
+  fullName: string;
+  phone: string;
+}
+AuthResponse:
+{
+  session: AuthSession | null;
+  requiresEmailConfirmation: boolean;
+  user: AuthUserContext;
+}
+Create a browser-safe fetch API client using NEXT_PUBLIC_API_URL.
+Normalize the configured base URL without silently inventing a fallback.
+Fail safely when NEXT_PUBLIC_API_URL is absent or invalid.
+Implement typed registration and login requests:
+POST /auth/register
+POST /auth/login
+Send JSON with Content-Type application/json.
+Support an optional bearer access token for later protected requests. When
+provided, send it through exactly one Authorization header.
+Parse successful JSON responses safely. Validate the expected authentication
+response shape before returning it.
+Create a typed safe API error containing only an HTTP status and an approved
+user-facing message.
+Preserve safe documented backend error messages where appropriate. Convert
+malformed JSON, unexpected response shapes, provider-detail responses,
+non-JSON responses, and network failures into generic safe messages.
+Never include or log passwords, access tokens, refresh tokens, Authorization
+headers, anonymous keys, service-role keys, cookies, provider response bodies,
+or environment values.
+Do not manage authentication sessions.
+Do not create a Supabase browser client.
+Do not modify login or registration pages.
+Do not redirect.
+Do not persist user information.
+Do not modify the backend.
+Do not contact hosted services.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Frontend tests run through an explicit package script.
+- The frontend test foundation supports CODE-024 unit tests and CODE-025 React
+  component tests.
+- Register requests use POST /auth/register and exactly the approved payload.
+- Login requests use POST /auth/login and exactly the approved payload.
+- Requests use the validated NEXT_PUBLIC_API_URL.
+- Successful authentication responses are parsed and validated.
+- Optional access tokens produce exactly one Bearer Authorization header.
+- No Authorization header is sent when no access token is provided.
+- Documented safe backend messages can be displayed.
+- Malformed, non-JSON, unexpected, and network failures return generic safe
+  errors.
+- Tests cover base URL validation, register requests, login requests,
+  successful responses, documented HTTP errors, malformed responses,
+  non-JSON responses, network failures, and bearer-header behavior.
+- Tests confirm credentials and session values never appear in errors or logs.
+- Only the seven authorized paths are modified.
+- No form integration, session storage, Supabase client, redirect, backend
+  change, or hosted operation is implemented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apps/web/lib/supabase.ts;
+apps/web/lib/auth.ts;
+apps/web/lib/auth.test.ts;
+apps/web/app/(auth)/login/page.tsx;
+apps/web/app/(auth)/login/page.test.tsx;
+apps/web/app/(auth)/register/page.tsx;
+apps/web/app/(auth)/register/page.test.tsx;
+apps/web/package.json;
+././pnpm-lock.yaml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connect registration and login pages to backend authentication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a browser-only Supabase client using the documented public
+NEXT_PUBLIC_SUPABASE_URL and NEXT_PUBLIC_SUPABASE_ANON_KEY configuration.
+Use the CODE-024 API client to call the completed NestJS authentication
+endpoints.
+Registration:
+- Remove the administrator/team-member role selector.
+- Do not send role.
+- Keep confirmPassword only for client-side validation.
+- Send exactly email, password, companyName, fullName, and phone.
+- Preserve loading state and prevent duplicate submission.
+- Display safe 409, 500, 503, malformed-response, and network errors.
+- When a session is returned, install the access and refresh tokens into the
+  browser Supabase client using its supported session API.
+- Retain the returned IAMONIT user context in memory for the current browser
+  lifecycle. Do not persist the user profile as an authorization source.
+- Temporarily redirect successful authenticated registration to / because
+  /dashboard is not implemented.
+- When session is null and requiresEmailConfirmation is true, do not establish
+  authenticated state. Show clear email-confirmation guidance and a link to
+  /login.
+Login:
+- Send exactly email and password.
+- Preserve loading state and prevent duplicate submission.
+- Display the generic safe 401 message for invalid credentials.
+- Display safe 403, 500, 503, malformed-response, and network errors.
+- Require a non-null approved session response.
+- Install the session into the browser Supabase client.
+- Retain the returned IAMONIT user context in memory for the current browser
+  lifecycle.
+- Temporarily redirect successful login to / because /dashboard and /my-tasks
+  are not implemented.
+Use Supabase-managed browser session persistence and refresh behavior. Do not
+manually write access or refresh tokens to localStorage, sessionStorage,
+cookies, or another custom token store.
+Frontend user context is display state only. Backend token verification and
+database-derived tenant/role context remain authoritative.
+If Supabase session installation fails, clear partial in-memory user state and
+show a safe generic error.
+Do not implement logout UI, protected-route middleware, dashboard state,
+custom refresh logic, custom JWTs, backend changes, RLS changes, CORS changes,
+or hosted operations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Register submits the exact approved backend request.
+- Registration role selection is removed.
+- confirmPassword is never sent.
+- Successful session registration establishes a Supabase browser session and
+  redirects to /.
+- Confirmation-required registration establishes no session and shows clear
+  guidance.
+- Login submits exactly email and password.
+- Successful login establishes a Supabase browser session and redirects to /.
+- Returned IAMONIT user context is available in memory to auth helpers.
+- Failed session establishment leaves no partial user state.
+- Loading and duplicate-submission protection remain functional.
+- Safe documented backend errors are displayed without exposing provider
+  details.
+- Tests cover registration payload, no role field, no confirmPassword field,
+  session registration, confirmation-required behavior, login payload,
+  session installation, user context, temporary redirects, validation,
+  duplicate submission, and safe failure handling.
+- No custom token persistence, logout UI, protected-route middleware, backend
+  change, RLS change, CORS change, or hosted operation is implemented.
+- Only the nine authorized paths are modified.</t>
   </si>
 </sst>
 </file>
@@ -19185,28 +19366,28 @@
     </row>
     <row r="13" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>525</v>
+        <v>586</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>526</v>
+        <v>587</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>978</v>
+        <v>1060</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>527</v>
+        <v>1061</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>528</v>
+        <v>1062</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>529</v>
+        <v>1063</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>25</v>
@@ -19214,57 +19395,57 @@
     </row>
     <row r="14" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>530</v>
+        <v>591</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>526</v>
+        <v>587</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>979</v>
+        <v>1064</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>531</v>
+        <v>1065</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>532</v>
+        <v>1066</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>533</v>
+        <v>1067</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
-        <v>534</v>
+        <v>525</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>535</v>
+        <v>526</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>980</v>
+        <v>978</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>536</v>
+        <v>527</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>537</v>
+        <v>528</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>538</v>
+        <v>161</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>539</v>
+        <v>529</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>25</v>
@@ -19272,94 +19453,94 @@
     </row>
     <row r="16" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>540</v>
+        <v>530</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>535</v>
+        <v>526</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>931</v>
+        <v>979</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>541</v>
+        <v>531</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>538</v>
+        <v>161</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>543</v>
+        <v>533</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>546</v>
+        <v>536</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>547</v>
+        <v>537</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>195</v>
+        <v>538</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>548</v>
+        <v>539</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
-        <v>549</v>
+        <v>540</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>982</v>
+        <v>931</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>551</v>
+        <v>542</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>552</v>
+        <v>538</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>553</v>
+        <v>543</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
-        <v>554</v>
+        <v>544</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>64</v>
@@ -19368,19 +19549,19 @@
         <v>545</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>939</v>
+        <v>981</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>555</v>
+        <v>546</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>556</v>
+        <v>547</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>552</v>
+        <v>195</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>557</v>
+        <v>548</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>25</v>
@@ -19388,7 +19569,7 @@
     </row>
     <row r="20" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
-        <v>558</v>
+        <v>549</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>64</v>
@@ -19397,254 +19578,254 @@
         <v>545</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>940</v>
+        <v>982</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>559</v>
+        <v>550</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>560</v>
+        <v>551</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>213</v>
+        <v>552</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>563</v>
+        <v>545</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>983</v>
+        <v>939</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>564</v>
+        <v>555</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>565</v>
+        <v>556</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>240</v>
+        <v>552</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>566</v>
+        <v>557</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
-        <v>567</v>
+        <v>558</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>563</v>
+        <v>545</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>984</v>
+        <v>940</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>568</v>
+        <v>559</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>569</v>
+        <v>560</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>240</v>
+        <v>213</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>570</v>
+        <v>561</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>571</v>
+        <v>562</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>572</v>
+        <v>563</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>985</v>
+        <v>983</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>573</v>
+        <v>564</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>574</v>
+        <v>565</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>575</v>
+        <v>566</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
-        <v>576</v>
+        <v>567</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C24" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>984</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>568</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A25" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>985</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>574</v>
+      </c>
+      <c r="G25" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>575</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="32" x14ac:dyDescent="0.2">
+      <c r="A26" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>577</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>950</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>578</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F26" s="5" t="s">
         <v>579</v>
       </c>
-      <c r="G24" s="5" t="s">
+      <c r="G26" s="5" t="s">
         <v>282</v>
       </c>
-      <c r="H24" s="5" t="s">
+      <c r="H26" s="5" t="s">
         <v>580</v>
       </c>
-      <c r="I24" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="112" x14ac:dyDescent="0.2">
-      <c r="A25" s="5" t="s">
+      <c r="I26" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="112" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
         <v>581</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>986</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>582</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>1022</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>1023</v>
-      </c>
-      <c r="I25" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="160" x14ac:dyDescent="0.2">
-      <c r="A26" s="5" t="s">
-        <v>584</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>987</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>585</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>1024</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>1025</v>
-      </c>
-      <c r="I26" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="5" t="s">
-        <v>586</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>587</v>
+        <v>490</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>588</v>
+        <v>582</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>589</v>
+        <v>1022</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>590</v>
+        <v>1023</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" ht="16" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="160" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>591</v>
+        <v>584</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>59</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>587</v>
+        <v>490</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>989</v>
+        <v>987</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>592</v>
+        <v>585</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>593</v>
+        <v>1024</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>594</v>
+        <v>1025</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="16" x14ac:dyDescent="0.2">
@@ -20816,10 +20997,10 @@
         <v>59</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>988</v>
+        <v>1060</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>588</v>
+        <v>1061</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>135</v>
@@ -20833,10 +21014,10 @@
         <v>59</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>989</v>
+        <v>1064</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>592</v>
+        <v>1065</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>135</v>

</xml_diff>

<commit_message>
CODE-025 Connect registration and login to backend authentication
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -7016,7 +7016,7 @@
         <v>5</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>138</v>
@@ -10360,7 +10360,7 @@
         <v>5</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>140</v>
@@ -19419,7 +19419,7 @@
         <v>1067</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="16" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
CODE-051 Define multi-tenant authentication repository foundation
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3465" uniqueCount="1073">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3479" uniqueCount="1078">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -1550,7 +1550,7 @@
     <t>Sprint 11</t>
   </si>
   <si>
-    <t>IAM-007,IAM-010,IAM-011</t>
+    <t>IAM-011,IAM-016,IAM-018</t>
   </si>
   <si>
     <t>supabase/migrations/20260808233000_multi_tenant_membership_foundation.sql</t>
@@ -2475,6 +2475,170 @@
 - No existing migration is edited.
 - No app_users cleanup is performed.
 - No backend/frontend source code is modified.
+- No hosted operation occurs.</t>
+  </si>
+  <si>
+    <t>CODE-051</t>
+  </si>
+  <si>
+    <t>apps/api/src/modules/auth/auth.repository.ts; apps/api/src/modules/auth/auth.repository.spec.ts; apps/api/src/modules/auth/auth.types.ts; apps/api/src/modules/auth/dto/auth-response.dto.ts</t>
+  </si>
+  <si>
+    <t>Create multi-tenant authentication repository and contract foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This task is a compatibility-first backend foundation.
+Do not change registration/login orchestration yet.
+Do not change controllers yet.
+Do not change frontend code.
+Do not change token verification yet.
+Do not change AuthGuard or RolesGuard yet.
+Do not remove public.app_users compatibility reads required by existing
+working authentication behavior.
+The purpose of CODE-051 is to introduce the correct multi-tenant repository
+queries and types alongside the currently working singular auth flow so later
+tasks can safely switch over.
+1. Add multi-tenant domain types.
+Keep the existing AuthRole definition.
+Add:
+MembershipStatus:
+- active
+- suspended
+- removed
+UserProfileRecord:
+- userId
+- fullName
+- phone
+MembershipSummary:
+- membershipId
+- tenantId
+- tenantName
+- role
+- status
+AuthenticatedIdentity:
+- userId
+TenantRequestContext:
+- userId
+- membershipId
+- tenantId
+- role
+Do not remove legacy AuthUserContext or AuthenticatedContext in this task if
+existing code still requires them.
+2. Add repository lookup for the person profile.
+Add a method equivalent to:
+findUserProfileById(userId)
+It must read from public.user_profiles.
+It must not use public.app_users as the authoritative source for this new
+method.
+Return null when no profile exists.
+3. Add repository lookup for all memberships belonging to a user.
+Add a method equivalent to:
+findMembershipsByUserId(userId)
+It must join:
+public.tenant_memberships
+public.tenants
+Return:
+- membershipId
+- tenantId
+- tenantName
+- role
+- membership status
+It must support zero, one, or multiple memberships.
+Do not assume one user has only one tenant.
+Do not collapse or overwrite memberships.
+Use deterministic ordering for testability.
+4. Add repository lookup for an active membership in a requested tenant.
+Add a method equivalent to:
+findActiveMembership(userId, tenantId)
+It must return the membership only when:
+- tenant_memberships.user_id matches
+- tenant_memberships.tenant_id matches
+- tenant_memberships.status = active
+- tenants.status = active
+It must return null when:
+- membership does not exist
+- membership is suspended
+- membership is removed
+- tenant is suspended
+- tenant is archived
+- user belongs to another tenant instead
+This method will later support TenantContextGuard.
+5. Add future multi-tenant response contract types without switching existing
+controllers/services to them yet.
+Within auth-response.dto.ts introduce compatible DTO definitions equivalent
+to:
+UserProfileDto:
+- userId
+- email
+- fullName
+- phone
+MembershipSummaryDto:
+- membershipId
+- tenantId
+- tenantName
+- role
+- status
+MultiTenantAuthResponseDto:
+- session
+- requiresEmailConfirmation
+- profile
+- memberships
+- selectedMembership
+selectedMembership must allow null.
+Do not remove or break the currently used AuthResponseDto yet.
+The existing auth flow must continue compiling and testing after this task.
+6. Repository tests must cover at minimum:
+- user profile lookup from user_profiles
+- missing profile returns null
+- zero memberships returns []
+- one membership
+- multiple memberships
+- same user with different roles in different tenants
+- membership tenant name returned from tenants
+- active membership lookup succeeds
+- suspended membership rejected
+- removed membership rejected
+- suspended tenant rejected
+- archived tenant rejected
+- membership belonging to another tenant is not returned
+- queries use tenant_memberships/user_profiles rather than relying on
+  singular app_users semantics
+7. This task must not:
+- write membership data
+- create tenants
+- create profiles
+- alter registration orchestration
+- alter login orchestration
+- alter Supabase Auth behavior
+- alter token verification
+- introduce tenant header parsing
+- introduce TenantContextGuard
+- alter RolesGuard
+- alter AuthGuard
+- alter RLS
+- modify migrations
+- modify frontend code
+- remove app_users compatibility code
+- contact hosted Supabase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- New user profile repository lookup reads public.user_profiles.
+- New membership repository lookup supports multiple tenant memberships.
+- One user may be represented with different roles in different tenants.
+- Active membership lookup validates both membership and tenant status.
+- No tenant is selected implicitly.
+- No role is derived globally for the user.
+- New types clearly separate identity, person profile, membership, and
+  tenant-request context.
+- Future multi-tenant auth response contract contains profile, memberships,
+  and selectedMembership.
+- Existing register/login behavior remains compatible.
+- Existing tests continue passing.
+- New repository tests pass.
+- API TypeScript build/typecheck passes.
+- No frontend files change.
+- No database migration changes.
+- No workbook modification occurs during eventual CODE-051 execution.
 - No hosted operation occurs.</t>
   </si>
   <si>
@@ -4740,22 +4904,22 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -4763,76 +4927,76 @@
         <v>619</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="D3" s="14" t="s">
+        <v>923</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>918</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>913</v>
-      </c>
       <c r="F3" s="14" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>120</v>
@@ -4840,79 +5004,79 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>936</v>
+        <v>941</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>937</v>
+        <v>942</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>939</v>
+        <v>944</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>941</v>
+        <v>946</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>942</v>
+        <v>947</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>943</v>
+        <v>948</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>944</v>
+        <v>949</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>945</v>
+        <v>950</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>273</v>
@@ -4920,59 +5084,59 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>948</v>
+        <v>953</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>951</v>
+        <v>956</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>952</v>
+        <v>957</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>953</v>
+        <v>958</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>954</v>
+        <v>959</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>955</v>
+        <v>960</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>957</v>
+        <v>962</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>959</v>
+        <v>964</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>362</v>
@@ -5004,25 +5168,25 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>960</v>
+        <v>965</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>961</v>
+        <v>966</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>962</v>
+        <v>967</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>963</v>
+        <v>968</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>964</v>
+        <v>969</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>22</v>
@@ -5030,25 +5194,25 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>965</v>
+        <v>970</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>966</v>
+        <v>971</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>967</v>
+        <v>972</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>968</v>
+        <v>973</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>969</v>
+        <v>974</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>970</v>
+        <v>975</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>971</v>
+        <v>976</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>25</v>
@@ -5056,25 +5220,25 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>972</v>
+        <v>977</v>
       </c>
       <c r="B3" s="14" t="s">
+        <v>978</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>979</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>973</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>974</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>968</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>975</v>
+        <v>980</v>
       </c>
       <c r="F3" s="14" t="s">
+        <v>981</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>976</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>971</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>25</v>
@@ -5082,22 +5246,22 @@
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>977</v>
+        <v>982</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>332</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>978</v>
+        <v>983</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>979</v>
+        <v>984</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>980</v>
+        <v>985</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>981</v>
+        <v>986</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>331</v>
@@ -5108,22 +5272,22 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>982</v>
+        <v>987</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>983</v>
+        <v>988</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>984</v>
+        <v>989</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>985</v>
+        <v>990</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>986</v>
+        <v>991</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>987</v>
+        <v>992</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>338</v>
@@ -5134,25 +5298,25 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>988</v>
+        <v>993</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>979</v>
+        <v>984</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>990</v>
+        <v>995</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>25</v>
@@ -5160,25 +5324,25 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>992</v>
+        <v>997</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>993</v>
+        <v>998</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>979</v>
+        <v>984</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>25</v>
@@ -5186,25 +5350,25 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>999</v>
+        <v>1004</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1000</v>
+        <v>1005</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1001</v>
+        <v>1006</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1002</v>
+        <v>1007</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1003</v>
+        <v>1008</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1004</v>
+        <v>1009</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>25</v>
@@ -5212,22 +5376,22 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1005</v>
+        <v>1010</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1006</v>
+        <v>1011</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1007</v>
+        <v>1012</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>985</v>
+        <v>990</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1009</v>
+        <v>1014</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>302</v>
@@ -5238,22 +5402,22 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1010</v>
+        <v>1015</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1011</v>
+        <v>1016</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1012</v>
+        <v>1017</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1013</v>
+        <v>1018</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>181</v>
@@ -5264,22 +5428,22 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1016</v>
+        <v>1021</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>1017</v>
+        <v>1022</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>1018</v>
+        <v>1023</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>194</v>
@@ -5290,22 +5454,22 @@
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1019</v>
+        <v>1024</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1020</v>
+        <v>1025</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1021</v>
+        <v>1026</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>968</v>
+        <v>973</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>1022</v>
+        <v>1027</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>1023</v>
+        <v>1028</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>325</v>
@@ -5365,19 +5529,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1024</v>
+        <v>1029</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1025</v>
+        <v>1030</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1026</v>
+        <v>1031</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1027</v>
+        <v>1032</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>1028</v>
+        <v>1033</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>500</v>
@@ -5388,163 +5552,163 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1031</v>
+        <v>1036</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1032</v>
+        <v>1037</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>130</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>67</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1037</v>
+        <v>1042</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>183</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1039</v>
+        <v>1044</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1042</v>
+        <v>1047</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1044</v>
+        <v>1049</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1046</v>
+        <v>1051</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>1049</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>1044</v>
-      </c>
       <c r="C7" s="14" t="s">
-        <v>1050</v>
+        <v>1055</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1051</v>
+        <v>1056</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1044</v>
+        <v>1049</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1054</v>
+        <v>1059</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
     </row>
   </sheetData>
@@ -5572,13 +5736,13 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>824</v>
+        <v>829</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1055</v>
+        <v>1060</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1056</v>
+        <v>1061</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>500</v>
@@ -5587,7 +5751,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5595,10 +5759,10 @@
         <v>130</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>130</v>
@@ -5613,10 +5777,10 @@
         <v>94</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1060</v>
+        <v>1065</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>67</v>
@@ -5631,10 +5795,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1061</v>
+        <v>1066</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>199</v>
@@ -5646,13 +5810,13 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1062</v>
+        <v>1067</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1063</v>
+        <v>1068</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>61</v>
@@ -5664,13 +5828,13 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>1064</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>1065</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1059</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>199</v>
@@ -5685,10 +5849,10 @@
         <v>309</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1066</v>
+        <v>1071</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1067</v>
+        <v>1072</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>199</v>
@@ -5703,10 +5867,10 @@
         <v>374</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1068</v>
+        <v>1073</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>378</v>
@@ -5721,10 +5885,10 @@
         <v>400</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>55</v>
@@ -5739,10 +5903,10 @@
         <v>400</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1070</v>
+        <v>1075</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>55</v>
@@ -5754,13 +5918,13 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1071</v>
+        <v>1076</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>1072</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>1067</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>433</v>
@@ -18985,7 +19149,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19433,7 +19597,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" ht="409.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>640</v>
       </c>
@@ -19441,22 +19605,22 @@
         <v>67</v>
       </c>
       <c r="C16" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D16" s="14" t="s">
         <v>641</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="E16" s="14" t="s">
         <v>642</v>
       </c>
-      <c r="E16" s="14" t="s">
+      <c r="F16" s="14" t="s">
         <v>643</v>
       </c>
-      <c r="F16" s="14" t="s">
+      <c r="G16" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="H16" s="14" t="s">
         <v>644</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>645</v>
       </c>
       <c r="I16" s="14" t="s">
         <v>25</v>
@@ -19464,13 +19628,13 @@
     </row>
     <row r="17" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B17" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="D17" s="14" t="s">
         <v>647</v>
@@ -19491,7 +19655,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>651</v>
       </c>
@@ -19499,39 +19663,39 @@
         <v>67</v>
       </c>
       <c r="C18" s="14" t="s">
+        <v>646</v>
+      </c>
+      <c r="D18" s="14" t="s">
         <v>652</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="E18" s="14" t="s">
         <v>653</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="F18" s="14" t="s">
         <v>654</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="G18" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H18" s="14" t="s">
         <v>655</v>
       </c>
-      <c r="G18" s="14" t="s">
+      <c r="I18" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="14" t="s">
         <v>656</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>657</v>
-      </c>
-      <c r="I18" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
-        <v>658</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>174</v>
+        <v>658</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>659</v>
@@ -19540,10 +19704,10 @@
         <v>660</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="I19" s="14" t="s">
         <v>25</v>
@@ -19551,42 +19715,42 @@
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
       <c r="D20" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="E20" s="14" t="s">
         <v>664</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="F20" s="14" t="s">
         <v>665</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="G20" s="14" t="s">
+        <v>661</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>666</v>
       </c>
-      <c r="G20" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="H20" s="14" t="s">
+      <c r="I20" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
         <v>667</v>
-      </c>
-      <c r="I20" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>668</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>669</v>
@@ -19598,10 +19762,10 @@
         <v>671</v>
       </c>
       <c r="G21" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="H21" s="14" t="s">
         <v>672</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>673</v>
       </c>
       <c r="I21" s="14" t="s">
         <v>25</v>
@@ -19609,16 +19773,16 @@
     </row>
     <row r="22" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>234</v>
+        <v>674</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>675</v>
@@ -19627,10 +19791,10 @@
         <v>676</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="I22" s="14" t="s">
         <v>25</v>
@@ -19638,57 +19802,57 @@
     </row>
     <row r="23" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>235</v>
+        <v>677</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="I23" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>683</v>
+        <v>668</v>
       </c>
       <c r="D24" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="E24" s="14" t="s">
         <v>684</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="F24" s="14" t="s">
         <v>685</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="G24" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="H24" s="14" t="s">
         <v>686</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>266</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>687</v>
       </c>
       <c r="I24" s="14" t="s">
         <v>25</v>
@@ -19696,13 +19860,13 @@
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="D25" s="14" t="s">
         <v>689</v>
@@ -19723,7 +19887,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>693</v>
       </c>
@@ -19731,22 +19895,22 @@
         <v>67</v>
       </c>
       <c r="C26" s="14" t="s">
+        <v>688</v>
+      </c>
+      <c r="D26" s="14" t="s">
         <v>694</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="E26" s="14" t="s">
         <v>695</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="F26" s="14" t="s">
         <v>696</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="G26" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="H26" s="14" t="s">
         <v>697</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>698</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>25</v>
@@ -19754,16 +19918,16 @@
     </row>
     <row r="27" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C27" s="14" t="s">
+        <v>699</v>
+      </c>
+      <c r="D27" s="14" t="s">
         <v>700</v>
-      </c>
-      <c r="D27" s="14" t="s">
-        <v>319</v>
       </c>
       <c r="E27" s="14" t="s">
         <v>701</v>
@@ -19772,7 +19936,7 @@
         <v>702</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="H27" s="14" t="s">
         <v>703</v>
@@ -19781,18 +19945,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>704</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>571</v>
+        <v>705</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>705</v>
+        <v>319</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>706</v>
@@ -19801,16 +19965,16 @@
         <v>707</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="H28" s="14" t="s">
         <v>708</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>709</v>
       </c>
@@ -19839,7 +20003,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>714</v>
       </c>
@@ -19847,36 +20011,36 @@
         <v>61</v>
       </c>
       <c r="C30" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D30" s="14" t="s">
         <v>715</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="E30" s="14" t="s">
         <v>716</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="F30" s="14" t="s">
         <v>717</v>
       </c>
-      <c r="F30" s="14" t="s">
+      <c r="G30" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H30" s="14" t="s">
         <v>718</v>
       </c>
-      <c r="G30" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>719</v>
-      </c>
       <c r="I30" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>721</v>
@@ -19888,10 +20052,10 @@
         <v>723</v>
       </c>
       <c r="G31" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="H31" s="14" t="s">
         <v>724</v>
-      </c>
-      <c r="H31" s="14" t="s">
-        <v>725</v>
       </c>
       <c r="I31" s="14" t="s">
         <v>25</v>
@@ -19899,19 +20063,19 @@
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>663</v>
+        <v>720</v>
       </c>
       <c r="D32" s="14" t="s">
+        <v>726</v>
+      </c>
+      <c r="E32" s="14" t="s">
         <v>727</v>
-      </c>
-      <c r="E32" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="F32" s="14" t="s">
         <v>728</v>
@@ -19934,22 +20098,22 @@
         <v>61</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>732</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="F33" s="14" t="s">
         <v>733</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>248</v>
+        <v>734</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="I33" s="14" t="s">
         <v>25</v>
@@ -19957,28 +20121,28 @@
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>25</v>
@@ -19986,25 +20150,25 @@
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>741</v>
+        <v>255</v>
       </c>
       <c r="F35" s="14" t="s">
         <v>742</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="H35" s="14" t="s">
         <v>743</v>
@@ -20021,22 +20185,22 @@
         <v>61</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>683</v>
+        <v>668</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>283</v>
+        <v>745</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="I36" s="14" t="s">
         <v>25</v>
@@ -20044,16 +20208,16 @@
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>749</v>
+        <v>688</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>750</v>
@@ -20062,7 +20226,7 @@
         <v>751</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="H37" s="14" t="s">
         <v>752</v>
@@ -20071,7 +20235,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>753</v>
       </c>
@@ -20079,109 +20243,109 @@
         <v>61</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>700</v>
+        <v>754</v>
       </c>
       <c r="D38" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>755</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>756</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>757</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A39" s="14" t="s">
+        <v>758</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>705</v>
+      </c>
+      <c r="D39" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="E38" s="14" t="s">
-        <v>754</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>755</v>
-      </c>
-      <c r="G38" s="14" t="s">
+      <c r="E39" s="14" t="s">
+        <v>759</v>
+      </c>
+      <c r="F39" s="14" t="s">
+        <v>760</v>
+      </c>
+      <c r="G39" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="H38" s="14" t="s">
-        <v>756</v>
-      </c>
-      <c r="I38" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="39" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
-        <v>757</v>
-      </c>
-      <c r="B39" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>758</v>
-      </c>
-      <c r="D39" s="14" t="s">
-        <v>759</v>
-      </c>
-      <c r="E39" s="14" t="s">
-        <v>760</v>
-      </c>
-      <c r="F39" s="14" t="s">
+      <c r="H39" s="14" t="s">
         <v>761</v>
       </c>
-      <c r="G39" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H39" s="14" t="s">
+      <c r="I39" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
         <v>762</v>
-      </c>
-      <c r="I39" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
-        <v>763</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>207</v>
+        <v>764</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="I40" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="I41" s="14" t="s">
         <v>25</v>
@@ -20189,16 +20353,16 @@
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>772</v>
+        <v>132</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>773</v>
@@ -20207,7 +20371,7 @@
         <v>774</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="H42" s="14" t="s">
         <v>775</v>
@@ -20221,25 +20385,25 @@
         <v>776</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="C43" s="14" t="s">
+        <v>763</v>
+      </c>
+      <c r="D43" s="14" t="s">
         <v>777</v>
       </c>
-      <c r="D43" s="14" t="s">
+      <c r="E43" s="14" t="s">
         <v>778</v>
       </c>
-      <c r="E43" s="14" t="s">
+      <c r="F43" s="14" t="s">
         <v>779</v>
       </c>
-      <c r="F43" s="14" t="s">
+      <c r="G43" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="H43" s="14" t="s">
         <v>780</v>
-      </c>
-      <c r="G43" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="H43" s="14" t="s">
-        <v>781</v>
       </c>
       <c r="I43" s="14" t="s">
         <v>25</v>
@@ -20247,16 +20411,16 @@
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>378</v>
       </c>
       <c r="C44" s="14" t="s">
+        <v>782</v>
+      </c>
+      <c r="D44" s="14" t="s">
         <v>783</v>
-      </c>
-      <c r="D44" s="14" t="s">
-        <v>398</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>784</v>
@@ -20265,7 +20429,7 @@
         <v>785</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="H44" s="14" t="s">
         <v>786</v>
@@ -20274,44 +20438,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>787</v>
       </c>
       <c r="B45" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="C45" s="14" t="s">
         <v>788</v>
       </c>
-      <c r="C45" s="14" t="s">
+      <c r="D45" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="E45" s="14" t="s">
         <v>789</v>
       </c>
-      <c r="D45" s="14" t="s">
+      <c r="F45" s="14" t="s">
         <v>790</v>
       </c>
-      <c r="E45" s="14" t="s">
+      <c r="G45" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="H45" s="14" t="s">
         <v>791</v>
       </c>
-      <c r="F45" s="14" t="s">
+      <c r="I45" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="46" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A46" s="14" t="s">
         <v>792</v>
       </c>
-      <c r="G45" s="14" t="s">
-        <v>471</v>
-      </c>
-      <c r="H45" s="14" t="s">
+      <c r="B46" s="14" t="s">
         <v>793</v>
       </c>
-      <c r="I45" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
+      <c r="C46" s="14" t="s">
         <v>794</v>
-      </c>
-      <c r="B46" s="14" t="s">
-        <v>788</v>
-      </c>
-      <c r="C46" s="14" t="s">
-        <v>789</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>795</v>
@@ -20323,7 +20487,7 @@
         <v>797</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
       <c r="H46" s="14" t="s">
         <v>798</v>
@@ -20332,76 +20496,76 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>799</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>788</v>
+        <v>793</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>789</v>
+        <v>794</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>491</v>
+        <v>800</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="I47" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="48" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>61</v>
+        <v>793</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>804</v>
+        <v>794</v>
       </c>
       <c r="D48" s="14" t="s">
+        <v>491</v>
+      </c>
+      <c r="E48" s="14" t="s">
         <v>805</v>
       </c>
-      <c r="E48" s="14" t="s">
+      <c r="F48" s="14" t="s">
         <v>806</v>
       </c>
-      <c r="F48" s="14" t="s">
+      <c r="G48" s="14" t="s">
+        <v>486</v>
+      </c>
+      <c r="H48" s="14" t="s">
         <v>807</v>
-      </c>
-      <c r="G48" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="H48" s="14" t="s">
-        <v>808</v>
       </c>
       <c r="I48" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="49" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
+        <v>808</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C49" s="14" t="s">
         <v>809</v>
       </c>
-      <c r="B49" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C49" s="14" t="s">
+      <c r="D49" s="14" t="s">
         <v>810</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>87</v>
       </c>
       <c r="E49" s="14" t="s">
         <v>811</v>
@@ -20410,7 +20574,7 @@
         <v>812</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="H49" s="14" t="s">
         <v>813</v>
@@ -20419,7 +20583,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
         <v>814</v>
       </c>
@@ -20427,10 +20591,10 @@
         <v>86</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>758</v>
+        <v>815</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>815</v>
+        <v>87</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>816</v>
@@ -20439,7 +20603,7 @@
         <v>817</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H50" s="14" t="s">
         <v>818</v>
@@ -20448,7 +20612,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
         <v>819</v>
       </c>
@@ -20456,7 +20620,7 @@
         <v>86</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="D51" s="14" t="s">
         <v>820</v>
@@ -20468,7 +20632,7 @@
         <v>822</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="H51" s="14" t="s">
         <v>823</v>
@@ -20477,9 +20641,38 @@
         <v>13</v>
       </c>
     </row>
+    <row r="52" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A52" s="14" t="s">
+        <v>824</v>
+      </c>
+      <c r="B52" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>763</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>825</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>826</v>
+      </c>
+      <c r="F52" s="14" t="s">
+        <v>827</v>
+      </c>
+      <c r="G52" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H52" s="14" t="s">
+        <v>828</v>
+      </c>
+      <c r="I52" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I51"/>
-  <conditionalFormatting sqref="I2:I51">
+  <autoFilter ref="A1:I52"/>
+  <conditionalFormatting sqref="I2:I52">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -20514,7 +20707,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -20526,19 +20719,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>824</v>
+        <v>829</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>825</v>
+        <v>830</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>827</v>
+        <v>832</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>828</v>
+        <v>833</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20745,18 +20938,18 @@
         <v>635</v>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" ht="45" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>67</v>
       </c>
       <c r="B14" s="14" t="s">
+        <v>641</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>642</v>
       </c>
-      <c r="C14" s="14" t="s">
-        <v>643</v>
-      </c>
       <c r="D14" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="E14" s="14" t="s">
         <v>640</v>
@@ -20776,7 +20969,7 @@
         <v>175</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20784,13 +20977,13 @@
         <v>67</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>652</v>
+      </c>
+      <c r="C16" s="14" t="s">
         <v>653</v>
       </c>
-      <c r="C16" s="14" t="s">
-        <v>654</v>
-      </c>
       <c r="D16" s="14" t="s">
-        <v>656</v>
+        <v>175</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>651</v>
@@ -20801,16 +20994,16 @@
         <v>67</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>174</v>
+        <v>658</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>659</v>
       </c>
       <c r="D17" s="14" t="s">
+        <v>661</v>
+      </c>
+      <c r="E17" s="14" t="s">
         <v>656</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>658</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20818,16 +21011,16 @@
         <v>67</v>
       </c>
       <c r="B18" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C18" s="14" t="s">
         <v>664</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>665</v>
-      </c>
       <c r="D18" s="14" t="s">
-        <v>213</v>
+        <v>661</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20841,10 +21034,10 @@
         <v>670</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>672</v>
+        <v>213</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20852,16 +21045,16 @@
         <v>67</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>234</v>
+        <v>674</v>
       </c>
       <c r="C20" s="14" t="s">
         <v>675</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20869,16 +21062,16 @@
         <v>67</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C21" s="14" t="s">
+        <v>680</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>677</v>
+      </c>
+      <c r="E21" s="14" t="s">
         <v>679</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>235</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>678</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20886,16 +21079,16 @@
         <v>67</v>
       </c>
       <c r="B22" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="C22" s="14" t="s">
         <v>684</v>
       </c>
-      <c r="C22" s="14" t="s">
-        <v>685</v>
-      </c>
       <c r="D22" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20912,7 +21105,7 @@
         <v>266</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20920,13 +21113,13 @@
         <v>67</v>
       </c>
       <c r="B24" s="14" t="s">
+        <v>694</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>695</v>
       </c>
-      <c r="C24" s="14" t="s">
-        <v>696</v>
-      </c>
       <c r="D24" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>693</v>
@@ -20937,30 +21130,30 @@
         <v>67</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>319</v>
+        <v>700</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>701</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>705</v>
+        <v>319</v>
       </c>
       <c r="C26" s="14" t="s">
         <v>706</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="E26" s="14" t="s">
         <v>704</v>
@@ -20988,16 +21181,16 @@
         <v>61</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>626</v>
+        <v>715</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>627</v>
+        <v>716</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>624</v>
+        <v>714</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21005,16 +21198,16 @@
         <v>61</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>145</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21022,16 +21215,16 @@
         <v>61</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>716</v>
+        <v>631</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>717</v>
+        <v>632</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>714</v>
+        <v>630</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21045,10 +21238,10 @@
         <v>722</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>724</v>
+        <v>188</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21056,16 +21249,16 @@
         <v>61</v>
       </c>
       <c r="B32" s="14" t="s">
+        <v>726</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>727</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>729</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21076,10 +21269,10 @@
         <v>732</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>248</v>
+        <v>734</v>
       </c>
       <c r="E33" s="14" t="s">
         <v>731</v>
@@ -21090,16 +21283,16 @@
         <v>61</v>
       </c>
       <c r="B34" s="14" t="s">
+        <v>737</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="E34" s="14" t="s">
         <v>736</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="E34" s="14" t="s">
-        <v>735</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21107,16 +21300,16 @@
         <v>61</v>
       </c>
       <c r="B35" s="14" t="s">
+        <v>741</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E35" s="14" t="s">
         <v>740</v>
-      </c>
-      <c r="C35" s="14" t="s">
-        <v>741</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>739</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21124,13 +21317,13 @@
         <v>61</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>283</v>
+        <v>745</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>744</v>
@@ -21141,16 +21334,16 @@
         <v>61</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="C37" s="14" t="s">
         <v>750</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21158,13 +21351,13 @@
         <v>61</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>753</v>
@@ -21172,19 +21365,19 @@
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>759</v>
       </c>
-      <c r="C39" s="14" t="s">
-        <v>760</v>
-      </c>
       <c r="D39" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21192,16 +21385,16 @@
         <v>86</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>207</v>
+        <v>764</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21209,16 +21402,16 @@
         <v>86</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="C41" s="14" t="s">
+        <v>769</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="E41" s="14" t="s">
         <v>768</v>
-      </c>
-      <c r="D41" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21226,30 +21419,30 @@
         <v>86</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>772</v>
+        <v>132</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>773</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="B43" s="14" t="s">
+        <v>777</v>
+      </c>
+      <c r="C43" s="14" t="s">
         <v>778</v>
       </c>
-      <c r="C43" s="14" t="s">
-        <v>779</v>
-      </c>
       <c r="D43" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="E43" s="14" t="s">
         <v>776</v>
@@ -21260,33 +21453,33 @@
         <v>378</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>398</v>
+        <v>783</v>
       </c>
       <c r="C44" s="14" t="s">
         <v>784</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>86</v>
+        <v>378</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>87</v>
+        <v>398</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>811</v>
+        <v>789</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>81</v>
+        <v>393</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>809</v>
+        <v>787</v>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21294,13 +21487,13 @@
         <v>86</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>815</v>
+        <v>87</v>
       </c>
       <c r="C46" s="14" t="s">
         <v>816</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>814</v>
@@ -21317,14 +21510,31 @@
         <v>821</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="E47" s="14" t="s">
         <v>819</v>
       </c>
     </row>
+    <row r="48" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B48" s="14" t="s">
+        <v>825</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>826</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>824</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E47"/>
+  <autoFilter ref="A1:E48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -21349,114 +21559,114 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>826</v>
+        <v>831</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
       <c r="C3" s="14" t="s">
+        <v>848</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>843</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>838</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="C5" s="14" t="s">
+        <v>859</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>854</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>849</v>
-      </c>
       <c r="E5" s="14" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>164</v>
@@ -21464,22 +21674,22 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>170</v>
@@ -21487,186 +21697,186 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-052 Define multi-tenant signup and login orchestration
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3479" uniqueCount="1078">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3493" uniqueCount="1083">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -2639,6 +2639,295 @@
 - No frontend files change.
 - No database migration changes.
 - No workbook modification occurs during eventual CODE-051 execution.
+- No hosted operation occurs.</t>
+  </si>
+  <si>
+    <t>CODE-052</t>
+  </si>
+  <si>
+    <t>apps/api/src/modules/auth/auth.repository.ts; apps/api/src/modules/auth/auth.repository.spec.ts; apps/api/src/modules/auth/auth.service.ts; apps/api/src/modules/auth/auth.service.spec.ts; apps/api/src/modules/auth/auth.types.ts; apps/api/src/modules/auth/dto/auth-response.dto.ts; apps/api/src/modules/auth/dto/register-transporter.dto.ts; apps/api/src/modules/auth/dto/register-car-puller.dto.ts</t>
+  </si>
+  <si>
+    <t>Create multi-tenant transporter and car-puller authentication orchestration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a compatibility-first service/repository task.
+Do not change controllers in this task.
+Do not change frontend code.
+Do not change token verification.
+Do not change AuthGuard.
+Do not change RolesGuard.
+Do not add TenantContextGuard yet.
+Do not remove the existing legacy register/login behavior required by the
+currently working frontend.
+The goal is to build the new multi-tenant authentication orchestration
+alongside the current flow so a later task can safely switch HTTP endpoints.
+1. TRANSPORTER REGISTRATION DTO
+Create RegisterTransporterDto.
+Required fields:
+- email
+- password
+- companyName
+- fullName
+- phone
+Requirements:
+- email must use existing email validation conventions
+- password must use existing approved password validation
+- companyName required
+- fullName required
+- phone must use the existing approved international/E.164-compatible
+  validation convention
+- do not accept a client-provided role
+- do not accept tenantId
+- do not accept membershipId
+2. CAR-PULLER REGISTRATION DTO
+Create RegisterCarPullerDto.
+Required fields:
+- email
+- password
+- fullName
+- phone
+Do NOT include:
+- companyName
+- role
+- tenantId
+- membershipId
+Car-puller signup represents an individual identity/profile and must not
+automatically create a transporter company.
+3. NEW TRANSPORTER ACCOUNT REPOSITORY WRITE
+Add a repository operation equivalent to:
+createTransporterAccount(...)
+Do not replace the existing compatibility createCompanyAccount method yet if
+the legacy authentication flow still uses it.
+The new operation must create in one PostgreSQL transaction:
+A. public.user_profiles
+B. public.tenants
+C. public.tenant_memberships
+Behavior:
+- user_profiles.user_id = Supabase Auth user ID
+- create one new tenant using companyName
+- duplicate company display names must be allowed
+- create exactly one membership for the registering user
+- membership role = admin
+- membership status = active
+- no public.app_users row is required for the new multi-tenant flow
+- rollback all database writes if any database step fails
+- return enough information to construct the profile and newly created
+  membership response
+Do not infer identity from company name.
+4. NEW CAR-PULLER PROFILE REPOSITORY WRITE
+Add a repository operation equivalent to:
+createUserProfile(...)
+For car-puller signup:
+- insert one public.user_profiles row
+- do not create a tenant
+- do not create a tenant_memberships row
+- do not create an app_users row for the new multi-tenant flow
+Return the created profile.
+5. ACTIVE MEMBERSHIP LIST LOOKUP
+Add a repository operation equivalent to:
+findActiveMembershipsByUserId(userId)
+It must join:
+public.tenant_memberships
+public.tenants
+It must return only memberships where:
+tenant_memberships.status = 'active'
+AND
+tenants.status = 'active'
+Return:
+- membershipId
+- tenantId
+- tenantName
+- role
+- status
+Use deterministic ordering.
+Zero memberships is valid.
+Do not select a tenant inside the repository.
+6. NEW MULTI-TENANT AUTH RESPONSE TYPE
+Add or complete a domain-level MultiTenantAuthResponse type compatible with
+the DTO foundation from CODE-051.
+It must contain:
+session
+requiresEmailConfirmation
+profile
+memberships
+selectedMembership
+Profile must contain:
+- userId
+- email
+- fullName
+- phone
+selectedMembership must allow null.
+Do not remove the legacy AuthResponse type yet.
+7. TRANSPORTER REGISTRATION SERVICE ORCHESTRATION
+Add a new service operation equivalent to:
+registerTransporter(...)
+Do not replace the currently used legacy register method yet.
+Flow:
+1. Create Supabase Auth identity using the existing public Supabase client.
+2. Respect Supabase email-confirmation behavior.
+3. Create user profile + tenant + admin membership atomically using the new
+   repository operation.
+4. Return MultiTenantAuthResponse.
+For successful transporter registration:
+memberships contains exactly the newly created membership.
+selectedMembership = newly created membership.
+role = admin.
+Company display-name duplication must NOT produce a conflict by itself.
+If the PostgreSQL operation fails after a NEW Auth identity was created:
+- rollback PostgreSQL transaction
+- attempt compensating deletion of only that newly created Auth identity using
+  the existing server-side/admin Supabase mechanism
+- preserve safe error mapping
+Do not expose provider internals or secrets.
+8. CAR-PULLER REGISTRATION SERVICE ORCHESTRATION
+Add a new service operation equivalent to:
+registerCarPuller(...)
+Flow:
+1. Create Supabase Auth identity.
+2. Respect email-confirmation behavior.
+3. Create public.user_profiles.
+4. Do not create a tenant.
+5. Do not create a membership.
+6. Return:
+memberships = []
+selectedMembership = null
+A car puller may later obtain tenant memberships through invitation/joining
+flows.
+If profile persistence fails after a NEW Auth identity was created:
+- attempt compensation using the existing safe Auth-user deletion mechanism
+Do not invent a company for a car puller.
+9. MULTI-TENANT LOGIN ORCHESTRATION
+Add a new service operation equivalent to:
+loginMultiTenant(...)
+Do not replace the currently used legacy login method yet.
+Flow:
+1. Authenticate with existing Supabase signInWithPassword behavior.
+2. Load public.user_profiles by Auth user ID.
+3. Load active memberships using findActiveMembershipsByUserId().
+4. Build MultiTenantAuthResponse.
+Selection behavior:
+ZERO active memberships:
+selectedMembership = null
+EXACTLY ONE active membership:
+selectedMembership = that membership
+MORE THAN ONE active membership:
+selectedMembership = null
+The server must not arbitrarily choose one membership when several exist.
+The Supabase access token remains tenant-agnostic.
+Do not encode tenantId or application role into a new token.
+10. LOGIN PROFILE REQUIREMENT
+If Supabase authentication succeeds but public.user_profiles does not exist:
+- fail safely using the existing application-profile-missing convention
+- do not invent a profile
+- do not fall back to public.app_users for the new multi-tenant login method
+11. ERROR HANDLING
+Preserve safe error semantics equivalent to existing authentication behavior.
+At minimum test:
+- invalid credentials -&gt; safe authentication error
+- duplicate email/Auth identity -&gt; safe conflict behavior
+- provider unavailable -&gt; safe service-unavailable behavior
+- database failure -&gt; safe server error
+- compensation behavior
+- no raw Supabase/PostgreSQL internals leaked to clients
+Duplicate company display name is NOT an error.
+12. EXISTING AUTHENTICATION COMPATIBILITY
+The current working frontend still uses the legacy endpoints.
+Therefore this CODE-052 task must preserve:
+- current register()
+- current login()
+- existing AuthResponse
+- existing app_users compatibility queries needed by those legacy methods
+- existing controllers
+- existing frontend behavior
+New multi-tenant operations exist alongside them.
+A later task will switch controllers/endpoints to the new operations.
+13. TESTS
+Repository/service tests must cover at minimum:
+TRANSPORTER:
+- creates profile
+- creates tenant
+- creates active admin membership
+- profile/tenant/membership are transactional
+- duplicate tenant display name does not create a conflict
+- response contains one admin membership
+- selectedMembership is that membership
+- email-confirmation session-null behavior
+- database failure triggers rollback/compensation
+- Auth identity compensation is attempted only for a newly created identity
+CAR PULLER:
+- creates Auth identity
+- creates profile
+- creates no tenant
+- creates no membership
+- memberships = []
+- selectedMembership = null
+- email-confirmation behavior
+- persistence failure compensation
+LOGIN:
+- invalid credentials safely rejected
+- missing profile safely rejected
+- zero memberships -&gt; selectedMembership null
+- one active membership -&gt; automatically selected
+- two or more active memberships -&gt; selectedMembership null
+- multiple memberships are all returned
+- same user may have different roles in different tenants
+- suspended membership excluded
+- removed membership excluded
+- suspended tenant excluded
+- archived tenant excluded
+- token/session remains tenant-agnostic
+REGRESSION:
+- legacy registration tests continue passing
+- legacy login tests continue passing
+- existing controller tests continue passing
+- full API suite passes
+14. OUT OF SCOPE
+Do NOT:
+- change auth.controller.ts
+- create the new HTTP endpoints yet
+- change frontend registration pages
+- change frontend login
+- introduce tenant selection UI
+- introduce tenant switcher
+- change jwt.strategy.ts
+- change auth.guard.ts
+- change roles.guard.ts
+- create TenantContextGuard
+- alter RLS
+- modify migrations
+- modify database schema
+- modify app_users migration
+- remove app_users
+- modify package dependencies
+- access hosted Supabase
+- modify .env files</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- New transporter signup orchestration creates:
+  Auth identity + profile + tenant + active admin membership.
+- New car-puller signup orchestration creates:
+  Auth identity + profile only.
+- Company name is absent from car-puller signup.
+- Duplicate company display names are allowed.
+- No client-selected role exists in either registration DTO.
+- Multi-tenant login returns profile and all active memberships.
+- Zero memberships is valid.
+- Exactly one active membership may be automatically selected.
+- Multiple active memberships never cause arbitrary tenant selection.
+- Different roles in different tenants are preserved.
+- Supabase token remains tenant-agnostic.
+- New flow does not rely on app_users as its authoritative profile or
+  membership source.
+- Legacy authentication remains operational.
+- Existing API tests continue passing.
+- New tests pass.
+- API build/typecheck passes.
+- Task-agent tests pass.
+- No frontend file changes.
+- No migration changes.
+- No controller changes.
+- No guard changes.
 - No hosted operation occurs.</t>
   </si>
   <si>
@@ -4904,22 +5193,22 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -4927,76 +5216,76 @@
         <v>619</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="D3" s="14" t="s">
+        <v>928</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>923</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>918</v>
-      </c>
       <c r="F3" s="14" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>928</v>
+        <v>933</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>120</v>
@@ -5004,79 +5293,79 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>936</v>
+        <v>941</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>937</v>
+        <v>942</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>939</v>
+        <v>944</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>941</v>
+        <v>946</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>942</v>
+        <v>947</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>943</v>
+        <v>948</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>944</v>
+        <v>949</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>945</v>
+        <v>950</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>948</v>
+        <v>953</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>273</v>
@@ -5084,59 +5373,59 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>951</v>
+        <v>956</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>952</v>
+        <v>957</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>953</v>
+        <v>958</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>954</v>
+        <v>959</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>955</v>
+        <v>960</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>957</v>
+        <v>962</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>959</v>
+        <v>964</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>960</v>
+        <v>965</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>961</v>
+        <v>966</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>962</v>
+        <v>967</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>963</v>
+        <v>968</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>964</v>
+        <v>969</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>945</v>
+        <v>950</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>362</v>
@@ -5168,25 +5457,25 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>965</v>
+        <v>970</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>966</v>
+        <v>971</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>967</v>
+        <v>972</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>968</v>
+        <v>973</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>969</v>
+        <v>974</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>22</v>
@@ -5194,25 +5483,25 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>970</v>
+        <v>975</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>971</v>
+        <v>976</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>972</v>
+        <v>977</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>973</v>
+        <v>978</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>974</v>
+        <v>979</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>975</v>
+        <v>980</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>976</v>
+        <v>981</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>25</v>
@@ -5220,25 +5509,25 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>977</v>
+        <v>982</v>
       </c>
       <c r="B3" s="14" t="s">
+        <v>983</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>984</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>978</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>979</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>973</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>980</v>
+        <v>985</v>
       </c>
       <c r="F3" s="14" t="s">
+        <v>986</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>981</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>976</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>25</v>
@@ -5246,22 +5535,22 @@
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>982</v>
+        <v>987</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>332</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>983</v>
+        <v>988</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>984</v>
+        <v>989</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>985</v>
+        <v>990</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>986</v>
+        <v>991</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>331</v>
@@ -5272,22 +5561,22 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>987</v>
+        <v>992</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>988</v>
+        <v>993</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>990</v>
+        <v>995</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>992</v>
+        <v>997</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>338</v>
@@ -5298,25 +5587,25 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>993</v>
+        <v>998</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>984</v>
+        <v>989</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>25</v>
@@ -5324,25 +5613,25 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>999</v>
+        <v>1004</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>984</v>
+        <v>989</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1000</v>
+        <v>1005</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>1001</v>
+        <v>1006</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1002</v>
+        <v>1007</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>25</v>
@@ -5350,25 +5639,25 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1003</v>
+        <v>1008</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1004</v>
+        <v>1009</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1005</v>
+        <v>1010</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1006</v>
+        <v>1011</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1007</v>
+        <v>1012</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1009</v>
+        <v>1014</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>25</v>
@@ -5376,22 +5665,22 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1010</v>
+        <v>1015</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1011</v>
+        <v>1016</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1012</v>
+        <v>1017</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>990</v>
+        <v>995</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>1013</v>
+        <v>1018</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>302</v>
@@ -5402,22 +5691,22 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1016</v>
+        <v>1021</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1017</v>
+        <v>1022</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1018</v>
+        <v>1023</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>181</v>
@@ -5428,22 +5717,22 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1019</v>
+        <v>1024</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1020</v>
+        <v>1025</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1021</v>
+        <v>1026</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>1022</v>
+        <v>1027</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>1023</v>
+        <v>1028</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>194</v>
@@ -5454,22 +5743,22 @@
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1024</v>
+        <v>1029</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1025</v>
+        <v>1030</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1026</v>
+        <v>1031</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>973</v>
+        <v>978</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>1027</v>
+        <v>1032</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>1028</v>
+        <v>1033</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>325</v>
@@ -5529,19 +5818,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1031</v>
+        <v>1036</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1032</v>
+        <v>1037</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>500</v>
@@ -5552,163 +5841,163 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1037</v>
+        <v>1042</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>130</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1039</v>
+        <v>1044</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>67</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1042</v>
+        <v>1047</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>183</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1044</v>
+        <v>1049</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1046</v>
+        <v>1051</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1050</v>
+        <v>1055</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1051</v>
+        <v>1056</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>1054</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>1049</v>
-      </c>
       <c r="C7" s="14" t="s">
-        <v>1055</v>
+        <v>1060</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1056</v>
+        <v>1061</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
     </row>
   </sheetData>
@@ -5736,13 +6025,13 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1060</v>
+        <v>1065</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1061</v>
+        <v>1066</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>500</v>
@@ -5751,7 +6040,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1062</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5759,10 +6048,10 @@
         <v>130</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1063</v>
+        <v>1068</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>130</v>
@@ -5777,10 +6066,10 @@
         <v>94</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1065</v>
+        <v>1070</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>67</v>
@@ -5795,10 +6084,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1066</v>
+        <v>1071</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>199</v>
@@ -5810,13 +6099,13 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1067</v>
+        <v>1072</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1068</v>
+        <v>1073</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>61</v>
@@ -5828,13 +6117,13 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>1069</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>1070</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1064</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>199</v>
@@ -5849,10 +6138,10 @@
         <v>309</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1071</v>
+        <v>1076</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1072</v>
+        <v>1077</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>199</v>
@@ -5867,10 +6156,10 @@
         <v>374</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>378</v>
@@ -5885,10 +6174,10 @@
         <v>400</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1074</v>
+        <v>1079</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>55</v>
@@ -5903,10 +6192,10 @@
         <v>400</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1075</v>
+        <v>1080</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>55</v>
@@ -5918,13 +6207,13 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>1077</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>1072</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>433</v>
@@ -19149,7 +19438,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19626,7 +19915,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" ht="409.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>645</v>
       </c>
@@ -19634,22 +19923,22 @@
         <v>67</v>
       </c>
       <c r="C17" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D17" s="14" t="s">
         <v>646</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>647</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="F17" s="14" t="s">
         <v>648</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="G17" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="H17" s="14" t="s">
         <v>649</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>650</v>
       </c>
       <c r="I17" s="14" t="s">
         <v>25</v>
@@ -19657,13 +19946,13 @@
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="B18" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>652</v>
@@ -19684,7 +19973,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>656</v>
       </c>
@@ -19692,39 +19981,39 @@
         <v>67</v>
       </c>
       <c r="C19" s="14" t="s">
+        <v>651</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>657</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="E19" s="14" t="s">
         <v>658</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="F19" s="14" t="s">
         <v>659</v>
       </c>
-      <c r="F19" s="14" t="s">
+      <c r="G19" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H19" s="14" t="s">
         <v>660</v>
       </c>
-      <c r="G19" s="14" t="s">
+      <c r="I19" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="14" t="s">
         <v>661</v>
-      </c>
-      <c r="H19" s="14" t="s">
-        <v>662</v>
-      </c>
-      <c r="I19" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>663</v>
       </c>
       <c r="B20" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>174</v>
+        <v>663</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>664</v>
@@ -19733,10 +20022,10 @@
         <v>665</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="I20" s="14" t="s">
         <v>25</v>
@@ -19744,42 +20033,42 @@
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>668</v>
+        <v>662</v>
       </c>
       <c r="D21" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="E21" s="14" t="s">
         <v>669</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="F21" s="14" t="s">
         <v>670</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="G21" s="14" t="s">
+        <v>666</v>
+      </c>
+      <c r="H21" s="14" t="s">
         <v>671</v>
       </c>
-      <c r="G21" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="H21" s="14" t="s">
+      <c r="I21" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
         <v>672</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>673</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="D22" s="14" t="s">
         <v>674</v>
@@ -19791,10 +20080,10 @@
         <v>676</v>
       </c>
       <c r="G22" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="H22" s="14" t="s">
         <v>677</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>678</v>
       </c>
       <c r="I22" s="14" t="s">
         <v>25</v>
@@ -19802,16 +20091,16 @@
     </row>
     <row r="23" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>234</v>
+        <v>679</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>680</v>
@@ -19820,10 +20109,10 @@
         <v>681</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="I23" s="14" t="s">
         <v>25</v>
@@ -19831,57 +20120,57 @@
     </row>
     <row r="24" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>235</v>
+        <v>682</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="I24" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="25" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>688</v>
+        <v>673</v>
       </c>
       <c r="D25" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="E25" s="14" t="s">
         <v>689</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="F25" s="14" t="s">
         <v>690</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="G25" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="H25" s="14" t="s">
         <v>691</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>266</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>692</v>
       </c>
       <c r="I25" s="14" t="s">
         <v>25</v>
@@ -19889,13 +20178,13 @@
     </row>
     <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>694</v>
@@ -19916,7 +20205,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>698</v>
       </c>
@@ -19924,22 +20213,22 @@
         <v>67</v>
       </c>
       <c r="C27" s="14" t="s">
+        <v>693</v>
+      </c>
+      <c r="D27" s="14" t="s">
         <v>699</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="E27" s="14" t="s">
         <v>700</v>
       </c>
-      <c r="E27" s="14" t="s">
+      <c r="F27" s="14" t="s">
         <v>701</v>
       </c>
-      <c r="F27" s="14" t="s">
+      <c r="G27" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="H27" s="14" t="s">
         <v>702</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>703</v>
       </c>
       <c r="I27" s="14" t="s">
         <v>25</v>
@@ -19947,16 +20236,16 @@
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C28" s="14" t="s">
+        <v>704</v>
+      </c>
+      <c r="D28" s="14" t="s">
         <v>705</v>
-      </c>
-      <c r="D28" s="14" t="s">
-        <v>319</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>706</v>
@@ -19965,7 +20254,7 @@
         <v>707</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="H28" s="14" t="s">
         <v>708</v>
@@ -19974,18 +20263,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
         <v>709</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>571</v>
+        <v>710</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>710</v>
+        <v>319</v>
       </c>
       <c r="E29" s="14" t="s">
         <v>711</v>
@@ -19994,16 +20283,16 @@
         <v>712</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="H29" s="14" t="s">
         <v>713</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>714</v>
       </c>
@@ -20032,7 +20321,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>719</v>
       </c>
@@ -20040,36 +20329,36 @@
         <v>61</v>
       </c>
       <c r="C31" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D31" s="14" t="s">
         <v>720</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="E31" s="14" t="s">
         <v>721</v>
       </c>
-      <c r="E31" s="14" t="s">
+      <c r="F31" s="14" t="s">
         <v>722</v>
       </c>
-      <c r="F31" s="14" t="s">
+      <c r="G31" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H31" s="14" t="s">
         <v>723</v>
       </c>
-      <c r="G31" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="H31" s="14" t="s">
-        <v>724</v>
-      </c>
       <c r="I31" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>726</v>
@@ -20081,10 +20370,10 @@
         <v>728</v>
       </c>
       <c r="G32" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="H32" s="14" t="s">
         <v>729</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>730</v>
       </c>
       <c r="I32" s="14" t="s">
         <v>25</v>
@@ -20092,19 +20381,19 @@
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>668</v>
+        <v>725</v>
       </c>
       <c r="D33" s="14" t="s">
+        <v>731</v>
+      </c>
+      <c r="E33" s="14" t="s">
         <v>732</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="F33" s="14" t="s">
         <v>733</v>
@@ -20127,22 +20416,22 @@
         <v>61</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="D34" s="14" t="s">
         <v>737</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="F34" s="14" t="s">
         <v>738</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>248</v>
+        <v>739</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>25</v>
@@ -20150,28 +20439,28 @@
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="I35" s="14" t="s">
         <v>25</v>
@@ -20179,25 +20468,25 @@
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>746</v>
+        <v>255</v>
       </c>
       <c r="F36" s="14" t="s">
         <v>747</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="H36" s="14" t="s">
         <v>748</v>
@@ -20214,22 +20503,22 @@
         <v>61</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>688</v>
+        <v>673</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>283</v>
+        <v>750</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>25</v>
@@ -20237,16 +20526,16 @@
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>754</v>
+        <v>693</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>755</v>
@@ -20255,7 +20544,7 @@
         <v>756</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="H38" s="14" t="s">
         <v>757</v>
@@ -20264,7 +20553,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
         <v>758</v>
       </c>
@@ -20272,109 +20561,109 @@
         <v>61</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>705</v>
+        <v>759</v>
       </c>
       <c r="D39" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>760</v>
+      </c>
+      <c r="F39" s="14" t="s">
+        <v>761</v>
+      </c>
+      <c r="G39" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="H39" s="14" t="s">
+        <v>762</v>
+      </c>
+      <c r="I39" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
+        <v>763</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>710</v>
+      </c>
+      <c r="D40" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="E39" s="14" t="s">
-        <v>759</v>
-      </c>
-      <c r="F39" s="14" t="s">
-        <v>760</v>
-      </c>
-      <c r="G39" s="14" t="s">
+      <c r="E40" s="14" t="s">
+        <v>764</v>
+      </c>
+      <c r="F40" s="14" t="s">
+        <v>765</v>
+      </c>
+      <c r="G40" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="H39" s="14" t="s">
-        <v>761</v>
-      </c>
-      <c r="I39" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="40" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
-        <v>762</v>
-      </c>
-      <c r="B40" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>763</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>764</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>765</v>
-      </c>
-      <c r="F40" s="14" t="s">
+      <c r="H40" s="14" t="s">
         <v>766</v>
       </c>
-      <c r="G40" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H40" s="14" t="s">
+      <c r="I40" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="14" t="s">
         <v>767</v>
-      </c>
-      <c r="I40" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
-        <v>768</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>207</v>
+        <v>769</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="I41" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="I42" s="14" t="s">
         <v>25</v>
@@ -20382,16 +20671,16 @@
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>777</v>
+        <v>132</v>
       </c>
       <c r="E43" s="14" t="s">
         <v>778</v>
@@ -20400,7 +20689,7 @@
         <v>779</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="H43" s="14" t="s">
         <v>780</v>
@@ -20414,25 +20703,25 @@
         <v>781</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="C44" s="14" t="s">
+        <v>768</v>
+      </c>
+      <c r="D44" s="14" t="s">
         <v>782</v>
       </c>
-      <c r="D44" s="14" t="s">
+      <c r="E44" s="14" t="s">
         <v>783</v>
       </c>
-      <c r="E44" s="14" t="s">
+      <c r="F44" s="14" t="s">
         <v>784</v>
       </c>
-      <c r="F44" s="14" t="s">
+      <c r="G44" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="H44" s="14" t="s">
         <v>785</v>
-      </c>
-      <c r="G44" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="H44" s="14" t="s">
-        <v>786</v>
       </c>
       <c r="I44" s="14" t="s">
         <v>25</v>
@@ -20440,16 +20729,16 @@
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>378</v>
       </c>
       <c r="C45" s="14" t="s">
+        <v>787</v>
+      </c>
+      <c r="D45" s="14" t="s">
         <v>788</v>
-      </c>
-      <c r="D45" s="14" t="s">
-        <v>398</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>789</v>
@@ -20458,7 +20747,7 @@
         <v>790</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="H45" s="14" t="s">
         <v>791</v>
@@ -20467,44 +20756,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
         <v>792</v>
       </c>
       <c r="B46" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="C46" s="14" t="s">
         <v>793</v>
       </c>
-      <c r="C46" s="14" t="s">
+      <c r="D46" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="E46" s="14" t="s">
         <v>794</v>
       </c>
-      <c r="D46" s="14" t="s">
+      <c r="F46" s="14" t="s">
         <v>795</v>
       </c>
-      <c r="E46" s="14" t="s">
+      <c r="G46" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="H46" s="14" t="s">
         <v>796</v>
       </c>
-      <c r="F46" s="14" t="s">
+      <c r="I46" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="47" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A47" s="14" t="s">
         <v>797</v>
       </c>
-      <c r="G46" s="14" t="s">
-        <v>471</v>
-      </c>
-      <c r="H46" s="14" t="s">
+      <c r="B47" s="14" t="s">
         <v>798</v>
       </c>
-      <c r="I46" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="47" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
+      <c r="C47" s="14" t="s">
         <v>799</v>
-      </c>
-      <c r="B47" s="14" t="s">
-        <v>793</v>
-      </c>
-      <c r="C47" s="14" t="s">
-        <v>794</v>
       </c>
       <c r="D47" s="14" t="s">
         <v>800</v>
@@ -20516,7 +20805,7 @@
         <v>802</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
       <c r="H47" s="14" t="s">
         <v>803</v>
@@ -20525,76 +20814,76 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
         <v>804</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>793</v>
+        <v>798</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>794</v>
+        <v>799</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>491</v>
+        <v>805</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="H48" s="14" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="I48" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="49" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>61</v>
+        <v>798</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>809</v>
+        <v>799</v>
       </c>
       <c r="D49" s="14" t="s">
+        <v>491</v>
+      </c>
+      <c r="E49" s="14" t="s">
         <v>810</v>
       </c>
-      <c r="E49" s="14" t="s">
+      <c r="F49" s="14" t="s">
         <v>811</v>
       </c>
-      <c r="F49" s="14" t="s">
+      <c r="G49" s="14" t="s">
+        <v>486</v>
+      </c>
+      <c r="H49" s="14" t="s">
         <v>812</v>
-      </c>
-      <c r="G49" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="H49" s="14" t="s">
-        <v>813</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="50" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
+        <v>813</v>
+      </c>
+      <c r="B50" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" s="14" t="s">
         <v>814</v>
       </c>
-      <c r="B50" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C50" s="14" t="s">
+      <c r="D50" s="14" t="s">
         <v>815</v>
-      </c>
-      <c r="D50" s="14" t="s">
-        <v>87</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>816</v>
@@ -20603,7 +20892,7 @@
         <v>817</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="H50" s="14" t="s">
         <v>818</v>
@@ -20612,7 +20901,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
         <v>819</v>
       </c>
@@ -20620,10 +20909,10 @@
         <v>86</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>763</v>
+        <v>820</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>820</v>
+        <v>87</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>821</v>
@@ -20632,7 +20921,7 @@
         <v>822</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H51" s="14" t="s">
         <v>823</v>
@@ -20641,7 +20930,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>824</v>
       </c>
@@ -20649,7 +20938,7 @@
         <v>86</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="D52" s="14" t="s">
         <v>825</v>
@@ -20661,7 +20950,7 @@
         <v>827</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="H52" s="14" t="s">
         <v>828</v>
@@ -20670,9 +20959,38 @@
         <v>13</v>
       </c>
     </row>
+    <row r="53" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A53" s="14" t="s">
+        <v>829</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C53" s="14" t="s">
+        <v>768</v>
+      </c>
+      <c r="D53" s="14" t="s">
+        <v>830</v>
+      </c>
+      <c r="E53" s="14" t="s">
+        <v>831</v>
+      </c>
+      <c r="F53" s="14" t="s">
+        <v>832</v>
+      </c>
+      <c r="G53" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H53" s="14" t="s">
+        <v>833</v>
+      </c>
+      <c r="I53" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I52"/>
-  <conditionalFormatting sqref="I2:I52">
+  <autoFilter ref="A1:I53"/>
+  <conditionalFormatting sqref="I2:I53">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -20707,7 +21025,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -20719,19 +21037,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>829</v>
+        <v>834</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>830</v>
+        <v>835</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>833</v>
+        <v>838</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20955,18 +21273,18 @@
         <v>640</v>
       </c>
     </row>
-    <row r="15" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" ht="60" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
         <v>67</v>
       </c>
       <c r="B15" s="14" t="s">
+        <v>646</v>
+      </c>
+      <c r="C15" s="14" t="s">
         <v>647</v>
       </c>
-      <c r="C15" s="14" t="s">
-        <v>648</v>
-      </c>
       <c r="D15" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>645</v>
@@ -20986,7 +21304,7 @@
         <v>175</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -20994,13 +21312,13 @@
         <v>67</v>
       </c>
       <c r="B17" s="14" t="s">
+        <v>657</v>
+      </c>
+      <c r="C17" s="14" t="s">
         <v>658</v>
       </c>
-      <c r="C17" s="14" t="s">
-        <v>659</v>
-      </c>
       <c r="D17" s="14" t="s">
-        <v>661</v>
+        <v>175</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>656</v>
@@ -21011,16 +21329,16 @@
         <v>67</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>174</v>
+        <v>663</v>
       </c>
       <c r="C18" s="14" t="s">
         <v>664</v>
       </c>
       <c r="D18" s="14" t="s">
+        <v>666</v>
+      </c>
+      <c r="E18" s="14" t="s">
         <v>661</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21028,16 +21346,16 @@
         <v>67</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>669</v>
       </c>
-      <c r="C19" s="14" t="s">
-        <v>670</v>
-      </c>
       <c r="D19" s="14" t="s">
-        <v>213</v>
+        <v>666</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21051,10 +21369,10 @@
         <v>675</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>677</v>
+        <v>213</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21062,16 +21380,16 @@
         <v>67</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>234</v>
+        <v>679</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>680</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21079,16 +21397,16 @@
         <v>67</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C22" s="14" t="s">
+        <v>685</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>682</v>
+      </c>
+      <c r="E22" s="14" t="s">
         <v>684</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>235</v>
-      </c>
-      <c r="E22" s="14" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21096,16 +21414,16 @@
         <v>67</v>
       </c>
       <c r="B23" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="C23" s="14" t="s">
         <v>689</v>
       </c>
-      <c r="C23" s="14" t="s">
-        <v>690</v>
-      </c>
       <c r="D23" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21122,7 +21440,7 @@
         <v>266</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21130,13 +21448,13 @@
         <v>67</v>
       </c>
       <c r="B25" s="14" t="s">
+        <v>699</v>
+      </c>
+      <c r="C25" s="14" t="s">
         <v>700</v>
       </c>
-      <c r="C25" s="14" t="s">
-        <v>701</v>
-      </c>
       <c r="D25" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>698</v>
@@ -21147,30 +21465,30 @@
         <v>67</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>319</v>
+        <v>705</v>
       </c>
       <c r="C26" s="14" t="s">
         <v>706</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>710</v>
+        <v>319</v>
       </c>
       <c r="C27" s="14" t="s">
         <v>711</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="E27" s="14" t="s">
         <v>709</v>
@@ -21198,16 +21516,16 @@
         <v>61</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>626</v>
+        <v>720</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>627</v>
+        <v>721</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>624</v>
+        <v>719</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21215,16 +21533,16 @@
         <v>61</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>145</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21232,16 +21550,16 @@
         <v>61</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>721</v>
+        <v>631</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>722</v>
+        <v>632</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>719</v>
+        <v>630</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21255,10 +21573,10 @@
         <v>727</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>729</v>
+        <v>188</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21266,16 +21584,16 @@
         <v>61</v>
       </c>
       <c r="B33" s="14" t="s">
+        <v>731</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>732</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>734</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21286,10 +21604,10 @@
         <v>737</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>248</v>
+        <v>739</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>736</v>
@@ -21300,16 +21618,16 @@
         <v>61</v>
       </c>
       <c r="B35" s="14" t="s">
+        <v>742</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="D35" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="E35" s="14" t="s">
         <v>741</v>
-      </c>
-      <c r="C35" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>740</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21317,16 +21635,16 @@
         <v>61</v>
       </c>
       <c r="B36" s="14" t="s">
+        <v>746</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E36" s="14" t="s">
         <v>745</v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>746</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="E36" s="14" t="s">
-        <v>744</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21334,13 +21652,13 @@
         <v>61</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>283</v>
+        <v>750</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>749</v>
@@ -21351,16 +21669,16 @@
         <v>61</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="C38" s="14" t="s">
         <v>755</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21368,13 +21686,13 @@
         <v>61</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="E39" s="14" t="s">
         <v>758</v>
@@ -21382,19 +21700,19 @@
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>764</v>
       </c>
-      <c r="C40" s="14" t="s">
-        <v>765</v>
-      </c>
       <c r="D40" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21402,16 +21720,16 @@
         <v>86</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>207</v>
+        <v>769</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21419,16 +21737,16 @@
         <v>86</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="C42" s="14" t="s">
+        <v>774</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="E42" s="14" t="s">
         <v>773</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="E42" s="14" t="s">
-        <v>772</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21436,30 +21754,30 @@
         <v>86</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>777</v>
+        <v>132</v>
       </c>
       <c r="C43" s="14" t="s">
         <v>778</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="B44" s="14" t="s">
+        <v>782</v>
+      </c>
+      <c r="C44" s="14" t="s">
         <v>783</v>
       </c>
-      <c r="C44" s="14" t="s">
-        <v>784</v>
-      </c>
       <c r="D44" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>781</v>
@@ -21470,33 +21788,33 @@
         <v>378</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>398</v>
+        <v>788</v>
       </c>
       <c r="C45" s="14" t="s">
         <v>789</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>86</v>
+        <v>378</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>87</v>
+        <v>398</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>816</v>
+        <v>794</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>81</v>
+        <v>393</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>814</v>
+        <v>792</v>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21504,13 +21822,13 @@
         <v>86</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>820</v>
+        <v>87</v>
       </c>
       <c r="C47" s="14" t="s">
         <v>821</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E47" s="14" t="s">
         <v>819</v>
@@ -21527,14 +21845,31 @@
         <v>826</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="E48" s="14" t="s">
         <v>824</v>
       </c>
     </row>
+    <row r="49" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>830</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>831</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>829</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E48"/>
+  <autoFilter ref="A1:E49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -21559,114 +21894,114 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="C3" s="14" t="s">
+        <v>853</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>848</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>843</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>853</v>
+        <v>858</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="C5" s="14" t="s">
+        <v>864</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>859</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>854</v>
-      </c>
       <c r="E5" s="14" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>164</v>
@@ -21674,22 +22009,22 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>864</v>
+        <v>869</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>170</v>
@@ -21697,186 +22032,186 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-053 Define identity-only token verification foundation
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3493" uniqueCount="1083">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3507" uniqueCount="1088">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -2927,6 +2927,144 @@
 - No frontend file changes.
 - No migration changes.
 - No controller changes.
+- No guard changes.
+- No hosted operation occurs.</t>
+  </si>
+  <si>
+    <t>CODE-053</t>
+  </si>
+  <si>
+    <t>apps/api/src/modules/auth/jwt.strategy.ts; apps/api/src/modules/auth/jwt.strategy.spec.ts; apps/api/src/modules/auth/auth.types.ts</t>
+  </si>
+  <si>
+    <t>Create identity-only Supabase token verification foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This task is compatibility-first.
+Do not change AuthGuard yet.
+Do not change RolesGuard yet.
+Do not add TenantContextGuard yet.
+Do not change controllers.
+Do not change frontend code.
+Do not change registration/login orchestration.
+Do not change migrations.
+Do not change RLS.
+The purpose of CODE-053 is to create the new identity-only token-verification
+path while preserving the legacy tenant-scoped verification path until the
+next authorization task switches the guards.
+1. IDENTITY-ONLY TOKEN VERIFICATION
+Add a new token verification method equivalent to:
+verifyIdentity(accessToken)
+Behavior:
+- Accept the bearer access token string.
+- Use the existing Supabase public client.
+- Verify the token using the existing trusted Supabase getClaims/token
+  verification mechanism already used by the application.
+- Obtain the authenticated Supabase user ID.
+- Return:
+{
+  userId: string
+}
+using the existing/new AuthenticatedIdentity type.
+Do not return:
+- tenantId
+- membershipId
+- role
+- tenant name
+- application permissions
+2. TOKEN REMAINS TENANT-AGNOSTIC
+The new verification method must not:
+- query public.app_users
+- query public.user_profiles
+- query public.tenant_memberships
+- query public.tenants
+- derive an application role
+- select a tenant
+- trust tenant/role from browser state
+- trust tenant/role from JWT metadata
+Supabase token verification establishes identity only.
+3. ERROR HANDLING
+Preserve existing safe authentication behavior.
+The new identity-only verifier must safely reject:
+- missing/empty token if invoked directly
+- invalid token
+- expired/rejected token
+- missing authenticated subject/user ID
+- provider verification failure
+Do not expose:
+- raw Supabase provider errors
+- access tokens
+- JWT contents
+- Supabase keys
+- database details
+4. LEGACY COMPATIBILITY
+Do not remove the currently used legacy token-verification behavior yet if
+AuthGuard still depends on it.
+Existing protected flow must continue compiling and testing.
+The old app_users-based tenant/role lookup may remain temporarily only for
+compatibility.
+Clearly separate the new identity-only path from the legacy tenant-scoped
+path.
+A later task will:
+- switch AuthGuard to identity-only
+- introduce TenantContextGuard
+- resolve active tenant membership
+- feed tenant-specific role into RolesGuard
+5. TYPES
+Reuse:
+AuthenticatedIdentity {
+  userId: string
+}
+Do not change TenantRequestContext in this task.
+Do not remove legacy AuthenticatedContext yet if existing code requires it.
+6. TESTS
+Add/update jwt.strategy.spec.ts tests covering at minimum:
+- valid Supabase token returns only userId
+- valid identity response contains no tenantId
+- valid identity response contains no role
+- valid identity response contains no membershipId
+- identity-only path performs no repository membership lookup
+- identity-only path performs no app_users lookup
+- invalid token safely rejected
+- provider verification error safely rejected
+- missing subject/user ID safely rejected
+- legacy verification behavior remains compatible
+- existing verifier tests continue passing
+7. OUT OF SCOPE
+Do NOT:
+- modify auth.guard.ts
+- modify auth.guard.spec.ts
+- modify roles.guard.ts
+- modify roles.guard.spec.ts
+- introduce tenant-context.guard.ts
+- introduce tenant selection header parsing
+- modify auth.repository.ts
+- modify auth.service.ts
+- modify controllers
+- modify DTOs
+- modify frontend
+- modify database schema
+- modify migrations
+- modify RLS
+- remove app_users compatibility
+- contact hosted Supabase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Identity-only token verifier exists.
+- Valid Supabase token returns AuthenticatedIdentity containing only userId.
+- New identity verification performs no tenant lookup.
+- New identity verification performs no role lookup.
+- New identity verification does not rely on app_users.
+- Supabase token remains tenant-agnostic.
+- Safe error handling is preserved.
+- Existing legacy verifier remains compatible temporarily.
+- Existing AuthGuard/RoleGuard behavior is not changed in this task.
+- Existing API tests continue passing.
+- New verifier tests pass.
+- API build/typecheck passes.
+- Task-agent tests pass.
+- No frontend files change.
+- No migration changes.
 - No guard changes.
 - No hosted operation occurs.</t>
   </si>
@@ -5193,22 +5331,22 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5216,76 +5354,76 @@
         <v>619</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="D3" s="14" t="s">
+        <v>933</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>928</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>923</v>
-      </c>
       <c r="F3" s="14" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>936</v>
+        <v>941</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>937</v>
+        <v>942</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>120</v>
@@ -5293,79 +5431,79 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>939</v>
+        <v>944</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>941</v>
+        <v>946</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>942</v>
+        <v>947</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>943</v>
+        <v>948</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>944</v>
+        <v>949</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>945</v>
+        <v>950</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>948</v>
+        <v>953</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>951</v>
+        <v>956</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>952</v>
+        <v>957</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>953</v>
+        <v>958</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>954</v>
+        <v>959</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>955</v>
+        <v>960</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>273</v>
@@ -5373,59 +5511,59 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>957</v>
+        <v>962</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>959</v>
+        <v>964</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>960</v>
+        <v>965</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>710</v>
+        <v>715</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>961</v>
+        <v>966</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>962</v>
+        <v>967</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>963</v>
+        <v>968</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>964</v>
+        <v>969</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>965</v>
+        <v>970</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>966</v>
+        <v>971</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>967</v>
+        <v>972</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>968</v>
+        <v>973</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>969</v>
+        <v>974</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>362</v>
@@ -5457,25 +5595,25 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>970</v>
+        <v>975</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>971</v>
+        <v>976</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>972</v>
+        <v>977</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>973</v>
+        <v>978</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>974</v>
+        <v>979</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>22</v>
@@ -5483,25 +5621,25 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>975</v>
+        <v>980</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>976</v>
+        <v>981</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>977</v>
+        <v>982</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>978</v>
+        <v>983</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>979</v>
+        <v>984</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>980</v>
+        <v>985</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>981</v>
+        <v>986</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>25</v>
@@ -5509,25 +5647,25 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>982</v>
+        <v>987</v>
       </c>
       <c r="B3" s="14" t="s">
+        <v>988</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>989</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>983</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>984</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>978</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>985</v>
+        <v>990</v>
       </c>
       <c r="F3" s="14" t="s">
+        <v>991</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>986</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>981</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>25</v>
@@ -5535,22 +5673,22 @@
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>987</v>
+        <v>992</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>332</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>988</v>
+        <v>993</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>990</v>
+        <v>995</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>331</v>
@@ -5561,22 +5699,22 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>992</v>
+        <v>997</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>993</v>
+        <v>998</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>338</v>
@@ -5587,25 +5725,25 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>999</v>
+        <v>1004</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1000</v>
+        <v>1005</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1001</v>
+        <v>1006</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>739</v>
+        <v>744</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>25</v>
@@ -5613,25 +5751,25 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1002</v>
+        <v>1007</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1003</v>
+        <v>1008</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1004</v>
+        <v>1009</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1005</v>
+        <v>1010</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>1006</v>
+        <v>1011</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1007</v>
+        <v>1012</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>25</v>
@@ -5639,25 +5777,25 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1009</v>
+        <v>1014</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1010</v>
+        <v>1015</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1011</v>
+        <v>1016</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1012</v>
+        <v>1017</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1013</v>
+        <v>1018</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>25</v>
@@ -5665,22 +5803,22 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1016</v>
+        <v>1021</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1017</v>
+        <v>1022</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>1018</v>
+        <v>1023</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1019</v>
+        <v>1024</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>302</v>
@@ -5691,22 +5829,22 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1020</v>
+        <v>1025</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1021</v>
+        <v>1026</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1022</v>
+        <v>1027</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1023</v>
+        <v>1028</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>181</v>
@@ -5717,22 +5855,22 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1024</v>
+        <v>1029</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1025</v>
+        <v>1030</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1026</v>
+        <v>1031</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>1027</v>
+        <v>1032</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>1028</v>
+        <v>1033</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>194</v>
@@ -5743,22 +5881,22 @@
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1031</v>
+        <v>1036</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>978</v>
+        <v>983</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>1032</v>
+        <v>1037</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>325</v>
@@ -5818,19 +5956,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1037</v>
+        <v>1042</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>500</v>
@@ -5841,163 +5979,163 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1039</v>
+        <v>1044</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1042</v>
+        <v>1047</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>130</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1044</v>
+        <v>1049</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>1046</v>
+        <v>1051</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>67</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>183</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1050</v>
+        <v>1055</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1051</v>
+        <v>1056</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1054</v>
+        <v>1059</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1055</v>
+        <v>1060</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1056</v>
+        <v>1061</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>1059</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>1054</v>
-      </c>
       <c r="C7" s="14" t="s">
-        <v>1060</v>
+        <v>1065</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1061</v>
+        <v>1066</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1062</v>
+        <v>1067</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1054</v>
+        <v>1059</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1063</v>
+        <v>1068</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
     </row>
   </sheetData>
@@ -6025,13 +6163,13 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1065</v>
+        <v>1070</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1066</v>
+        <v>1071</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>500</v>
@@ -6040,7 +6178,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1067</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6048,10 +6186,10 @@
         <v>130</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1068</v>
+        <v>1073</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>130</v>
@@ -6066,10 +6204,10 @@
         <v>94</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1070</v>
+        <v>1075</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>67</v>
@@ -6084,10 +6222,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1071</v>
+        <v>1076</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>199</v>
@@ -6099,13 +6237,13 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1072</v>
+        <v>1077</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>61</v>
@@ -6117,13 +6255,13 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>1080</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>1074</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>1075</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1069</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>199</v>
@@ -6138,10 +6276,10 @@
         <v>309</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1077</v>
+        <v>1082</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>199</v>
@@ -6156,10 +6294,10 @@
         <v>374</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1078</v>
+        <v>1083</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>378</v>
@@ -6174,10 +6312,10 @@
         <v>400</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1079</v>
+        <v>1084</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>55</v>
@@ -6192,10 +6330,10 @@
         <v>400</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1080</v>
+        <v>1085</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>55</v>
@@ -6207,13 +6345,13 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1081</v>
+        <v>1086</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>1082</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>1077</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>433</v>
@@ -19438,7 +19576,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -19944,7 +20082,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" ht="409.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>650</v>
       </c>
@@ -19952,22 +20090,22 @@
         <v>67</v>
       </c>
       <c r="C18" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D18" s="14" t="s">
         <v>651</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="E18" s="14" t="s">
         <v>652</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="F18" s="14" t="s">
         <v>653</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="G18" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="H18" s="14" t="s">
         <v>654</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>655</v>
       </c>
       <c r="I18" s="14" t="s">
         <v>25</v>
@@ -19975,13 +20113,13 @@
     </row>
     <row r="19" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>657</v>
@@ -20002,7 +20140,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>661</v>
       </c>
@@ -20010,39 +20148,39 @@
         <v>67</v>
       </c>
       <c r="C20" s="14" t="s">
+        <v>656</v>
+      </c>
+      <c r="D20" s="14" t="s">
         <v>662</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="E20" s="14" t="s">
         <v>663</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="F20" s="14" t="s">
         <v>664</v>
       </c>
-      <c r="F20" s="14" t="s">
+      <c r="G20" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>665</v>
       </c>
-      <c r="G20" s="14" t="s">
+      <c r="I20" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="14" t="s">
         <v>666</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>667</v>
-      </c>
-      <c r="I20" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>668</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>174</v>
+        <v>668</v>
       </c>
       <c r="E21" s="14" t="s">
         <v>669</v>
@@ -20051,10 +20189,10 @@
         <v>670</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="I21" s="14" t="s">
         <v>25</v>
@@ -20062,42 +20200,42 @@
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="D22" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="E22" s="14" t="s">
         <v>674</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="F22" s="14" t="s">
         <v>675</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="G22" s="14" t="s">
+        <v>671</v>
+      </c>
+      <c r="H22" s="14" t="s">
         <v>676</v>
       </c>
-      <c r="G22" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="H22" s="14" t="s">
+      <c r="I22" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
         <v>677</v>
-      </c>
-      <c r="I22" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>678</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>679</v>
@@ -20109,10 +20247,10 @@
         <v>681</v>
       </c>
       <c r="G23" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="H23" s="14" t="s">
         <v>682</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>683</v>
       </c>
       <c r="I23" s="14" t="s">
         <v>25</v>
@@ -20120,16 +20258,16 @@
     </row>
     <row r="24" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>234</v>
+        <v>684</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>685</v>
@@ -20138,10 +20276,10 @@
         <v>686</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="I24" s="14" t="s">
         <v>25</v>
@@ -20149,57 +20287,57 @@
     </row>
     <row r="25" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>235</v>
+        <v>687</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="I25" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>693</v>
+        <v>678</v>
       </c>
       <c r="D26" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="E26" s="14" t="s">
         <v>694</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="F26" s="14" t="s">
         <v>695</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="G26" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="H26" s="14" t="s">
         <v>696</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>266</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>697</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>25</v>
@@ -20207,13 +20345,13 @@
     </row>
     <row r="27" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>699</v>
@@ -20234,7 +20372,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>703</v>
       </c>
@@ -20242,22 +20380,22 @@
         <v>67</v>
       </c>
       <c r="C28" s="14" t="s">
+        <v>698</v>
+      </c>
+      <c r="D28" s="14" t="s">
         <v>704</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="E28" s="14" t="s">
         <v>705</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="F28" s="14" t="s">
         <v>706</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="G28" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="H28" s="14" t="s">
         <v>707</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>708</v>
       </c>
       <c r="I28" s="14" t="s">
         <v>25</v>
@@ -20265,16 +20403,16 @@
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="14" t="s">
+        <v>709</v>
+      </c>
+      <c r="D29" s="14" t="s">
         <v>710</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>319</v>
       </c>
       <c r="E29" s="14" t="s">
         <v>711</v>
@@ -20283,7 +20421,7 @@
         <v>712</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="H29" s="14" t="s">
         <v>713</v>
@@ -20292,18 +20430,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
         <v>714</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>571</v>
+        <v>715</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>715</v>
+        <v>319</v>
       </c>
       <c r="E30" s="14" t="s">
         <v>716</v>
@@ -20312,16 +20450,16 @@
         <v>717</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="H30" s="14" t="s">
         <v>718</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
         <v>719</v>
       </c>
@@ -20350,7 +20488,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
         <v>724</v>
       </c>
@@ -20358,36 +20496,36 @@
         <v>61</v>
       </c>
       <c r="C32" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D32" s="14" t="s">
         <v>725</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="E32" s="14" t="s">
         <v>726</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="F32" s="14" t="s">
         <v>727</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="G32" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H32" s="14" t="s">
         <v>728</v>
       </c>
-      <c r="G32" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>729</v>
-      </c>
       <c r="I32" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>731</v>
@@ -20399,10 +20537,10 @@
         <v>733</v>
       </c>
       <c r="G33" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="H33" s="14" t="s">
         <v>734</v>
-      </c>
-      <c r="H33" s="14" t="s">
-        <v>735</v>
       </c>
       <c r="I33" s="14" t="s">
         <v>25</v>
@@ -20410,19 +20548,19 @@
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>673</v>
+        <v>730</v>
       </c>
       <c r="D34" s="14" t="s">
+        <v>736</v>
+      </c>
+      <c r="E34" s="14" t="s">
         <v>737</v>
-      </c>
-      <c r="E34" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="F34" s="14" t="s">
         <v>738</v>
@@ -20445,22 +20583,22 @@
         <v>61</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>742</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="F35" s="14" t="s">
         <v>743</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="I35" s="14" t="s">
         <v>25</v>
@@ -20468,28 +20606,28 @@
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="I36" s="14" t="s">
         <v>25</v>
@@ -20497,25 +20635,25 @@
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>751</v>
+        <v>255</v>
       </c>
       <c r="F37" s="14" t="s">
         <v>752</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="H37" s="14" t="s">
         <v>753</v>
@@ -20532,22 +20670,22 @@
         <v>61</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>693</v>
+        <v>678</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>283</v>
+        <v>755</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="I38" s="14" t="s">
         <v>25</v>
@@ -20555,16 +20693,16 @@
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>759</v>
+        <v>698</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="E39" s="14" t="s">
         <v>760</v>
@@ -20573,7 +20711,7 @@
         <v>761</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="H39" s="14" t="s">
         <v>762</v>
@@ -20582,7 +20720,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
         <v>763</v>
       </c>
@@ -20590,109 +20728,109 @@
         <v>61</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>710</v>
+        <v>764</v>
       </c>
       <c r="D40" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>765</v>
+      </c>
+      <c r="F40" s="14" t="s">
+        <v>766</v>
+      </c>
+      <c r="G40" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="H40" s="14" t="s">
+        <v>767</v>
+      </c>
+      <c r="I40" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="41" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A41" s="14" t="s">
+        <v>768</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>715</v>
+      </c>
+      <c r="D41" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="E40" s="14" t="s">
-        <v>764</v>
-      </c>
-      <c r="F40" s="14" t="s">
-        <v>765</v>
-      </c>
-      <c r="G40" s="14" t="s">
+      <c r="E41" s="14" t="s">
+        <v>769</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>770</v>
+      </c>
+      <c r="G41" s="14" t="s">
         <v>325</v>
       </c>
-      <c r="H40" s="14" t="s">
-        <v>766</v>
-      </c>
-      <c r="I40" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="41" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
-        <v>767</v>
-      </c>
-      <c r="B41" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>768</v>
-      </c>
-      <c r="D41" s="14" t="s">
-        <v>769</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>770</v>
-      </c>
-      <c r="F41" s="14" t="s">
+      <c r="H41" s="14" t="s">
         <v>771</v>
       </c>
-      <c r="G41" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H41" s="14" t="s">
+      <c r="I41" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="14" t="s">
         <v>772</v>
-      </c>
-      <c r="I41" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>773</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>207</v>
+        <v>774</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="I43" s="14" t="s">
         <v>25</v>
@@ -20700,16 +20838,16 @@
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>782</v>
+        <v>132</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>783</v>
@@ -20718,7 +20856,7 @@
         <v>784</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="H44" s="14" t="s">
         <v>785</v>
@@ -20732,25 +20870,25 @@
         <v>786</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="C45" s="14" t="s">
+        <v>773</v>
+      </c>
+      <c r="D45" s="14" t="s">
         <v>787</v>
       </c>
-      <c r="D45" s="14" t="s">
+      <c r="E45" s="14" t="s">
         <v>788</v>
       </c>
-      <c r="E45" s="14" t="s">
+      <c r="F45" s="14" t="s">
         <v>789</v>
       </c>
-      <c r="F45" s="14" t="s">
+      <c r="G45" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="H45" s="14" t="s">
         <v>790</v>
-      </c>
-      <c r="G45" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="H45" s="14" t="s">
-        <v>791</v>
       </c>
       <c r="I45" s="14" t="s">
         <v>25</v>
@@ -20758,16 +20896,16 @@
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>378</v>
       </c>
       <c r="C46" s="14" t="s">
+        <v>792</v>
+      </c>
+      <c r="D46" s="14" t="s">
         <v>793</v>
-      </c>
-      <c r="D46" s="14" t="s">
-        <v>398</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>794</v>
@@ -20776,7 +20914,7 @@
         <v>795</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="H46" s="14" t="s">
         <v>796</v>
@@ -20785,44 +20923,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
         <v>797</v>
       </c>
       <c r="B47" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="C47" s="14" t="s">
         <v>798</v>
       </c>
-      <c r="C47" s="14" t="s">
+      <c r="D47" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="E47" s="14" t="s">
         <v>799</v>
       </c>
-      <c r="D47" s="14" t="s">
+      <c r="F47" s="14" t="s">
         <v>800</v>
       </c>
-      <c r="E47" s="14" t="s">
+      <c r="G47" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="H47" s="14" t="s">
         <v>801</v>
       </c>
-      <c r="F47" s="14" t="s">
+      <c r="I47" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
         <v>802</v>
       </c>
-      <c r="G47" s="14" t="s">
-        <v>471</v>
-      </c>
-      <c r="H47" s="14" t="s">
+      <c r="B48" s="14" t="s">
         <v>803</v>
       </c>
-      <c r="I47" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
+      <c r="C48" s="14" t="s">
         <v>804</v>
-      </c>
-      <c r="B48" s="14" t="s">
-        <v>798</v>
-      </c>
-      <c r="C48" s="14" t="s">
-        <v>799</v>
       </c>
       <c r="D48" s="14" t="s">
         <v>805</v>
@@ -20834,7 +20972,7 @@
         <v>807</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
       <c r="H48" s="14" t="s">
         <v>808</v>
@@ -20843,76 +20981,76 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
         <v>809</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>798</v>
+        <v>803</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>799</v>
+        <v>804</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>491</v>
+        <v>810</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="50" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>61</v>
+        <v>803</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>814</v>
+        <v>804</v>
       </c>
       <c r="D50" s="14" t="s">
+        <v>491</v>
+      </c>
+      <c r="E50" s="14" t="s">
         <v>815</v>
       </c>
-      <c r="E50" s="14" t="s">
+      <c r="F50" s="14" t="s">
         <v>816</v>
       </c>
-      <c r="F50" s="14" t="s">
+      <c r="G50" s="14" t="s">
+        <v>486</v>
+      </c>
+      <c r="H50" s="14" t="s">
         <v>817</v>
-      </c>
-      <c r="G50" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="H50" s="14" t="s">
-        <v>818</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="51" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
+        <v>818</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" s="14" t="s">
         <v>819</v>
       </c>
-      <c r="B51" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C51" s="14" t="s">
+      <c r="D51" s="14" t="s">
         <v>820</v>
-      </c>
-      <c r="D51" s="14" t="s">
-        <v>87</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>821</v>
@@ -20921,7 +21059,7 @@
         <v>822</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="H51" s="14" t="s">
         <v>823</v>
@@ -20930,7 +21068,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>824</v>
       </c>
@@ -20938,10 +21076,10 @@
         <v>86</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>768</v>
+        <v>825</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>825</v>
+        <v>87</v>
       </c>
       <c r="E52" s="14" t="s">
         <v>826</v>
@@ -20950,7 +21088,7 @@
         <v>827</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H52" s="14" t="s">
         <v>828</v>
@@ -20959,7 +21097,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
         <v>829</v>
       </c>
@@ -20967,7 +21105,7 @@
         <v>86</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="D53" s="14" t="s">
         <v>830</v>
@@ -20979,7 +21117,7 @@
         <v>832</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="H53" s="14" t="s">
         <v>833</v>
@@ -20988,9 +21126,38 @@
         <v>13</v>
       </c>
     </row>
+    <row r="54" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="14" t="s">
+        <v>834</v>
+      </c>
+      <c r="B54" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C54" s="14" t="s">
+        <v>773</v>
+      </c>
+      <c r="D54" s="14" t="s">
+        <v>835</v>
+      </c>
+      <c r="E54" s="14" t="s">
+        <v>836</v>
+      </c>
+      <c r="F54" s="14" t="s">
+        <v>837</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>838</v>
+      </c>
+      <c r="I54" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I53"/>
-  <conditionalFormatting sqref="I2:I53">
+  <autoFilter ref="A1:I54"/>
+  <conditionalFormatting sqref="I2:I54">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -21025,7 +21192,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -21037,19 +21204,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>834</v>
+        <v>839</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>835</v>
+        <v>840</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>837</v>
+        <v>842</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>838</v>
+        <v>843</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21290,18 +21457,18 @@
         <v>645</v>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" ht="45" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
         <v>67</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>651</v>
+      </c>
+      <c r="C16" s="14" t="s">
         <v>652</v>
       </c>
-      <c r="C16" s="14" t="s">
-        <v>653</v>
-      </c>
       <c r="D16" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>650</v>
@@ -21321,7 +21488,7 @@
         <v>175</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21329,13 +21496,13 @@
         <v>67</v>
       </c>
       <c r="B18" s="14" t="s">
+        <v>662</v>
+      </c>
+      <c r="C18" s="14" t="s">
         <v>663</v>
       </c>
-      <c r="C18" s="14" t="s">
-        <v>664</v>
-      </c>
       <c r="D18" s="14" t="s">
-        <v>666</v>
+        <v>175</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>661</v>
@@ -21346,16 +21513,16 @@
         <v>67</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>174</v>
+        <v>668</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>669</v>
       </c>
       <c r="D19" s="14" t="s">
+        <v>671</v>
+      </c>
+      <c r="E19" s="14" t="s">
         <v>666</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21363,16 +21530,16 @@
         <v>67</v>
       </c>
       <c r="B20" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>674</v>
       </c>
-      <c r="C20" s="14" t="s">
-        <v>675</v>
-      </c>
       <c r="D20" s="14" t="s">
-        <v>213</v>
+        <v>671</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21386,10 +21553,10 @@
         <v>680</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>682</v>
+        <v>213</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21397,16 +21564,16 @@
         <v>67</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>234</v>
+        <v>684</v>
       </c>
       <c r="C22" s="14" t="s">
         <v>685</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21414,16 +21581,16 @@
         <v>67</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C23" s="14" t="s">
+        <v>690</v>
+      </c>
+      <c r="D23" s="14" t="s">
+        <v>687</v>
+      </c>
+      <c r="E23" s="14" t="s">
         <v>689</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>235</v>
-      </c>
-      <c r="E23" s="14" t="s">
-        <v>688</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21431,16 +21598,16 @@
         <v>67</v>
       </c>
       <c r="B24" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>694</v>
       </c>
-      <c r="C24" s="14" t="s">
-        <v>695</v>
-      </c>
       <c r="D24" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21457,7 +21624,7 @@
         <v>266</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21465,13 +21632,13 @@
         <v>67</v>
       </c>
       <c r="B26" s="14" t="s">
+        <v>704</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>705</v>
       </c>
-      <c r="C26" s="14" t="s">
-        <v>706</v>
-      </c>
       <c r="D26" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="E26" s="14" t="s">
         <v>703</v>
@@ -21482,30 +21649,30 @@
         <v>67</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>319</v>
+        <v>710</v>
       </c>
       <c r="C27" s="14" t="s">
         <v>711</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>715</v>
+        <v>319</v>
       </c>
       <c r="C28" s="14" t="s">
         <v>716</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>714</v>
@@ -21533,16 +21700,16 @@
         <v>61</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>626</v>
+        <v>725</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>627</v>
+        <v>726</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>624</v>
+        <v>724</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21550,16 +21717,16 @@
         <v>61</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>145</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21567,16 +21734,16 @@
         <v>61</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>726</v>
+        <v>631</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>727</v>
+        <v>632</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>724</v>
+        <v>630</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21590,10 +21757,10 @@
         <v>732</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>734</v>
+        <v>188</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21601,16 +21768,16 @@
         <v>61</v>
       </c>
       <c r="B34" s="14" t="s">
+        <v>736</v>
+      </c>
+      <c r="C34" s="14" t="s">
         <v>737</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>243</v>
       </c>
       <c r="D34" s="14" t="s">
         <v>739</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21621,10 +21788,10 @@
         <v>742</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="E35" s="14" t="s">
         <v>741</v>
@@ -21635,16 +21802,16 @@
         <v>61</v>
       </c>
       <c r="B36" s="14" t="s">
+        <v>747</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="E36" s="14" t="s">
         <v>746</v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="E36" s="14" t="s">
-        <v>745</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21652,16 +21819,16 @@
         <v>61</v>
       </c>
       <c r="B37" s="14" t="s">
+        <v>751</v>
+      </c>
+      <c r="C37" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E37" s="14" t="s">
         <v>750</v>
-      </c>
-      <c r="C37" s="14" t="s">
-        <v>751</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="E37" s="14" t="s">
-        <v>749</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21669,13 +21836,13 @@
         <v>61</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>283</v>
+        <v>755</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>754</v>
@@ -21686,16 +21853,16 @@
         <v>61</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="C39" s="14" t="s">
         <v>760</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21703,13 +21870,13 @@
         <v>61</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="E40" s="14" t="s">
         <v>763</v>
@@ -21717,19 +21884,19 @@
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>769</v>
       </c>
-      <c r="C41" s="14" t="s">
-        <v>770</v>
-      </c>
       <c r="D41" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21737,16 +21904,16 @@
         <v>86</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>207</v>
+        <v>774</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21754,16 +21921,16 @@
         <v>86</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="C43" s="14" t="s">
+        <v>779</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="E43" s="14" t="s">
         <v>778</v>
-      </c>
-      <c r="D43" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="E43" s="14" t="s">
-        <v>777</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21771,30 +21938,30 @@
         <v>86</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>782</v>
+        <v>132</v>
       </c>
       <c r="C44" s="14" t="s">
         <v>783</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="B45" s="14" t="s">
+        <v>787</v>
+      </c>
+      <c r="C45" s="14" t="s">
         <v>788</v>
       </c>
-      <c r="C45" s="14" t="s">
-        <v>789</v>
-      </c>
       <c r="D45" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>786</v>
@@ -21805,33 +21972,33 @@
         <v>378</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>398</v>
+        <v>793</v>
       </c>
       <c r="C46" s="14" t="s">
         <v>794</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>86</v>
+        <v>378</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>87</v>
+        <v>398</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>821</v>
+        <v>799</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>81</v>
+        <v>393</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>819</v>
+        <v>797</v>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21839,13 +22006,13 @@
         <v>86</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>825</v>
+        <v>87</v>
       </c>
       <c r="C48" s="14" t="s">
         <v>826</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E48" s="14" t="s">
         <v>824</v>
@@ -21862,14 +22029,31 @@
         <v>831</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="E49" s="14" t="s">
         <v>829</v>
       </c>
     </row>
+    <row r="50" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B50" s="14" t="s">
+        <v>835</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>836</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>834</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E49"/>
+  <autoFilter ref="A1:E50"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -21894,114 +22078,114 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>839</v>
+        <v>844</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>840</v>
+        <v>845</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>836</v>
+        <v>841</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>841</v>
+        <v>846</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>842</v>
+        <v>847</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>843</v>
+        <v>848</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>844</v>
+        <v>849</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>846</v>
+        <v>851</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>847</v>
+        <v>852</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>848</v>
+        <v>853</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>849</v>
+        <v>854</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>851</v>
+        <v>856</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>852</v>
+        <v>857</v>
       </c>
       <c r="C3" s="14" t="s">
+        <v>858</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>853</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>848</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>854</v>
+        <v>859</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>850</v>
+        <v>855</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>855</v>
+        <v>860</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>858</v>
+        <v>863</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>859</v>
+        <v>864</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>860</v>
+        <v>865</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>861</v>
+        <v>866</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>862</v>
+        <v>867</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>863</v>
+        <v>868</v>
       </c>
       <c r="C5" s="14" t="s">
+        <v>869</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>864</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>859</v>
-      </c>
       <c r="E5" s="14" t="s">
-        <v>865</v>
+        <v>870</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>866</v>
+        <v>871</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>164</v>
@@ -22009,22 +22193,22 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>170</v>
@@ -22032,186 +22216,186 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>886</v>
+        <v>891</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>897</v>
+        <v>902</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>845</v>
+        <v>850</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>856</v>
+        <v>861</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-054 Define verified tenant-context authorization
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3507" uniqueCount="1088">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3521" uniqueCount="1094">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3066,6 +3066,256 @@
 - No frontend files change.
 - No migration changes.
 - No guard changes.
+- No hosted operation occurs.</t>
+  </si>
+  <si>
+    <t>CODE-054</t>
+  </si>
+  <si>
+    <t>authorization</t>
+  </si>
+  <si>
+    <t>apps/api/src/common/guards/auth.guard.ts; apps/api/src/common/guards/auth.guard.spec.ts; apps/api/src/common/guards/tenant-context.guard.ts; apps/api/src/common/guards/tenant-context.guard.spec.ts; apps/api/src/common/guards/roles.guard.ts; apps/api/src/common/guards/roles.guard.spec.ts; apps/api/src/modules/auth/auth.module.ts</t>
+  </si>
+  <si>
+    <t>Create identity AuthGuard and verified tenant-context authorization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This task performs the guard-layer architecture transition.
+Do not expose the new transporter/car-puller HTTP endpoints yet.
+Do not modify controllers.
+Do not modify frontend code.
+Do not modify registration/login service orchestration.
+Do not modify migrations or RLS.
+Do not remove legacy JwtStrategy.verify() yet.
+Supabase identity and tenant authorization must be separate concerns.
+1. AUTHGUARD BECOMES IDENTITY-ONLY
+Update AuthGuard so it:
+1. Extracts the Bearer token using the existing approved behavior.
+2. Calls:
+JwtStrategy.verifyIdentity(accessToken)
+NOT the legacy tenant-scoped verify() method.
+3. Attaches exactly an authenticated identity equivalent to:
+{
+  userId
+}
+to request.user.
+AuthGuard must NOT attach:
+- tenantId
+- membershipId
+- role
+AuthGuard must NOT:
+- query public.app_users
+- query public.tenant_memberships
+- select a tenant
+- derive an application role
+Keep existing safe Bearer-token validation.
+Missing/malformed credentials remain Unauthorized.
+2. CREATE TENANTCONTEXTGUARD
+Create:
+apps/api/src/common/guards/tenant-context.guard.ts
+The guard operates AFTER AuthGuard.
+It must require a valid authenticated identity already attached to
+request.user.
+Read the requested tenant from this HTTP header:
+X-IAMONIT-Tenant-Id
+Header lookup must work using the normal lowercase Node/Nest representation:
+x-iamonit-tenant-id
+3. TENANT HEADER VALIDATION
+TenantContextGuard must safely reject:
+- no authenticated identity -&gt; Unauthorized
+- missing tenant header -&gt; Bad Request
+- blank tenant header -&gt; Bad Request
+- multiple tenant-header values -&gt; Bad Request
+- malformed tenant UUID -&gt; Bad Request
+Do not silently select a tenant.
+Do not infer a tenant from:
+- JWT
+- role
+- previous request
+- first membership
+- browser state
+- company name
+4. VERIFY MEMBERSHIP SERVER-SIDE
+TenantContextGuard must call the existing repository method equivalent to:
+findActiveMembership(userId, tenantId)
+The repository method already requires:
+- membership user matches authenticated user
+- membership tenant matches requested tenant
+- membership status = active
+- tenant status = active
+If no active membership is returned:
+Forbidden
+A tenant ID supplied by the browser is only a request for context.
+It is never proof of authorization.
+5. ATTACH VERIFIED TENANT REQUEST CONTEXT
+After membership validation succeeds, replace/enrich request.user with:
+{
+  userId,
+  membershipId,
+  tenantId,
+  role
+}
+using the existing TenantRequestContext type.
+The values must come from the verified Auth identity and database membership.
+Do not trust role or membershipId supplied by the client.
+6. DATABASE FAILURE HANDLING
+If membership verification fails because the database is unavailable:
+return a safe ServiceUnavailable response.
+Unexpected repository failures:
+return a safe InternalServerError response.
+Do not expose:
+- SQL
+- database URLs
+- stack traces
+- PostgreSQL internals
+7. ROLESGUARD BECOMES TENANT-CONTEXT AWARE
+Update RolesGuard so application role authorization is based only on the
+verified TenantRequestContext produced by TenantContextGuard.
+For handlers with no @Roles metadata:
+allow the request without requiring tenant role metadata.
+For handlers requiring roles:
+request.user must contain a valid tenant request context.
+Required context:
+- userId
+- membershipId
+- tenantId
+- role
+If tenant context is missing:
+Unauthorized
+If context exists but role is not one of the required roles:
+Forbidden
+RolesGuard must:
+- perform no database lookup
+- perform no JWT parsing
+- perform no tenant selection
+- not trust browser-provided role values
+8. MULTI-COMPANY ROLE BEHAVIOR
+The guard architecture must support:
+Same Auth user:
+Tenant A -&gt; admin
+Tenant B -&gt; dispatcher
+Tenant C -&gt; car_puller
+Authorization must depend on the membership belonging to the requested tenant.
+There must be no globally cached or globally assigned application role for the
+person.
+9. AUTHMODULE
+Update auth.module.ts only as necessary to make the new guard/repository
+dependencies resolvable through Nest dependency injection.
+Register/export guard providers only where required.
+Do not modify controllers or apply the guards to routes in this task.
+10. LEGACY JWT COMPATIBILITY
+JwtStrategy.verify() may remain temporarily for compatibility/testing.
+Do not delete it in CODE-054.
+However:
+AuthGuard must no longer use legacy verify().
+AuthGuard must use verifyIdentity().
+11. TESTS — AUTHGUARD
+Cover at minimum:
+- valid Bearer token calls verifyIdentity()
+- attaches only { userId }
+- does not attach tenantId
+- does not attach membershipId
+- does not attach role
+- does not call legacy verify()
+- missing Authorization header -&gt; Unauthorized
+- malformed Bearer scheme -&gt; Unauthorized
+- blank token -&gt; Unauthorized
+- identity-verification error safely propagated/mapped
+12. TESTS — TENANTCONTEXTGUARD
+Cover at minimum:
+- missing authenticated identity -&gt; Unauthorized
+- missing X-IAMONIT-Tenant-Id -&gt; Bad Request
+- blank header -&gt; Bad Request
+- malformed UUID -&gt; Bad Request
+- multiple header values -&gt; Bad Request
+- active membership succeeds
+- repository called with authenticated userId + requested tenantId
+- request.user becomes TenantRequestContext
+- different tenant/no membership -&gt; Forbidden
+- suspended membership -&gt; Forbidden
+- removed membership -&gt; Forbidden
+- suspended tenant -&gt; Forbidden
+- archived tenant -&gt; Forbidden
+- database unavailable -&gt; ServiceUnavailable
+- unexpected repository error -&gt; safe InternalServerError
+13. TESTS — ROLESGUARD
+Cover at minimum:
+- no @Roles metadata -&gt; allow
+- admin requirement with admin membership -&gt; allow
+- dispatcher requirement with dispatcher membership -&gt; allow
+- car_puller requirement with car_puller membership -&gt; allow
+- wrong tenant-specific role -&gt; Forbidden
+- identity-only request without tenant context on role-protected handler -&gt;
+  Unauthorized
+- role check uses request.user tenant context
+- no repository calls
+- same user may pass different role checks under different tenant contexts
+14. CHAINING TEST
+Add at least one focused test demonstrating the intended sequence:
+AuthGuard
+  -&gt; identity only
+TenantContextGuard
+  -&gt; verified tenant membership
+RolesGuard
+  -&gt; role from that membership
+The test must demonstrate that changing the requested tenant for the same user
+can result in a different authorized role.
+15. SECURITY RULES
+Do not trust:
+- tenantId from JWT claims
+- role from JWT claims
+- tenantId from request body
+- role from request body
+- membershipId from client
+- company name as tenant identity
+The only accepted tenant selector in this task is:
+X-IAMONIT-Tenant-Id
+and it must always be checked against the authenticated user's active
+membership.
+16. OUT OF SCOPE
+Do NOT:
+- modify auth.controller.ts
+- modify users.controller.ts
+- apply guards to HTTP endpoints yet
+- modify auth.service.ts
+- modify auth.repository.ts
+- modify jwt.strategy.ts unless compilation absolutely requires a type-only
+  compatibility change
+- modify registration DTOs
+- modify login DTO
+- modify frontend
+- modify migrations
+- modify RLS
+- remove app_users
+- create tenant-switcher UI
+- access hosted Supabase
+- modify package dependencies
+- modify environment files</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- AuthGuard authenticates identity only.
+- AuthGuard uses verifyIdentity(), not legacy verify().
+- request.user after AuthGuard contains only userId.
+- TenantContextGuard requires explicit X-IAMONIT-Tenant-Id.
+- Missing/malformed tenant context is safely rejected.
+- Requested tenant is verified against active PostgreSQL membership.
+- Inactive membership does not grant access.
+- Inactive tenant does not grant access.
+- Successful tenant verification produces:
+  userId, membershipId, tenantId, role.
+- RolesGuard uses the verified tenant-specific role.
+- Same user can have different authorization roles in different tenants.
+- No global application role is assumed.
+- Supabase access token remains tenant-agnostic.
+- Existing registration/login behavior remains operational.
+- Existing API tests continue passing.
+- New guard tests pass.
+- API build/typecheck passes.
+- Task-agent tests pass.
+- No frontend changes.
+- No controller changes.
+- No migration/RLS changes.
 - No hosted operation occurs.</t>
   </si>
   <si>
@@ -5331,22 +5581,22 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>921</v>
+        <v>927</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>922</v>
+        <v>928</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>923</v>
+        <v>929</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5354,76 +5604,76 @@
         <v>619</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>926</v>
+        <v>932</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>927</v>
+        <v>933</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>929</v>
+        <v>935</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>930</v>
+        <v>936</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>931</v>
+        <v>937</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>932</v>
+        <v>938</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>933</v>
+        <v>939</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>934</v>
+        <v>940</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>935</v>
+        <v>941</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>939</v>
+        <v>945</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>941</v>
+        <v>947</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>120</v>
@@ -5431,79 +5681,79 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>944</v>
+        <v>950</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>273</v>
@@ -5511,59 +5761,59 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>968</v>
+        <v>974</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>969</v>
+        <v>975</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>970</v>
+        <v>976</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>971</v>
+        <v>977</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>362</v>
@@ -5595,25 +5845,25 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>978</v>
+        <v>984</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>22</v>
@@ -5621,25 +5871,25 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>25</v>
@@ -5647,25 +5897,25 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>987</v>
+        <v>993</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>988</v>
+        <v>994</v>
       </c>
       <c r="C3" s="14" t="s">
+        <v>995</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>989</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>983</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>991</v>
+        <v>997</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>25</v>
@@ -5673,22 +5923,22 @@
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>992</v>
+        <v>998</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>332</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>993</v>
+        <v>999</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>995</v>
+        <v>1001</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>331</v>
@@ -5699,22 +5949,22 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>997</v>
+        <v>1003</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>998</v>
+        <v>1004</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>999</v>
+        <v>1005</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>1000</v>
+        <v>1006</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>1002</v>
+        <v>1008</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>338</v>
@@ -5725,25 +5975,25 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1003</v>
+        <v>1009</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1005</v>
+        <v>1011</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1006</v>
+        <v>1012</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>25</v>
@@ -5751,25 +6001,25 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1007</v>
+        <v>1013</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1008</v>
+        <v>1014</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1009</v>
+        <v>1015</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>1011</v>
+        <v>1017</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1012</v>
+        <v>1018</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>25</v>
@@ -5777,25 +6027,25 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1013</v>
+        <v>1019</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1014</v>
+        <v>1020</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1015</v>
+        <v>1021</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1016</v>
+        <v>1022</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1017</v>
+        <v>1023</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1018</v>
+        <v>1024</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1019</v>
+        <v>1025</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>25</v>
@@ -5803,22 +6053,22 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1020</v>
+        <v>1026</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1021</v>
+        <v>1027</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1022</v>
+        <v>1028</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>1000</v>
+        <v>1006</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>1023</v>
+        <v>1029</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1024</v>
+        <v>1030</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>302</v>
@@ -5829,22 +6079,22 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1025</v>
+        <v>1031</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1026</v>
+        <v>1032</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>181</v>
@@ -5855,22 +6105,22 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1029</v>
+        <v>1035</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1030</v>
+        <v>1036</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1031</v>
+        <v>1037</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>1032</v>
+        <v>1038</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>1033</v>
+        <v>1039</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>194</v>
@@ -5881,22 +6131,22 @@
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1034</v>
+        <v>1040</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1035</v>
+        <v>1041</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1036</v>
+        <v>1042</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>1037</v>
+        <v>1043</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>1038</v>
+        <v>1044</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>325</v>
@@ -5956,19 +6206,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1039</v>
+        <v>1045</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1041</v>
+        <v>1047</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1042</v>
+        <v>1048</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>1043</v>
+        <v>1049</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>500</v>
@@ -5979,163 +6229,163 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1044</v>
+        <v>1050</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1046</v>
+        <v>1052</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1047</v>
+        <v>1053</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>130</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1049</v>
+        <v>1055</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1050</v>
+        <v>1056</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>1051</v>
+        <v>1057</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>67</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1052</v>
+        <v>1058</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1053</v>
+        <v>1059</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>183</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1054</v>
+        <v>1060</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1059</v>
+        <v>1065</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1061</v>
+        <v>1067</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1062</v>
+        <v>1068</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>1063</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1064</v>
+        <v>1070</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1059</v>
+        <v>1065</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1065</v>
+        <v>1071</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1066</v>
+        <v>1072</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1063</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1067</v>
+        <v>1073</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1059</v>
+        <v>1065</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="14" t="s">
+        <v>1075</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>1068</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>1069</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>1062</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>1063</v>
       </c>
     </row>
   </sheetData>
@@ -6163,13 +6413,13 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1070</v>
+        <v>1076</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1071</v>
+        <v>1077</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>500</v>
@@ -6178,7 +6428,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6186,10 +6436,10 @@
         <v>130</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1073</v>
+        <v>1079</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>130</v>
@@ -6204,10 +6454,10 @@
         <v>94</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1075</v>
+        <v>1081</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>67</v>
@@ -6222,10 +6472,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1076</v>
+        <v>1082</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>199</v>
@@ -6237,13 +6487,13 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1077</v>
+        <v>1083</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1078</v>
+        <v>1084</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>61</v>
@@ -6255,13 +6505,13 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1079</v>
+        <v>1085</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>1080</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1074</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>199</v>
@@ -6276,10 +6526,10 @@
         <v>309</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1081</v>
+        <v>1087</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1082</v>
+        <v>1088</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>199</v>
@@ -6294,10 +6544,10 @@
         <v>374</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1083</v>
+        <v>1089</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>378</v>
@@ -6312,10 +6562,10 @@
         <v>400</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>55</v>
@@ -6330,10 +6580,10 @@
         <v>400</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1085</v>
+        <v>1091</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>55</v>
@@ -6345,13 +6595,13 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1086</v>
+        <v>1092</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1087</v>
+        <v>1093</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1082</v>
+        <v>1088</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>433</v>
@@ -19576,7 +19826,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -20111,7 +20361,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" ht="409.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
         <v>655</v>
       </c>
@@ -20131,7 +20381,7 @@
         <v>659</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="H19" s="14" t="s">
         <v>660</v>
@@ -20148,36 +20398,36 @@
         <v>67</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="G20" s="14" t="s">
         <v>175</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="I20" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="D21" s="14" t="s">
         <v>668</v>
@@ -20189,39 +20439,39 @@
         <v>670</v>
       </c>
       <c r="G21" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H21" s="14" t="s">
         <v>671</v>
       </c>
-      <c r="H21" s="14" t="s">
+      <c r="I21" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
         <v>672</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>673</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>174</v>
+        <v>674</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G22" s="14" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="I22" s="14" t="s">
         <v>25</v>
@@ -20229,16 +20479,16 @@
     </row>
     <row r="23" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>679</v>
+        <v>174</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>680</v>
@@ -20247,7 +20497,7 @@
         <v>681</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>213</v>
+        <v>677</v>
       </c>
       <c r="H23" s="14" t="s">
         <v>682</v>
@@ -20256,7 +20506,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>683</v>
       </c>
@@ -20264,19 +20514,19 @@
         <v>67</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>687</v>
+        <v>213</v>
       </c>
       <c r="H24" s="14" t="s">
         <v>688</v>
@@ -20293,22 +20543,22 @@
         <v>67</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>234</v>
+        <v>690</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="I25" s="14" t="s">
         <v>25</v>
@@ -20316,45 +20566,45 @@
     </row>
     <row r="26" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>235</v>
+        <v>693</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>698</v>
+        <v>684</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>699</v>
+        <v>240</v>
       </c>
       <c r="E27" s="14" t="s">
         <v>700</v>
@@ -20363,7 +20613,7 @@
         <v>701</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="H27" s="14" t="s">
         <v>702</v>
@@ -20380,36 +20630,36 @@
         <v>67</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>266</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="I28" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>710</v>
@@ -20421,7 +20671,7 @@
         <v>712</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="H29" s="14" t="s">
         <v>713</v>
@@ -20441,56 +20691,56 @@
         <v>715</v>
       </c>
       <c r="D30" s="14" t="s">
+        <v>716</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>717</v>
+      </c>
+      <c r="F30" s="14" t="s">
+        <v>718</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="H30" s="14" t="s">
+        <v>719</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="14" t="s">
+        <v>720</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>721</v>
+      </c>
+      <c r="D31" s="14" t="s">
         <v>319</v>
       </c>
-      <c r="E30" s="14" t="s">
-        <v>716</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>717</v>
-      </c>
-      <c r="G30" s="14" t="s">
+      <c r="E31" s="14" t="s">
+        <v>722</v>
+      </c>
+      <c r="F31" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="G31" s="14" t="s">
         <v>314</v>
       </c>
-      <c r="H30" s="14" t="s">
-        <v>718</v>
-      </c>
-      <c r="I30" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="31" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
-        <v>719</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>571</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>720</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>722</v>
-      </c>
-      <c r="G31" s="14" t="s">
-        <v>99</v>
-      </c>
       <c r="H31" s="14" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>61</v>
@@ -20499,33 +20749,33 @@
         <v>571</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="G32" s="14" t="s">
         <v>99</v>
       </c>
       <c r="H32" s="14" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="I32" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>730</v>
+        <v>571</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>731</v>
@@ -20537,13 +20787,13 @@
         <v>733</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>188</v>
+        <v>99</v>
       </c>
       <c r="H33" s="14" t="s">
         <v>734</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -20554,19 +20804,19 @@
         <v>61</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>739</v>
+        <v>188</v>
       </c>
       <c r="H34" s="14" t="s">
         <v>740</v>
@@ -20583,22 +20833,22 @@
         <v>61</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>678</v>
+        <v>736</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>742</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>243</v>
+        <v>743</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="I35" s="14" t="s">
         <v>25</v>
@@ -20606,28 +20856,28 @@
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>248</v>
+        <v>750</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="I36" s="14" t="s">
         <v>25</v>
@@ -20635,28 +20885,28 @@
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>25</v>
@@ -20664,28 +20914,28 @@
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>756</v>
+        <v>255</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="I38" s="14" t="s">
         <v>25</v>
@@ -20693,28 +20943,28 @@
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>698</v>
+        <v>684</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>283</v>
+        <v>761</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>25</v>
@@ -20722,74 +20972,74 @@
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>764</v>
+        <v>704</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="I40" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="41" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>715</v>
+        <v>770</v>
       </c>
       <c r="D41" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>771</v>
+      </c>
+      <c r="F41" s="14" t="s">
+        <v>772</v>
+      </c>
+      <c r="G41" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="H41" s="14" t="s">
+        <v>773</v>
+      </c>
+      <c r="I41" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="14" t="s">
+        <v>774</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>721</v>
+      </c>
+      <c r="D42" s="14" t="s">
         <v>330</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>769</v>
-      </c>
-      <c r="F41" s="14" t="s">
-        <v>770</v>
-      </c>
-      <c r="G41" s="14" t="s">
-        <v>325</v>
-      </c>
-      <c r="H41" s="14" t="s">
-        <v>771</v>
-      </c>
-      <c r="I41" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>772</v>
-      </c>
-      <c r="B42" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C42" s="14" t="s">
-        <v>773</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>774</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>775</v>
@@ -20798,16 +21048,16 @@
         <v>776</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="H42" s="14" t="s">
         <v>777</v>
       </c>
       <c r="I42" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="43" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
         <v>778</v>
       </c>
@@ -20815,51 +21065,51 @@
         <v>86</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>207</v>
+        <v>780</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="I43" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="F44" s="14" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="H44" s="14" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="I44" s="14" t="s">
         <v>25</v>
@@ -20867,28 +21117,28 @@
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>787</v>
+        <v>132</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="H45" s="14" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="I45" s="14" t="s">
         <v>25</v>
@@ -20896,13 +21146,13 @@
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>792</v>
+        <v>779</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>793</v>
@@ -20914,7 +21164,7 @@
         <v>795</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="H46" s="14" t="s">
         <v>796</v>
@@ -20934,123 +21184,123 @@
         <v>798</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>398</v>
+        <v>799</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="I47" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="48" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>803</v>
+        <v>378</v>
       </c>
       <c r="C48" s="14" t="s">
         <v>804</v>
       </c>
       <c r="D48" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="E48" s="14" t="s">
         <v>805</v>
       </c>
-      <c r="E48" s="14" t="s">
+      <c r="F48" s="14" t="s">
         <v>806</v>
       </c>
-      <c r="F48" s="14" t="s">
+      <c r="G48" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="H48" s="14" t="s">
         <v>807</v>
       </c>
-      <c r="G48" s="14" t="s">
+      <c r="I48" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="49" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
+        <v>808</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>809</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>810</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>811</v>
+      </c>
+      <c r="E49" s="14" t="s">
+        <v>812</v>
+      </c>
+      <c r="F49" s="14" t="s">
+        <v>813</v>
+      </c>
+      <c r="G49" s="14" t="s">
         <v>471</v>
       </c>
-      <c r="H48" s="14" t="s">
-        <v>808</v>
-      </c>
-      <c r="I48" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="49" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="14" t="s">
-        <v>809</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>803</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>804</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>810</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>811</v>
-      </c>
-      <c r="F49" s="14" t="s">
-        <v>812</v>
-      </c>
-      <c r="G49" s="14" t="s">
-        <v>480</v>
-      </c>
       <c r="H49" s="14" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="50" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>804</v>
+        <v>810</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>491</v>
+        <v>816</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="51" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>61</v>
+        <v>809</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>819</v>
+        <v>810</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>820</v>
+        <v>491</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>821</v>
@@ -21059,7 +21309,7 @@
         <v>822</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>57</v>
+        <v>486</v>
       </c>
       <c r="H51" s="14" t="s">
         <v>823</v>
@@ -21068,96 +21318,125 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>824</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="C52" s="14" t="s">
         <v>825</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>87</v>
+        <v>826</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="I52" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="53" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="B53" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>773</v>
+        <v>831</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>830</v>
+        <v>87</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H53" s="14" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="I53" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="54" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B54" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="I54" s="14" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="55" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A55" s="14" t="s">
+        <v>840</v>
+      </c>
+      <c r="B55" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C55" s="14" t="s">
+        <v>779</v>
+      </c>
+      <c r="D55" s="14" t="s">
+        <v>841</v>
+      </c>
+      <c r="E55" s="14" t="s">
+        <v>842</v>
+      </c>
+      <c r="F55" s="14" t="s">
+        <v>843</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H55" s="14" t="s">
+        <v>844</v>
+      </c>
+      <c r="I55" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I54"/>
-  <conditionalFormatting sqref="I2:I54">
+  <autoFilter ref="A1:I55"/>
+  <conditionalFormatting sqref="I2:I55">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -21192,7 +21471,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -21204,19 +21483,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>840</v>
+        <v>846</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>842</v>
+        <v>848</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21474,7 +21753,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" ht="60" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
         <v>67</v>
       </c>
@@ -21485,7 +21764,7 @@
         <v>658</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="E17" s="14" t="s">
         <v>655</v>
@@ -21496,10 +21775,10 @@
         <v>67</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D18" s="14" t="s">
         <v>175</v>
@@ -21519,10 +21798,10 @@
         <v>669</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>671</v>
+        <v>175</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21530,16 +21809,16 @@
         <v>67</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>174</v>
+        <v>674</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21547,16 +21826,16 @@
         <v>67</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>679</v>
+        <v>174</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>680</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>213</v>
+        <v>677</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21564,13 +21843,13 @@
         <v>67</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>687</v>
+        <v>213</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>683</v>
@@ -21581,13 +21860,13 @@
         <v>67</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>234</v>
+        <v>690</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>689</v>
@@ -21598,16 +21877,16 @@
         <v>67</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>235</v>
+        <v>693</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21615,16 +21894,16 @@
         <v>67</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>699</v>
+        <v>240</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>700</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21632,10 +21911,10 @@
         <v>67</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="D26" s="14" t="s">
         <v>266</v>
@@ -21655,10 +21934,10 @@
         <v>711</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21666,13 +21945,13 @@
         <v>67</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>319</v>
+        <v>716</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="E28" s="14" t="s">
         <v>714</v>
@@ -21680,19 +21959,19 @@
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B29" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>722</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="E29" s="14" t="s">
         <v>720</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>719</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21700,16 +21979,16 @@
         <v>61</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D30" s="14" t="s">
         <v>99</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21717,16 +21996,16 @@
         <v>61</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>626</v>
+        <v>731</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>627</v>
+        <v>732</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>624</v>
+        <v>730</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21734,16 +22013,16 @@
         <v>61</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>145</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21751,16 +22030,16 @@
         <v>61</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>731</v>
+        <v>631</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>732</v>
+        <v>632</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>729</v>
+        <v>630</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21768,13 +22047,13 @@
         <v>61</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>739</v>
+        <v>188</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>735</v>
@@ -21788,10 +22067,10 @@
         <v>742</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>243</v>
+        <v>743</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="E35" s="14" t="s">
         <v>741</v>
@@ -21802,16 +22081,16 @@
         <v>61</v>
       </c>
       <c r="B36" s="14" t="s">
+        <v>748</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>750</v>
+      </c>
+      <c r="E36" s="14" t="s">
         <v>747</v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>248</v>
-      </c>
-      <c r="E36" s="14" t="s">
-        <v>746</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21819,16 +22098,16 @@
         <v>61</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21836,16 +22115,16 @@
         <v>61</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="C38" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E38" s="14" t="s">
         <v>756</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>754</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21853,16 +22132,16 @@
         <v>61</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>283</v>
+        <v>761</v>
       </c>
       <c r="C39" s="14" t="s">
+        <v>762</v>
+      </c>
+      <c r="D39" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="E39" s="14" t="s">
         <v>760</v>
-      </c>
-      <c r="D39" s="14" t="s">
-        <v>278</v>
-      </c>
-      <c r="E39" s="14" t="s">
-        <v>759</v>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21870,16 +22149,16 @@
         <v>61</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="C40" s="14" t="s">
+        <v>766</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="E40" s="14" t="s">
         <v>765</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>763</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21887,33 +22166,33 @@
         <v>61</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="C41" s="14" t="s">
+        <v>771</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="E41" s="14" t="s">
         <v>769</v>
-      </c>
-      <c r="D41" s="14" t="s">
-        <v>325</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>768</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>774</v>
+        <v>330</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>775</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21921,13 +22200,13 @@
         <v>86</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>207</v>
+        <v>780</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="E43" s="14" t="s">
         <v>778</v>
@@ -21938,16 +22217,16 @@
         <v>86</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21955,21 +22234,21 @@
         <v>86</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>787</v>
+        <v>132</v>
       </c>
       <c r="C45" s="14" t="s">
+        <v>789</v>
+      </c>
+      <c r="D45" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E45" s="14" t="s">
         <v>788</v>
-      </c>
-      <c r="D45" s="14" t="s">
-        <v>260</v>
-      </c>
-      <c r="E45" s="14" t="s">
-        <v>786</v>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>793</v>
@@ -21978,10 +22257,10 @@
         <v>794</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21989,13 +22268,13 @@
         <v>378</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>398</v>
+        <v>799</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E47" s="14" t="s">
         <v>797</v>
@@ -22003,19 +22282,19 @@
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>86</v>
+        <v>378</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>87</v>
+        <v>398</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>826</v>
+        <v>805</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>81</v>
+        <v>393</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>824</v>
+        <v>803</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22023,16 +22302,16 @@
         <v>86</v>
       </c>
       <c r="B49" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>832</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="E49" s="14" t="s">
         <v>830</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>831</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>829</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22040,20 +22319,37 @@
         <v>86</v>
       </c>
       <c r="B50" s="14" t="s">
+        <v>836</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>837</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E50" s="14" t="s">
         <v>835</v>
       </c>
-      <c r="C50" s="14" t="s">
-        <v>836</v>
-      </c>
-      <c r="D50" s="14" t="s">
+    </row>
+    <row r="51" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>841</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>842</v>
+      </c>
+      <c r="D51" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="E50" s="14" t="s">
-        <v>834</v>
+      <c r="E51" s="14" t="s">
+        <v>840</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E50"/>
+  <autoFilter ref="A1:E51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -22078,114 +22374,114 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>845</v>
+        <v>851</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>846</v>
+        <v>852</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>848</v>
+        <v>854</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>866</v>
+        <v>872</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>867</v>
+        <v>873</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>868</v>
+        <v>874</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>164</v>
@@ -22193,22 +22489,22 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>876</v>
+        <v>882</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>170</v>
@@ -22216,186 +22512,186 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>879</v>
+        <v>885</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>881</v>
+        <v>887</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>882</v>
+        <v>888</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>883</v>
+        <v>889</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>885</v>
+        <v>891</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>886</v>
+        <v>892</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>888</v>
+        <v>894</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>889</v>
+        <v>895</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>891</v>
+        <v>897</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>893</v>
+        <v>899</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>896</v>
+        <v>902</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>897</v>
+        <v>903</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>898</v>
+        <v>904</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>899</v>
+        <v>905</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>900</v>
+        <v>906</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>901</v>
+        <v>907</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>902</v>
+        <v>908</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>904</v>
+        <v>910</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>908</v>
+        <v>914</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>909</v>
+        <v>915</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>910</v>
+        <v>916</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>911</v>
+        <v>917</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>912</v>
+        <v>918</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>914</v>
+        <v>920</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>915</v>
+        <v>921</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>916</v>
+        <v>922</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>917</v>
+        <v>923</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>919</v>
+        <v>925</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>916</v>
+        <v>922</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-055 Define multi-tenant authentication endpoints
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3521" uniqueCount="1094">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3535" uniqueCount="1098">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3315,6 +3315,188 @@
 - Task-agent tests pass.
 - No frontend changes.
 - No controller changes.
+- No migration/RLS changes.
+- No hosted operation occurs.</t>
+  </si>
+  <si>
+    <t>CODE-055</t>
+  </si>
+  <si>
+    <t>Expose multi-tenant authentication HTTP endpoints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a controller-only compatibility task.
+Do not change frontend code.
+Do not change AuthService orchestration.
+Do not change AuthRepository.
+Do not change guards.
+Do not change JwtStrategy.
+Do not change migrations or RLS.
+Do not remove legacy authentication endpoints.
+The goal is to expose the already-implemented CODE-052 multi-tenant service
+methods through HTTP while preserving the currently working frontend.
+1. TRANSPORTER REGISTRATION ENDPOINT
+Add:
+POST /auth/register/transporter
+Request DTO:
+RegisterTransporterDto
+Delegate directly to:
+AuthService.registerTransporter()
+Success status:
+201 Created
+Response:
+MultiTenantAuthResponseDto
+The controller must not:
+- accept a role
+- accept tenantId
+- accept membershipId
+- derive an application role
+- perform database operations directly
+- perform Supabase operations directly
+The service remains responsible for orchestration.
+2. CAR-PULLER REGISTRATION ENDPOINT
+Add:
+POST /auth/register/car-puller
+Request DTO:
+RegisterCarPullerDto
+Delegate directly to:
+AuthService.registerCarPuller()
+Success status:
+201 Created
+Response:
+MultiTenantAuthResponseDto
+Company name must not be required or accepted by the DTO.
+The controller must not create or select a tenant.
+3. MULTI-TENANT LOGIN ENDPOINT
+Add a transitional endpoint:
+POST /auth/login/multi-tenant
+Request DTO:
+LoginDto
+Delegate directly to:
+AuthService.loginMultiTenant()
+Success status:
+200 OK
+Response:
+MultiTenantAuthResponseDto
+This route is transitional so the frontend can migrate safely without
+breaking the existing POST /auth/login route.
+Do not perform tenant selection in the controller.
+Service behavior remains:
+- zero active memberships -&gt; selectedMembership = null
+- exactly one active membership -&gt; selected automatically
+- multiple active memberships -&gt; selectedMembership = null
+4. PRESERVE LEGACY ROUTES
+The following existing routes must remain unchanged:
+POST /auth/register
+POST /auth/login
+They currently support the existing frontend and must continue to delegate to
+the existing legacy AuthService methods.
+Do not rename them.
+Do not remove them.
+Do not change their request DTOs.
+Do not change their response contracts in CODE-055.
+5. ROUTE SECURITY
+All registration/login endpoints in this task remain public authentication
+entry points.
+Do not apply:
+AuthGuard
+TenantContextGuard
+RolesGuard
+to these registration/login routes.
+Tenant-context authorization belongs on authenticated tenant-scoped business
+APIs, not login/register endpoints.
+6. SWAGGER / RESPONSE CONTRACT
+Document the new endpoints consistently with existing controller conventions.
+Use MultiTenantAuthResponseDto for:
+POST /auth/register/transporter
+POST /auth/register/car-puller
+POST /auth/login/multi-tenant
+Preserve legacy AuthResponseDto documentation for legacy endpoints.
+7. CONTROLLER RESPONSIBILITY
+Keep the controller thin.
+Allowed responsibility:
+- accept validated DTO
+- call corresponding AuthService method
+- return service result
+Do not add:
+- business orchestration
+- membership lookup
+- profile lookup
+- tenant creation logic
+- Supabase logic
+- token parsing
+- compensation logic
+8. TESTS
+Update auth.controller.spec.ts to cover at minimum:
+TRANSPORTER
+- POST-equivalent controller method delegates to registerTransporter()
+- exact RegisterTransporterDto-shaped input is passed through
+- service result is returned unchanged
+- no client role field is introduced
+CAR PULLER
+- delegates to registerCarPuller()
+- input contains no companyName requirement
+- service result is returned unchanged
+MULTI-TENANT LOGIN
+- delegates to loginMultiTenant()
+- exact LoginDto-shaped input is passed through
+- multi-tenant result is returned unchanged
+LEGACY REGRESSION
+- existing register controller behavior still works
+- existing login controller behavior still works
+- existing controller tests continue passing
+METADATA / ROUTING
+Verify through controller metadata/testing as appropriate:
+- transporter registration route exists
+- car-puller registration route exists
+- multi-tenant login route exists
+- transporter registration uses 201
+- car-puller registration uses 201
+- multi-tenant login uses 200
+- legacy routes still exist
+9. OUT OF SCOPE
+Do NOT:
+- modify auth.service.ts
+- modify auth.repository.ts
+- modify jwt.strategy.ts
+- modify AuthGuard
+- modify TenantContextGuard
+- modify RolesGuard
+- modify registration DTO implementations
+- modify auth response DTO implementations
+- modify frontend
+- remove legacy routes
+- alter database schema
+- modify migrations
+- alter RLS
+- modify package dependencies
+- modify environment files
+- access hosted Supabase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- POST /auth/register/transporter exists.
+- It accepts RegisterTransporterDto.
+- It returns the multi-tenant auth response.
+- It delegates only to registerTransporter().
+- POST /auth/register/car-puller exists.
+- It accepts RegisterCarPullerDto.
+- It returns the multi-tenant auth response.
+- It delegates only to registerCarPuller().
+- POST /auth/login/multi-tenant exists.
+- It accepts LoginDto.
+- It delegates only to loginMultiTenant().
+- It returns the multi-tenant auth response.
+- Legacy POST /auth/register remains operational.
+- Legacy POST /auth/login remains operational.
+- No tenant or role is selected in the controller.
+- No auth guard is applied to registration/login routes.
+- Existing API tests continue passing.
+- New controller tests pass.
+- API build/typecheck passes.
+- Task-agent tests pass.
+- No frontend files change.
+- No guard changes.
+- No service/repository changes.
 - No migration/RLS changes.
 - No hosted operation occurs.</t>
   </si>
@@ -5581,22 +5763,22 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5604,76 +5786,76 @@
         <v>619</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="C3" s="14" t="s">
+        <v>942</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>943</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>938</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>939</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>934</v>
-      </c>
       <c r="F3" s="14" t="s">
-        <v>940</v>
+        <v>944</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>944</v>
+        <v>948</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="C5" s="14" t="s">
+        <v>952</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>948</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>944</v>
-      </c>
       <c r="E5" s="14" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>120</v>
@@ -5681,79 +5863,79 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>958</v>
+        <v>962</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>959</v>
+        <v>963</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>273</v>
@@ -5761,59 +5943,59 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>969</v>
+        <v>973</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>975</v>
+        <v>979</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>976</v>
+        <v>980</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>977</v>
+        <v>981</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>978</v>
+        <v>982</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>979</v>
+        <v>983</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>980</v>
+        <v>984</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>362</v>
@@ -5845,25 +6027,25 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>981</v>
+        <v>985</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>983</v>
+        <v>987</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>22</v>
@@ -5871,25 +6053,25 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>987</v>
+        <v>991</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>990</v>
+        <v>994</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>991</v>
+        <v>995</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>992</v>
+        <v>996</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>25</v>
@@ -5897,25 +6079,25 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
+        <v>997</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>998</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>999</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>993</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>994</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>995</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>989</v>
-      </c>
       <c r="E3" s="14" t="s">
+        <v>1000</v>
+      </c>
+      <c r="F3" s="14" t="s">
+        <v>1001</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>996</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>997</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>992</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>25</v>
@@ -5923,22 +6105,22 @@
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>998</v>
+        <v>1002</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>332</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>331</v>
@@ -5949,22 +6131,22 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1005</v>
+        <v>1009</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>1006</v>
+        <v>1010</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>338</v>
@@ -5975,25 +6157,25 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1011</v>
+        <v>1015</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>25</v>
@@ -6001,25 +6183,25 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1013</v>
+        <v>1017</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1014</v>
+        <v>1018</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1015</v>
+        <v>1019</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1018</v>
+        <v>1022</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>25</v>
@@ -6027,25 +6209,25 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1021</v>
+        <v>1025</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1025</v>
+        <v>1029</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>25</v>
@@ -6053,22 +6235,22 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1027</v>
+        <v>1031</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>1006</v>
+        <v>1010</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>1029</v>
+        <v>1033</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1030</v>
+        <v>1034</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>302</v>
@@ -6079,22 +6261,22 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1031</v>
+        <v>1035</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1032</v>
+        <v>1036</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1033</v>
+        <v>1037</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>181</v>
@@ -6105,22 +6287,22 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>1039</v>
+        <v>1043</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>194</v>
@@ -6131,22 +6313,22 @@
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>1044</v>
+        <v>1048</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>325</v>
@@ -6206,19 +6388,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1045</v>
+        <v>1049</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1046</v>
+        <v>1050</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1047</v>
+        <v>1051</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>500</v>
@@ -6229,163 +6411,163 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1052</v>
+        <v>1056</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>130</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>1055</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>1051</v>
-      </c>
       <c r="C3" s="14" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>1057</v>
+        <v>1061</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>67</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1058</v>
+        <v>1062</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1059</v>
+        <v>1063</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>183</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1061</v>
+        <v>1065</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1062</v>
+        <v>1066</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1063</v>
+        <v>1067</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1066</v>
+        <v>1070</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1067</v>
+        <v>1071</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1068</v>
+        <v>1072</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1071</v>
+        <v>1075</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1073</v>
+        <v>1077</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1075</v>
+        <v>1079</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1068</v>
+        <v>1072</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
     </row>
   </sheetData>
@@ -6413,13 +6595,13 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1076</v>
+        <v>1080</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1077</v>
+        <v>1081</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>500</v>
@@ -6428,7 +6610,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1078</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6436,10 +6618,10 @@
         <v>130</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1079</v>
+        <v>1083</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>130</v>
@@ -6454,10 +6636,10 @@
         <v>94</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1081</v>
+        <v>1085</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>67</v>
@@ -6472,10 +6654,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1082</v>
+        <v>1086</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>199</v>
@@ -6487,13 +6669,13 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1083</v>
+        <v>1087</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>1088</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>1084</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>1080</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>61</v>
@@ -6505,13 +6687,13 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1085</v>
+        <v>1089</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1086</v>
+        <v>1090</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>199</v>
@@ -6526,10 +6708,10 @@
         <v>309</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1087</v>
+        <v>1091</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1088</v>
+        <v>1092</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>199</v>
@@ -6544,10 +6726,10 @@
         <v>374</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1089</v>
+        <v>1093</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>378</v>
@@ -6562,10 +6744,10 @@
         <v>400</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1090</v>
+        <v>1094</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>55</v>
@@ -6580,10 +6762,10 @@
         <v>400</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1091</v>
+        <v>1095</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>55</v>
@@ -6595,13 +6777,13 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>1092</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>1093</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>1088</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>433</v>
@@ -19826,7 +20008,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -20390,7 +20572,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" ht="409.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
         <v>661</v>
       </c>
@@ -20398,22 +20580,22 @@
         <v>67</v>
       </c>
       <c r="C20" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>598</v>
+      </c>
+      <c r="E20" s="14" t="s">
         <v>662</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="F20" s="14" t="s">
         <v>663</v>
       </c>
-      <c r="E20" s="14" t="s">
+      <c r="G20" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="H20" s="14" t="s">
         <v>664</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>665</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="H20" s="14" t="s">
-        <v>666</v>
       </c>
       <c r="I20" s="14" t="s">
         <v>25</v>
@@ -20421,83 +20603,83 @@
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="B21" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="D21" s="14" t="s">
+        <v>667</v>
+      </c>
+      <c r="E21" s="14" t="s">
         <v>668</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="F21" s="14" t="s">
         <v>669</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>670</v>
       </c>
       <c r="G21" s="14" t="s">
         <v>175</v>
       </c>
       <c r="H21" s="14" t="s">
+        <v>670</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="14" t="s">
         <v>671</v>
-      </c>
-      <c r="I21" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>672</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="14" t="s">
+        <v>666</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>672</v>
+      </c>
+      <c r="E22" s="14" t="s">
         <v>673</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="F22" s="14" t="s">
         <v>674</v>
       </c>
-      <c r="E22" s="14" t="s">
+      <c r="G22" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H22" s="14" t="s">
         <v>675</v>
       </c>
-      <c r="F22" s="14" t="s">
+      <c r="I22" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
         <v>676</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>677</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>678</v>
-      </c>
-      <c r="I22" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>679</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>174</v>
+        <v>678</v>
       </c>
       <c r="E23" s="14" t="s">
+        <v>679</v>
+      </c>
+      <c r="F23" s="14" t="s">
         <v>680</v>
       </c>
-      <c r="F23" s="14" t="s">
+      <c r="G23" s="14" t="s">
         <v>681</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>677</v>
       </c>
       <c r="H23" s="14" t="s">
         <v>682</v>
@@ -20514,51 +20696,51 @@
         <v>67</v>
       </c>
       <c r="C24" s="14" t="s">
+        <v>677</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="E24" s="14" t="s">
         <v>684</v>
       </c>
-      <c r="D24" s="14" t="s">
+      <c r="F24" s="14" t="s">
         <v>685</v>
       </c>
-      <c r="E24" s="14" t="s">
+      <c r="G24" s="14" t="s">
+        <v>681</v>
+      </c>
+      <c r="H24" s="14" t="s">
         <v>686</v>
       </c>
-      <c r="F24" s="14" t="s">
+      <c r="I24" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="14" t="s">
         <v>687</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>213</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>688</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>689</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D25" s="14" t="s">
+        <v>689</v>
+      </c>
+      <c r="E25" s="14" t="s">
         <v>690</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="F25" s="14" t="s">
         <v>691</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="G25" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="H25" s="14" t="s">
         <v>692</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>693</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>694</v>
       </c>
       <c r="I25" s="14" t="s">
         <v>25</v>
@@ -20566,25 +20748,25 @@
     </row>
     <row r="26" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>234</v>
+        <v>694</v>
       </c>
       <c r="E26" s="14" t="s">
+        <v>695</v>
+      </c>
+      <c r="F26" s="14" t="s">
         <v>696</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="G26" s="14" t="s">
         <v>697</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>693</v>
       </c>
       <c r="H26" s="14" t="s">
         <v>698</v>
@@ -20601,10 +20783,10 @@
         <v>67</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E27" s="14" t="s">
         <v>700</v>
@@ -20613,7 +20795,7 @@
         <v>701</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>235</v>
+        <v>697</v>
       </c>
       <c r="H27" s="14" t="s">
         <v>702</v>
@@ -20622,7 +20804,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
         <v>703</v>
       </c>
@@ -20630,22 +20812,22 @@
         <v>67</v>
       </c>
       <c r="C28" s="14" t="s">
+        <v>688</v>
+      </c>
+      <c r="D28" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="E28" s="14" t="s">
         <v>704</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="F28" s="14" t="s">
         <v>705</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="G28" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="H28" s="14" t="s">
         <v>706</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>707</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>266</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>708</v>
       </c>
       <c r="I28" s="14" t="s">
         <v>25</v>
@@ -20653,57 +20835,57 @@
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="D29" s="14" t="s">
+        <v>709</v>
+      </c>
+      <c r="E29" s="14" t="s">
         <v>710</v>
       </c>
-      <c r="E29" s="14" t="s">
+      <c r="F29" s="14" t="s">
         <v>711</v>
-      </c>
-      <c r="F29" s="14" t="s">
-        <v>712</v>
       </c>
       <c r="G29" s="14" t="s">
         <v>266</v>
       </c>
       <c r="H29" s="14" t="s">
+        <v>712</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
         <v>713</v>
-      </c>
-      <c r="I29" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="30" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
-        <v>714</v>
       </c>
       <c r="B30" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C30" s="14" t="s">
+        <v>708</v>
+      </c>
+      <c r="D30" s="14" t="s">
+        <v>714</v>
+      </c>
+      <c r="E30" s="14" t="s">
         <v>715</v>
       </c>
-      <c r="D30" s="14" t="s">
+      <c r="F30" s="14" t="s">
         <v>716</v>
       </c>
-      <c r="E30" s="14" t="s">
+      <c r="G30" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="H30" s="14" t="s">
         <v>717</v>
-      </c>
-      <c r="F30" s="14" t="s">
-        <v>718</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>291</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>719</v>
       </c>
       <c r="I30" s="14" t="s">
         <v>25</v>
@@ -20711,65 +20893,65 @@
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C31" s="14" t="s">
+        <v>719</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>720</v>
+      </c>
+      <c r="E31" s="14" t="s">
         <v>721</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="F31" s="14" t="s">
+        <v>722</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="H31" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="14" t="s">
+        <v>724</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>725</v>
+      </c>
+      <c r="D32" s="14" t="s">
         <v>319</v>
       </c>
-      <c r="E31" s="14" t="s">
-        <v>722</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>723</v>
-      </c>
-      <c r="G31" s="14" t="s">
+      <c r="E32" s="14" t="s">
+        <v>726</v>
+      </c>
+      <c r="F32" s="14" t="s">
+        <v>727</v>
+      </c>
+      <c r="G32" s="14" t="s">
         <v>314</v>
       </c>
-      <c r="H31" s="14" t="s">
-        <v>724</v>
-      </c>
-      <c r="I31" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="32" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
-        <v>725</v>
-      </c>
-      <c r="B32" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>571</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>726</v>
-      </c>
-      <c r="E32" s="14" t="s">
-        <v>727</v>
-      </c>
-      <c r="F32" s="14" t="s">
+      <c r="H32" s="14" t="s">
         <v>728</v>
       </c>
-      <c r="G32" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="H32" s="14" t="s">
+      <c r="I32" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="14" t="s">
         <v>729</v>
-      </c>
-      <c r="I32" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>730</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>61</v>
@@ -20778,77 +20960,77 @@
         <v>571</v>
       </c>
       <c r="D33" s="14" t="s">
+        <v>730</v>
+      </c>
+      <c r="E33" s="14" t="s">
         <v>731</v>
       </c>
-      <c r="E33" s="14" t="s">
+      <c r="F33" s="14" t="s">
         <v>732</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>733</v>
       </c>
       <c r="G33" s="14" t="s">
         <v>99</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="I33" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="34" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C34" s="14" t="s">
+        <v>571</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>735</v>
+      </c>
+      <c r="E34" s="14" t="s">
         <v>736</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="F34" s="14" t="s">
         <v>737</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="G34" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H34" s="14" t="s">
         <v>738</v>
       </c>
-      <c r="F34" s="14" t="s">
-        <v>739</v>
-      </c>
-      <c r="G34" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="H34" s="14" t="s">
-        <v>740</v>
-      </c>
       <c r="I34" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="D35" s="14" t="s">
+        <v>741</v>
+      </c>
+      <c r="E35" s="14" t="s">
         <v>742</v>
       </c>
-      <c r="E35" s="14" t="s">
+      <c r="F35" s="14" t="s">
         <v>743</v>
       </c>
-      <c r="F35" s="14" t="s">
+      <c r="G35" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="H35" s="14" t="s">
         <v>744</v>
-      </c>
-      <c r="G35" s="14" t="s">
-        <v>745</v>
-      </c>
-      <c r="H35" s="14" t="s">
-        <v>746</v>
       </c>
       <c r="I35" s="14" t="s">
         <v>25</v>
@@ -20856,28 +21038,28 @@
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>684</v>
+        <v>740</v>
       </c>
       <c r="D36" s="14" t="s">
+        <v>746</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>747</v>
+      </c>
+      <c r="F36" s="14" t="s">
         <v>748</v>
       </c>
-      <c r="E36" s="14" t="s">
-        <v>243</v>
-      </c>
-      <c r="F36" s="14" t="s">
+      <c r="G36" s="14" t="s">
         <v>749</v>
       </c>
-      <c r="G36" s="14" t="s">
+      <c r="H36" s="14" t="s">
         <v>750</v>
-      </c>
-      <c r="H36" s="14" t="s">
-        <v>751</v>
       </c>
       <c r="I36" s="14" t="s">
         <v>25</v>
@@ -20885,25 +21067,25 @@
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D37" s="14" t="s">
+        <v>752</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="F37" s="14" t="s">
         <v>753</v>
       </c>
-      <c r="E37" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="F37" s="14" t="s">
+      <c r="G37" s="14" t="s">
         <v>754</v>
-      </c>
-      <c r="G37" s="14" t="s">
-        <v>248</v>
       </c>
       <c r="H37" s="14" t="s">
         <v>755</v>
@@ -20920,19 +21102,19 @@
         <v>61</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D38" s="14" t="s">
         <v>757</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F38" s="14" t="s">
         <v>758</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="H38" s="14" t="s">
         <v>759</v>
@@ -20949,22 +21131,22 @@
         <v>61</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D39" s="14" t="s">
         <v>761</v>
       </c>
       <c r="E39" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="F39" s="14" t="s">
         <v>762</v>
       </c>
-      <c r="F39" s="14" t="s">
+      <c r="G39" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="H39" s="14" t="s">
         <v>763</v>
-      </c>
-      <c r="G39" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="H39" s="14" t="s">
-        <v>764</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>25</v>
@@ -20972,16 +21154,16 @@
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>704</v>
+        <v>688</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>283</v>
+        <v>765</v>
       </c>
       <c r="E40" s="14" t="s">
         <v>766</v>
@@ -20990,7 +21172,7 @@
         <v>767</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="H40" s="14" t="s">
         <v>768</v>
@@ -21007,39 +21189,39 @@
         <v>61</v>
       </c>
       <c r="C41" s="14" t="s">
+        <v>708</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="E41" s="14" t="s">
         <v>770</v>
       </c>
-      <c r="D41" s="14" t="s">
-        <v>307</v>
-      </c>
-      <c r="E41" s="14" t="s">
+      <c r="F41" s="14" t="s">
         <v>771</v>
       </c>
-      <c r="F41" s="14" t="s">
+      <c r="G41" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="H41" s="14" t="s">
         <v>772</v>
       </c>
-      <c r="G41" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="H41" s="14" t="s">
+      <c r="I41" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="14" t="s">
         <v>773</v>
-      </c>
-      <c r="I41" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="42" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>774</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>721</v>
+        <v>774</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="E42" s="14" t="s">
         <v>775</v>
@@ -21048,7 +21230,7 @@
         <v>776</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="H42" s="14" t="s">
         <v>777</v>
@@ -21057,47 +21239,47 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
         <v>778</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="C43" s="14" t="s">
+        <v>725</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="E43" s="14" t="s">
         <v>779</v>
       </c>
-      <c r="D43" s="14" t="s">
+      <c r="F43" s="14" t="s">
         <v>780</v>
       </c>
-      <c r="E43" s="14" t="s">
+      <c r="G43" s="14" t="s">
+        <v>325</v>
+      </c>
+      <c r="H43" s="14" t="s">
         <v>781</v>
       </c>
-      <c r="F43" s="14" t="s">
+      <c r="I43" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A44" s="14" t="s">
         <v>782</v>
-      </c>
-      <c r="G43" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H43" s="14" t="s">
-        <v>783</v>
-      </c>
-      <c r="I43" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>784</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>207</v>
+        <v>784</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>785</v>
@@ -21106,13 +21288,13 @@
         <v>786</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="H44" s="14" t="s">
         <v>787</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -21123,10 +21305,10 @@
         <v>86</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>789</v>
@@ -21135,7 +21317,7 @@
         <v>790</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="H45" s="14" t="s">
         <v>791</v>
@@ -21152,22 +21334,22 @@
         <v>86</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="D46" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="E46" s="14" t="s">
         <v>793</v>
       </c>
-      <c r="E46" s="14" t="s">
+      <c r="F46" s="14" t="s">
         <v>794</v>
       </c>
-      <c r="F46" s="14" t="s">
+      <c r="G46" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="H46" s="14" t="s">
         <v>795</v>
-      </c>
-      <c r="G46" s="14" t="s">
-        <v>260</v>
-      </c>
-      <c r="H46" s="14" t="s">
-        <v>796</v>
       </c>
       <c r="I46" s="14" t="s">
         <v>25</v>
@@ -21175,28 +21357,28 @@
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
+        <v>796</v>
+      </c>
+      <c r="B47" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C47" s="14" t="s">
+        <v>783</v>
+      </c>
+      <c r="D47" s="14" t="s">
         <v>797</v>
       </c>
-      <c r="B47" s="14" t="s">
-        <v>378</v>
-      </c>
-      <c r="C47" s="14" t="s">
+      <c r="E47" s="14" t="s">
         <v>798</v>
       </c>
-      <c r="D47" s="14" t="s">
+      <c r="F47" s="14" t="s">
         <v>799</v>
       </c>
-      <c r="E47" s="14" t="s">
+      <c r="G47" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="H47" s="14" t="s">
         <v>800</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>801</v>
-      </c>
-      <c r="G47" s="14" t="s">
-        <v>381</v>
-      </c>
-      <c r="H47" s="14" t="s">
-        <v>802</v>
       </c>
       <c r="I47" s="14" t="s">
         <v>25</v>
@@ -21204,103 +21386,103 @@
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>378</v>
       </c>
       <c r="C48" s="14" t="s">
+        <v>802</v>
+      </c>
+      <c r="D48" s="14" t="s">
+        <v>803</v>
+      </c>
+      <c r="E48" s="14" t="s">
         <v>804</v>
       </c>
-      <c r="D48" s="14" t="s">
+      <c r="F48" s="14" t="s">
+        <v>805</v>
+      </c>
+      <c r="G48" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="H48" s="14" t="s">
+        <v>806</v>
+      </c>
+      <c r="I48" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A49" s="14" t="s">
+        <v>807</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>378</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>808</v>
+      </c>
+      <c r="D49" s="14" t="s">
         <v>398</v>
       </c>
-      <c r="E48" s="14" t="s">
-        <v>805</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>806</v>
-      </c>
-      <c r="G48" s="14" t="s">
+      <c r="E49" s="14" t="s">
+        <v>809</v>
+      </c>
+      <c r="F49" s="14" t="s">
+        <v>810</v>
+      </c>
+      <c r="G49" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="H48" s="14" t="s">
-        <v>807</v>
-      </c>
-      <c r="I48" s="14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="49" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="14" t="s">
-        <v>808</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>809</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>810</v>
-      </c>
-      <c r="D49" s="14" t="s">
+      <c r="H49" s="14" t="s">
         <v>811</v>
       </c>
-      <c r="E49" s="14" t="s">
+      <c r="I49" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50" s="14" t="s">
         <v>812</v>
       </c>
-      <c r="F49" s="14" t="s">
+      <c r="B50" s="14" t="s">
         <v>813</v>
       </c>
-      <c r="G49" s="14" t="s">
+      <c r="C50" s="14" t="s">
+        <v>814</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>815</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>816</v>
+      </c>
+      <c r="F50" s="14" t="s">
+        <v>817</v>
+      </c>
+      <c r="G50" s="14" t="s">
         <v>471</v>
       </c>
-      <c r="H49" s="14" t="s">
-        <v>814</v>
-      </c>
-      <c r="I49" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="50" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="14" t="s">
-        <v>815</v>
-      </c>
-      <c r="B50" s="14" t="s">
-        <v>809</v>
-      </c>
-      <c r="C50" s="14" t="s">
-        <v>810</v>
-      </c>
-      <c r="D50" s="14" t="s">
-        <v>816</v>
-      </c>
-      <c r="E50" s="14" t="s">
-        <v>817</v>
-      </c>
-      <c r="F50" s="14" t="s">
+      <c r="H50" s="14" t="s">
         <v>818</v>
-      </c>
-      <c r="G50" s="14" t="s">
-        <v>480</v>
-      </c>
-      <c r="H50" s="14" t="s">
-        <v>819</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="51" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
+        <v>819</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>813</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>814</v>
+      </c>
+      <c r="D51" s="14" t="s">
         <v>820</v>
-      </c>
-      <c r="B51" s="14" t="s">
-        <v>809</v>
-      </c>
-      <c r="C51" s="14" t="s">
-        <v>810</v>
-      </c>
-      <c r="D51" s="14" t="s">
-        <v>491</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>821</v>
@@ -21309,7 +21491,7 @@
         <v>822</v>
       </c>
       <c r="G51" s="14" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="H51" s="14" t="s">
         <v>823</v>
@@ -21318,125 +21500,154 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
         <v>824</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>61</v>
+        <v>813</v>
       </c>
       <c r="C52" s="14" t="s">
+        <v>814</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>491</v>
+      </c>
+      <c r="E52" s="14" t="s">
         <v>825</v>
       </c>
-      <c r="D52" s="14" t="s">
+      <c r="F52" s="14" t="s">
         <v>826</v>
       </c>
-      <c r="E52" s="14" t="s">
+      <c r="G52" s="14" t="s">
+        <v>486</v>
+      </c>
+      <c r="H52" s="14" t="s">
         <v>827</v>
-      </c>
-      <c r="F52" s="14" t="s">
-        <v>828</v>
-      </c>
-      <c r="G52" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="H52" s="14" t="s">
-        <v>829</v>
       </c>
       <c r="I52" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="53" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
+        <v>828</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" s="14" t="s">
+        <v>829</v>
+      </c>
+      <c r="D53" s="14" t="s">
         <v>830</v>
       </c>
-      <c r="B53" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C53" s="14" t="s">
+      <c r="E53" s="14" t="s">
         <v>831</v>
       </c>
-      <c r="D53" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="E53" s="14" t="s">
+      <c r="F53" s="14" t="s">
         <v>832</v>
       </c>
-      <c r="F53" s="14" t="s">
+      <c r="G53" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="H53" s="14" t="s">
         <v>833</v>
-      </c>
-      <c r="G53" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="H53" s="14" t="s">
-        <v>834</v>
       </c>
       <c r="I53" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="54" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="B54" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>779</v>
+        <v>835</v>
       </c>
       <c r="D54" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="E54" s="14" t="s">
         <v>836</v>
       </c>
-      <c r="E54" s="14" t="s">
+      <c r="F54" s="14" t="s">
         <v>837</v>
       </c>
-      <c r="F54" s="14" t="s">
+      <c r="G54" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="H54" s="14" t="s">
         <v>838</v>
-      </c>
-      <c r="G54" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="H54" s="14" t="s">
-        <v>839</v>
       </c>
       <c r="I54" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="55" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="D55" s="14" t="s">
+        <v>840</v>
+      </c>
+      <c r="E55" s="14" t="s">
         <v>841</v>
       </c>
-      <c r="E55" s="14" t="s">
+      <c r="F55" s="14" t="s">
         <v>842</v>
       </c>
-      <c r="F55" s="14" t="s">
+      <c r="G55" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H55" s="14" t="s">
         <v>843</v>
-      </c>
-      <c r="G55" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="H55" s="14" t="s">
-        <v>844</v>
       </c>
       <c r="I55" s="14" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="56" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A56" s="14" t="s">
+        <v>844</v>
+      </c>
+      <c r="B56" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C56" s="14" t="s">
+        <v>783</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>845</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>846</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>847</v>
+      </c>
+      <c r="G56" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H56" s="14" t="s">
+        <v>848</v>
+      </c>
+      <c r="I56" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I55"/>
-  <conditionalFormatting sqref="I2:I55">
+  <autoFilter ref="A1:I56"/>
+  <conditionalFormatting sqref="I2:I56">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -21471,7 +21682,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -21483,19 +21694,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21770,18 +21981,18 @@
         <v>655</v>
       </c>
     </row>
-    <row r="18" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
         <v>67</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>663</v>
+        <v>598</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="E18" s="14" t="s">
         <v>661</v>
@@ -21792,16 +22003,16 @@
         <v>67</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>667</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>668</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>669</v>
       </c>
       <c r="D19" s="14" t="s">
         <v>175</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21809,16 +22020,16 @@
         <v>67</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>677</v>
+        <v>175</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21826,16 +22037,16 @@
         <v>67</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>174</v>
+        <v>678</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21843,13 +22054,13 @@
         <v>67</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>685</v>
+        <v>174</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>213</v>
+        <v>681</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>683</v>
@@ -21860,16 +22071,16 @@
         <v>67</v>
       </c>
       <c r="B23" s="14" t="s">
+        <v>689</v>
+      </c>
+      <c r="C23" s="14" t="s">
         <v>690</v>
       </c>
-      <c r="C23" s="14" t="s">
-        <v>691</v>
-      </c>
       <c r="D23" s="14" t="s">
-        <v>693</v>
+        <v>213</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21877,16 +22088,16 @@
         <v>67</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>234</v>
+        <v>694</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="D24" s="14" t="s">
+        <v>697</v>
+      </c>
+      <c r="E24" s="14" t="s">
         <v>693</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>695</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21894,13 +22105,13 @@
         <v>67</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>700</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>235</v>
+        <v>697</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>699</v>
@@ -21911,13 +22122,13 @@
         <v>67</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>705</v>
+        <v>240</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="E26" s="14" t="s">
         <v>703</v>
@@ -21928,16 +22139,16 @@
         <v>67</v>
       </c>
       <c r="B27" s="14" t="s">
+        <v>709</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>710</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>711</v>
       </c>
       <c r="D27" s="14" t="s">
         <v>266</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21945,16 +22156,16 @@
         <v>67</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21962,33 +22173,33 @@
         <v>67</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>319</v>
+        <v>720</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B30" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>726</v>
       </c>
-      <c r="C30" s="14" t="s">
-        <v>727</v>
-      </c>
       <c r="D30" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21996,16 +22207,16 @@
         <v>61</v>
       </c>
       <c r="B31" s="14" t="s">
+        <v>730</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>731</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>732</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>99</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22013,16 +22224,16 @@
         <v>61</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>626</v>
+        <v>735</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>627</v>
+        <v>736</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>624</v>
+        <v>734</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22030,16 +22241,16 @@
         <v>61</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>145</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22047,16 +22258,16 @@
         <v>61</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>737</v>
+        <v>631</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>738</v>
+        <v>632</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>735</v>
+        <v>630</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22064,16 +22275,16 @@
         <v>61</v>
       </c>
       <c r="B35" s="14" t="s">
+        <v>741</v>
+      </c>
+      <c r="C35" s="14" t="s">
         <v>742</v>
       </c>
-      <c r="C35" s="14" t="s">
-        <v>743</v>
-      </c>
       <c r="D35" s="14" t="s">
-        <v>745</v>
+        <v>188</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22081,16 +22292,16 @@
         <v>61</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>243</v>
+        <v>747</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22098,16 +22309,16 @@
         <v>61</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>248</v>
+        <v>754</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22118,10 +22329,10 @@
         <v>757</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>756</v>
@@ -22135,10 +22346,10 @@
         <v>761</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>762</v>
+        <v>255</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="E39" s="14" t="s">
         <v>760</v>
@@ -22149,16 +22360,16 @@
         <v>61</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>283</v>
+        <v>765</v>
       </c>
       <c r="C40" s="14" t="s">
         <v>766</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22166,13 +22377,13 @@
         <v>61</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="E41" s="14" t="s">
         <v>769</v>
@@ -22183,30 +22394,30 @@
         <v>61</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="C42" s="14" t="s">
         <v>775</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>780</v>
+        <v>330</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="E43" s="14" t="s">
         <v>778</v>
@@ -22217,16 +22428,16 @@
         <v>86</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>207</v>
+        <v>784</v>
       </c>
       <c r="C44" s="14" t="s">
         <v>785</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22234,13 +22445,13 @@
         <v>86</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="C45" s="14" t="s">
         <v>789</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>788</v>
@@ -22251,13 +22462,13 @@
         <v>86</v>
       </c>
       <c r="B46" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C46" s="14" t="s">
         <v>793</v>
       </c>
-      <c r="C46" s="14" t="s">
-        <v>794</v>
-      </c>
       <c r="D46" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>792</v>
@@ -22265,19 +22476,19 @@
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22285,33 +22496,33 @@
         <v>378</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>398</v>
+        <v>803</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>86</v>
+        <v>378</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>87</v>
+        <v>398</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>832</v>
+        <v>809</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>81</v>
+        <v>393</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>830</v>
+        <v>807</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22319,16 +22530,16 @@
         <v>86</v>
       </c>
       <c r="B50" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C50" s="14" t="s">
         <v>836</v>
       </c>
-      <c r="C50" s="14" t="s">
-        <v>837</v>
-      </c>
       <c r="D50" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22336,20 +22547,37 @@
         <v>86</v>
       </c>
       <c r="B51" s="14" t="s">
+        <v>840</v>
+      </c>
+      <c r="C51" s="14" t="s">
         <v>841</v>
       </c>
-      <c r="C51" s="14" t="s">
-        <v>842</v>
-      </c>
       <c r="D51" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B52" s="14" t="s">
+        <v>845</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>846</v>
+      </c>
+      <c r="D52" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="E51" s="14" t="s">
-        <v>840</v>
+      <c r="E52" s="14" t="s">
+        <v>844</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E51"/>
+  <autoFilter ref="A1:E52"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -22374,114 +22602,114 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>855</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>851</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>847</v>
-      </c>
       <c r="D1" s="10" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B3" s="14" t="s">
+        <v>867</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>868</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>863</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>864</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>859</v>
-      </c>
       <c r="E3" s="14" t="s">
+        <v>869</v>
+      </c>
+      <c r="F3" s="14" t="s">
         <v>865</v>
       </c>
-      <c r="F3" s="14" t="s">
-        <v>861</v>
-      </c>
       <c r="G3" s="14" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>878</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>879</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>874</v>
       </c>
-      <c r="C5" s="14" t="s">
-        <v>875</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>870</v>
-      </c>
       <c r="E5" s="14" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>164</v>
@@ -22489,22 +22717,22 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>170</v>
@@ -22512,186 +22740,186 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
       <c r="F14" s="14" t="s">
+        <v>930</v>
+      </c>
+      <c r="G14" s="14" t="s">
         <v>926</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>922</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-056 Define multi-tenant frontend authentication migration
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3535" uniqueCount="1098">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3549" uniqueCount="1104">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -3497,6 +3497,403 @@
 - No frontend files change.
 - No guard changes.
 - No service/repository changes.
+- No migration/RLS changes.
+- No hosted operation occurs.</t>
+  </si>
+  <si>
+    <t>CODE-056</t>
+  </si>
+  <si>
+    <t>authentication</t>
+  </si>
+  <si>
+    <t>apps/web/lib/auth.types.ts; apps/web/lib/api.ts; apps/web/lib/api.test.ts; apps/web/lib/auth.ts; apps/web/lib/auth.test.ts; apps/web/app/(auth)/login/page.tsx; apps/web/app/(auth)/login/page.test.tsx; apps/web/app/(auth)/register/page.tsx; apps/web/app/(auth)/register/page.test.tsx; apps/web/app/(auth)/register/transporter/page.tsx; apps/web/app/(auth)/register/transporter/page.test.tsx; apps/web/app/(auth)/register/car-puller/page.tsx; apps/web/app/(auth)/register/car-puller/page.test.tsx</t>
+  </si>
+  <si>
+    <t>Migrate frontend authentication to transporter and car-puller multi-tenant flows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This task migrates the browser authentication experience to the new
+multi-tenant backend contracts.
+Do not modify backend code.
+Do not modify migrations or RLS.
+Do not modify Supabase server configuration.
+Do not implement dashboards yet.
+Do not implement invitations yet.
+Do not implement the existing-user-create-second-transporter flow yet.
+Do not implement tenant-scoped business APIs yet.
+1. FRONTEND MULTI-TENANT TYPES
+Update auth.types.ts to represent the backend multi-tenant response.
+Keep or temporarily preserve legacy frontend types only where required for
+compatibility tests.
+Add types equivalent to:
+AuthSession:
+- accessToken
+- refreshToken
+- expiresIn
+- expiresAt
+- tokenType
+UserProfile:
+- userId
+- email
+- fullName
+- phone
+MembershipStatus:
+- active
+- suspended
+- removed
+MembershipSummary:
+- membershipId
+- tenantId
+- tenantName
+- role
+- status
+MultiTenantAuthResponse:
+- session
+- requiresEmailConfirmation
+- profile
+- memberships
+- selectedMembership
+selectedMembership must allow null.
+Supported roles remain:
+- admin
+- dispatcher
+- car_puller
+2. FRONTEND API CLIENT
+Add/update API functions for exactly:
+registerTransporter(...)
+  -&gt; POST /auth/register/transporter
+registerCarPuller(...)
+  -&gt; POST /auth/register/car-puller
+loginMultiTenant(...)
+  -&gt; POST /auth/login/multi-tenant
+Transporter request payload:
+{
+  email,
+  password,
+  companyName,
+  fullName,
+  phone
+}
+Car-puller payload:
+{
+  email,
+  password,
+  fullName,
+  phone
+}
+Login payload:
+{
+  email,
+  password
+}
+Do not send:
+- confirmPassword
+- role
+- tenantId
+- membershipId
+Validate the multi-tenant response shape safely.
+Do not accept malformed profile/membership/session responses.
+3. SESSION INSTALLATION
+Continue using the existing browser Supabase client/session mechanism.
+When the backend returns a non-null session:
+install the Supabase session using the existing safe browser-session approach.
+Do NOT manually store access tokens or refresh tokens in localStorage.
+Do NOT invent custom JWT handling.
+Email-confirmation behavior must continue working when session is null.
+4. FRONTEND AUTH APPLICATION STATE
+Update the existing auth helper/state so it can retain:
+- profile
+- memberships
+- selectedMembership
+The application context is not an authorization source.
+Tenant authorization will always be revalidated by the backend.
+Do not treat selectedMembership as proof of authorization.
+Do not place role or tenant identity inside the Supabase token.
+5. REGISTER LANDING PAGE
+Change:
+/register
+from the current single transporter-style form into the account-type choice
+screen matching the proposed IAMONIT product design.
+Present two clear actions:
+"Sign Up as a Transporter"
+and
+"Sign Up as a Car Puller"
+Transporter action navigates to:
+/register/transporter
+Car Puller action navigates to:
+/register/car-puller
+The page itself must not submit an authentication request.
+6. TRANSPORTER REGISTRATION PAGE
+Create:
+/register/transporter
+Use the existing IAMONIT registration styling where practical.
+Fields:
+- Full name
+- Company name
+- Email address
+- Phone number
+- Password
+- Confirm password
+Do not show a role selector.
+Client validation:
+- required fields
+- valid email
+- existing approved password rule
+- password confirmation
+- phone in international/E.164-compatible format
+Example accepted phone format:
++14694681177
+confirmPassword is client-only.
+Submit exactly:
+{
+  email,
+  password,
+  companyName,
+  fullName,
+  phone
+}
+to registerTransporter().
+7. TRANSPORTER SUCCESS BEHAVIOR
+On successful transporter registration:
+- install returned Supabase session when non-null
+- retain returned profile
+- retain memberships
+- retain selectedMembership
+The backend should normally return exactly one active admin membership.
+Do not recalculate or manufacture admin role in the browser.
+Use the backend response.
+Until the transporter dashboard is implemented:
+redirect successful authenticated registration to:
+/
+If email confirmation is required:
+do not pretend the user is authenticated.
+Show the existing clear confirmation-required guidance.
+8. CAR-PULLER REGISTRATION PAGE
+Create:
+/register/car-puller
+Fields:
+- Full name
+- Email address
+- Phone number
+- Password
+- Confirm password
+Do NOT show:
+- Company name
+- Role
+- Tenant
+- Membership
+Use the same email/password/phone/confirmation validation conventions.
+Submit exactly:
+{
+  email,
+  password,
+  fullName,
+  phone
+}
+to registerCarPuller().
+9. CAR-PULLER SUCCESS BEHAVIOR
+A newly registered car puller is valid with:
+memberships = []
+selectedMembership = null
+Do not treat zero memberships as registration failure.
+Do not invent a transporter/company.
+Do not invent a car_puller membership.
+Membership will be created later through invitation/joining.
+Install session when provided.
+Until the car-puller task/dashboard experience is implemented:
+redirect authenticated success to:
+/
+If email confirmation is required:
+show confirmation guidance instead.
+10. LOGIN PAGE MIGRATION
+Change the frontend login flow to call:
+POST /auth/login/multi-tenant
+through loginMultiTenant().
+Stop using the legacy login endpoint from the active login UI.
+Do not remove backend legacy endpoint compatibility in this task.
+11. LOGIN WITH ZERO MEMBERSHIPS
+Zero active memberships is valid.
+Example:
+new independent car puller.
+Behavior:
+- install Supabase session
+- retain profile
+- memberships = []
+- selectedMembership = null
+- allow successful authentication
+Until zero-membership onboarding/dashboard exists:
+redirect to /.
+Do not display "account not configured" merely because memberships are empty.
+12. LOGIN WITH EXACTLY ONE MEMBERSHIP
+When backend returns exactly one active membership and selectedMembership is
+that membership:
+- retain the membership
+- retain selectedMembership
+- redirect to /
+Do not independently recalculate selection if the backend response is valid.
+13. LOGIN WITH MULTIPLE MEMBERSHIPS
+When more than one active membership is returned and:
+selectedMembership = null
+do NOT arbitrarily choose the first membership.
+Do NOT silently choose a tenant by:
+- array order
+- role
+- company name
+- previous tenant
+- JWT content
+Instead, display a tenant/company selection UI after successful login.
+The selection UI may remain within the login flow for this task rather than
+introducing a separate route.
+Display each membership using at least:
+- tenantName
+- role
+When the user selects one:
+- choose that exact returned MembershipSummary as the active client context
+- do not alter the Supabase token
+- do not send a server authorization request merely to select it in this task
+- redirect to / after selection
+The selected tenant will later be supplied as X-IAMONIT-Tenant-Id to
+tenant-scoped API calls, where the backend will revalidate membership.
+14. SAFE MEMBERSHIP SELECTION
+A selected membership must exist in the memberships returned by the backend.
+Do not allow arbitrary tenantId text entry.
+Do not allow arbitrary role selection.
+Do not construct a fake membership object from user input.
+15. ERROR HANDLING
+Continue displaying safe user-facing errors.
+Do not display:
+- Supabase internals
+- raw PostgreSQL errors
+- JWTs
+- access tokens
+- refresh tokens
+- stack traces
+Preserve duplicate-email and authentication error behavior.
+Duplicate transporter company display name must not be treated as a frontend
+validation conflict.
+16. DOUBLE SUBMISSION
+Preserve existing loading/double-submit protection on:
+- transporter registration
+- car-puller registration
+- login
+17. LEGACY FRONTEND AUTH COMPATIBILITY
+The active UI should now use the new multi-tenant APIs.
+Legacy frontend helpers/types may remain only if required temporarily by
+unrelated code, but must not drive the active login/register pages.
+Do not modify backend legacy routes.
+18. TESTS — API CLIENT
+Cover:
+- transporter endpoint/path
+- exact transporter payload
+- car-puller endpoint/path
+- exact car-puller payload
+- multi-tenant login endpoint/path
+- exact login payload
+- valid multi-tenant response
+- malformed profile rejected
+- malformed membership rejected
+- malformed selectedMembership rejected
+- session-null confirmation response accepted
+19. TESTS — REGISTER LANDING
+Cover:
+- displays Sign Up as a Transporter
+- displays Sign Up as a Car Puller
+- transporter navigation target
+- car-puller navigation target
+- no registration API call from account-type selection page
+20. TESTS — TRANSPORTER REGISTRATION
+Cover:
+- company name exists
+- no role selector
+- phone format validation
+- confirm password client-only
+- exact backend payload
+- calls registerTransporter()
+- double-submit prevention
+- confirmation-required guidance
+- session installation
+- successful redirect
+21. TESTS — CAR-PULLER REGISTRATION
+Cover:
+- company name absent
+- role selector absent
+- exact backend payload
+- calls registerCarPuller()
+- zero memberships accepted
+- selectedMembership null accepted
+- confirmation behavior
+- session installation
+- successful redirect
+22. TESTS — LOGIN
+Cover:
+- calls loginMultiTenant()
+- session installation
+- zero memberships succeeds
+- one membership succeeds
+- one selected membership retained
+- multiple memberships do not auto-select first membership
+- membership chooser is displayed for multiple memberships
+- chooser displays tenant name and role
+- selecting a returned membership stores that exact membership
+- arbitrary/fake membership cannot be selected
+- successful selection redirects
+- loading/double-submit behavior preserved
+- safe errors preserved
+23. SECURITY
+Do not:
+- persist accessToken manually
+- persist refreshToken manually
+- trust tenant/role as authorization
+- create JWT claims
+- accept arbitrary membership/tenant selection
+- send X-IAMONIT-Tenant-Id to login/register endpoints
+- expose secret values
+24. OUT OF SCOPE
+Do NOT:
+- modify backend files
+- modify database schema
+- modify migrations
+- modify RLS
+- implement transporter dashboard
+- implement car-puller dashboard
+- implement work orders
+- implement invitations
+- implement tenant switcher in application navigation
+- implement existing-user create-new-transporter flow
+- implement protected-route framework
+- implement logout changes unless compilation requires compatibility
+- install unrelated dependencies
+- modify environment files
+- access hosted Supabase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- /register presents Transporter and Car Puller signup choices.
+- /register/transporter exists.
+- /register/car-puller exists.
+- Transporter form includes companyName.
+- Car Puller form excludes companyName.
+- Neither form includes a role selector.
+- Transporter form calls /auth/register/transporter.
+- Car Puller form calls /auth/register/car-puller.
+- Login uses /auth/login/multi-tenant.
+- Frontend understands profile + memberships + selectedMembership.
+- Zero-membership login succeeds.
+- Exactly one membership can remain selected from backend response.
+- Multiple memberships are not arbitrarily auto-selected.
+- Multiple memberships produce explicit company-selection UI.
+- Membership choice comes only from server-returned memberships.
+- Supabase session installation continues working.
+- Email-confirmation behavior continues working.
+- Existing safe error behavior continues working.
+- Phone E.164-compatible validation remains.
+- Double-submit prevention remains.
+- Frontend tests pass.
+- Frontend TypeScript check passes.
+- Frontend lint passes.
+- Frontend production build passes.
+- Task-agent tests pass.
+- No backend files change.
 - No migration/RLS changes.
 - No hosted operation occurs.</t>
   </si>
@@ -5763,22 +6160,22 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>931</v>
+        <v>937</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>932</v>
+        <v>938</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>933</v>
+        <v>939</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>934</v>
+        <v>940</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -5786,76 +6183,76 @@
         <v>619</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>935</v>
+        <v>941</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>939</v>
+        <v>945</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>941</v>
+        <v>947</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>944</v>
+        <v>950</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>120</v>
@@ -5863,79 +6260,79 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>968</v>
+        <v>974</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>969</v>
+        <v>975</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>970</v>
+        <v>976</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>273</v>
@@ -5943,59 +6340,59 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>971</v>
+        <v>977</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>978</v>
+        <v>984</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>362</v>
@@ -6027,25 +6424,25 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>987</v>
+        <v>993</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>988</v>
+        <v>994</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>989</v>
+        <v>995</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>22</v>
@@ -6053,25 +6450,25 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>991</v>
+        <v>997</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>992</v>
+        <v>998</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>993</v>
+        <v>999</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>995</v>
+        <v>1001</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>25</v>
@@ -6079,25 +6476,25 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>997</v>
+        <v>1003</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>998</v>
+        <v>1004</v>
       </c>
       <c r="C3" s="14" t="s">
+        <v>1005</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>999</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>993</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>1000</v>
+        <v>1006</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>25</v>
@@ -6105,22 +6502,22 @@
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1002</v>
+        <v>1008</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>332</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1003</v>
+        <v>1009</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1005</v>
+        <v>1011</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>1006</v>
+        <v>1012</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>331</v>
@@ -6131,22 +6528,22 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1007</v>
+        <v>1013</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1008</v>
+        <v>1014</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1009</v>
+        <v>1015</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1011</v>
+        <v>1017</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>1012</v>
+        <v>1018</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>338</v>
@@ -6157,25 +6554,25 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1013</v>
+        <v>1019</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1014</v>
+        <v>1020</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1015</v>
+        <v>1021</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1016</v>
+        <v>1022</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>25</v>
@@ -6183,25 +6580,25 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1017</v>
+        <v>1023</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1018</v>
+        <v>1024</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1019</v>
+        <v>1025</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1020</v>
+        <v>1026</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>1021</v>
+        <v>1027</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1022</v>
+        <v>1028</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>25</v>
@@ -6209,25 +6606,25 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1023</v>
+        <v>1029</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1024</v>
+        <v>1030</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1025</v>
+        <v>1031</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1026</v>
+        <v>1032</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1027</v>
+        <v>1033</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1028</v>
+        <v>1034</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1029</v>
+        <v>1035</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>25</v>
@@ -6235,22 +6632,22 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1030</v>
+        <v>1036</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1031</v>
+        <v>1037</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1032</v>
+        <v>1038</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>1033</v>
+        <v>1039</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1034</v>
+        <v>1040</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>302</v>
@@ -6261,22 +6658,22 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1035</v>
+        <v>1041</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1036</v>
+        <v>1042</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1037</v>
+        <v>1043</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1038</v>
+        <v>1044</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>181</v>
@@ -6287,22 +6684,22 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1039</v>
+        <v>1045</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1040</v>
+        <v>1046</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1041</v>
+        <v>1047</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>1042</v>
+        <v>1048</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>1043</v>
+        <v>1049</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>194</v>
@@ -6313,22 +6710,22 @@
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1044</v>
+        <v>1050</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1045</v>
+        <v>1051</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1046</v>
+        <v>1052</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>993</v>
+        <v>999</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>1047</v>
+        <v>1053</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>1048</v>
+        <v>1054</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>325</v>
@@ -6388,19 +6785,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1049</v>
+        <v>1055</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1050</v>
+        <v>1056</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1051</v>
+        <v>1057</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1052</v>
+        <v>1058</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>1053</v>
+        <v>1059</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>500</v>
@@ -6411,163 +6808,163 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1054</v>
+        <v>1060</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1057</v>
+        <v>1063</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>130</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1059</v>
+        <v>1065</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1060</v>
+        <v>1066</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>1061</v>
+        <v>1067</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>67</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1062</v>
+        <v>1068</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1063</v>
+        <v>1069</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>183</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1064</v>
+        <v>1070</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1065</v>
+        <v>1071</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1055</v>
+        <v>1061</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1066</v>
+        <v>1072</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1067</v>
+        <v>1073</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>433</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>1058</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1068</v>
+        <v>1074</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1070</v>
+        <v>1076</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1071</v>
+        <v>1077</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1072</v>
+        <v>1078</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>1073</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1074</v>
+        <v>1080</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1075</v>
+        <v>1081</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1076</v>
+        <v>1082</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1073</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1077</v>
+        <v>1083</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1069</v>
+        <v>1075</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1078</v>
+        <v>1084</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="14" t="s">
+        <v>1085</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>1078</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>1079</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>1072</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>1073</v>
       </c>
     </row>
   </sheetData>
@@ -6595,13 +6992,13 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1080</v>
+        <v>1086</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1081</v>
+        <v>1087</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>500</v>
@@ -6610,7 +7007,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1082</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6618,10 +7015,10 @@
         <v>130</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1083</v>
+        <v>1089</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>130</v>
@@ -6636,10 +7033,10 @@
         <v>94</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1085</v>
+        <v>1091</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>67</v>
@@ -6654,10 +7051,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1086</v>
+        <v>1092</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>199</v>
@@ -6669,13 +7066,13 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1087</v>
+        <v>1093</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1088</v>
+        <v>1094</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>61</v>
@@ -6687,13 +7084,13 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1089</v>
+        <v>1095</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>1090</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1084</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>199</v>
@@ -6708,10 +7105,10 @@
         <v>309</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1091</v>
+        <v>1097</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1092</v>
+        <v>1098</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>199</v>
@@ -6726,10 +7123,10 @@
         <v>374</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1093</v>
+        <v>1099</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>378</v>
@@ -6744,10 +7141,10 @@
         <v>400</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1094</v>
+        <v>1100</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>55</v>
@@ -6762,10 +7159,10 @@
         <v>400</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1095</v>
+        <v>1101</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>55</v>
@@ -6777,13 +7174,13 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1096</v>
+        <v>1102</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1097</v>
+        <v>1103</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1092</v>
+        <v>1098</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>433</v>
@@ -20008,7 +20405,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -20601,12 +20998,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" ht="409.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="14" t="s">
         <v>665</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>666</v>
@@ -20621,7 +21018,7 @@
         <v>669</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="H21" s="14" t="s">
         <v>670</v>
@@ -20638,36 +21035,36 @@
         <v>67</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="G22" s="14" t="s">
         <v>175</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="I22" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="14" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B23" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="D23" s="14" t="s">
         <v>678</v>
@@ -20679,39 +21076,39 @@
         <v>680</v>
       </c>
       <c r="G23" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H23" s="14" t="s">
         <v>681</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>682</v>
       </c>
       <c r="I23" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>174</v>
+        <v>684</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="I24" s="14" t="s">
         <v>25</v>
@@ -20719,16 +21116,16 @@
     </row>
     <row r="25" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="14" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="B25" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>689</v>
+        <v>174</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>690</v>
@@ -20737,7 +21134,7 @@
         <v>691</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>213</v>
+        <v>687</v>
       </c>
       <c r="H25" s="14" t="s">
         <v>692</v>
@@ -20746,7 +21143,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>693</v>
       </c>
@@ -20754,19 +21151,19 @@
         <v>67</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>697</v>
+        <v>213</v>
       </c>
       <c r="H26" s="14" t="s">
         <v>698</v>
@@ -20783,22 +21180,22 @@
         <v>67</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>234</v>
+        <v>700</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="I27" s="14" t="s">
         <v>25</v>
@@ -20806,45 +21203,45 @@
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="G28" s="14" t="s">
-        <v>235</v>
+        <v>703</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="I28" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>708</v>
+        <v>694</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>709</v>
+        <v>240</v>
       </c>
       <c r="E29" s="14" t="s">
         <v>710</v>
@@ -20853,7 +21250,7 @@
         <v>711</v>
       </c>
       <c r="G29" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="H29" s="14" t="s">
         <v>712</v>
@@ -20870,36 +21267,36 @@
         <v>67</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="G30" s="14" t="s">
         <v>266</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="I30" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="31" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="D31" s="14" t="s">
         <v>720</v>
@@ -20911,7 +21308,7 @@
         <v>722</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="H31" s="14" t="s">
         <v>723</v>
@@ -20931,56 +21328,56 @@
         <v>725</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>319</v>
+        <v>726</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="G32" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="H32" s="14" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="I32" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="33" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>571</v>
+        <v>731</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>730</v>
+        <v>319</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="G33" s="14" t="s">
-        <v>99</v>
+        <v>314</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>61</v>
@@ -20989,33 +21386,33 @@
         <v>571</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="G34" s="14" t="s">
         <v>99</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>740</v>
+        <v>571</v>
       </c>
       <c r="D35" s="14" t="s">
         <v>741</v>
@@ -21027,13 +21424,13 @@
         <v>743</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>188</v>
+        <v>99</v>
       </c>
       <c r="H35" s="14" t="s">
         <v>744</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -21044,19 +21441,19 @@
         <v>61</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="F36" s="14" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>749</v>
+        <v>188</v>
       </c>
       <c r="H36" s="14" t="s">
         <v>750</v>
@@ -21073,22 +21470,22 @@
         <v>61</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>688</v>
+        <v>746</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>752</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>243</v>
+        <v>753</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="G37" s="14" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>25</v>
@@ -21096,28 +21493,28 @@
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="B38" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="F38" s="14" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="G38" s="14" t="s">
-        <v>248</v>
+        <v>760</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="I38" s="14" t="s">
         <v>25</v>
@@ -21125,28 +21522,28 @@
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="G39" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>25</v>
@@ -21154,28 +21551,28 @@
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D40" s="14" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>766</v>
+        <v>255</v>
       </c>
       <c r="F40" s="14" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>296</v>
+        <v>254</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="I40" s="14" t="s">
         <v>25</v>
@@ -21183,28 +21580,28 @@
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>708</v>
+        <v>694</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>283</v>
+        <v>771</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="I41" s="14" t="s">
         <v>25</v>
@@ -21212,74 +21609,74 @@
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>774</v>
+        <v>714</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>302</v>
+        <v>278</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="I42" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="43" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>725</v>
+        <v>780</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="H43" s="14" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="I43" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="44" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>783</v>
+        <v>731</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>784</v>
+        <v>330</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>785</v>
@@ -21288,16 +21685,16 @@
         <v>786</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="H44" s="14" t="s">
         <v>787</v>
       </c>
       <c r="I44" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="45" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="45" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
         <v>788</v>
       </c>
@@ -21305,51 +21702,51 @@
         <v>86</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>207</v>
+        <v>790</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="H45" s="14" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="I45" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="H46" s="14" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="I46" s="14" t="s">
         <v>25</v>
@@ -21357,28 +21754,28 @@
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>797</v>
+        <v>132</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="G47" s="14" t="s">
-        <v>260</v>
+        <v>125</v>
       </c>
       <c r="H47" s="14" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="I47" s="14" t="s">
         <v>25</v>
@@ -21386,13 +21783,13 @@
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>802</v>
+        <v>789</v>
       </c>
       <c r="D48" s="14" t="s">
         <v>803</v>
@@ -21404,7 +21801,7 @@
         <v>805</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="H48" s="14" t="s">
         <v>806</v>
@@ -21424,123 +21821,123 @@
         <v>808</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>398</v>
+        <v>809</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="50" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>813</v>
+        <v>378</v>
       </c>
       <c r="C50" s="14" t="s">
         <v>814</v>
       </c>
       <c r="D50" s="14" t="s">
+        <v>398</v>
+      </c>
+      <c r="E50" s="14" t="s">
         <v>815</v>
       </c>
-      <c r="E50" s="14" t="s">
+      <c r="F50" s="14" t="s">
         <v>816</v>
       </c>
-      <c r="F50" s="14" t="s">
+      <c r="G50" s="14" t="s">
+        <v>393</v>
+      </c>
+      <c r="H50" s="14" t="s">
         <v>817</v>
       </c>
-      <c r="G50" s="14" t="s">
+      <c r="I50" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="51" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51" s="14" t="s">
+        <v>818</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>819</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>820</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>821</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>822</v>
+      </c>
+      <c r="F51" s="14" t="s">
+        <v>823</v>
+      </c>
+      <c r="G51" s="14" t="s">
         <v>471</v>
       </c>
-      <c r="H50" s="14" t="s">
-        <v>818</v>
-      </c>
-      <c r="I50" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="51" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="14" t="s">
-        <v>819</v>
-      </c>
-      <c r="B51" s="14" t="s">
-        <v>813</v>
-      </c>
-      <c r="C51" s="14" t="s">
-        <v>814</v>
-      </c>
-      <c r="D51" s="14" t="s">
-        <v>820</v>
-      </c>
-      <c r="E51" s="14" t="s">
-        <v>821</v>
-      </c>
-      <c r="F51" s="14" t="s">
-        <v>822</v>
-      </c>
-      <c r="G51" s="14" t="s">
-        <v>480</v>
-      </c>
       <c r="H51" s="14" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="I51" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="52" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>813</v>
+        <v>819</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>491</v>
+        <v>826</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="F52" s="14" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>486</v>
+        <v>480</v>
       </c>
       <c r="H52" s="14" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="I52" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="53" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>61</v>
+        <v>819</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>829</v>
+        <v>820</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>830</v>
+        <v>491</v>
       </c>
       <c r="E53" s="14" t="s">
         <v>831</v>
@@ -21549,7 +21946,7 @@
         <v>832</v>
       </c>
       <c r="G53" s="14" t="s">
-        <v>57</v>
+        <v>486</v>
       </c>
       <c r="H53" s="14" t="s">
         <v>833</v>
@@ -21558,96 +21955,125 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="14" t="s">
         <v>834</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="C54" s="14" t="s">
         <v>835</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>87</v>
+        <v>836</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="I54" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="55" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>783</v>
+        <v>841</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>840</v>
+        <v>87</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H55" s="14" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="I55" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="56" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="B56" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="F56" s="14" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="G56" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="H56" s="14" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="I56" s="14" t="s">
         <v>13</v>
       </c>
     </row>
+    <row r="57" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="14" t="s">
+        <v>850</v>
+      </c>
+      <c r="B57" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C57" s="14" t="s">
+        <v>789</v>
+      </c>
+      <c r="D57" s="14" t="s">
+        <v>851</v>
+      </c>
+      <c r="E57" s="14" t="s">
+        <v>852</v>
+      </c>
+      <c r="F57" s="14" t="s">
+        <v>853</v>
+      </c>
+      <c r="G57" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H57" s="14" t="s">
+        <v>854</v>
+      </c>
+      <c r="I57" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I56"/>
-  <conditionalFormatting sqref="I2:I56">
+  <autoFilter ref="A1:I57"/>
+  <conditionalFormatting sqref="I2:I57">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -21682,7 +22108,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -21694,19 +22120,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -21998,9 +22424,9 @@
         <v>661</v>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" ht="90" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B19" s="14" t="s">
         <v>667</v>
@@ -22009,7 +22435,7 @@
         <v>668</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>175</v>
+        <v>493</v>
       </c>
       <c r="E19" s="14" t="s">
         <v>665</v>
@@ -22020,10 +22446,10 @@
         <v>67</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="D20" s="14" t="s">
         <v>175</v>
@@ -22043,10 +22469,10 @@
         <v>679</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>681</v>
+        <v>175</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22054,16 +22480,16 @@
         <v>67</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>174</v>
+        <v>684</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22071,16 +22497,16 @@
         <v>67</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>689</v>
+        <v>174</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>690</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>213</v>
+        <v>687</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22088,13 +22514,13 @@
         <v>67</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>697</v>
+        <v>213</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>693</v>
@@ -22105,13 +22531,13 @@
         <v>67</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>234</v>
+        <v>700</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="E25" s="14" t="s">
         <v>699</v>
@@ -22122,16 +22548,16 @@
         <v>67</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>235</v>
+        <v>703</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22139,16 +22565,16 @@
         <v>67</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>709</v>
+        <v>240</v>
       </c>
       <c r="C27" s="14" t="s">
         <v>710</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>266</v>
+        <v>235</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22156,10 +22582,10 @@
         <v>67</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="D28" s="14" t="s">
         <v>266</v>
@@ -22179,10 +22605,10 @@
         <v>721</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>291</v>
+        <v>266</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22190,13 +22616,13 @@
         <v>67</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>319</v>
+        <v>726</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="E30" s="14" t="s">
         <v>724</v>
@@ -22204,19 +22630,19 @@
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B31" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>732</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="E31" s="14" t="s">
         <v>730</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>731</v>
-      </c>
-      <c r="D31" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22224,16 +22650,16 @@
         <v>61</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="D32" s="14" t="s">
         <v>99</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22241,16 +22667,16 @@
         <v>61</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>626</v>
+        <v>741</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>627</v>
+        <v>742</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>624</v>
+        <v>740</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22258,16 +22684,16 @@
         <v>61</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="D34" s="14" t="s">
         <v>145</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22275,16 +22701,16 @@
         <v>61</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>741</v>
+        <v>631</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>742</v>
+        <v>632</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>188</v>
+        <v>145</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>739</v>
+        <v>630</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22292,13 +22718,13 @@
         <v>61</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>749</v>
+        <v>188</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>745</v>
@@ -22312,10 +22738,10 @@
         <v>752</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>243</v>
+        <v>753</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>751</v>
@@ -22326,16 +22752,16 @@
         <v>61</v>
       </c>
       <c r="B38" s="14" t="s">
+        <v>758</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>760</v>
+      </c>
+      <c r="E38" s="14" t="s">
         <v>757</v>
-      </c>
-      <c r="C38" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>248</v>
-      </c>
-      <c r="E38" s="14" t="s">
-        <v>756</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22343,16 +22769,16 @@
         <v>61</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22360,16 +22786,16 @@
         <v>61</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="C40" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E40" s="14" t="s">
         <v>766</v>
-      </c>
-      <c r="D40" s="14" t="s">
-        <v>296</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22377,16 +22803,16 @@
         <v>61</v>
       </c>
       <c r="B41" s="14" t="s">
-        <v>283</v>
+        <v>771</v>
       </c>
       <c r="C41" s="14" t="s">
+        <v>772</v>
+      </c>
+      <c r="D41" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="E41" s="14" t="s">
         <v>770</v>
-      </c>
-      <c r="D41" s="14" t="s">
-        <v>278</v>
-      </c>
-      <c r="E41" s="14" t="s">
-        <v>769</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22394,16 +22820,16 @@
         <v>61</v>
       </c>
       <c r="B42" s="14" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
       <c r="C42" s="14" t="s">
+        <v>776</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="E42" s="14" t="s">
         <v>775</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>302</v>
-      </c>
-      <c r="E42" s="14" t="s">
-        <v>773</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22411,33 +22837,33 @@
         <v>61</v>
       </c>
       <c r="B43" s="14" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="C43" s="14" t="s">
+        <v>781</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="E43" s="14" t="s">
         <v>779</v>
-      </c>
-      <c r="D43" s="14" t="s">
-        <v>325</v>
-      </c>
-      <c r="E43" s="14" t="s">
-        <v>778</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>784</v>
+        <v>330</v>
       </c>
       <c r="C44" s="14" t="s">
         <v>785</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>104</v>
+        <v>325</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22445,13 +22871,13 @@
         <v>86</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>207</v>
+        <v>790</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>202</v>
+        <v>104</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>788</v>
@@ -22462,16 +22888,16 @@
         <v>86</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>132</v>
+        <v>207</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>125</v>
+        <v>202</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22479,21 +22905,21 @@
         <v>86</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>797</v>
+        <v>132</v>
       </c>
       <c r="C47" s="14" t="s">
+        <v>799</v>
+      </c>
+      <c r="D47" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E47" s="14" t="s">
         <v>798</v>
-      </c>
-      <c r="D47" s="14" t="s">
-        <v>260</v>
-      </c>
-      <c r="E47" s="14" t="s">
-        <v>796</v>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="14" t="s">
-        <v>378</v>
+        <v>86</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>803</v>
@@ -22502,10 +22928,10 @@
         <v>804</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>381</v>
+        <v>260</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22513,13 +22939,13 @@
         <v>378</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>398</v>
+        <v>809</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E49" s="14" t="s">
         <v>807</v>
@@ -22527,19 +22953,19 @@
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>86</v>
+        <v>378</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>87</v>
+        <v>398</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>836</v>
+        <v>815</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>81</v>
+        <v>393</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>834</v>
+        <v>813</v>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22547,16 +22973,16 @@
         <v>86</v>
       </c>
       <c r="B51" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>842</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="E51" s="14" t="s">
         <v>840</v>
-      </c>
-      <c r="C51" s="14" t="s">
-        <v>841</v>
-      </c>
-      <c r="D51" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="E51" s="14" t="s">
-        <v>839</v>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -22564,20 +22990,37 @@
         <v>86</v>
       </c>
       <c r="B52" s="14" t="s">
+        <v>846</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>847</v>
+      </c>
+      <c r="D52" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="E52" s="14" t="s">
         <v>845</v>
       </c>
-      <c r="C52" s="14" t="s">
-        <v>846</v>
-      </c>
-      <c r="D52" s="14" t="s">
+    </row>
+    <row r="53" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>851</v>
+      </c>
+      <c r="C53" s="14" t="s">
+        <v>852</v>
+      </c>
+      <c r="D53" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="E52" s="14" t="s">
-        <v>844</v>
+      <c r="E53" s="14" t="s">
+        <v>850</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E52"/>
+  <autoFilter ref="A1:E53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -22602,114 +23045,114 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>866</v>
+        <v>872</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>867</v>
+        <v>873</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>868</v>
+        <v>874</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>876</v>
+        <v>882</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>879</v>
+        <v>885</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>881</v>
+        <v>887</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>164</v>
@@ -22717,22 +23160,22 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>882</v>
+        <v>888</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>883</v>
+        <v>889</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>885</v>
+        <v>891</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>886</v>
+        <v>892</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>170</v>
@@ -22740,186 +23183,186 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>888</v>
+        <v>894</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>889</v>
+        <v>895</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>891</v>
+        <v>897</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>893</v>
+        <v>899</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>896</v>
+        <v>902</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>897</v>
+        <v>903</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>898</v>
+        <v>904</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>899</v>
+        <v>905</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>900</v>
+        <v>906</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>901</v>
+        <v>907</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>902</v>
+        <v>908</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>904</v>
+        <v>910</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>908</v>
+        <v>914</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>909</v>
+        <v>915</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>910</v>
+        <v>916</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>911</v>
+        <v>917</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>912</v>
+        <v>918</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>914</v>
+        <v>920</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>915</v>
+        <v>921</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>916</v>
+        <v>922</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>917</v>
+        <v>923</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>900</v>
+        <v>906</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>919</v>
+        <v>925</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>921</v>
+        <v>927</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>922</v>
+        <v>928</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>923</v>
+        <v>929</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>926</v>
+        <v>932</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>904</v>
+        <v>910</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>927</v>
+        <v>933</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>929</v>
+        <v>935</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>930</v>
+        <v>936</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>926</v>
+        <v>932</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CODE-059 Define frontend auth rehydration
</commit_message>
<xml_diff>
--- a/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
+++ b/planning/IAMONIT_Full_Project_Control_Workbook.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3577" uniqueCount="1116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3591" uniqueCount="1121">
   <si>
     <t>IAMONIT Project Control Workbook</t>
   </si>
@@ -4381,6 +4381,323 @@
 - git diff --check passes.
 - No frontend changes occur.
 - No migration/RLS changes occur.</t>
+  </si>
+  <si>
+    <t>CODE-059</t>
+  </si>
+  <si>
+    <t>apps/web/app/layout.tsx; apps/web/components/auth/AuthBootstrap.tsx; apps/web/components/auth/AuthBootstrap.test.tsx; apps/web/lib/auth.types.ts; apps/web/lib/api.ts; apps/web/lib/api.test.ts; apps/web/lib/auth.ts; apps/web/lib/auth.test.ts</t>
+  </si>
+  <si>
+    <t>Rehydrate frontend multi-tenant authentication from verified session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. PURPOSE
+Implement frontend authentication rehydration after browser refresh.
+The browser-managed Supabase session remains the authentication credential.
+IAMONIT application state must be reconstructed from:
+Supabase browser session
+        |
+        | access token
+        v
+GET /auth/me
+        |
+        v
+verified backend profile + memberships
+        |
+        v
+frontend AuthState
+Do not reconstruct tenant or role information from Supabase JWT claims.
+Do not store a custom copy of access or refresh tokens.
+2. FRONTEND BOOTSTRAP RESPONSE TYPE
+Add a frontend type equivalent to:
+AuthBootstrapResponse
+containing exactly:
+profile
+memberships
+selectedMembership
+It must NOT contain:
+session
+accessToken
+refreshToken
+requiresEmailConfirmation
+Reuse existing:
+UserProfile
+MembershipSummary
+where practical.
+3. FRONTEND API CLIENT
+Add an API function equivalent to:
+getCurrentUser(accessToken)
+or:
+getAuthBootstrap(accessToken)
+It must call:
+GET /auth/me
+Use the configured NEXT_PUBLIC_API_URL through the existing API-client
+base-URL validation.
+Send the Supabase access token only through:
+Authorization: Bearer &lt;accessToken&gt;
+Do not send:
+- X-IAMONIT-Tenant-Id
+- tenantId query parameter
+- tenantId request body
+- role header
+- membership header
+GET /auth/me must have no request body.
+Do not log or expose the access token.
+4. RESPONSE VALIDATION
+Strictly validate the GET /auth/me JSON response.
+The response must contain exactly:
+profile
+memberships
+selectedMembership
+Validate:
+profile:
+- userId
+- email
+- fullName
+- phone
+membership:
+- membershipId
+- tenantId
+- tenantName
+- role
+- status
+selectedMembership:
+- may be null
+- when non-null, it must correspond to one of the returned memberships
+Do not accept extra session/token fields.
+Malformed responses must become the existing safe generic frontend API error.
+5. SESSION REHYDRATION
+Update apps/web/lib/auth.ts with a method equivalent to:
+rehydrateAuthSession()
+or:
+rehydrateAuthState()
+Use:
+getBrowserSupabaseClient().auth.getSession()
+The frontend must allow Supabase itself to restore/manage its browser session.
+Do not implement custom token refresh logic.
+If there is no Supabase session:
+- clear IAMONIT application auth state
+- do not call GET /auth/me
+- return an unauthenticated/null result normally
+If there is a Supabase session:
+- obtain its current access token
+- call GET /auth/me
+- reconstruct currentAuthState only from that verified backend response
+6. AUTH STATE
+The reconstructed AuthState must contain:
+profile
+memberships
+selectedMembership
+Do not populate role or tenant information from:
+- JWT claims
+- Supabase user metadata
+- localStorage role values
+- query parameters
+- URL values
+Membership and role information must come only from GET /auth/me.
+7. MEMBERSHIP SELECTION RULES
+Respect the backend bootstrap response.
+Zero memberships:
+selectedMembership = null
+Exactly one active membership:
+selectedMembership = that exact membership
+Multiple active memberships:
+selectedMembership = null unless a future explicitly verified tenant-selection
+mechanism selects one.
+Do not arbitrarily choose:
+memberships[0]
+for multiple memberships.
+8. FIX CURRENT MEMBERSHIP OBJECT-IDENTITY WEAKNESS
+The existing selectMembership implementation currently depends on JavaScript
+object identity.
+Remove that requirement.
+Selection should resolve the requested membership through its stable:
+membershipId
+against currentAuthState.memberships.
+The selected object stored in currentAuthState must be the canonical membership
+already contained in the current verified memberships array.
+Do not trust role, tenantName, tenantId, or status from an arbitrary caller
+object.
+A membershipId not present in currentAuthState.memberships must be rejected.
+Keep the existing login page behavior compatible without modifying the login
+page in CODE-059.
+9. AUTH BOOTSTRAP COMPONENT
+Create:
+apps/web/components/auth/AuthBootstrap.tsx
+It must be a client component.
+Its responsibility is only to initialize/reconstruct frontend auth state from
+the Supabase browser session when the application starts.
+It should call the auth rehydration function once during initial application
+bootstrap.
+It must not:
+- perform role authorization
+- choose an arbitrary tenant
+- decode JWT tenant/role claims
+- call protected business endpoints
+- redirect users based on role
+- implement sidebar navigation
+- implement logout
+- implement tenant switching UI
+It must handle the absence of a Supabase session normally.
+Bootstrap failures must not cause an unhandled promise rejection or expose
+token/provider/database details.
+10. ROOT LAYOUT
+Integrate AuthBootstrap into:
+apps/web/app/layout.tsx
+so frontend auth reconstruction occurs after a full browser reload.
+Do not convert authentication responsibility to server-side cookie parsing.
+Do not add custom middleware.
+Do not add protected-route middleware in CODE-059.
+11. EXISTING LOGIN / REGISTRATION
+Do not modify:
+apps/web/app/(auth)/login/page.tsx
+apps/web/app/(auth)/register/page.tsx
+apps/web/app/(auth)/register/transporter/page.tsx
+apps/web/app/(auth)/register/car-puller/page.tsx
+Existing behavior must remain compatible.
+After normal login/register with a returned session:
+establishAuthSession()
+must continue setting:
+profile
+memberships
+selectedMembership
+using the backend response.
+CODE-059 supplements this with browser-refresh reconstruction.
+12. API TESTS
+Cover at minimum:
+- GET /auth/me uses HTTP GET
+- correct configured API base URL is used
+- Authorization header contains the provided access token
+- exactly one Bearer Authorization header is sent
+- no tenant header is sent
+- no role header is sent
+- GET request has no request body
+- valid bootstrap response is accepted
+- zero memberships is accepted
+- one selected membership is accepted
+- multiple memberships with selectedMembership=null is accepted
+- selectedMembership not contained in memberships is rejected
+- malformed profile is rejected
+- malformed membership is rejected
+- unexpected session/token fields are rejected
+- non-JSON response becomes safe generic error
+- network failure becomes safe generic error
+- sensitive access token is never included in thrown error text
+13. AUTH STATE TESTS
+Cover at minimum:
+- no Supabase session returns null/unauthenticated state
+- no-session path does not call GET /auth/me
+- existing application auth state is cleared when no session exists
+- Supabase session access token is passed to GET /auth/me
+- bootstrap profile becomes current profile
+- bootstrap memberships become current memberships
+- zero memberships preserves selectedMembership=null
+- exactly one backend-selected membership is preserved
+- multiple memberships with null selection remain unselected
+- role is taken from backend membership data
+- tenant information is taken from backend membership data
+- bootstrap failure clears unsafe/stale application auth state
+- bootstrap failure does not expose token values
+- no JWT payload decoding is used
+- no custom refresh token handling is introduced
+14. MEMBERSHIP SELECTION TESTS
+Cover:
+- selection succeeds for a verified membership
+- selection is resolved by membershipId rather than object identity
+- a different object instance with the same membershipId resolves to the
+  canonical current membership
+- forged role/tenant/status fields on the caller object are not persisted
+- unknown membershipId is rejected
+- no auth state returns false
+15. AUTH BOOTSTRAP COMPONENT TESTS
+Cover at minimum:
+- bootstrap calls rehydration during initial mount
+- it runs only once for one mount
+- no-session completion is handled normally
+- successful rehydration completes normally
+- rejected bootstrap does not create an unhandled rejection
+- child/application rendering behavior remains deterministic
+- component does not perform redirects
+- component does not choose tenants
+16. SECURITY BOUNDARY
+The resulting refresh flow must be:
+Browser Supabase session
+        |
+        | current access token
+        v
+GET /auth/me
+        |
+        | AuthGuard / verifyIdentity
+        v
+Backend verified identity
+        |
+        v
+user_profiles
+tenant_memberships
+tenants
+        |
+        v
+AuthBootstrapResponse
+        |
+        v
+Frontend AuthState
+Never:
+Browser storage/JWT role
+        -&gt;
+trusted role/tenant
+17. OUT OF SCOPE
+Do NOT:
+- modify backend files
+- modify GET /auth/me
+- modify login/register pages
+- implement GET /users
+- implement sidebar
+- modify CODE-026
+- implement dashboard
+- add protected-route middleware
+- implement tenant switcher UI
+- implement logout UI
+- remove legacy backend authentication
+- remove app_users
+- change authentication endpoints
+- modify database migrations
+- modify RLS
+- modify Supabase configuration
+- modify environment files
+- access hosted Supabase
+- install unrelated dependencies
+- store custom copies of access/refresh tokens
+- commit or push</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Frontend AuthBootstrapResponse type exists.
+- Frontend API client supports GET /auth/me.
+- GET /auth/me uses Bearer authentication.
+- No tenant header is sent to /auth/me.
+- No role/tenant value is derived from JWT claims.
+- Browser Supabase session is used as the credential source.
+- No custom token persistence is added.
+- No custom token refresh logic is added.
+- Browser refresh can reconstruct IAMONIT AuthState.
+- No session results in a clean unauthenticated state.
+- Profile comes from verified /auth/me response.
+- Memberships come from verified /auth/me response.
+- selectedMembership behavior preserves backend rules.
+- Multiple memberships are never arbitrarily auto-selected.
+- selectMembership no longer depends on object identity.
+- Membership selection uses canonical verified membership data.
+- Root application integrates the bootstrap component.
+- Existing login/register behavior remains compatible.
+- Frontend API tests pass.
+- Frontend auth tests pass.
+- AuthBootstrap component tests pass.
+- Frontend typecheck passes.
+- Frontend tests pass.
+- Frontend build passes locally.
+- Task-agent tests pass.
+- git diff --check passes.
+- No backend/migration/RLS changes occur.</t>
   </si>
   <si>
     <t>CODE-010</t>
@@ -6642,22 +6959,22 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>950</v>
+        <v>955</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>951</v>
+        <v>956</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>952</v>
+        <v>957</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -6665,76 +6982,76 @@
         <v>621</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>953</v>
+        <v>958</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>954</v>
+        <v>959</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>955</v>
+        <v>960</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>957</v>
+        <v>962</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>958</v>
+        <v>963</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>959</v>
+        <v>964</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>960</v>
+        <v>965</v>
       </c>
       <c r="D3" s="14" t="s">
+        <v>966</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>961</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>956</v>
-      </c>
       <c r="F3" s="14" t="s">
-        <v>962</v>
+        <v>967</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>963</v>
+        <v>968</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>964</v>
+        <v>969</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>965</v>
+        <v>970</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>966</v>
+        <v>971</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>967</v>
+        <v>972</v>
       </c>
     </row>
     <row r="5" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>968</v>
+        <v>973</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>969</v>
+        <v>974</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>970</v>
+        <v>975</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>966</v>
+        <v>971</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>120</v>
@@ -6742,79 +7059,79 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>971</v>
+        <v>976</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>972</v>
+        <v>977</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>973</v>
+        <v>978</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>974</v>
+        <v>979</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>975</v>
+        <v>980</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>976</v>
+        <v>981</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>977</v>
+        <v>982</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>978</v>
+        <v>983</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>979</v>
+        <v>984</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>980</v>
+        <v>985</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>981</v>
+        <v>986</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>982</v>
+        <v>987</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>983</v>
+        <v>988</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>984</v>
+        <v>989</v>
       </c>
     </row>
     <row r="9" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>985</v>
+        <v>990</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>986</v>
+        <v>991</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>987</v>
+        <v>992</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>988</v>
+        <v>993</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F9" s="14" t="s">
         <v>275</v>
@@ -6822,59 +7139,59 @@
     </row>
     <row r="10" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>990</v>
+        <v>995</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>992</v>
+        <v>997</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>956</v>
+        <v>961</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>993</v>
+        <v>998</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>999</v>
+        <v>1004</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1000</v>
+        <v>1005</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1001</v>
+        <v>1006</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>1002</v>
+        <v>1007</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>983</v>
+        <v>988</v>
       </c>
       <c r="F12" s="14" t="s">
         <v>364</v>
@@ -6906,25 +7223,25 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1003</v>
+        <v>1008</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1004</v>
+        <v>1009</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1005</v>
+        <v>1010</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1006</v>
+        <v>1011</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1007</v>
+        <v>1012</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
       <c r="H1" s="10" t="s">
         <v>22</v>
@@ -6932,25 +7249,25 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1009</v>
+        <v>1014</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1010</v>
+        <v>1015</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>1011</v>
+        <v>1016</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1012</v>
+        <v>1017</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>1013</v>
+        <v>1018</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>25</v>
@@ -6958,25 +7275,25 @@
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="B3" s="14" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>1016</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>1017</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>1011</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>1018</v>
+        <v>1023</v>
       </c>
       <c r="F3" s="14" t="s">
+        <v>1024</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>1019</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>1014</v>
       </c>
       <c r="H3" s="14" t="s">
         <v>25</v>
@@ -6984,22 +7301,22 @@
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1020</v>
+        <v>1025</v>
       </c>
       <c r="B4" s="14" t="s">
         <v>334</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1021</v>
+        <v>1026</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>1022</v>
+        <v>1027</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1023</v>
+        <v>1028</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>1024</v>
+        <v>1029</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>333</v>
@@ -7010,22 +7327,22 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1025</v>
+        <v>1030</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1026</v>
+        <v>1031</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1027</v>
+        <v>1032</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>1028</v>
+        <v>1033</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>340</v>
@@ -7036,25 +7353,25 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1031</v>
+        <v>1036</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1032</v>
+        <v>1037</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>1022</v>
+        <v>1027</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="H6" s="14" t="s">
         <v>25</v>
@@ -7062,25 +7379,25 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1037</v>
+        <v>1042</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>1022</v>
+        <v>1027</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>1039</v>
+        <v>1044</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="H7" s="14" t="s">
         <v>25</v>
@@ -7088,25 +7405,25 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1042</v>
+        <v>1047</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1044</v>
+        <v>1049</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1046</v>
+        <v>1051</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>25</v>
@@ -7114,22 +7431,22 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1050</v>
+        <v>1055</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>1028</v>
+        <v>1033</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>1051</v>
+        <v>1056</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="G9" s="14" t="s">
         <v>304</v>
@@ -7140,22 +7457,22 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1054</v>
+        <v>1059</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>1055</v>
+        <v>1060</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>1056</v>
+        <v>1061</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>182</v>
@@ -7166,22 +7483,22 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>1060</v>
+        <v>1065</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>1061</v>
+        <v>1066</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>196</v>
@@ -7192,22 +7509,22 @@
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>1062</v>
+        <v>1067</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>1063</v>
+        <v>1068</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>1011</v>
+        <v>1016</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>1065</v>
+        <v>1070</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>1066</v>
+        <v>1071</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>327</v>
@@ -7267,19 +7584,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>1067</v>
+        <v>1072</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1068</v>
+        <v>1073</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>1070</v>
+        <v>1075</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>1071</v>
+        <v>1076</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>502</v>
@@ -7290,163 +7607,163 @@
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>1072</v>
+        <v>1077</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1074</v>
+        <v>1079</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>1075</v>
+        <v>1080</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>130</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>1077</v>
+        <v>1082</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1078</v>
+        <v>1083</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>1079</v>
+        <v>1084</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>67</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>1080</v>
+        <v>1085</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1081</v>
+        <v>1086</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>184</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>1082</v>
+        <v>1087</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>435</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1083</v>
+        <v>1088</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1084</v>
+        <v>1089</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>1085</v>
+        <v>1090</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>435</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>1086</v>
+        <v>1091</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>1087</v>
+        <v>1092</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>1088</v>
+        <v>1093</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>1089</v>
+        <v>1094</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>1090</v>
+        <v>1095</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>1091</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>1092</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>1087</v>
-      </c>
       <c r="C7" s="14" t="s">
-        <v>1093</v>
+        <v>1098</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>1094</v>
+        <v>1099</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>86</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>1091</v>
+        <v>1096</v>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>1095</v>
+        <v>1100</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1087</v>
+        <v>1092</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1096</v>
+        <v>1101</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>1097</v>
+        <v>1102</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>1090</v>
+        <v>1095</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>1091</v>
+        <v>1096</v>
       </c>
     </row>
   </sheetData>
@@ -7474,13 +7791,13 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1098</v>
+        <v>1103</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>1099</v>
+        <v>1104</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>502</v>
@@ -7489,7 +7806,7 @@
         <v>22</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>1100</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -7497,10 +7814,10 @@
         <v>130</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1101</v>
+        <v>1106</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>130</v>
@@ -7515,10 +7832,10 @@
         <v>94</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>1103</v>
+        <v>1108</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>67</v>
@@ -7533,10 +7850,10 @@
         <v>19</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>1104</v>
+        <v>1109</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="D4" s="14" t="s">
         <v>201</v>
@@ -7548,13 +7865,13 @@
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>1105</v>
+        <v>1110</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>1106</v>
+        <v>1111</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="D5" s="14" t="s">
         <v>61</v>
@@ -7566,13 +7883,13 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>1107</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>1108</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>1102</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>201</v>
@@ -7587,10 +7904,10 @@
         <v>311</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>1109</v>
+        <v>1114</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>1110</v>
+        <v>1115</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>201</v>
@@ -7605,10 +7922,10 @@
         <v>376</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>1111</v>
+        <v>1116</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>380</v>
@@ -7623,10 +7940,10 @@
         <v>402</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>1112</v>
+        <v>1117</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="D9" s="14" t="s">
         <v>55</v>
@@ -7641,10 +7958,10 @@
         <v>402</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>1113</v>
+        <v>1118</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>1102</v>
+        <v>1107</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>55</v>
@@ -7656,13 +7973,13 @@
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>1114</v>
+        <v>1119</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>1115</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>1110</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>435</v>
@@ -20887,7 +21204,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -21567,15 +21884,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" ht="409.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="14" t="s">
         <v>684</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>674</v>
+        <v>668</v>
       </c>
       <c r="D24" s="14" t="s">
         <v>685</v>
@@ -21587,7 +21904,7 @@
         <v>687</v>
       </c>
       <c r="G24" s="14" t="s">
-        <v>175</v>
+        <v>495</v>
       </c>
       <c r="H24" s="14" t="s">
         <v>688</v>
@@ -21625,7 +21942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
         <v>694</v>
       </c>
@@ -21633,39 +21950,39 @@
         <v>67</v>
       </c>
       <c r="C26" s="14" t="s">
+        <v>674</v>
+      </c>
+      <c r="D26" s="14" t="s">
         <v>695</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="E26" s="14" t="s">
         <v>696</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="F26" s="14" t="s">
         <v>697</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="G26" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="H26" s="14" t="s">
         <v>698</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>699</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>700</v>
       </c>
       <c r="I26" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="B27" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>174</v>
+        <v>701</v>
       </c>
       <c r="E27" s="14" t="s">
         <v>702</v>
@@ -21674,10 +21991,10 @@
         <v>703</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="I27" s="14" t="s">
         <v>25</v>
@@ -21685,42 +22002,42 @@
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="D28" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="E28" s="14" t="s">
         <v>707</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="F28" s="14" t="s">
         <v>708</v>
       </c>
-      <c r="F28" s="14" t="s">
+      <c r="G28" s="14" t="s">
+        <v>704</v>
+      </c>
+      <c r="H28" s="14" t="s">
         <v>709</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="H28" s="14" t="s">
-        <v>710</v>
       </c>
       <c r="I28" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B29" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="D29" s="14" t="s">
         <v>712</v>
@@ -21732,10 +22049,10 @@
         <v>714</v>
       </c>
       <c r="G29" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="H29" s="14" t="s">
         <v>715</v>
-      </c>
-      <c r="H29" s="14" t="s">
-        <v>716</v>
       </c>
       <c r="I29" s="14" t="s">
         <v>25</v>
@@ -21743,16 +22060,16 @@
     </row>
     <row r="30" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B30" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>236</v>
+        <v>717</v>
       </c>
       <c r="E30" s="14" t="s">
         <v>718</v>
@@ -21761,10 +22078,10 @@
         <v>719</v>
       </c>
       <c r="G30" s="14" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="I30" s="14" t="s">
         <v>25</v>
@@ -21772,57 +22089,57 @@
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="B31" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="G31" s="14" t="s">
-        <v>237</v>
+        <v>720</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="I31" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="32" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>726</v>
+        <v>711</v>
       </c>
       <c r="D32" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="E32" s="14" t="s">
         <v>727</v>
       </c>
-      <c r="E32" s="14" t="s">
+      <c r="F32" s="14" t="s">
         <v>728</v>
       </c>
-      <c r="F32" s="14" t="s">
+      <c r="G32" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="H32" s="14" t="s">
         <v>729</v>
-      </c>
-      <c r="G32" s="14" t="s">
-        <v>268</v>
-      </c>
-      <c r="H32" s="14" t="s">
-        <v>730</v>
       </c>
       <c r="I32" s="14" t="s">
         <v>25</v>
@@ -21830,13 +22147,13 @@
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="D33" s="14" t="s">
         <v>732</v>
@@ -21857,7 +22174,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
         <v>736</v>
       </c>
@@ -21865,22 +22182,22 @@
         <v>67</v>
       </c>
       <c r="C34" s="14" t="s">
+        <v>731</v>
+      </c>
+      <c r="D34" s="14" t="s">
         <v>737</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="E34" s="14" t="s">
         <v>738</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="F34" s="14" t="s">
         <v>739</v>
       </c>
-      <c r="F34" s="14" t="s">
+      <c r="G34" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="H34" s="14" t="s">
         <v>740</v>
-      </c>
-      <c r="G34" s="14" t="s">
-        <v>293</v>
-      </c>
-      <c r="H34" s="14" t="s">
-        <v>741</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>25</v>
@@ -21888,16 +22205,16 @@
     </row>
     <row r="35" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>67</v>
       </c>
       <c r="C35" s="14" t="s">
+        <v>742</v>
+      </c>
+      <c r="D35" s="14" t="s">
         <v>743</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>321</v>
       </c>
       <c r="E35" s="14" t="s">
         <v>744</v>
@@ -21906,7 +22223,7 @@
         <v>745</v>
       </c>
       <c r="G35" s="14" t="s">
-        <v>316</v>
+        <v>293</v>
       </c>
       <c r="H35" s="14" t="s">
         <v>746</v>
@@ -21915,18 +22232,18 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>747</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>573</v>
+        <v>748</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>748</v>
+        <v>321</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>749</v>
@@ -21935,16 +22252,16 @@
         <v>750</v>
       </c>
       <c r="G36" s="14" t="s">
-        <v>99</v>
+        <v>316</v>
       </c>
       <c r="H36" s="14" t="s">
         <v>751</v>
       </c>
       <c r="I36" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" ht="112" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>752</v>
       </c>
@@ -21973,7 +22290,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" ht="160" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>757</v>
       </c>
@@ -21981,36 +22298,36 @@
         <v>61</v>
       </c>
       <c r="C38" s="14" t="s">
+        <v>573</v>
+      </c>
+      <c r="D38" s="14" t="s">
         <v>758</v>
       </c>
-      <c r="D38" s="14" t="s">
+      <c r="E38" s="14" t="s">
         <v>759</v>
       </c>
-      <c r="E38" s="14" t="s">
+      <c r="F38" s="14" t="s">
         <v>760</v>
       </c>
-      <c r="F38" s="14" t="s">
+      <c r="G38" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H38" s="14" t="s">
         <v>761</v>
       </c>
-      <c r="G38" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="H38" s="14" t="s">
-        <v>762</v>
-      </c>
       <c r="I38" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="D39" s="14" t="s">
         <v>764</v>
@@ -22022,10 +22339,10 @@
         <v>766</v>
       </c>
       <c r="G39" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="H39" s="14" t="s">
         <v>767</v>
-      </c>
-      <c r="H39" s="14" t="s">
-        <v>768</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>25</v>
@@ -22033,19 +22350,19 @@
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>706</v>
+        <v>763</v>
       </c>
       <c r="D40" s="14" t="s">
+        <v>769</v>
+      </c>
+      <c r="E40" s="14" t="s">
         <v>770</v>
-      </c>
-      <c r="E40" s="14" t="s">
-        <v>245</v>
       </c>
       <c r="F40" s="14" t="s">
         <v>771</v>
@@ -22068,22 +22385,22 @@
         <v>61</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="D41" s="14" t="s">
         <v>775</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="F41" s="14" t="s">
         <v>776</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>250</v>
+        <v>777</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="I41" s="14" t="s">
         <v>25</v>
@@ -22091,28 +22408,28 @@
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="14" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="G42" s="14" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="H42" s="14" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="I42" s="14" t="s">
         <v>25</v>
@@ -22120,25 +22437,25 @@
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>784</v>
+        <v>257</v>
       </c>
       <c r="F43" s="14" t="s">
         <v>785</v>
       </c>
       <c r="G43" s="14" t="s">
-        <v>298</v>
+        <v>256</v>
       </c>
       <c r="H43" s="14" t="s">
         <v>786</v>
@@ -22155,22 +22472,22 @@
         <v>61</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>726</v>
+        <v>711</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>285</v>
+        <v>788</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="F44" s="14" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="G44" s="14" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
       <c r="H44" s="14" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="I44" s="14" t="s">
         <v>25</v>
@@ -22178,16 +22495,16 @@
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>61</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>792</v>
+        <v>731</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>309</v>
+        <v>285</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>793</v>
@@ -22196,7 +22513,7 @@
         <v>794</v>
       </c>
       <c r="G45" s="14" t="s">
-        <v>304</v>
+        <v>280</v>
       </c>
       <c r="H45" s="14" t="s">
         <v>795</v>
@@ -22205,7 +22522,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="14" t="s">
         <v>796</v>
       </c>
@@ -22213,109 +22530,109 @@
         <v>61</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>743</v>
+        <v>797</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>332</v>
+        <v>309</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="G46" s="14" t="s">
-        <v>327</v>
+        <v>304</v>
       </c>
       <c r="H46" s="14" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="I46" s="14" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="47" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>801</v>
+        <v>748</v>
       </c>
       <c r="D47" s="14" t="s">
+        <v>332</v>
+      </c>
+      <c r="E47" s="14" t="s">
         <v>802</v>
       </c>
-      <c r="E47" s="14" t="s">
+      <c r="F47" s="14" t="s">
         <v>803</v>
       </c>
-      <c r="F47" s="14" t="s">
+      <c r="G47" s="14" t="s">
+        <v>327</v>
+      </c>
+      <c r="H47" s="14" t="s">
         <v>804</v>
       </c>
-      <c r="G47" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="H47" s="14" t="s">
+      <c r="I47" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A48" s="14" t="s">
         <v>805</v>
-      </c>
-      <c r="I47" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
-        <v>806</v>
       </c>
       <c r="B48" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>209</v>
+        <v>807</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="G48" s="14" t="s">
-        <v>204</v>
+        <v>104</v>
       </c>
       <c r="H48" s="14" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="I48" s="14" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>132</v>
+        <v>209</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="G49" s="14" t="s">
-        <v>125</v>
+        <v>204</v>
       </c>
       <c r="H49" s="14" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>25</v>
@@ -22323,16 +22640,16 @@
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="B50" s="14" t="s">
         <v>86</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>815</v>
+        <v>132</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>816</v>
@@ -22341,7 +22658,7 @@
         <v>817</v>
       </c>
       <c r="G50" s="14" t="s">
-        <v>262</v>
+        <v>125</v>
       </c>
       <c r="H50" s="14" t="s">
         <v>818</v>
@@ -22355,25 +22672,25 @@
         <v>819</v>
       </c>
       <c r="B51" s="14" t="s">
-        <v>380</v>
+        <v>86</v>
       </c>
       <c r="C51" s="14" t="s">
+        <v>806</v>
+      </c>
+      <c r="D51" s="14" t="s">
         <v>820</v>
       </c>
-      <c r="D51" s="14" t="s">
+      <c r="E51" s="14" t="s">
         <v>821</v>
       </c>
-      <c r="E51" s="14" t="s">
+      <c r="F51" s="14" t="s">
         <v>822</v>
       </c>
-      <c r="F51" s="14" t="s">
+      <c r="G51" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="H51" s="14" t="s">
         <v>823</v>
-      </c>
-      <c r="G51" s="14" t="s">
-        <v>383</v>
-      </c>
-      <c r="H51" s="14" t="s">
-        <v>824</v>
       </c>
       <c r="I51" s="14" t="s">
         <v>25</v>
@@ -22381,16 +22698,16 @@
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="14" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B52" s="14" t="s">
         <v>380</v>
       </c>
       <c r="C52" s="14" t="s">
+        <v>825</v>
+      </c>
+      <c r="D52" s="14" t="s">
         <v>826</v>
-      </c>
-      <c r="D52" s="14" t="s">
-        <v>400</v>
       </c>
       <c r="E52" s="14" t="s">
         <v>827</v>
@@ -22399,7 +22716,7 @@
         <v>828</v>
       </c>
       <c r="G52" s="14" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="H52" s="14" t="s">
         <v>829</v>
@@ -22408,44 +22725,44 @@
         <v>25</v>
       </c>
     </row>
-    <row r="53" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
         <v>830</v>
       </c>
       <c r="B53" s="14" t="s">
+        <v>380</v>
+      </c>
+      <c r="C53" s="14" t="s">
         <v>831</v>
       </c>
-      <c r="C53" s="14" t="s">
+      <c r="D53" s="14" t="s">
+        <v>400</v>
+      </c>
+      <c r="E53" s="14" t="s">
         <v>832</v>
       </c>
-      <c r="D53" s="14" t="s">
+      <c r="F53" s="14" t="s">
         <v>833</v>
       </c>
-      <c r="E53" s="14" t="s">
+      <c r="G53" s="14" t="s">
+        <v>395</v>
+      </c>
+      <c r="H53" s="14" t="s">
         <v>834</v>
       </c>
-      <c r="F53" s="14" t="s">
+      <c r="I53" s="14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="54" ht="64" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="14" t="s">
         <v>835</v>
       </c>
-      <c r="G53" s="14" t="s">
-        <v>473</v>
-      </c>
-      <c r="H53" s="14" t="s">
+      <c r="B54" s="14" t="s">
         <v>836</v>
       </c>
-      <c r="I53" s="14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="54" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="14" t="s">
+      <c r="C54" s="14" t="s">
         <v>837</v>
-      </c>
-      <c r="B54" s="14" t="s">
-        <v>831</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>832</v>
       </c>
       <c r="D54" s="14" t="s">
         <v>838</v>
@@ -22457,7 +22774,7 @@
         <v>840</v>
       </c>
       <c r="G54" s="14" t="s">
-        <v>482</v>
+        <v>473</v>
       </c>
       <c r="H54" s="14" t="s">
         <v>841</v>
@@ -22466,76 +22783,76 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" ht="80" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
         <v>842</v>
       </c>
       <c r="B55" s="14" t="s">
-        <v>831</v>
+        <v>836</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>832</v>
+        <v>837</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>493</v>
+        <v>843</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="G55" s="14" t="s">
-        <v>488</v>
+        <v>482</v>
       </c>
       <c r="H55" s="14" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="I55" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="56" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="B56" s="14" t="s">
-        <v>61</v>
+        <v>836</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>847</v>
+        <v>837</v>
       </c>
       <c r="D56" s="14" t="s">
+        <v>493</v>
+      </c>
+      <c r="E56" s="14" t="s">
         <v>848</v>
       </c>
-      <c r="E56" s="14" t="s">
+      <c r="F56" s="14" t="s">
         <v>849</v>
       </c>
-      <c r="F56" s="14" t="s">
+      <c r="G56" s="14" t="s">
+        <v>488</v>
+      </c>
+      <c r="H56" s="14" t="s">
         <v>850</v>
-      </c>
-      <c r="G56" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="H56" s="14" t="s">
-        <v>851</v>
       </c>
       <c r="I56" s="14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="57" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" ht="96" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
+        <v>851</v>
+      </c>
+      <c r="B57" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C57" s="14" t="s">
         <v>852</v>
       </c>
-      <c r="B57" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="C57" s="14" t="s">
+      <c r="D57" s="14" t="s">
         <v>853</v>
-      </c>
-      <c r="D57" s="14" t="s">
-        <v>87</v>
       </c>
       <c r="E57" s="14" t="s">
         <v>854</v>
@@ -22544,7 +22861,7 @@
         <v>855</v>
       </c>
       <c r="G57" s="14" t="s">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="H57" s="14" t="s">
         <v>856</v>
@@ -22553,7 +22870,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="58" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" ht="128" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
         <v>857</v>
       </c>
@@ -22561,10 +22878,10 @@
         <v>86</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>801</v>
+        <v>858</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>858</v>
+        <v>87</v>
       </c>
       <c r="E58" s="14" t="s">
         <v>859</v>
@@ -22573,7 +22890,7 @@
         <v>860</v>
       </c>
       <c r="G58" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H58" s="14" t="s">
         <v>861</v>
@@ -22582,7 +22899,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="59" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" ht="144" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
         <v>862</v>
       </c>
@@ -22590,7 +22907,7 @@
         <v>86</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>801</v>
+        <v>806</v>
       </c>
       <c r="D59" s="14" t="s">
         <v>863</v>
@@ -22602,7 +22919,7 @@
         <v>865</v>
       </c>
       <c r="G59" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="H59" s="14" t="s">
         <v>866</v>
@@ -22611,9 +22928,38 @@
         <v>13</v>
       </c>
     </row>
+    <row r="60" ht="409.6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A60" s="14" t="s">
+        <v>867</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C60" s="14" t="s">
+        <v>806</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>868</v>
+      </c>
+      <c r="E60" s="14" t="s">
+        <v>869</v>
+      </c>
+      <c r="F60" s="14" t="s">
+        <v>870</v>
+      </c>
+      <c r="G60" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="H60" s="14" t="s">
+        <v>871</v>
+      </c>
+      <c r="I60" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I59"/>
-  <conditionalFormatting sqref="I2:I59">
+  <autoFilter ref="A1:I60"/>
+  <conditionalFormatting sqref="I2:I60">
     <cfRule type="expression" dxfId="15" priority="1">
       <formula>$I2="Done"</formula>
     </cfRule>
@@ -22648,7 +22994,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -22660,19 +23006,19 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>867</v>
+        <v>872</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>868</v>
+        <v>873</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>870</v>
+        <v>875</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>871</v>
+        <v>876</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23015,9 +23361,9 @@
         <v>679</v>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" ht="70" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="14" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="B22" s="14" t="s">
         <v>685</v>
@@ -23026,7 +23372,7 @@
         <v>686</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>175</v>
+        <v>495</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>684</v>
@@ -23054,13 +23400,13 @@
         <v>67</v>
       </c>
       <c r="B24" s="14" t="s">
+        <v>695</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>696</v>
       </c>
-      <c r="C24" s="14" t="s">
-        <v>697</v>
-      </c>
       <c r="D24" s="14" t="s">
-        <v>699</v>
+        <v>175</v>
       </c>
       <c r="E24" s="14" t="s">
         <v>694</v>
@@ -23071,16 +23417,16 @@
         <v>67</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>174</v>
+        <v>701</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>702</v>
       </c>
       <c r="D25" s="14" t="s">
+        <v>704</v>
+      </c>
+      <c r="E25" s="14" t="s">
         <v>699</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>701</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23088,16 +23434,16 @@
         <v>67</v>
       </c>
       <c r="B26" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>707</v>
       </c>
-      <c r="C26" s="14" t="s">
-        <v>708</v>
-      </c>
       <c r="D26" s="14" t="s">
-        <v>215</v>
+        <v>704</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23111,10 +23457,10 @@
         <v>713</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>715</v>
+        <v>215</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23122,16 +23468,16 @@
         <v>67</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>236</v>
+        <v>717</v>
       </c>
       <c r="C28" s="14" t="s">
         <v>718</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23139,16 +23485,16 @@
         <v>67</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C29" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>720</v>
+      </c>
+      <c r="E29" s="14" t="s">
         <v>722</v>
-      </c>
-      <c r="D29" s="14" t="s">
-        <v>237</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23156,16 +23502,16 @@
         <v>67</v>
       </c>
       <c r="B30" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>727</v>
       </c>
-      <c r="C30" s="14" t="s">
-        <v>728</v>
-      </c>
       <c r="D30" s="14" t="s">
-        <v>268</v>
+        <v>237</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23182,7 +23528,7 @@
         <v>268</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23190,13 +23536,13 @@
         <v>67</v>
       </c>
       <c r="B32" s="14" t="s">
+        <v>737</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>738</v>
       </c>
-      <c r="C32" s="14" t="s">
-        <v>739</v>
-      </c>
       <c r="D32" s="14" t="s">
-        <v>293</v>
+        <v>268</v>
       </c>
       <c r="E32" s="14" t="s">
         <v>736</v>
@@ -23207,30 +23553,30 @@
         <v>67</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>321</v>
+        <v>743</v>
       </c>
       <c r="C33" s="14" t="s">
         <v>744</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>316</v>
+        <v>293</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>748</v>
+        <v>321</v>
       </c>
       <c r="C34" s="14" t="s">
         <v>749</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>99</v>
+        <v>316</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>747</v>
@@ -23258,16 +23604,16 @@
         <v>61</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>628</v>
+        <v>758</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>629</v>
+        <v>759</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>145</v>
+        <v>99</v>
       </c>
       <c r="E36" s="14" t="s">
-        <v>626</v>
+        <v>757</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23275,16 +23621,16 @@
         <v>61</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="D37" s="14" t="s">
         <v>145</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>632</v>
+        <v>626</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23292,16 +23638,16 @@
         <v>61</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>759</v>
+        <v>633</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>760</v>
+        <v>634</v>
       </c>
       <c r="D38" s="14" t="s">
-        <v>189</v>
+        <v>145</v>
       </c>
       <c r="E38" s="14" t="s">
-        <v>757</v>
+        <v>632</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23315,10 +23661,10 @@
         <v>765</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>767</v>
+        <v>189</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23326,16 +23672,16 @@
         <v>61</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>769</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>770</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>245</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>772</v>
       </c>
       <c r="E40" s="14" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23346,10 +23692,10 @@
         <v>775</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>250</v>
+        <v>777</v>
       </c>
       <c r="E41" s="14" t="s">
         <v>774</v>
@@ -23360,16 +23706,16 @@
         <v>61</v>
       </c>
       <c r="B42" s="14" t="s">
+        <v>780</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="D42" s="14" t="s">
+        <v>250</v>
+      </c>
+      <c r="E42" s="14" t="s">
         <v>779</v>
-      </c>
-      <c r="C42" s="14" t="s">
-        <v>257</v>
-      </c>
-      <c r="D42" s="14" t="s">
-        <v>256</v>
-      </c>
-      <c r="E42" s="14" t="s">
-        <v>778</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23377,16 +23723,16 @@
         <v>61</v>
       </c>
       <c r="B43" s="14" t="s">
+        <v>784</v>
+      </c>
+      <c r="C43" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="D43" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="E43" s="14" t="s">
         <v>783</v>
-      </c>
-      <c r="C43" s="14" t="s">
-        <v>784</v>
-      </c>
-      <c r="D43" s="14" t="s">
-        <v>298</v>
-      </c>
-      <c r="E43" s="14" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23394,13 +23740,13 @@
         <v>61</v>
       </c>
       <c r="B44" s="14" t="s">
-        <v>285</v>
+        <v>788</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>787</v>
@@ -23411,16 +23757,16 @@
         <v>61</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>309</v>
+        <v>285</v>
       </c>
       <c r="C45" s="14" t="s">
         <v>793</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>304</v>
+        <v>280</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23428,13 +23774,13 @@
         <v>61</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>332</v>
+        <v>309</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>327</v>
+        <v>304</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>796</v>
@@ -23442,19 +23788,19 @@
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>86</v>
+        <v>61</v>
       </c>
       <c r="B47" s="14" t="s">
+        <v>332</v>
+      </c>
+      <c r="C47" s="14" t="s">
         <v>802</v>
       </c>
-      <c r="C47" s="14" t="s">
-        <v>803</v>
-      </c>
       <c r="D47" s="14" t="s">
-        <v>104</v>
+        <v>327</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23462,16 +23808,16 @@
         <v>86</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>209</v>
+        <v>807</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>204</v>
+        <v>104</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23479,16 +23825,16 @@
         <v>86</v>
       </c>
       <c r="B49" s="14" t="s">
-        <v>132</v>
+        <v>209</v>
       </c>
       <c r="C49" s="14" t="s">
+        <v>812</v>
+      </c>
+      <c r="D49" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="E49" s="14" t="s">
         <v>811</v>
-      </c>
-      <c r="D49" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="E49" s="14" t="s">
-        <v>810</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23496,30 +23842,30 @@
         <v>86</v>
       </c>
       <c r="B50" s="14" t="s">
-        <v>815</v>
+        <v>132</v>
       </c>
       <c r="C50" s="14" t="s">
         <v>816</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>262</v>
+        <v>125</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>380</v>
+        <v>86</v>
       </c>
       <c r="B51" s="14" t="s">
+        <v>820</v>
+      </c>
+      <c r="C51" s="14" t="s">
         <v>821</v>
       </c>
-      <c r="C51" s="14" t="s">
-        <v>822</v>
-      </c>
       <c r="D51" s="14" t="s">
-        <v>383</v>
+        <v>262</v>
       </c>
       <c r="E51" s="14" t="s">
         <v>819</v>
@@ -23530,33 +23876,33 @@
         <v>380</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>400</v>
+        <v>826</v>
       </c>
       <c r="C52" s="14" t="s">
         <v>827</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>86</v>
+        <v>380</v>
       </c>
       <c r="B53" s="14" t="s">
-        <v>87</v>
+        <v>400</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>854</v>
+        <v>832</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>81</v>
+        <v>395</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>852</v>
+        <v>830</v>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -23564,13 +23910,13 @@
         <v>86</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>858</v>
+        <v>87</v>
       </c>
       <c r="C54" s="14" t="s">
         <v>859</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E54" s="14" t="s">
         <v>857</v>
@@ -23587,14 +23933,31 @@
         <v>864</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>110</v>
+        <v>88</v>
       </c>
       <c r="E55" s="14" t="s">
         <v>862</v>
       </c>
     </row>
+    <row r="56" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B56" s="14" t="s">
+        <v>868</v>
+      </c>
+      <c r="C56" s="14" t="s">
+        <v>869</v>
+      </c>
+      <c r="D56" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="E56" s="14" t="s">
+        <v>867</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E55"/>
+  <autoFilter ref="A1:E56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -23619,114 +23982,114 @@
   <sheetData>
     <row r="1" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>872</v>
+        <v>877</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>873</v>
+        <v>878</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>869</v>
+        <v>874</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>874</v>
+        <v>879</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>875</v>
+        <v>880</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>876</v>
+        <v>881</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>877</v>
+        <v>882</v>
       </c>
     </row>
     <row r="2" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>879</v>
+        <v>884</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>880</v>
+        <v>885</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>881</v>
+        <v>886</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>882</v>
+        <v>887</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>884</v>
+        <v>889</v>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>885</v>
+        <v>890</v>
       </c>
       <c r="C3" s="14" t="s">
+        <v>891</v>
+      </c>
+      <c r="D3" s="14" t="s">
         <v>886</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>881</v>
-      </c>
       <c r="E3" s="14" t="s">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="F3" s="14" t="s">
-        <v>883</v>
+        <v>888</v>
       </c>
       <c r="G3" s="14" t="s">
-        <v>888</v>
+        <v>893</v>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>890</v>
+        <v>895</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>891</v>
+        <v>896</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>892</v>
+        <v>897</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>893</v>
+        <v>898</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>894</v>
+        <v>899</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>895</v>
+        <v>900</v>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>896</v>
+        <v>901</v>
       </c>
       <c r="C5" s="14" t="s">
+        <v>902</v>
+      </c>
+      <c r="D5" s="14" t="s">
         <v>897</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>892</v>
-      </c>
       <c r="E5" s="14" t="s">
-        <v>898</v>
+        <v>903</v>
       </c>
       <c r="F5" s="14" t="s">
-        <v>899</v>
+        <v>904</v>
       </c>
       <c r="G5" s="14" t="s">
         <v>164</v>
@@ -23734,22 +24097,22 @@
     </row>
     <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>900</v>
+        <v>905</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>901</v>
+        <v>906</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>902</v>
+        <v>907</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>903</v>
+        <v>908</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>904</v>
+        <v>909</v>
       </c>
       <c r="G6" s="14" t="s">
         <v>170</v>
@@ -23757,186 +24120,186 @@
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>906</v>
+        <v>911</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>907</v>
+        <v>912</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>908</v>
+        <v>913</v>
       </c>
       <c r="F7" s="14" t="s">
-        <v>909</v>
+        <v>914</v>
       </c>
       <c r="G7" s="14" t="s">
-        <v>910</v>
+        <v>915</v>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>905</v>
+        <v>910</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>911</v>
+        <v>916</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>912</v>
+        <v>917</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>913</v>
+        <v>918</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>914</v>
+        <v>919</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>915</v>
+        <v>920</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>916</v>
+        <v>921</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>917</v>
+        <v>922</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>919</v>
+        <v>924</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>920</v>
+        <v>925</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>921</v>
+        <v>926</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>923</v>
+        <v>928</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>924</v>
+        <v>929</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>925</v>
+        <v>930</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>926</v>
+        <v>931</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>927</v>
+        <v>932</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>928</v>
+        <v>933</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>929</v>
+        <v>934</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>930</v>
+        <v>935</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>932</v>
+        <v>937</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>933</v>
+        <v>938</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>934</v>
+        <v>939</v>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>878</v>
+        <v>883</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>935</v>
+        <v>940</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>936</v>
+        <v>941</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>918</v>
+        <v>923</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>937</v>
+        <v>942</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>938</v>
+        <v>943</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>939</v>
+        <v>944</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>889</v>
+        <v>894</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>940</v>
+        <v>945</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>941</v>
+        <v>946</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>942</v>
+        <v>947</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>943</v>
+        <v>948</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>944</v>
+        <v>949</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>922</v>
+        <v>927</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>945</v>
+        <v>950</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>946</v>
+        <v>951</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>931</v>
+        <v>936</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>947</v>
+        <v>952</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>948</v>
+        <v>953</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>944</v>
+        <v>949</v>
       </c>
     </row>
   </sheetData>

</xml_diff>